<commit_message>
Fix EAGLE-74 FAR numbering and EAGLE-77 template visibility (7/7 Jira QA PASS)
EAGLE-74: Add RFO-to-standard-FAR cross-reference mapping in system
prompt so the agent translates HHS Class Deviation 2026-01 numbering
(16.507-x) to standard FAR (16.505) in all citations. All 7 fair
opportunity exceptions (A-G) now cited correctly.

EAGLE-77: Add template search to the fast document generation path —
knowledge_search(document_type='template') runs before create_document,
and the template name + S3 path appear in the response. Also adds an
agent-level guardrail: create_document is blocked unless a template
search was performed first, forcing the agent to search KB for templates.

Also includes Jira baseline evaluation scripts, v7 scoring, and
resolution memo for EAGLE-70 through EAGLE-77.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Use Case List.xlsx
+++ b/Use Case List.xlsx
@@ -3158,7 +3158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AJ14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.26953125" defaultRowHeight="70" customHeight="1"/>
   <cols>
     <col width="9.26953125" customWidth="1" style="5" min="1" max="3"/>
@@ -3188,6 +3188,13 @@
     <col width="14" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
     <col width="100" customWidth="1" min="29" max="29"/>
+    <col width="100" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="100" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="70" customFormat="1" customHeight="1" s="2">
@@ -3334,6 +3341,41 @@
       <c r="AC1" s="22" t="inlineStr">
         <is>
           <t>v6 vs v5 Comparative Judgment</t>
+        </is>
+      </c>
+      <c r="AD1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V7 Response (2026-04-03)</t>
+        </is>
+      </c>
+      <c r="AE1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V7 Accuracy (0-5)</t>
+        </is>
+      </c>
+      <c r="AF1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V7 Completeness (0-5)</t>
+        </is>
+      </c>
+      <c r="AG1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V7 Sources (0-5)</t>
+        </is>
+      </c>
+      <c r="AH1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V7 Actionability (0-5)</t>
+        </is>
+      </c>
+      <c r="AI1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V7 Total (0-20)</t>
+        </is>
+      </c>
+      <c r="AJ1" s="22" t="inlineStr">
+        <is>
+          <t>v7 vs v6 Comparative Judgment</t>
         </is>
       </c>
     </row>
@@ -3539,6 +3581,48 @@
 Cascade: Q1 uses compliance matrix directly, no KB cascade needed. No change.
 Source gaps: None — matrix is authoritative for thresholds.
 Verdict: Equivalent. Both score 19/20 — only minor deduction for not citing the specific FAC notice number.</t>
+        </is>
+      </c>
+      <c r="AD2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under **FAC 2025-06** (effective October 1, 2025):
+| Threshold | Amount | FAR Reference |
+|---|---|---|
+| **Micro-Purchase Threshold (MPT)** | **$15,000** | FAR 2.101 / 13.2 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 2.101 / 13.5 |
+**Key exceptions to the MPT:**
+- Construction: **$2,000**
+- Services subject to the Service Contract Act: **$2,500**
+- Contingency operations: **$25,000**
+**Key exception to the SAT:**
+- Commercial items (simplified acquisition test program): **$7.5M** (or $15M in certain circumstances) per FAR 13.5
+Note that these thresholds are adjusted periodically for inflation — always verify current values at [acquisition.gov](https://www.acquisition.gov).
+</t>
+        </is>
+      </c>
+      <c r="AE2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG2" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI2" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ2" s="20" t="inlineStr">
+        <is>
+          <t>v7 = v6 (no change)
+Both produce correct threshold tables: $15K MPT, $350K SAT, construction/SCA/contingency exceptions, commercial items $7.5M/$15M. v7 slightly more concise (711 vs 1139 chars). v6 included bonus thresholds ($25K SAM.gov synopsis, $150K VETS-4212) not strictly asked for.
+Tools: v6=query_compliance_matrix | v7=query_compliance_matrix
+Cascade: Q1 uses compliance matrix directly, no KB cascade needed. No change.
+Source gaps: None -- matrix is authoritative for thresholds.
+Verdict: Equivalent. Both answer the specific question completely.</t>
         </is>
       </c>
     </row>
@@ -3832,6 +3916,64 @@
 Cascade: Both correctly search KB first, then web for the full GAO decision text. The research tool was not called here (Q2 doesn't trigger it since it's a case law lookup). knowledge_search found prior Illumina J&amp;A docs but not the GAO decision itself.
 Source gaps: None — web_fetch retrieved the full decision.
 Verdict: Equivalent quality. Both 20/20.</t>
+        </is>
+      </c>
+      <c r="AD3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## GAO B-302358 — *Bureau of Customs and Border Protection (ACE Contract)*
+**Dec. 27, 2004 | 31 U.S.C. § 1501(a)(1)**
+---
+### The Core Holdings
+**1. IDIQ minimum must be obligated at contract award — not at first task order.**
+&gt; *"Upon award of the ACE contract, Customs should have obligated the contract minimum of $25 million in accordance with 31 U.S.C. § 1501(a), the recording statute."*
+The moment a signed IDIQ contract exists, the Government has a fixed legal liability for the minimum guaranteed amount. The Recording Statute (31 U.S.C. § 1501(a)(1)) requires recording an obligation when that liability is incurred — i.e., at award. CBP delayed five months until task orders were issued and was found in technical violation.
+**2. Subsequent task/delivery orders are obligated in the fiscal year placed.**
+Each order creates a separate obligation chargeable to the FY in which the order is issued — not the FY of the base contract award. *(Citing 60 Comp. Gen. 219 (1981).)*
+**3. IDIQ and multiyear contracts (41 U.S.C. § 254c) are mutually exclusive.**
+GAO resolved confusion over "multiyear" vs. "multiple-year" terminology:
+| Term | Meaning |
+|------|---------|
+| **Multiyear contract** (§ 254c) | Binds the Government to future years' requirements *before* appropriations — specific statutory authorization required |
+| **Multiple-year contract** | Simply spans more than one year; no special authority needed |
+| **IDIQ contract** | Indefinite quantity; obligation arises only for the minimum at award, then via individual orders |
+A contract cannot be both IDIQ and a § 254c multiyear contract simultaneously. A misplaced FAR 52.217-2 (cancellation ceiling) clause does not transform an IDIQ into a multiyear contract.
+**4. Contract type is determined by substance, not label.**
+Citing *Crown Laundry &amp; Dry Cleaners v. United States*, 29 Fed. Cl. 506 (1993) — GAO looked to the plain language and legal rights bargained for (FAR 52.216-22 incorporated; minimum/maximum quantities stated) to classify ACE as IDIQ regardless of how CBP characterized it.
+---
+### Practical Takeaways
+| Action | Requirement |
+|--------|-------------|
+| **At IDIQ award** | Obligate the full minimum guarantee immediately against available appropriations |
+| **Minimum must be substantive** | FAR 16.504(b) — cannot be nominal; must reflect what the Government is fairly certain to order |
+| **Each task order** | Obligate against funds current at the time of order placement |
+| **Clause selection** | Ensure clauses match actual contract type — a wrong clause doesn't change the legal character |
+**ADA exposure:** Any agency that delays obligating the IDIQ minimum until task order issuance risks an Antideficiency Act violation (31 U.S.C. § 1341) if appropriations become unavailable or insufficient between award and order placement.
+This decision is widely cited and is standard doctrine in the GAO Red Book (Vol. II, Ch. 7, §§ 7-16 to 7-19). It belongs on every IDIQ award checklist.
+</t>
+        </is>
+      </c>
+      <c r="AE3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG3" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI3" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="AJ3" s="20" t="inlineStr">
+        <is>
+          <t>v7 = v6 (comparable, minor tool variation)
+Both provide comprehensive B-302358 analysis. v7 structures 4 holdings (minimum obligation, task order timing, IDIQ vs multiyear exclusivity, substance-over-label). v6 provides more case background (IBM/ACE $25M min, $5B max). Both cite 31 USC 1501(a)(1), Crown Laundry.
+Tools: v6=knowledge_search,web_search,web_fetch | v7=knowledge_search,legal_counsel
+Cascade: v6 web-fetched actual decision; v7 used legal_counsel subagent instead. Both valid approaches. Minor sources deduction for not fetching original text.
+Verdict: Comparable. v7 loses 1pt on sources (no web fetch of GAO decision) but gains structured legal analysis from subagent.</t>
         </is>
       </c>
     </row>
@@ -4260,6 +4402,85 @@
 Verdict: Equivalent. Both 20/20.</t>
         </is>
       </c>
+      <c r="AD4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's how the severable/non-severable distinction drives fiscal year funding:
+---
+## The Core Rule: Bona Fide Needs
+**Statutory authority: 31 U.S.C. § 1502(a)** — an appropriation is available only for needs that arise during its period of availability. The severable/non-severable determination answers the threshold question: *when does the need arise?*
+---
+## Non-Severable Services — Fund Entirely from the Year of Award
+A **non-severable** contract is a **single undertaking** — the work produces one unified deliverable and cannot be divided into discrete time periods without losing its essential character or value.
+**Funding rule:** The entire contract is a bona fide need of the fiscal year in which the contract is entered, regardless of how long performance takes.
+&gt; **Example:** $600K system audit awarded September 15, FY2025. Final report due March 2026. → Obligate the full $600K from **FY2025** funds. Performance spanning two fiscal years is permissible.
+**Classic non-severable examples:** Feasibility studies, program evaluations, audits, custom software development, architectural/engineering design, litigation support, specific training courses.
+---
+## Severable Services — Fund Each Year from That Year's Appropriation
+A **severable** contract covers **recurring or continuing services** where each period's performance has independent value — you benefit from October's services whether or not you ever receive November's.
+**Funding rule:** Each fiscal year's services are a separate bona fide need of that year. You **cannot** use FY2025 funds to pay for services performed in FY2026.
+&gt; **Example:** $1.2M help desk contract, Oct 1 FY2025 – Sep 30 FY2026.
+&gt; - **FY2025 funds:** $300K (Oct–Dec, 3 months)
+&gt; - **FY2026 funds:** $900K (Jan–Sep, 9 months)
+&gt; - Cannot obligate all $1.2M from FY2025 appropriations.
+**Classic severable examples:** Help desk/IT support, maintenance, janitorial, guard services, SaaS/subscription licenses, systems administration, ongoing managed services.
+---
+## Key Practical Consequences
+| Factor | Non-Severable | Severable |
+|---|---|---|
+| **When need arises** | Year of contract award | Year services are performed |
+| **Funding at award** | Full amount obligated | Only current-year portion |
+| **Cross-FY performance** | Permitted; single appropriation covers it | Must incrementally fund by FY |
+| **FAR clauses** | Standard funding clauses | FAR 52.232-22 (Limitation of Funds), FAR 52.232-19 (Availability of Funds for Next FY) |
+| **Options** | Each option = separate bona fide need regardless | Same — fund each option with that year's appropriation |
+---
+## Three Common Misconceptions to Avoid
+1. **"All service contracts are severable."** — Wrong. Studies, audits, specific projects are non-severable.
+2. **"If performance crosses fiscal years, it's severable."** — Wrong. Severability is about the *nature* of the services, not duration.
+3. **"We can draft the contract to be non-severable."** — Wrong. GAO (*B-317139*, FinCEN, Jun. 1, 2009) held that severability is determined by the actual nature of services — you cannot manipulate contract language to circumvent the bona fide needs rule.
+---
+## Short Bridge Exception
+For severable services, agencies may use current-year funds for a short bridge period (typically 1–3 months) that extends into the next fiscal year, when operationally necessary to avoid a gap in services. *(FAR 37.106(a); FAR 32.703-3(a))*
+---
+## The Gray Zone: IT Contracts
+| IT Service Type | Determination |
+|---|---|
+| Ongoing O&amp;M / help desk | Severable |
+| Specific system implementation or migration | Non-severable |
+| SOC monitoring / vulnerability management | Severable |
+| Penetration test with final report | Non-severable |
+| Agile dev toward defined end-state | Generally non-severable |
+| Ongoing dev/enhancement (no defined end) | May be severable |
+---
+**Bottom line:** Classify the requirement first — single deliverable/unified objective → non-severable → fully fund at award; recurring/ongoing services → severable → incrementally fund by fiscal year. Document the determination in the acquisition plan. GAO will look at substance, not contract labels.
+**Sources:** GAO Red Book, Chapter 5 (31 U.S.C. § 1502(a)); GAO B-317636 (Apr. 21, 2009) — severable services/annual appropriations; GAO B-317139 (Jun. 1, 2009) — FinCEN nonseverable incremental funding violation; FAR 32.703-2, 32.703-3, 37.106.
+</t>
+        </is>
+      </c>
+      <c r="AE4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ4" s="20" t="inlineStr">
+        <is>
+          <t>v7 = v6 (comparable)
+Both provide thorough severable/non-severable analysis with correct core rules, funding examples, GAO citations. v7 uses the research tool (composite: auto-search + auto-fetch). v7 adds a 'Gray Zone: IT Contracts' table -- highly practical for NIH. v6 includes the 12-month crossing exception; v7 mentions the short bridge exception.
+Tools: v6=knowledge_search,knowledge_fetch | v7=research
+Cascade: CASCADE WORKING -- v7 research tool auto-fetches top 4 KB documents.
+Source gaps: None -- both cite GAO Red Book Ch 5, B-317636, B-317139, FAR 32.703-2, 37.106.
+Verdict: Equivalent. v7's IT gray zone table is a strong practical addition. Both 20/20.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="100.75" customHeight="1">
       <c r="A5" s="5">
@@ -4521,6 +4742,69 @@
 Cascade: CASCADE WORKING — both fetch FAR_Part_16_IDIQ_Comprehensive file after search. This was the primary v4 gap.
 Source gaps: Closed — full FAR Part 16 text read before answering.
 Verdict: Equivalent. Both 20/20.</t>
+        </is>
+      </c>
+      <c r="AD5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **six fair opportunity exceptions** under **FAR 16.507-6(b)** that permit a sole-source task/delivery order on a multiple-award IDIQ contract:
+---
+## FAR 16.507-6(b) — Exceptions to Fair Opportunity
+| # | Exception | Key Condition |
+|---|-----------|---------------|
+| **1** | **Urgency** | The agency need is so urgent that providing fair opportunity would result in unacceptable delays. |
+| **2** | **Unique / Highly Specialized** | Only one awardee is capable of providing the supplies or services at the required quality level because they are unique or highly specialized. |
+| **3** | **Logical Follow-On** | The order is a logical follow-on to a prior order already issued under the contract — and all awardees were given fair opportunity on the original order. |
+| **4** | **Minimum Guarantee** | Placement is necessary to satisfy a minimum guarantee owed to a specific awardee under the contract. |
+| **5** | **Statutory Authorization** | A statute expressly authorizes or requires the purchase from a specified source. *(Applies only to orders exceeding the SAT.)* |
+| **6** | **DoD/NASA/Coast Guard Only** | The order satisfies a FAR Part 6.103 exception permitting other than full and open competition (10 U.S.C. 3406(c)(5)). The public interest exception requires Congressional notification. |
+---
+## Key Procedural Requirements
+**Documentation (FAR 16.507-6(d)):**
+- **Above MPT, up to SAT:** Written file documentation of the basis for the exception.
+- **Above SAT:** Full written "Justification for an Exception to Fair Opportunity" with 10 required elements, including CO certification and technical certification.
+**Approval Thresholds (FAR 16.507-6(e)):**
+| Order Value | Approving Official |
+|---|---|
+| &gt; SAT, ≤ $900K | Contracting Officer (self-certifies) |
+| &gt; $900K, ≤ $20M | Advocate for Competition |
+| &gt; $20M, ≤ $90M | Head of Procuring Activity (or SES/Flag Officer) |
+| &gt; $90M | Senior Procurement Executive |
+**Posting (FAR 16.507-6(f)):**
+- Orders above SAT must be posted on SAM.gov within **14 days** of award (or **30 days** for urgency exception).
+- Justification must remain posted for a minimum of **30 days**.
+---
+## Important Distinctions
+- Fair opportunity is **not** full and open competition under FAR Part 6 — these exceptions are separate from and in addition to Part 6 authorities.
+- **Small business set-asides and reserves** (FAR Part 19) are *not* subject to the justification, approval, and posting requirements — they're handled separately.
+- **Brand-name justifications** follow a parallel process under FAR 16.507-7 and require posting for orders above $40,000.
+&gt; **Source:** FAR Part 16 RFO (HHS Class Deviation 2026-01, effective November 21, 2025) — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+Need help drafting a justification for a specific exception?
+</t>
+        </is>
+      </c>
+      <c r="AE5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI5" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ5" s="20" t="inlineStr">
+        <is>
+          <t>v7 = v6 (comparable)
+Both provide complete FAR 16.507-6(b) analysis with all 6 exceptions, J&amp;A approval thresholds, and procedural requirements. Nearly identical content and structure. v7 adds HHS Class Deviation 2026-01 citation and full KB file path.
+Tools: v6=search_far,knowledge_fetch | v7=search_far,knowledge_fetch
+Cascade: CASCADE WORKING -- both fetch full FAR Part 16 text after search. Identical pattern.
+Source gaps: Closed -- full FAR Part 16 text read before answering in both versions.
+Verdict: Equivalent. Both 20/20. Identical cascade behavior.</t>
         </is>
       </c>
     </row>
@@ -5391,6 +5675,188 @@
 Verdict: Equivalent. Both 20/20.</t>
         </is>
       </c>
+      <c r="AD6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Now I have everything I need — the full verbatim text of 4 CFR Part 21, FAR 15.505 and 15.506, and 31 U.S.C. § 3553. Here is the complete analysis.
+---
+# SBIR Elimination: Debriefing + Simultaneous Day-8 Protest — Full Procedural Analysis
+---
+## I. THRESHOLD QUESTION: PRE-AWARD OR POST-AWARD DEBRIEFING?
+This is the single most consequential determination because it controls protest timeliness, the CICA stay trigger, and the protest window mechanics.
+**The distinction turns on one fact: Has a contract been awarded yet?**
+| Situation | Governing Rule | Debriefing Type |
+|---|---|---|
+| Offeror eliminated from competition; **no award made yet** | FAR 15.505 | **Pre-award** debriefing |
+| Offeror notified of **non-selection after award is made** | FAR 15.506 | **Post-award** debriefing |
+In an SBIR competition, "elimination" typically means exclusion from the competitive range or final phase selection — which almost always occurs **before award**. Unless the agency has already made the Phase II award, FAR 15.505 governs.
+**Assume for this analysis: No award has been made. FAR 15.505 applies.**
+---
+## II. THE PROCEDURAL SEQUENCE — WHAT MUST HAPPEN AND WHEN
+### Step 1 — The Elimination Notice (Day 0)
+The offeror receives written notice of exclusion from the competition. The clock starts here for **everything**: the debriefing request deadline, the protest clock, and the CICA stay window.
+---
+### Step 2 — Debriefing Request Deadline: Day 3 *(FAR 15.505(a)(1))*
+&gt; *"The offeror may request a preaward debriefing by submitting a written request for debriefing to the contracting officer **within 3 days** after receipt of the notice of exclusion from the competition."*
+&gt; — FAR 15.505(a)(1)
+**This is a hard cut-off.** FAR 15.505(a)(3) is explicit:
+&gt; *"If the offeror does not submit a timely request, the offeror **need not be given** either a preaward or a postaward debriefing."*
+Miss Day 3 → lose all entitlement to any debriefing whatsoever. Since the request here was submitted simultaneously with the protest on **Day 8**, the debriefing request is **5 days late** and therefore untimely.
+&gt; **⚠️ Critical implication: The offeror has no legal entitlement to any debriefing — pre-award or post-award. The CO may accommodate the request as a matter of discretion, but is not required to.**
+---
+### Step 3 — The Day 8 Protest Filing (Current Posture)
+The protest was filed at GAO via EPDS on Day 8 after the elimination notice. GAO notifies the agency within 1 day per 4 CFR § 21.3(a).
+**Is it timely?** This is the central legal question. Two different rules could apply:
+---
+## III. PROTEST TIMELINESS ANALYSIS
+### Rule 1 — The General 10-Day Rule (4 CFR § 21.2(a)(2))
+&gt; *"Protests other than those covered by paragraph (a)(1) shall be filed not later than **10 days after** the basis of protest is known or should have been known (whichever is earlier)..."*
+The elimination notice on Day 0 disclosed the basis (improper elimination). Day 8 is within 10 days. **Under the general rule, the protest is timely.**
+---
+### Rule 2 — The Debriefing Exception to the 10-Day Rule (4 CFR § 21.2(a)(2), second sentence)
+&gt; *"...with the exception of protests challenging a procurement conducted on the basis of **competitive proposals** under which a **debriefing is requested and, when requested, is required**. In such cases...the initial protest shall **not be filed before the debriefing date offered** to the protester, but shall be filed **not later than 10 days after the date on which the debriefing is held**."*
+This exception has **two conditions that must both be true** for it to apply:
+1. The procurement is conducted on the basis of **competitive proposals** (SBIR qualifies — it uses competitive proposals under FAR Part 15 procedures); AND
+2. A debriefing is **requested AND, when requested, is required.**
+**The second condition is the problem here.** A debriefing is only "required when requested" if the request was timely. Here the request was submitted on Day 8 — 5 days after the FAR 15.505(a)(1) deadline expired. Because the request is untimely, **no debriefing is required**, and the exception cannot be invoked to toll the 10-day protest clock.
+**The Day 8 protest therefore runs under the general rule, not the debriefing exception.** It is timely only if filed within 10 days of the elimination notice. Day 8 falls within that window — the protest survives timeliness review.
+&gt; **⚠️ But there is a risk trap:** GAO must determine whether the basis of protest was known or should have been known earlier. If the solicitation itself contained the alleged deficiency, the pre-proposal impropriety rule under 4 CFR § 21.2(a)(1) could apply, potentially requiring filing before proposals were due.
+---
+## IV. COULD THE PROTEST HAVE BEEN FILED TOO EARLY?
+The debriefing exception contains a **floor, not just a ceiling**: a protest covered by that exception *"shall not be filed before the debriefing date offered."* But as established above, the exception doesn't apply here because the debriefing request was untimely. So the protest filed on Day 8 is not procedurally premature under the debriefing rule.
+**Compare this to a scenario where the debriefing was timely requested:** If the offeror had requested the debriefing on Day 2, received a debriefing scheduled for Day 14, and then filed protest on Day 8 — that protest *would be premature* under the exception (filed before the debriefing date offered). GAO would likely dismiss it or treat it as prematurely filed. The offeror would have to refile after the debriefing.
+---
+## V. THE CICA AUTOMATIC STAY — WHAT TRIGGERS IT AND WHAT GOVERNS IT
+### Statutory Framework (31 U.S.C. § 3553(c)–(d))
+Two stay provisions operate depending on whether award has been made:
+#### Pre-Award Stay (31 U.S.C. § 3553(c))
+&gt; *"A contract may not be awarded in any procurement after the Federal agency has received notice of a protest...from the Comptroller General and while the protest is pending."*
+**This is automatic.** Once GAO notifies the agency (within 1 day of protest filing), the agency **cannot make the award** while the protest is pending — unless the head of the procuring activity makes a written "urgent and compelling circumstances" finding under § 3553(c)(2).
+#### Post-Award Stay (31 U.S.C. § 3553(d))
+&gt; *"...the contracting officer shall immediately direct the contractor to cease performance..."* if the agency receives notice of protest within the **protected period** under § 3553(d)(4).
+The protected period for post-award stays ends on **the later of**:
+- **(i)** 10 calendar days after contract award, OR
+- **(ii)** 5 calendar days after the **debriefing date offered** to an unsuccessful offeror for any debriefing that is **requested and, when requested, is required.**
+---
+## VI. HOW THE DEBRIEFING CHOICE RESHAPES EVERYTHING
+### Scenario A: Debriefing Was Timely Requested (Day 2) — Hypothetical
+| Event | Calendar Effect |
+|---|---|
+| Day 0: Elimination notice | Clock starts |
+| Day 2: Written debriefing request (timely, per FAR 15.505(a)(1)) | Obligates agency to debrief |
+| Day ~7: Agency offers debriefing date (e.g., Day 12) | CICA window anchors to Day 12 |
+| Agency makes award | Cannot award while protest pending |
+| Protest filed within 10 days of Day 12 debriefing | Timely — debriefing exception governs |
+| Post-award CICA stay: expires Day 12 + 5 = Day 17 | Protest filed within this window triggers mandatory stay |
+**Pre-award protest timeliness:** Must file within 10 days of the debriefing (Day 12), so no later than **Day 22** from elimination notice.
+**Post-award stay protection (if award is made before protest):** The § 3553(d)(4)(A)(ii) window extends to **Day 17** — 5 days after the offered debriefing date. A protest filed before Day 17 triggers the mandatory post-award stay.
+---
+### Scenario B: Actual Facts — Untimely Debriefing Request (Day 8)
+| Event | Calendar Effect |
+|---|---|
+| Day 0: Elimination notice | Clock starts |
+| Day 3: FAR 15.505 deadline expires (no request made) | Debriefing entitlement lost |
+| Day 8: Untimely debriefing request + protest filed simultaneously | Protest runs under general 10-day rule |
+| Protest timeliness: | Within 10 days of Day 0 → **Timely** |
+| Post-award stay window: | 10 days after award, **not extended** by § 3553(d)(4)(A)(ii) (no required debriefing) |
+| CICA pre-award stay: | **Automatic** — agency cannot award while protest pending |
+**Key degradation:** By missing the debriefing deadline, the offeror:
+1. **Lost the extended protest window** — forfeits the right to wait for a debriefing before having to file
+2. **Lost the extended CICA post-award protection** — the § 3553(d)(4) window does not stretch past Day 10 post-award
+3. **Lost full debriefing content** — no entitlement to know the full evaluation rationale before GAO closes the record
+---
+## VII. THE AGENCY'S OBLIGATIONS AND OPTIONALITY
+### Pre-Award Phase (No Award Yet)
+| Action | Obligation |
+|---|---|
+| Award the contract | **Prohibited** while protest pending (31 U.S.C. § 3553(c)) |
+| Provide debriefing | Not required (untimely request) — discretionary accommodation only |
+| Respond to GAO | Agency report due within **30 days** of GAO notice (4 CFR § 21.3(c)) |
+| Override the pre-award stay | HCA written finding of "urgent and compelling circumstances" + GAO notification required (§ 3553(c)(2)) |
+### If Agency Wishes to Override the Pre-Award Stay
+At NIH, per NIH Manual 6033-2 and HHSAR 333.104(b)(1):
+1. CO prepares D&amp;F with background, protest grounds, and urgent/compelling justification
+2. Routed: IC Director of Acquisitions → NIH Protest Control Officer → **HCA** (non-delegable)
+3. HCA executes; **DASAMP (HHS OS) approval required**
+4. OGC-GLD concurrence and notification to GAO
+5. Written finding that award is likely within **30 days** of the finding
+---
+## VIII. WHAT HAPPENS IF THE AGENCY NOW PROVIDES THE DEBRIEFING (VOLUNTARILY)?
+FAR 15.505(a)(1) note and FAR 15.506(a)(4)(ii) both address this:
+&gt; *"Government accommodation of a request for delayed debriefing...does not automatically extend the deadlines for filing protests."*
+So if the CO voluntarily debriefs on Day 14:
+- **It does NOT restart or extend the protest clock.** The protest filed on Day 8 remains subject to its Day 8 filing date.
+- The offeror cannot file a supplemental protest beyond Day 18 (10 days from elimination notice) unless new grounds emerge from the debriefing that were **not known and could not have been known** before.
+- Supplemental grounds from the debriefing must be filed within **10 days of the debriefing** per 4 CFR § 21.2(a)(2). GAO will scrutinize whether those grounds were truly new.
+---
+## IX. SBIR-SPECIFIC JURISDICTION NOTE
+One additional issue that must be addressed for SBIR protests: **GAO has had jurisdiction questions** over certain SBIR proceedings, particularly where the program uses Other Transaction Agreements (OTAs) rather than procurement contracts. GAO's jurisdiction under 31 U.S.C. § 3551 extends to "procurement contracts." If the SBIR award instrument is an OTA or cooperative agreement, **GAO may lack jurisdiction entirely** — per 4 CFR § 21.5(m). Verify the instrument type before filing at GAO; the Court of Federal Claims may be the correct forum.
+If the SBIR is structured as a standard procurement contract (most Phase II SBIR awards are), GAO jurisdiction is proper.
+---
+## X. CONSOLIDATED TIMELINE SUMMARY
+```
+Day 0    Elimination notice received
+Day 1    GAO notified by agency (1 day after protest, once filed)
+Day 3    ← FAR 15.505 debriefing request deadline (MISSED)
+Day 8    Protest filed at GAO + untimely debriefing request submitted
+Day 9    GAO notifies agency; pre-award stay triggers automatically
+Day 9    Agency notifies other offerors with substantial prospect of award
+Day 10   ← General 10-day protest window closes (Day 8 protest is timely)
+Day 14   Agency document production list due to GAO (5 days before report)
+Day 16   Document objections due (2 days after list)
+Day 38   Agency report due (30 days after GAO notice on Day 9)
+Day 48   Protester comments due (10 days after agency report)
+Day 108  GAO decision deadline (100 days from Day 8 filing)
+Day 73   Express option decision (65 days, if requested by Day 13)
+```
+---
+## XI. KEY TAKEAWAYS FOR THE CO
+| Issue | Answer |
+|---|---|
+| Is the Day 8 protest timely? | **Yes** — within 10-day general rule; debriefing exception inapplicable |
+| Must you provide a debriefing? | **No** — request was untimely; accommodation is discretionary |
+| If you accommodate the debriefing, does it extend protest rights? | **No** — FAR 15.506(a)(4)(ii) is explicit |
+| Can you award while protest is pending? | **No** — automatic pre-award CICA stay, 31 U.S.C. § 3553(c) |
+| Can you override the stay? | Yes — HCA D&amp;F + DASAMP approval at NIH; "urgent and compelling" standard |
+| Does the lost debriefing request harm the offeror's protest? | Yes — no full debriefing facts, narrower supplemental grounds available, no extended CICA window |
+| SBIR-specific risk? | Check instrument type — OTA/cooperative agreement may divest GAO of jurisdiction |
+---
+**Sources:**
+- 4 CFR Part 21 (GAO Bid Protest Regulations) — eCFR (verified April 2026)
+- 31 U.S.C. § 3553 — CICA Stay Provisions (verified April 2026)
+- FAR 15.505 — Preaward Debriefings (acquisition.gov, FAC effective 03/17/2026)
+- FAR 15.506 — Postaward Debriefings (acquisition.gov, FAC effective 03/17/2026)
+- GAO Bid Protests Essential Guide for COs (GAO-18-510SP) — EAGLE KB
+- NIH Manual 6033-2 — Stay Provisions for Protests — EAGLE KB
+- GAO B-423341 (SMS Data Products) — Enhanced debriefing timeliness — EAGLE KB
+- *Threat Tec, LLC v. United States*, No. 26-150C (COFC Feb. 2026) — CICA stay override standard
+</t>
+        </is>
+      </c>
+      <c r="AE6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI6" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ6" s="20" t="inlineStr">
+        <is>
+          <t>v7 = v6 (comparable)
+Both produce exceptional SBIR protest analysis (13-15K chars). v7 uses 5 tools including web_search/web_fetch to verify primary sources (4 CFR Part 21, 31 USC 3553, FAR 15.505/15.506). v7 adds SBIR-specific OTA jurisdiction note and consolidated timeline with specific day counts. v6 structured as Parts I-IV; v7 has 11 sections with more granular analysis.
+Tools: v6=knowledge_search,search_far,knowledge_fetch | v7=search_far,research,knowledge_fetch,web_search,web_fetch
+Cascade: CASCADE WORKING -- both go deep. v7 adds web verification of primary statutory sources.
+Source gaps: None -- both cite 4 CFR Part 21, 31 USC 3553, FAR 15.505/15.506, GAO-18-510SP.
+Verdict: Equivalent. Both 20/20. v7 adds web-verified primary sources and SBIR jurisdiction nuance.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="159" customHeight="1">
       <c r="A7" s="5">
@@ -5597,17 +6063,785 @@
 Verdict: Equivalent. Both 18/20.</t>
         </is>
       </c>
+      <c r="AD7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is the core tension in the intake design — **action bias vs. informed accuracy**.
+The shoot-first approach (SOW in 3 questions) creates rework loops. The deep-intake approach gets lost in theory. Neither is right by itself.
+The real problem is **sequencing**: you need enough information to price before you commit to scope, but users don't want to answer 20 questions before seeing anything.
+Here's what I think the architecture should look like:
+---
+**The Gating Problem**
+Before generating any substantive document, you need three things locked:
+1. **What** — scope (SOW territory)
+2. **How much** — budget/IGCE (determines FAR part, competition, vehicle)
+3. **How** — acquisition strategy (contract type, vehicle, set-aside)
+These are interdependent. SOW scope drives IGCE. IGCE drives strategy. Strategy constrains SOW. The current approach breaks this by generating SOW before the other two exist.
+---
+**A Staged Gate Model**
+```
+Stage 1 — Framing (2-3 questions, instant)
+  What are you acquiring?
+  Rough budget order of magnitude? ($10K / $100K / $1M / $10M+)
+  Timeline?
+  → Output: FAR part determination + acquisition path
+  → NOT a document yet
+Stage 2 — Strategy Check (before any document)
+  Existing vehicles checked automatically
+  Small business applicability determined
+  Contract type recommended
+  → Output: "Here's your acquisition approach" — user confirms or adjusts
+  → Still no document
+Stage 3 — Document Generation
+  NOW generate documents in dependency order:
+  IGCE first (or parallel with SOW)
+  SOW scoped to match budget reality
+  Then AP, MRR, etc.
+```
+---
+**The Key Insight**
+The mistake is treating the SOW as the *entry point* when it's actually downstream of strategy. The **IGCE is the anchor document** — everything else sizes to fit it.
+If price comes back too high, you're back at Stage 2 (scope or strategy), not Stage 1. That's a much shorter loop.
+---
+**Tuning the Theory Problem**
+The reason deep intake gets chatty is that questions don't have a *destination*. If every question is explicitly tied to a gate condition ("I need this to determine FAR part" / "I need this to check vehicles"), the agent stops asking when the gate is satisfied — not when it runs out of questions.
+Gate-based intake = self-terminating. Theory-based intake = open-ended.
+---
+Want to prototype what Stage 1-2 questions + output would look like for the cloud services example? That would make it concrete enough to tune against.
+</t>
+        </is>
+      </c>
+      <c r="AE7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI7" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="AJ7" s="20" t="inlineStr">
+        <is>
+          <t>v7 = v6 (comparable)
+Both correctly diagnose the SOW-first rework problem and propose cost-validation gating. v7 offers a concrete 3-stage gating model (Framing -&gt; Strategy Check -&gt; Document Generation) with the insight that IGCE is the anchor document. v6 offers a 3-failure-modes diagnostic.
+Tools: v6=get_intake_status | v7=none
+Cascade: N/A -- design discussion. v7 correctly uses no tools. v6 called get_intake_status (unnecessary).
+Source gaps: N/A -- design discussion, no regulatory sources expected.
+Verdict: Equivalent. Both 18/20. v7 staged gate model slightly more concrete.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="5">
-        <f>A7+1</f>
-        <v/>
+      <c r="A8" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-70</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Cascade / KB Search</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>I need to sole-source a $280,000 annual software maintenance contract to Illumina Inc. for our BaseSpace Sequence Hub platform. Only Illumina can maintain this proprietary genomic analysis software. What documents do I need and what's the justification authority?</t>
+        </is>
+      </c>
+      <c r="AD8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete breakdown for your Illumina BaseSpace Sequence Hub sole-source maintenance contract:
+---
+## Sole-Source Acquisition: Illumina BaseSpace Sequence Hub
+**$280,000 Annual Maintenance | FAR Part 13 Simplified Acquisition**
+---
+### ✅ Justification Authority
+**FAR 6.302-1 — Only One Responsible Source (41 U.S.C. 3304(a)(1))**
+This is your authority. Proprietary software maintenance is the textbook case: only the OEM (Illumina) can maintain the BaseSpace Sequence Hub platform without substantial duplication of costs or unacceptable delays. Specific grounds:
+- **Proprietary architecture** — Source code, APIs, and platform internals are Illumina's IP; no third party can perform maintenance
+- **No equivalent substitute** — BaseSpace Sequence Hub is a unique cloud-based genomic analysis platform; alternative software would require re-validation and workflow re-development
+- **Follow-on maintenance** — Consistent with FAR 6.302-1(b)(1), continuation of support for an existing platform
+---
+### 📋 Required Documents
+At $280,000, this falls **below the SAT ($350,000)**, so you do **not** need a formal J&amp;A per FAR 6.3. You need a **Single Source Justification (SSJ) for simplified acquisitions** per **FAR 13.106-1(b)**:
+| Document | Required? | Notes |
+|---|---|---|
+| **Single Source Justification (SSJ)** | ✅ Required | FAR 13.106-1(b) — written determination in file |
+| **Statement of Work (SOW)** | ✅ Required | Describes maintenance scope, deliverables, SLAs |
+| **IGCE** | ✅ Required | NIH policy requires for all acquisitions &gt;MPT |
+| **Market Research Memo** | ✅ Required | Documents why competition not feasible |
+| **Purchase Request w/ Funds Certification** | ✅ Required | Budget office certifies funds availability |
+| **Required Sources Checklist** | ✅ Required | FAR 8.002 priority order check (AbilityOne, GSA, etc.) |
+| **SAM.gov Synopsis** | ✅ Required | Required for actions &gt;$25,000 (FAR 5.201) |
+| **NIH Information Security Checklist** | ✅ Required | IT acquisition — HHSAM 339.101(c)(1) |
+| **Section 508 Assessment** | ✅ Required | Cloud-based software platform |
+| **SAM.gov Exclusions Check** | ✅ Required | Verify Illumina active, not excluded |
+| **HHS-653 Small Business Form** | ✅ Required | All actions &gt;MPT ($15K) per AA 2023-02 |
+&gt; **No formal J&amp;A (FAR 6.304 package) is required** — that threshold kicks in above SAT. Your CO can approve the SSJ directly since $280,000 is within CO authority.
+---
+### ✅ J&amp;A Approval Level (if value grows above SAT)
+For your reference:
+| Value | Approval Authority |
+|---|---|
+| ≤ $350K (SAT) | CO approves SSJ — no J&amp;A required |
+| $350K–$900K | CO approves J&amp;A (FAR 6.304(a)(1)) |
+| $900K–$20M | HCA + Competition Advocate |
+| &gt;$20M | Head of Procuring Activity + additional reviews |
+---
+### ⚠️ Key Compliance Flags
+1. **SAM.gov Presolicitation Notice Required** — FAR 6.102-1 excludes FAR 5.101(b)(2) for "only one source" justifications. You **must** post a presolicitation notice on SAM.gov (not exempt from this requirement).
+2. **IT Clearances** — BaseSpace is a cloud-based SaaS platform. HHSAM 339.101(c)(1) requires an **Information Security &amp; Privacy Certification Checklist** before award.
+3. **NIH Policy 6027** — As a proprietary software licensing/maintenance agreement, CO must review the license terms for compliance with federal law (no unilateral termination clauses, no indemnification, no Antideficiency Act conflicts). Order of Precedence clause required.
+4. **SAM.gov Post-Award Posting** — Within 14 days of award, post the SSJ justification to SAM.gov (FAR 6.301 equivalent; redact Illumina's proprietary data first).
+5. **Price Reasonableness** — Document basis: prior contract pricing, Illumina's published maintenance rates, or Illumina's written quote compared to market benchmarks.
+---
+### 🚀 Ready to Generate Documents?
+I can immediately draft any of the following for this acquisition:
+1. **Single Source Justification (SSJ)** — core document
+2. **Statement of Work** — maintenance scope, response times, deliverables
+3. **IGCE** — based on Illumina quote + market benchmarks
+4. **Market Research Memo** — documenting Illumina as only viable source
+What do you have on hand — a quote from Illumina, existing contract, or SOW draft? That will let me generate the package right away.
+</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="5">
-        <f>A8+1</f>
-        <v/>
+      <c r="A9" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-71</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>NIH Policy Layer</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>What are the simplified acquisition threshold and micro-purchase threshold under current FAR? Also pull any NIH-specific policies that supplement these thresholds, including local purchase card policies, HCA approval requirements, and NIH procedural steps beyond standard FAR Part 13.</t>
+        </is>
+      </c>
+      <c r="AD9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete reference, pulling directly from FAR, HHS, and NIH primary sources:
+---
+# Simplified Acquisition &amp; Micro-Purchase Thresholds: FAR + HHS/NIH Policy Reference
+**Current as of FAC 2025-06, effective October 1, 2025**
+---
+## Part 1: FAR Thresholds (Statutory Baseline)
+| Threshold | Dollar Value | Authority |
+|-----------|-------------|-----------|
+| **Micro-Purchase Threshold (MPT)** | **$15,000** | FAR 13.2 |
+| MPT – Services subject to Service Contract Act (SCLS) | $2,500 | FAR 13.2 |
+| MPT – Construction (Davis-Bacon) | $2,000 | FAR 13.2 |
+| MPT – Contingency/OCONUS operations | $25,000–$40,000 | FAR 13.2 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 13.000 |
+| Commercial Simplified Acquisition Test Ceiling | $9,000,000 ($15M in certain cases) | FAR 13.5 |
+&gt; **Threshold Change Note:** The MPT increased from $10,000 to $15,000 effective October 1, 2025 per FAC 2025-06. The SAT increased from $250,000 to $350,000 simultaneously.
+---
+## Part 2: What the FAR Requires at Each Band
+### ≤ $15,000 — Micro-Purchase (FAR Subpart 13.2)
+| Requirement | Rule |
+|-------------|------|
+| Competition | **Not required** — award to single source if price is reasonable |
+| Preferred method | Government-wide commercial purchase card |
+| Small business set-aside | Not required; equitable distribution *encouraged* |
+| Synopsis (SAM.gov) | Not required |
+| Contract clauses | Minimal (FAR 13.202) |
+| Documentation | Minimal; purchase card monthly statement sufficient |
+| Price reasonableness | CO determines; no formal analysis required unless price is suspect |
+| Split-purchase prohibition | Required — cannot artificially divide requirement to stay at/below MPT (FAR 13.003(c)(2)) |
+### $15,001 – $350,000 — Simplified Acquisition (FAR Part 13)
+| Requirement | Rule |
+|-------------|------|
+| Competition | Promote to maximum extent practicable; consider ≥ 3 sources |
+| Small business set-aside | **Mandatory** — SHALL be set aside for small business (FAR 19.502-2); exceptions for 8(a), HUBZone, SDVOSB, WOSB |
+| Synopsis | Generally not required below $25K; above $25K, SAM.gov synopsis or documented exception required |
+| Price reasonableness | Required; document basis (comparison, prior prices, market data) |
+| Documentation | Keep to minimum; oral solicitations require notes of prices/sources; written: abstract or notes only |
+| Award basis | Most advantageous quote (price + other factors at CO discretion) |
+| Solicitation forms | Streamlined; no formal FAR Part 15 procedures required |
+### $350,001 – $9,000,000 — Commercial SAP (FAR Subpart 13.5)
+| Requirement | Rule |
+|-------------|------|
+| Authority | 41 U.S.C. 1901/1903; FAR Subpart 13.5 |
+| Applies to | Commercial products/services only |
+| Synopsis | Generally required (FAR 5.101) |
+| Small business | CO discretion (set-aside not mandatory) |
+| FAR Part 12 | Applies (commercial terms and conditions govern) |
+| Documentation | More than standard SAP; less than FAR Part 15 |
+---
+## Part 3: HHS-Specific Policies Supplementing FAR Part 13
+These requirements layer on top of FAR and are NIH/HHS-specific obligations.
+### 3.1 Key Dollar Triggers at HHS (HHSAM / HHS PMR Checklist)
+| Threshold | HHS-Added Requirement | Authority |
+|-----------|----------------------|-----------|
+| **&gt; MPT ($15K)** | HHS-653 Small Business Review Form required | AA 2023-02 Amendment 3 |
+| **&gt; $25K** | SAM.gov synopsis or documented exception | FAR 5.101; HHSAM 305.202 |
+| **&gt; SAT ($350K)** | Full Acquisition Plan (HHS template required) | FAR 7.105; HHSAM 307.105 |
+| **&gt; SAT ($350K)** | HHS Market Research Report Template required (not just notes) | HHSAM 310.000 |
+| **&gt; SAT ($350K)** | SPE approval required before solicitation for **non-commercial** products/services | EO 14271; HHS AA 2026-01 |
+| **&gt; $750K** | Subcontracting plan (other-than-small-business primes) | FAR 19.702 |
+| **&gt; $900K** | HCA approval for J&amp;A (sole source) | FAR 6.304(a)(2) |
+| **&gt; $2.5M** | Certified cost or pricing data (TINA) | FAR 15.403 |
+| **&gt; $4.5M** | Congressional notification to Assistant Secretary for Legislation (email: grantfax@hhs.gov) | HHS policy |
+| **&gt; $20M** | Written Acquisition Plan required (HHS threshold; FAR threshold is $7M new/$50M task orders) | HHSAM 307.105 |
+| **&gt; $90M** | SPE-level J&amp;A approval | FAR 6.304(a)(4) |
+| **&gt; $100M** | SPE approval for single-award IDIQ or BPA | HHS PMR |
+### 3.2 Mandatory Source Checks Before Any Purchase (FAR Part 8 / HHS)
+Before going to open market at **any** dollar level, purchasing officials must check required sources **in priority order**:
+**For Products:**
+1. HHS/OPDIV inventories and excess property
+2. Excess from other agencies (GSAXcess)
+3. Federal Prison Industries / UNICOR *(only required above MPT = $15K)*
+4. AbilityOne Program
+5. GSA Wholesale supply sources
+6. HHS Category Management BPAs
+7. GSA Multiple Award Schedules (MAS)
+8. HHS preferred IDIQ/BPA contracts
+9a. GSA Commercial Platforms (Amazon Business, Fisher Scientific) — MPT only
+9b. Open market (small businesses preferred)
+**For Services:**
+1. AbilityOne Program
+2. HHS Category Management BPAs
+3. GSA MAS
+4. HHS preferred IDIQ/BPAs
+5. Open market
+### 3.3 Mandatory Cross-Cutting Compliance Items (All Purchase Levels)
+These apply regardless of dollar value:
+| Requirement | Trigger |
+|-------------|---------|
+| **Bona fide needs rule** | All purchases — funds must match fiscal year of need (31 U.S.C. § 1502(a)) |
+| **Section 889 compliance** | All purchases — cannot buy from or contract with entities using Huawei, ZTE, Hytera, Hikvision, Dahua equipment |
+| **Section 508 (EIT)** | All purchases involving Electronic &amp; Information Technology |
+| **Sustainable acquisitions** | All purchases — energy-efficient, recycled content, biobased, EPEAT |
+| **Split-purchase prohibition** | All — cannot artificially split to stay below threshold (FAR 13.003(c)(2)) |
+| **Buy American Act** | Products/construction above MPT; GSA Schedule orders and micro-purchases &lt; $15K **exempt** |
+---
+## Part 4: NIH-Specific Procedural Requirements
+### 4.1 Purchase Card (GPC) — NIH Policies
+| Rule | NIH Requirement |
+|------|----------------|
+| **Pre-approval** | Written pre-approval from supervisor/AO required before every purchase |
+| **Price reasonableness documentation** | Required in writing for **all purchases ≥ $5,000** (NIH-specific — stricter than FAR) |
+| **Segregation of duties** | Funds Approving Official, Cardholder (CH), and Receiving Official must be **three different individuals** (FRC Checklist Q4) |
+| **SCLS cap for purchase card** | Services subject to Service Contract Act (janitorial, security, temp services) capped at **$2,500** — cannot exceed on GPC |
+| **Recurring requirements** | If aggregate exceeds MPT ($15K) over 12 months → must be processed by contracting office, not GPC |
+| **Convenience checks** | Capped at $7,500 (half of MPT); $2,500 for SCLS services; $2,000 for construction |
+### 4.2 NIH-Unique Clearance Requirements (Purchase Card Supplement v6.2)
+Many purchase categories require NIH-specific approvals before obligation:
+| Category | NIH-Specific Requirement |
+|----------|--------------------------|
+| **IT products (laptops/desktops)** | Must use NITAAC first → then NASA SEWP → then GSA; CIO approval for non-standard configs |
+| **IT products generally** | OCIO/IC Information Systems Security Officer (ISSO) guidance required |
+| **Construction** | Limited to $2,000; only by cardholders in OA/ORF or ORF pre-approved; Davis-Bacon applies |
+| **Conference/meeting space + food** | NIH Form 827-1 (Non-Delegable Attachment A) required; must be approved BEFORE obligation; OFM/DDM review |
+| **Food outside of conference** | IC's Executive Officer signs NIH Form 2408-1; DDM review and approval required BEFORE funds obligated |
+| **Custom antibodies** | Must purchase from vendor with active PHS Assurance (verify on OLAW website) |
+| **Radioactive materials** | Deliver to Building 21, Room 107; DRS clearance number on packing slip; Form 88-1 to Radiation Safety 24 hrs prior |
+| **Sensitive/accountable property** | Report to Property Management Office; specific NBS data fields required (OC code = 31x; Custodial Code; Property Description) |
+| **Kitchen appliances** | IC EO or delegee concurrence in writing required; must be common area only; no consumables |
+| **Microsoft software** | Must use Microsoft Enterprise Agreement BPA — no open market purchases |
+| **Printing/copying devices** | Must use FSSI Print Management BPAs or NIH ECS III; Executive Officer approval if deviation |
+| **Ergonomics** | ORS ergonomic evaluation required BEFORE purchasing equipment |
+| **Space heaters/fans** | ORF must attempt building fix first; written ORF Facility Manager approval required |
+| **Cellular devices** | Must use FSSI Wireless BPAs; IC IT approval before purchase |
+### 4.3 HCA Approval Requirements
+The Head of Contracting Activity (HCA) at NIH/HHS has specific approval authorities:
+| Action | HCA Requirement |
+|--------|----------------|
+| J&amp;A for sole source | $900K – $20M range (CO approves &lt; $900K; Competition Advocate approves $900K – $20M; HCA for higher) |
+| T&amp;M/LH BPAs &gt; 3 years | HCA approval required |
+| Single-award BPAs &gt; $100M | SPE approval (above HCA level) |
+| Non-commercial procurements &gt; SAT | SPE approval before solicitation per EO 14271 / HHS AA 2026-01 |
+| Buy American waiver (nonavailability) | HCA signature on D&amp;F required (OALM Communication 23-65 template) |
+### 4.4 NIH File Review Standards (FRC — OALM Checklist)
+OALM's Acquisition Compliance Reviews (ACRs) commonly cite these as findings. Avoid them:
+| Common Red Finding | Requirement |
+|-------------------|-------------|
+| Segregation of duties failure | FA and CO must be different people |
+| Competition documentation absent | Oral quotes require notes of who was called, what was requested, prices received |
+| Sole source justification insufficient | Must explain why vendor is uniquely qualified and why competition is not feasible |
+| Price reasonableness inadequate | Analysis must support conclusion; "competitive bid" alone without comparison data is insufficient |
+| SAM/exclusions check missing | Must document exclusion check at receipt of offer AND prior to award |
+| FPDS not finalized timely | Required within 3 business days of award |
+| Award date after delivery date | Timeline must be logical |
+| Receiving report incomplete | Must include contract number, description, quantities, dates, inspector signature |
+---
+## Quick Reference Summary
+```
+≤ $15K    → Micro-purchase | No competition required | GPC preferred
+              NIH adds: pre-approval, price reasonableness ≥ $5K, segregation of duties
+$15K–$350K → Simplified Acquisition | SB set-aside mandatory | ≥3 sources
+              HHS adds: HHS-653 form, synopsis &gt;$25K, FAR Part 8 source check
+&gt; $350K   → Full AP + HHS MRR template + FAR Part 8 + full competition
+              Non-commercial: SPE approval required before solicitation (EO 14271)
+              Sole source $900K–$20M: Competition Advocate approval
+```
+---
+**Sources:**
+- FAR Part 13 (FAC 2025-06) — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Acquisition_Procedures.txt`
+- HHS GPC Program Directive v7.0 (updated Nov 2025) — `eagle-knowledge-base/approved/compliance-strategist/SOPs/HHS_GPC_Streamlined_Guide_2025.txt`
+- NIH Purchase Card Supplement v6.2 (updated Nov 2025) — `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Purchase_Card_Supplement_Streamlined_2025.txt`
+- HHS PMR Threshold Matrix (FAC 2025-06) — `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Threshold_Matrix.txt`
+- HHS AA 2026-01 (EO 14271 SPE Approval) — `eagle-knowledge-base/approved/compliance-strategist/regulatory-policies/HHS_AA_2026_01_EO_14271_Non_Commercial_Approval.txt`
+- NIH FRC / OALM Acquisition Compliance Review Standards — research tool (fetched)
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-72</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>GAO KB Retrieval</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>What did GAO hold in B-302358 regarding IDIQ minimum obligation requirements? Search the knowledge base for the full decision text and cite the specific KB documents you find.</t>
+        </is>
+      </c>
+      <c r="AD10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I now have the full decision text directly from GAO.gov. Here is a complete, source-cited analysis:
+---
+## GAO B-302358 — *Bureau of Customs and Border Protection — Automated Commercial Environment Contract*
+**December 27, 2004 | Decided by: Anthony H. Gamboa, General Counsel**
+---
+### Case Background
+The Bureau of Customs and Border Protection (CBP) awarded its Automated Commercial Environment (ACE) contract to IBM Global Services on April 27, 2001. The contract had:
+- A **$25 million minimum order amount**
+- A **$5 billion maximum order amount**
+- A base period of 5 years plus two 5-year options
+The DHS Inspector General argued the contract was a **multiyear contract** subject to 41 U.S.C. § 254c (which requires obligating estimated termination costs at award). CBP maintained it was an **IDIQ contract** not subject to those requirements.
+---
+### GAO Holdings — Two Distinct Issues
+#### Holding 1: The ACE Contract Is an IDIQ, Not a Multiyear Contract
+GAO held that the ACE contract was plainly an **IDIQ contract** governed by 41 U.S.C. §§ 253h–253k and FAR Subpart 16.5 — not a multiyear contract under 41 U.S.C. § 254c. Key reasoning:
+&gt; *"An IDIQ contract is a contract 'that does not procure or specify a firm quantity' of supplies or services, other than a minimum or maximum quantity... A single contract cannot satisfy these wholly inconsistent sets of statutory and regulatory requirements."*
+GAO drew a sharp line between **"multiyear contracting"** (FAR Subpart 17.1 — buys multiple years' requirements up front, requires termination cost obligations) and **"multiple year contracts"** (contracts that simply extend over more than one year, including IDIQ contracts). The ACE contract's multi-year term did not make it a § 254c multiyear contract. Therefore, **CBP was not required to obligate estimated termination costs at award**.
+#### Holding 2: The Minimum Guarantee Must Be Obligated at Contract Award — Per 31 U.S.C. § 1501(a)(1)
+This is the holding directly on point for IDIQ minimum obligations:
+&gt; *"When an agency executes an indefinite-quantity contract such as an IDIQ contract, the agency must record an obligation in the amount of the required minimum purchase... At the time of award, the government has a fixed liability for the minimum amount to which it committed itself."*
+&gt; *"Customs should have recorded an obligation against a currently available appropriation for the authorized purpose in an amount reflecting the liability incurred as a result of a binding written agreement at the time the contract was awarded."*
+**The Rule:** The obligation for the minimum guaranteed amount (here, $25 million) must be recorded against a currently available appropriation **at the time of contract execution** — not when task orders are later placed. CBP waited 5 months (until it issued the first three task orders) to record the obligation. GAO found this violated the recording statute, 31 U.S.C. § 1501(a)(1), even though CBP happened to have sufficient funds available both at award and 5 months later.
+**Beyond the minimum:** Further obligations are incurred only as task or delivery orders are placed and are chargeable to the fiscal year appropriation current **at the time each order is placed** (citing 60 Comp. Gen. 219 (1981)).
+---
+### GAO's Recommendation
+&gt; *"We recommend that Customs take the necessary steps to ensure timely obligation of the minimum financial liability represented by IDIQ contracts."*
+---
+### Key Legal Authorities Cited in the Decision
+| Authority | Purpose |
+|-----------|---------|
+| **31 U.S.C. § 1501(a)(1)** — Recording Statute | Requires agencies to record obligations when a binding written agreement incurs a legal liability |
+| **FAR 16.504(a)** | IDIQ minimum: "The contract must require the Government to order and the contractor to furnish at least a stated minimum quantity" |
+| **FAR 52.216-22** | IDIQ clause — quantities are estimates only, not purchased by the contract |
+| **41 U.S.C. § 254c** (now 41 U.S.C. § 3903) | Multiyear contracting authority — held inapplicable to IDIQ contracts |
+| **65 Comp. Gen. 4 (1985); B-242974.6 (1991)** | Agency must record obligation at time of legal liability incurrence |
+| **63 Comp. Gen. 129 (1983)** | Mere signing of IDIQ agreement ≠ obligation for future orders; additional obligations arise only when orders are placed |
+| **GAO Red Book, Vol. II, Ch. 7** | Appropriations law principles for variable-quantity contracts |
+---
+### Practical Significance for NIH/HHS IDIQ Acquisitions
+Three rules flow directly from B-302358:
+1. **Obligate the minimum at award.** When an IDIQ contract is executed, the minimum guaranteed amount must be obligated against a currently available appropriation on the day of award. It cannot be deferred until the first task order is issued.
+2. **Match fiscal year for each task order.** Obligations for amounts above the minimum are recorded when each individual task or delivery order is placed, and must be charged to appropriations current at that time — not to the appropriation year when the base contract was awarded.
+3. **IDIQ ≠ Multiyear.** A multi-year IDIQ contract (e.g., base + options spanning 10+ years) is not subject to 41 U.S.C. § 254c and does not require termination cost obligations at award. The structural distinction is controlling; labels in the contract file are not.
+---
+### Sources
+| Source | Citation |
+|--------|----------|
+| **Primary — Full GAO Decision Text** | GAO B-302358, Dec. 27, 2004 · https://www.gao.gov/products/b-302358 |
+| **KB — FAR Part 16 IDIQ Guidance** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt` |
+| **KB — GAO Bid Protests Essential Guide** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt` |
+&gt; **KB Note:** GAO B-302358 does not have a standalone document in the EAGLE knowledge base. The decision text was retrieved directly from the GAO website (gao.gov). The KB does contain comprehensive FAR Part 16 IDIQ guidance (cited above) that is fully consistent with the B-302358 holding on minimum guarantee obligations.
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-73</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>Bona Fide Needs</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Explain how the bona fide needs rule under 31 U.S.C. 1502(a) interacts with the severable vs. non-severable distinction when funding a service contract that crosses fiscal years. Include both the severable services rules and the time-based bona fide needs rules.</t>
+        </is>
+      </c>
+      <c r="AD11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is a comprehensive explanation of how the bona fide needs rule under 31 U.S.C. § 1502(a) interacts with the severable/non-severable distinction for service contracts crossing fiscal years.
+---
+# The Bona Fide Needs Rule &amp; Severable vs. Non-Severable Services
+## I. The Foundational Statute
+**31 U.S.C. § 1502(a)** provides:
+&gt; *"The balance of an appropriation or fund limited for obligation to a definite period is available only for payment of expenses properly incurred during the period of availability or to complete contracts properly made within that period of availability."*
+The practical rule: **FY 2026 appropriations fund FY 2026 needs. FY 2025 appropriations fund FY 2025 needs.** You cannot use current-year funds to pay for future-year requirements, nor future-year funds for past requirements. This is a matter of congressional control over the power of the purse — using one year's money to satisfy another year's needs circumvents the annual appropriations process.
+For **services**, the operative question is: *when does the bona fide need arise?*
+The answer is: **when the services are performed** — not when the contract is signed. This is the **performance period rule**, and it is where the severable/non-severable distinction becomes critical.
+---
+## II. The Severable vs. Non-Severable Distinction
+These are not FAR concepts — they are **appropriations law** concepts rooted in GAO precedent. Contract language cannot manufacture one classification or the other; the determination is made on the **nature of the services**.
+### Non-Severable Services ("Single Undertaking")
+Services are non-severable when they constitute a **single undertaking** — tasks that are interdependent, build toward a unified outcome, and cannot be divided into discrete time periods without losing their essential character or value.
+**GAO Standard:** *"The question is whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."*
+**Identifying factors:**
+- Single final deliverable (report, design, system, opinion)
+- Tasks are interdependent — earlier phases are prerequisites for later ones
+- Value is derived from **complete performance**, not from any given period's increment
+- The time period is arbitrary or administrative, not definitional of scope
+**Clear examples:** Feasibility study, program evaluation, financial audit, custom software development for a specific system, architectural/engineering design, one-time legal representation in specific litigation, a defined training course.
+### Severable Services ("Recurring/Continuing")
+Services are severable when each unit of service has **independent value** regardless of what came before or after — the services can be logically divided by time period, and each period's performance stands alone.
+**Identifying factors:**
+- Recurring or ongoing outputs
+- Each day/week/month of performance is a discrete deliverable
+- Interrupting the contract partway through does not destroy the value of what has already been delivered
+- The performance period *defines the scope* of each increment rather than just scheduling it
+**Clear examples:** Help desk support, facilities maintenance, guard services, systems administration (monitoring, patching, user management), janitorial services, SaaS/database subscriptions, ongoing administrative support.
+---
+## III. How the Bona Fide Needs Rule Applies to Each Category
+### Non-Severable Services — The "Year of Award" Rule
+For non-severable services, the **entire contract represents a single bona fide need** arising in the fiscal year the contract is entered. Because the undertaking cannot be divided, the whole effort is treated as the need of the year when the Government commits to it.
+**Consequence:** You may **obligate the full contract value from the appropriation current at award**, even if performance extends into the next fiscal year (or beyond).
+&gt; **Example:** A $600K program evaluation is awarded September 15, FY2025. Fieldwork begins October 2025, and the final report is due March 2026. → **Entire $600K obligated from FY2025 funds.** The evaluation is a single undertaking; the bona fide need arose in FY2025 when the Government committed to the study.
+This is the statutory basis in § 1502(a)'s phrase: *"to complete contracts properly made within that period of availability."* The contract was properly made in FY2025; completion simply extends into FY2026.
+### Severable Services — The "Year of Performance" Rule
+For severable services, each fiscal year's portion of performance is a **separate bona fide need** belonging to that fiscal year. You cannot use FY2025 appropriations to pay for FY2026 services, because those services don't arise as a need until FY2026.
+**Consequence:** If a severable services contract crosses fiscal years, it **must be incrementally funded** — each year's appropriation covers only that year's services.
+&gt; **Example:** A $1.2M/year help desk support contract runs October 1, FY2025 – September 30, FY2026 (12 months at $100K/month). Contract is awarded in mid-FY2025:
+&gt; - **FY2025 funds: $300K** (October–December 2025, 3 months)
+&gt; - **FY2026 funds: $900K** (January–September 2026, 9 months)
+&gt; - **Cannot** obligate the full $1.2M from FY2025 — doing so would use FY2025 money to pay for FY2026 services, violating § 1502(a).
+---
+## IV. The Interaction: Time-Based Bona Fide Needs Rules for Each Category
+The two categories produce different time-based obligation rules:
+| Factor | Non-Severable | Severable |
+|---|---|---|
+| **When does the need arise?** | Year the contract is awarded | Year services are **performed** |
+| **Obligation timing** | Full amount at award | Incrementally, fiscal year by fiscal year |
+| **Crossing fiscal years** | Permissible; single appropriation | Requires incremental funding |
+| **Governing principle** | "Contracts properly made" within availability | Services performed = need arising |
+| **Key risk** | Awarding contract without genuine current need | Using prior-year funds for out-year services |
+| **FAR clauses (if cost-type)** | Standard funding clauses | FAR 52.232-22 (Limitation of Funds); FAR 52.232-19 (Availability of Funds for Next FY) |
+---
+## V. The Short Bridge Exception (Severable Services)
+There is a recognized, narrow exception for severable services: if a severable contract **crosses a fiscal year boundary by only a short period** (typically 1–3 months), the agency may fund the entire contract from the prior fiscal year's appropriation, provided:
+1. The bridge period is genuinely short (the exception is not unlimited)
+2. The award is necessary to avoid a gap in services
+3. There is documented operational necessity
+&gt; **Example:** A 3-month bridge contract runs August 1 – October 31, FY2025/FY2026. Even though October falls in FY2026, the **entire $150K may be funded from FY2025 appropriations** as a short bridge to prevent a service gap.
+This exception is administrative necessity, not a general license to fund severable out-year services with prior-year money.
+---
+## VI. The Option Year Overlay
+Options add a third layer. Each option period is a **separate bona fide need** of the fiscal year in which that option period is performed — regardless of whether the underlying service is severable or non-severable.
+- Option for FY2026 performance = FY2026 bona fide need = must use **FY2026 funds** to exercise it
+- You **cannot** exercise a FY2026 option in September FY2025 using FY2025 funds just to avoid losing year-end money
+**Advance exercise exception:** A CO may exercise an option using prior-year funds if:
+- Operational necessity requires advance notice to the contractor (e.g., a 60-day notice clause)
+- The exercise occurs close to the start of the option period (generally within 90 days)
+- The purpose is to avoid a service gap, not to circumvent the bona fide needs rule
+---
+## VII. The Classification Cannot Be Manipulated
+This is perhaps the most important practical point: **you cannot engineer the determination through contract language.** GAO has held that severability is determined by the nature of the services, not by how the contract characterizes them. Writing a help desk support contract as a "unified integrated service delivery undertaking" does not make it non-severable. Attempting this is itself a potential bona fide needs violation.
+---
+## VIII. Common Violations
+| Violation | What Happens | Prevention |
+|---|---|---|
+| Severable services fully funded with single-year funds | FY25 funds used to pay for FY26 services on an ongoing IT support contract | Analyze severability; fund incrementally |
+| End-of-year "parking" on non-severable contract | Award study contract September 29 without genuine current need | Document that need genuinely arose in current FY |
+| Advance option exercise without operational necessity | Exercise FY26 option in August FY25 to avoid losing FY25 money | Only advance-exercise when contractually required lead time necessitates it |
+| Misclassifying severable services as non-severable | SOW written to appear as "single undertaking" for ongoing maintenance | Classification based on nature of services, not drafting choices |
+---
+## IX. Practical Decision Framework
+**Step 1 — What is the primary deliverable?**
+- Single final product/report/system → likely **non-severable**
+- Ongoing outputs with independent periodic value → likely **severable**
+**Step 2 — Can you logically divide the work by time period?**
+- Cannot divide without losing essential value → **non-severable**
+- Each period stands alone → **severable**
+**Step 3 — Are the tasks interdependent?**
+- Each phase prerequisite to the next toward a unified goal → **non-severable**
+- Repetitive, independent tasks → **severable**
+**Step 4 — Apply the funding rule:**
+- Non-severable: Obligate full amount at award; document that the undertaking is a bona fide need of the current fiscal year
+- Severable: Fund incrementally; document the rationale for the pro-rata split across fiscal years
+---
+## X. Acquisition Plan Language
+**Non-severable:** *"The services required under this acquisition constitute a non-severable undertaking. The contract will produce [specific deliverable] through interdependent tasks that cannot be meaningfully divided into discrete time periods. The entire contract value will be obligated from FY [XXXX] appropriations, even though performance extends into FY [XXXX+1], in compliance with the bona fide needs rule because the entire undertaking represents a bona fide need of FY [XXXX] when the contract is entered."*
+**Severable:** *"The services required under this acquisition are severable, consisting of recurring [describe services] where each period's performance has independent value. Incremental funding is required: FY [XXXX] appropriations fund services from [dates] ($[amount]); FY [XXXX+1] appropriations will fund services from [dates] ($[amount]). This matches each fiscal year's appropriation to that year's bona fide need."*
+---
+## Sources
+| Document | Location |
+|---|---|
+| GAO Red Book, Ch. 5 — Bona Fide Needs Rule | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt` |
+| GAO Red Book, Ch. 5 — Severable vs. Non-Severable | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt` |
+| Contract Obligation Timing GAO Guidance | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt` |
+| Army Contract Attorneys Deskbook 2025, Ch. 4 | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt` |
+| Option Exercise Timing and Funding | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_options.txt` |
+| 31 U.S.C. § 1502(a) | Statute |
+| GAO Decision B-321640 (Sep. 19, 2011) | GAO — SBA parking funds case |
+| FAR 32.703-2, FAR 52.232-19, FAR 52.232-22 | FAR — Cross-fiscal-year funding clauses |
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-74</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>FAR 16.505 Exceptions</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>List every exception to the fair opportunity requirement for task orders under FAR 16.505(b)(2)(i), including the small business set-aside exception at subparagraph (F). There should be seven exceptions (A through G). Cite the exact FAR paragraph for each.</t>
+        </is>
+      </c>
+      <c r="AD12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are all seven exceptions to the fair opportunity requirement for task orders under multiple-award IDIQ contracts, drawn verbatim from **FAR 16.507-6(b)** (FAR RFO, effective HHS November 21, 2025 / HHS Class Deviation 2026-01):
+---
+## FAR 16.507-6(b) — Exceptions to Fair Opportunity
+&gt; Orders placed against multiple-award contracts are exempt from the competition requirements in FAR Part 6, but the contracting officer **must justify** placing any order above the micro-purchase threshold on a sole-source basis under one of these seven exceptions:
+---
+### **(b)(1) — Urgency**
+&gt; "The agency need for the supplies or services is **so urgent** that providing a fair opportunity would result in unacceptable delays."
+*Posting note: Justification must be posted within **30 days** after award (not the standard 14 days) — FAR 16.507-6(f)(2).*
+---
+### **(b)(2) — Unique / Highly Specialized Capability**
+&gt; "**Only one awardee is capable** of providing the supplies or services required at the level of quality required because the supplies or services ordered are unique or highly specialized."
+---
+### **(b)(3) — Logical Follow-On**
+&gt; "The order must be issued on a sole-source basis in the interest of economy and efficiency because it is a **logical follow-on** to an order already issued under the contract, provided that all awardees were given a fair opportunity to be considered for the original order."
+*Justification must describe why the relationship between the initial order and the follow-on is logical (e.g., scope, period of performance, or value) — FAR 16.507-6(d)(1) and (d)(2)(iv).*
+---
+### **(b)(4) — Minimum Guarantee**
+&gt; "It is necessary to place an order to **satisfy a minimum guarantee**."
+---
+### **(b)(5) — Statutory Authorization** *(orders exceeding the SAT only)*
+&gt; "For orders exceeding the SAT, a **statute expressly authorizes or requires** that the purchase be made from a specified source."
+*Note: This exception applies only to orders above the Simplified Acquisition Threshold ($350,000).*
+---
+### **(b)(6) — DoD/NASA/Coast Guard: FAR Part 6 Exceptions** *(agency-limited)*
+&gt; "For DoD, NASA, and the Coast Guard, the order satisfies one of the exceptions permitting the use of other than full and open competition listed in **part 6.103** (10 U.S.C. 3406(c)(5)). The public interest exception must not be used unless Congress is notified in accordance with 10 U.S.C. 3204(a)(7)."
+*Note: This exception is **limited to DoD, NASA, and the Coast Guard**. It is not available to civilian agencies such as NIH/HHS.*
+---
+### **(c) — Small Business Set-Aside / Reserves** *(not subject to J&amp;A requirements)*
+&gt; "Part 19 and Public Law 111-240 (15 U.S.C. 644(r)) provide authority for **setting aside orders** and placing orders under reserves, which are **not subject to** the justification, approval, and posting requirements in paragraphs (d)–(f)."
+*This is the small business exception. Unlike exceptions (b)(1)–(b)(6), small business set-asides under FAR Part 19 / 15 U.S.C. 644(r) are expressly carved out from the sole-source J&amp;A, approval, and posting requirements.*
+---
+## Summary Table
+| # | Citation | Exception | J&amp;A Required? |
+|---|----------|-----------|---------------|
+| 1 | FAR 16.507-6(b)(1) | Urgency — unacceptable delay | Yes (post within 30 days) |
+| 2 | FAR 16.507-6(b)(2) | Unique/highly specialized — only one awardee capable | Yes |
+| 3 | FAR 16.507-6(b)(3) | Logical follow-on to prior competed order | Yes |
+| 4 | FAR 16.507-6(b)(4) | Satisfy minimum guarantee | Yes |
+| 5 | FAR 16.507-6(b)(5) | Statutory authorization/requirement *(&gt;SAT only)* | Yes |
+| 6 | FAR 16.507-6(b)(6) | FAR Part 6 exception *(DoD/NASA/Coast Guard only)* | Yes |
+| 7 | FAR 16.507-6(c) | Small business set-aside/reserve (FAR Part 19 / 15 U.S.C. 644(r)) | **No** — exempt from J&amp;A, approval &amp; posting |
+---
+### Key Points for NIH/HHS Practitioners:
+- **Exception (b)(6) is not available to NIH/HHS** — it applies only to DoD, NASA, and the Coast Guard.
+- **Exception (c) (small business) is uniquely favorable** — it is the only exception that does not require a written justification, approval chain, or SAM.gov posting.
+- Approval thresholds for exceptions (b)(1)–(b)(5): CO self-certifies up to $900K; Advocate for Competition up to $20M; Head of Procuring Activity up to $90M; Senior Procurement Executive above $90M — per FAR 16.507-6(e).
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-76</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>SBIR KB vs Web</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>An offeror eliminated from a SBIR Phase II competition wants to protest at GAO. Search the knowledge base for all relevant protest guidance documents, including GAO bid protest guides, NIH stay provision policies, and debriefing requirements. List each KB document found with its file path before analyzing the protest process.</t>
+        </is>
+      </c>
+      <c r="AD13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is the complete picture — all KB documents listed first, followed by a thorough analysis.
+---
+## 📚 Knowledge Base Documents Found — Protest Guidance Folder
+All documents located at: `eagle-knowledge-base/approved/legal-counselor/protest-guidance/`
+| # | Title | File Path (S3 Key) | Type | Authority |
+|---|-------|-------------------|------|-----------|
+| 1 | **GAO Bid Protests – Essential Guide for COs** | `...protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt` | Guidance (GAO-18-510SP) | Regulation |
+| 2 | **NIH Manual 6033-1: CO's Statement of Facts in GAO Protests** | `...protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt` | NIH Manual Chapter | Policy/Guidance |
+| 3 | **NIH Manual 6033-2: Stay Provisions for Protests** | `...protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt` | NIH Manual Chapter | Policy/Guidance |
+| 4 | **NIH Policy Manual 6033-2: Stay Provisions (2008 Version)** | `...protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt` | Policy | Policy/Guidance |
+| 5 | **GAO Decision B-419956.258: EPDS Filing Timeliness** | `...protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt` | GAO Case Decision | Precedent |
+---
+## ⚖️ SBIR Phase II GAO Protest — Complete Analysis
+### 1. Threshold Issue: Is This Protestable at GAO?
+**SBIR Phase II competitions present a significant jurisdictional hurdle.** GAO's bid protest authority under the Competition in Contracting Act (31 U.S.C. §§ 3551–3556) covers whether agencies complied with statutes and regulations governing procurements. For SBIR programs, the critical question is **how the Phase II was conducted**:
+- **If awarded via a standard FAR-based competitive acquisition** (e.g., RFP, competitive range, proposals, source selection under FAR Part 15) → **GAO has jurisdiction**. The elimination of an offeror from competition is reviewable.
+- **If conducted under SBA's SBIR Policy Directive as a non-FAR agency determination** → GAO's jurisdiction may be limited, and challenges to SBA programmatic decisions are generally **outside GAO's jurisdiction** (per 4 C.F.R. § 21.5).
+Assuming the Phase II was conducted as a FAR-based competitive acquisition (which is the NIH norm for SBIR Phase II), the protest analysis below applies in full.
+---
+### 2. Standing — Interested Party Requirement (4 C.F.R. § 21.0(a))
+The eliminated offeror must be an **"interested party"**: an actual or prospective offeror with a **direct economic interest** in the procurement — specifically, a company that would be in line for award if the protest is sustained. An offeror eliminated from a Phase II competition who had a reasonable prospect of award generally qualifies. However, if the protester was eliminated early in a multi-step evaluation and other offerors remain ahead, GAO may find they lack the requisite direct economic interest.
+---
+### 3. Timeliness — The Most Critical Factor (4 C.F.R. § 21.2)
+⚠️ **GAO strictly enforces timeliness — it is the most common reason for dismissal.**
+For a competitive Phase II elimination, the specific rule depends on the protest basis:
+| Protest Basis | Filing Deadline |
+|---|---|
+| Solicitation impropriety apparent before proposals were due | **Before proposal due date** |
+| Award-related grounds (evaluation errors, discussions, source selection) | **10 calendar days** after basis known or should have been known |
+| **With required debriefing (FAR 15.505 or 15.506)** | **NOT before debriefing date offered**; then **10 calendar days after debriefing held** |
+| After agency-level protest | **10 calendar days** after adverse agency action |
+&gt; **Key rule for SBIR Phase II:** If a debriefing was required (FAR 15.506 for post-award) and offered, the protester **must request and attend the debriefing first**, and then has 10 days from the date the debriefing was held to file at GAO. The 10-day clock does not start running before the debriefing if one was required.
+Days are **calendar days**. Day one is the day after the triggering event. If day 10 falls on a weekend or federal holiday, the deadline extends to the next business day.
+---
+### 4. Debriefing Requirements — FAR 15.505 &amp; 15.506
+Debriefings are central to the protest timeline and serve as the primary source of protest grounds. Under FAR:
+- **FAR 15.505 — Preaward Debriefing:** For offerors excluded from the competitive range. Must be requested within 3 days of notice of exclusion. Agency must debrief within 5 days of the request.
+- **FAR 15.506 — Postaward Debriefing:** For unsuccessful offerors after award. Must be requested within 3 days of learning of award. Agency must debrief within 5 days.
+**Critical debriefing content requirements (FAR 15.506(d)):**
+- Agency's evaluation of significant weaknesses or deficiencies in the protester's proposal
+- Overall evaluated cost/price and technical rating of the protester and the awardee (if applicable)
+- Overall ranking of all offerors (if a ranking was created)
+- Summary of rationale for award
+- Reasonable responses to relevant questions
+**NIH Stay Provision Tie-in:** The CICA stay clock (see below) specifically references "5 calendar days after the debriefing date offered" as an alternative trigger for the stay, meaning debriefing timing is not just a protest rights issue — it affects NIH's operational options.
+---
+### 5. Filing Requirements (4 C.F.R. § 21.1)
+The protest **must be filed in GAO's Electronic Protest Docketing System (EPDS)** at `epds.gao.gov`. A complete protest filing must include:
+1. Protester's name, address, email, phone/fax
+2. Electronic signature
+3. Agency name, solicitation/contract number
+4. **Detailed statement of legal and factual grounds** (including copies of relevant documents)
+5. Information establishing interested party status
+6. Information establishing timeliness
+7. Specific request for ruling by the Comptroller General
+8. Form of relief requested
+**A complete copy must be furnished to the CO (or designated protest recipient) no later than 1 day after filing with GAO.**
+&gt; ⚠️ **Per GAO Decision B-419956.258 (Optimo IT, involving NIH CIO-SP4):** Email to protests@gao.gov is **NOT a valid filing** unless EPDS is experiencing a confirmed system-wide outage. A filing 10 minutes past the 5:30 PM EPDS deadline was dismissed. There are no grace periods or equitable exceptions.
+---
+### 6. CICA Automatic Stay — What Happens After Filing
+Under CICA (31 U.S.C. § 3553), when GAO receives a protest filed **within 10 calendar days of contract award** (or **within 5 calendar days after the debriefing date offered**, whichever is later):
+- **Pre-award:** Award is **automatically stayed** pending GAO's decision
+- **Post-award:** Contract performance is **automatically suspended** pending GAO's decision
+**NIH/HHS may override the stay**, but only through a formal Determination &amp; Findings (D&amp;F) process under NIH Manual 6033-2:
+| Override Type | Standard | Approval Level |
+|---|---|---|
+| **Pre-award (GAO protest)** | Urgent and compelling circumstances + award likely within 30 days | HCA (non-delegable) **+ DASAMP, OS, DHHS approval** |
+| **Post-award (GAO protest)** | Performance in best interests of U.S. **or** urgent and compelling circumstances | HCA (non-delegable) **+ DASAMP, OS, DHHS approval** |
+| **Pre-award (agency protest)** | Urgent/compelling or best interest of Government | CO, with PCO + OGC-GLD concurrence |
+| **Post-award (agency protest)** | Urgent/compelling or best interest | HCA approval |
+The routing chain for a GAO protest stay override at NIH is: **CO → IC Director of Acquisitions → NIH PCO → HCA → DASAMP (HHS)**. This is a multi-day process — mission criticality must be pre-documented in the acquisition plan to support it.
+---
+### 7. GAO Decision Timeline (4 C.F.R. § 21.9)
+| Track | Decision Issued |
+|---|---|
+| Standard | ≤ **100 calendar days** after protest filed |
+| Express Option | ≤ **65 calendar days** (must request within 5 days of filing; agency report due in 20 days; comments due in 5 days) |
+Under the standard track: Agency report due in **30 days**; protester comments due **10 days** after report.
+**Failure to file timely comments = mandatory dismissal of the protest** (no exceptions per B-419956.258).
+---
+### 8. NIH Internal Response Timeline (NIH Manual 6033-1)
+Once the CO receives a GAO protest notice:
+| Action | Deadline |
+|---|---|
+| Complete protest file (all docs except CO Statement) → 4 copies to OGC-GLD (DPCO) + 1 to NIH PCO | **5 calendar days** |
+| CO's Statement of Facts and Circumstances | **14 calendar days** |
+| OGC-GLD submits complete Agency Report to GAO | **30 calendar days** |
+| **Litigation hold imposed on ALL relevant records** | **Immediately upon receipt** |
+Files marked: *"Immediate Action – GAO Protest B – [case number]"*
+---
+### 9. Possible Outcomes
+| Outcome | Meaning | Potential Relief |
+|---|---|---|
+| **Dismiss** | Procedural defect (untimely, no standing, SBA jurisdiction, etc.) | None |
+| **Deny** | Agency complied with law, or violation did not prejudice protester | None |
+| **Sustain** | Agency violated statute/regulation and protester was prejudiced | Recompete, new evaluation, terminate contract, award to protester, **cost reimbursement (including attorney fees)** |
+**Cost reimbursement caveat:** If the agency takes voluntary corrective action *after* the report due date on a clearly meritorious protest, GAO may recommend cost reimbursement. If the agency acts *by* the report due date, no costs are recommended.
+---
+### 10. Summary: Action Checklist for the Eliminated SBIR Phase II Offeror
+- [ ] **Confirm GAO jurisdiction** — was Phase II conducted under FAR Part 15 competitive procedures?
+- [ ] **Confirm interested party status** — would you be next in line for award?
+- [ ] **Request debriefing immediately** — within 3 days of elimination notice (FAR 15.505 or 15.506 as applicable)
+- [ ] **Identify all protest grounds before or during debriefing**
+- [ ] **File at GAO within 10 calendar days after debriefing**
+- [ ] **Use EPDS only** — file well before 5:30 PM, do not wait until the deadline day
+- [ ] **Serve complete copy on CO** within 1 day of GAO filing
+- [ ] **File comments on Agency Report within 10 calendar days** of report — mandatory, no exceptions
+---
+*Sources: All five documents fully retrieved from `eagle-knowledge-base/approved/legal-counselor/protest-guidance/`. GAO citations: 4 C.F.R. Part 21; 31 U.S.C. §§ 3551–3556; FAR 33.104; HHSAR 333.104; NIH Manual Chapters 6033-1, 6033-2; GAO Decision B-419956.258 (NIH CIO-SP4, June 21, 2023).*
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE-77</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>Template Path</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Generate a Statement of Work for a $200,000 annual IT help desk support contract for the NCI Center for Biomedical Informatics and Information Technology (CBIIT). Requirements: 5 FTEs providing Tier 1-3 support, 24/7 coverage, SLA of 15-minute response for Tier 1. Before generating, identify which SOW template from the knowledge base you will use and show its full S3 path in your reasoning.</t>
+        </is>
+      </c>
+      <c r="AD14" s="20" t="inlineStr">
+        <is>
+          <t>[RERUN] Tools: create_document | Response: Generated a draft sow document. You can open it from the document card. | ISSUE: Agent generated SOW correctly but did NOT show template name or S3 path before generating. This confirms EAGLE-77 is still open.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V9 baseline: dynamic questions, HTML report, 250/260 across 13 questions
- run_baseline.py reads questions from Excel dynamically (not hardcoded 6)
- generate_report.py supports any number of questions, labels "read" not "cited"
- SKILL.md adds Phase 4 (HTML report generation) as mandatory step
- V9 results: 117/120 Q1-Q6 (+1 vs V8), 133/140 Q7-Q13 (new questions)
- Q2 source gap closed: 0→2 KB docs via subagent tracking (f0d5060)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Use Case List.xlsx
+++ b/Use Case List.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline questions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <pivotCaches>
     <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="0" r:id="rId4"/>
   </pivotCaches>
@@ -54,12 +54,6 @@
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
       <scheme val="minor"/>
@@ -85,11 +79,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -122,14 +122,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
-        <bgColor rgb="00C00000"/>
+        <fgColor rgb="FFC00000"/>
+        <bgColor rgb="FFC00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E7D32"/>
+        <bgColor rgb="FF2E7D32"/>
       </patternFill>
     </fill>
     <fill>
@@ -166,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -192,13 +198,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -207,7 +213,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="1" quotePrefix="0" xfId="0"/>
@@ -217,17 +223,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1184,7 +1193,8 @@
     <col width="15.453125" customWidth="1" style="5" min="1" max="1"/>
     <col width="7.7265625" customWidth="1" style="10" min="2" max="2"/>
     <col width="49.453125" customWidth="1" style="10" min="3" max="3"/>
-    <col width="33" customWidth="1" style="5" min="4" max="16384"/>
+    <col width="33" customWidth="1" style="5" min="4" max="4"/>
+    <col width="33" customWidth="1" style="5" min="5" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.5" customFormat="1" customHeight="1" s="2">
@@ -3158,7 +3168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ14"/>
+  <dimension ref="A1:AX14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.26953125" defaultRowHeight="70" customHeight="1"/>
   <cols>
     <col width="9.26953125" customWidth="1" style="5" min="1" max="3"/>
@@ -3166,35 +3176,33 @@
     <col width="110.453125" customWidth="1" style="5" min="5" max="5"/>
     <col width="14.81640625" customWidth="1" style="5" min="6" max="6"/>
     <col width="80.453125" customWidth="1" style="5" min="7" max="7"/>
-    <col width="9.26953125" customWidth="1" style="5" min="8" max="16384"/>
+    <col width="9.26953125" customWidth="1" style="5" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="80" customWidth="1" min="14" max="14"/>
-    <col width="100" customWidth="1" min="15" max="15"/>
-    <col width="100" customWidth="1" min="16" max="16"/>
+    <col width="100" customWidth="1" min="15" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="100" customWidth="1" min="22" max="22"/>
-    <col width="100" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="100" customWidth="1" min="29" max="29"/>
-    <col width="100" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
-    <col width="14" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-    <col width="14" customWidth="1" min="35" max="35"/>
-    <col width="100" customWidth="1" min="36" max="36"/>
+    <col width="100" customWidth="1" min="22" max="23"/>
+    <col width="14" customWidth="1" min="24" max="28"/>
+    <col width="100" customWidth="1" min="29" max="30"/>
+    <col width="14" customWidth="1" min="31" max="35"/>
+    <col width="100" customWidth="1" min="36" max="37"/>
+    <col width="14" customWidth="1" min="38" max="42"/>
+    <col width="100" customWidth="1" min="43" max="43"/>
+    <col width="100" customWidth="1" style="5" min="44" max="16384"/>
+    <col width="14" customWidth="1" min="45" max="45"/>
+    <col width="14" customWidth="1" min="46" max="46"/>
+    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="14" customWidth="1" min="48" max="48"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="100" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1" ht="70" customFormat="1" customHeight="1" s="2">
@@ -3376,6 +3384,76 @@
       <c r="AJ1" s="22" t="inlineStr">
         <is>
           <t>v7 vs v6 Comparative Judgment</t>
+        </is>
+      </c>
+      <c r="AK1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V8 Response (2026-04-06)</t>
+        </is>
+      </c>
+      <c r="AL1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V8 Accuracy (0-5)</t>
+        </is>
+      </c>
+      <c r="AM1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V8 Completeness (0-5)</t>
+        </is>
+      </c>
+      <c r="AN1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V8 Sources (0-5)</t>
+        </is>
+      </c>
+      <c r="AO1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V8 Actionability (0-5)</t>
+        </is>
+      </c>
+      <c r="AP1" s="22" t="inlineStr">
+        <is>
+          <t>EAGLE V8 Total (0-20)</t>
+        </is>
+      </c>
+      <c r="AQ1" s="22" t="inlineStr">
+        <is>
+          <t>V8 vs RO + V7 Comparative Judgment</t>
+        </is>
+      </c>
+      <c r="AR1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V9 Response (2026-04-06)</t>
+        </is>
+      </c>
+      <c r="AS1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V9 Accuracy (0-5)</t>
+        </is>
+      </c>
+      <c r="AT1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V9 Completeness (0-5)</t>
+        </is>
+      </c>
+      <c r="AU1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V9 Sources (0-5)</t>
+        </is>
+      </c>
+      <c r="AV1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V9 Actionability (0-5)</t>
+        </is>
+      </c>
+      <c r="AW1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V9 Total (0-20)</t>
+        </is>
+      </c>
+      <c r="AX1" s="23" t="inlineStr">
+        <is>
+          <t>V9 vs RO + V8 Comparative Judgment</t>
         </is>
       </c>
     </row>
@@ -3623,6 +3701,98 @@
 Cascade: Q1 uses compliance matrix directly, no KB cascade needed. No change.
 Source gaps: None -- matrix is authoritative for thresholds.
 Verdict: Equivalent. Both answer the specific question completely.</t>
+        </is>
+      </c>
+      <c r="AK2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under **FAC 2025-06** (effective October 1, 2025), the two key thresholds are:
+| Threshold | Amount | FAR Reference |
+|---|---|---|
+| **Micro-Purchase Threshold (MPT)** | **$15,000** | FAR 2.101 / FAR 13.2 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 2.101 / FAR 13.3 |
+**A few important MPT exceptions:**
+- **Construction:** $2,000 (Davis-Bacon applies above this)
+- **Services subject to the Service Contract Act:** $2,500
+- **Contingency operations:** $25,000
+**A few important SAT extensions:**
+- **Commercial items (simplified test):** $7.5M
+- **Commercial items (certain acquisitions):** $15M
+**Practical implications:**
+- **Under $15K** → No competition required; use purchase card or micro-purchase order (FAR 13.202)
+- **$15K–$350K** → Simplified acquisition procedures apply; competition generally required
+- **Above $350K** → Full competition and written acquisition plan requirements kick in
+Let me know if you need guidance on a specific acquisition scenario.
+</t>
+        </is>
+      </c>
+      <c r="AL2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN2" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP2" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="AQ2" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V8 = RO (comparable)
+RO comparison: Both correctly cite $15K MPT, $350K SAT under FAC 2025-06. V8 adds MPT exceptions (construction $2K, SCA $2.5K, contingency $25K) and SAT extensions ($7.5M/$15M commercial) that RO omits. RO includes HHS-specific practical notes (HHS-653 form) not in V8.
+V7 vs V8: Essentially identical quality. V8 slightly longer (1001 vs 711 chars) with more practical implications section.
+Tools: v7=query_compliance_matrix | v8=query_compliance_matrix (unchanged)
+Cascade effect: N/A -- threshold lookup via compliance matrix, no KB cascade needed.
+Source gap: RO cites HHS PMR Threshold Matrix file path; V8 cites FAR references but no KB file path. Minor gap.
+Verdict: Stable, no regression. V8 matches RO accuracy with better exception coverage.</t>
+        </is>
+      </c>
+      <c r="AR2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under **FAC 2025-06** (effective October 1, 2025):
+| Threshold | Amount | FAR Reference |
+|---|---|---|
+| **Micro-Purchase Threshold (MPT)** | **$15,000** | FAR 2.101 / FAR 13.2 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 2.101 / FAR 13.3 |
+**A few important MPT nuances:**
+- **Construction:** $2,000 (Davis-Bacon applies above this)
+- **Services subject to the Service Contract Act:** $2,500
+- **Contingency operations:** $25,000
+**SAT commercial item extensions:**
+- Commercial items (simplified test): up to **$7.5M**
+- Certain commercial items (special test): up to **$15M**
+At or below the MPT, competition is not required (FAR 13.202(a)). Above the SAT, full and open competition requirements under FAR Part 6 apply. Let me know if you need anything else.
+</t>
+        </is>
+      </c>
+      <c r="AS2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU2" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW2" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="AX2" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 = RO (comparable)
+RO comparison: Both correctly cite $15K MPT, $350K SAT under FAC 2025-06. V9 adds MPT exceptions (construction $2K, SCA $2.5K, contingency $25K) and SAT commercial extensions ($7.5M/$15M). RO adds practical notes about HHS-653 form and CPARS requirements.
+v8 vs v9: Identical response quality. No change in tool usage or output.
+Tools: v8=[query_compliance_matrix] | v9=[query_compliance_matrix]
+Cascade: N/A -- threshold lookup, no KB cascade needed.
+KB docs cited: V8=0 | V9=0 (unchanged, expected for compliance_matrix queries)
+Verdict: Stable -- compliance matrix tool delivers accurate threshold data.</t>
         </is>
       </c>
     </row>
@@ -3974,6 +4144,140 @@
 Tools: v6=knowledge_search,web_search,web_fetch | v7=knowledge_search,legal_counsel
 Cascade: v6 web-fetched actual decision; v7 used legal_counsel subagent instead. Both valid approaches. Minor sources deduction for not fetching original text.
 Verdict: Comparable. v7 loses 1pt on sources (no web fetch of GAO decision) but gains structured legal analysis from subagent.</t>
+        </is>
+      </c>
+      <c r="AK3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## GAO B-302358 — *Bureau of Customs and Border Protection* (Dec. 27, 2004)
+Two holdings, both still good law:
+---
+### Holding 1 — IDIQ ≠ Multiyear Contract
+The ACE contract was an IDIQ under FAR 16.504, **not** a multiyear contract subject to 41 U.S.C. § 254c. GAO held the two are **mutually exclusive instruments** — a single contract cannot satisfy both sets of requirements. Critically, the label on the contract doesn't control; the operative terms do. (*Crown Laundry and Dry Cleaners v. United States*, 29 Fed. Cl. 506 (1993).)
+---
+### Holding 2 — Minimum Must Be Obligated at Award *(the operationally significant one)*
+Under **31 U.S.C. § 1501(a)(1)** (the Recording Statute), an agency **must obligate the IDIQ minimum guarantee at the moment of contract execution** — not when the first task order is issued.
+CBP awarded a $25M minimum / $5B maximum IDIQ to IBM and waited five months to record the minimum obligation. GAO held this was improper.
+---
+### The Two-Stage Obligation Framework Confirmed
+| Stage | Trigger | Appropriation Charged |
+|---|---|---|
+| **Minimum guarantee** | Contract award/execution | FY of contract award |
+| **Orders above minimum** | Each individual task/delivery order | FY the order is placed |
+This two-stage model was anchored in *60 Comp. Gen. 219 (1981)* and the GAO Red Book, Vol. II, Ch. 7.
+---
+### Key Practical Rules for COs
+1. **Verify funds are available** in the amount of the minimum *before* signing the IDIQ
+2. **Record the obligation immediately** at execution — waiting for the first task order is a recording statute violation
+3. **Labels don't control** — if the contract functions as an IDIQ (FAR 52.216-22 included, order-based structure), it *is* an IDIQ regardless of what the cover page says
+4. **Multiple-award IDIQs**: each awardee's individual minimum must be separately funded and recorded at award
+---
+### ADA Disposition
+GAO did **not** find an Antideficiency Act violation on these facts because CBP had sufficient budget authority when it eventually recorded the obligation. But GAO issued a formal recommendation to implement controls — making clear that if funds had been *unavailable* at award, an ADA violation would have ripened.
+---
+**Relevant authorities:** 31 U.S.C. § 1501(a)(1); 31 U.S.C. § 1341 (ADA); FAR 16.504; FAR 52.216-22; OMB Circular A-11 § 20.5(c); GAO Red Book Vol. II, Ch. 7.
+</t>
+        </is>
+      </c>
+      <c r="AL3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN3" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP3" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="AQ3" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V8 = RO (comparable)
+RO comparison: Both correctly identify both holdings -- IDIQ minimum obligation at award (31 USC 1501(a)) and IDIQ != multiyear (41 USC 254c). V8 adds ADA disposition analysis and Crown Laundry citation beyond RO. RO includes more specific remedies detail (deobligate $955K, re-obligate from FY03).
+V7 vs V8: Same tools and quality. V8 slightly shorter (2389 vs 3003 chars) but equally comprehensive with cleaner table formatting.
+Tools: v7=knowledge_search,legal_counsel | v8=knowledge_search,legal_counsel (unchanged)
+Cascade effect: legal_counsel subagent engaged -- deep research path working correctly.
+Source gap: RO cites specific KB file paths (GAO_B-302358_IDIQ_Min_Fund.txt, appropriations_law_IDIQ_funding.txt); V8 cites legal authorities but no KB file paths. Minor gap.
+Verdict: Stable, comprehensive analysis with good two-stage obligation framework table.</t>
+        </is>
+      </c>
+      <c r="AR3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## GAO B-302358 — *Bureau of Customs and Border Protection* (Dec. 27, 2004)
+This is a foundational fiscal law decision on IDIQ minimum guarantees. Here's what GAO held:
+---
+### Two Core Holdings
+**1. IDIQ ≠ Multiyear Contract**
+GAO held that the ACE contract (IBM Global Services, $25M min / $5B max) was an **IDIQ contract, not a multiyear contract under 41 U.S.C. § 254c**, despite spanning multiple years. Contract *type* is determined by **substance, not labels** — the presence of FAR 52.216-22, indefinite quantities, and ordering procedures per FAR 16.504 controlled. The inclusion of a multiyear cancellation clause (FAR 52.217-2) was attributed to "imprecise usage" and didn't change the contract's legal character.
+**2. The Minimum Guarantee Must Be Obligated at Contract Award**
+This is the decision's most-cited holding. GAO held under **31 U.S.C. § 1501(a)(1)** (the Recording Statute):
+&gt; *"When an agency executes an indefinite-quantity contract such as an IDIQ contract, the agency must record an obligation in the amount of the required minimum purchase... At the time of award, the government has a fixed liability for the minimum amount to which it committed itself."*
+CBP had waited 5 months (until it issued task orders on September 28, 2001) before recording the $25M minimum. That violated the Recording Statute.
+---
+### The Creating vs. Recording Distinction
+| Concept | What Happened |
+|---|---|
+| **Creating the obligation** | Occurred at award (April 27, 2001) — CBP was legally bound for $25M |
+| **Recording the obligation** | Did NOT occur until September 28, 2001 — **5 months late** |
+GAO confirmed: failing to *record* doesn't extinguish the obligation — it still exists from the day of award. But the recording failure is a statutory violation.
+**Why no Antideficiency Act violation here:** CBP used **no-year funds** (available until expended), so there was no lapse risk. Had they used **annual (1-year) appropriations**, the failure to record the minimum at award could have been an ADA violation under 31 U.S.C. § 1341 if the fiscal year closed before recording.
+---
+### Fiscal Year Charging Rule for Subsequent Orders
+GAO reaffirmed the rule for orders placed after award:
+&gt; *"Further obligations occur as task or delivery orders are placed and are chargeable to the fiscal year in which the order is placed."* (citing 60 Comp. Gen. 219 (1981))
+So:
+- **Minimum guarantee** → obligated and charged to appropriations **available at contract award**
+- **Each task/delivery order** → obligated and charged to appropriations **available when the order is placed**
+---
+### FAR 16.504(b) Framework Validated
+The decision grounds in **FAR 16.504(b)**, which requires:
+1. The minimum must **exist** — no minimum = no binding contract (contract lacks consideration)
+2. The minimum must be **more than nominal** — a token $1 minimum is challengeable
+3. The minimum **should not exceed** what the Government is fairly certain to order
+---
+### Practitioner Takeaways
+| Risk | Severity |
+|---|---|
+| Nominal/illusory minimum ($1) | **HIGH** — contract lacks consideration, protestable |
+| Failing to obligate minimum on Day 1 (annual funds) | **HIGH** — potential ADA violation |
+| Including FAR 52.217-2 in an IDIQ contract | **MEDIUM** — clause mismatch creates legal ambiguity |
+| Using sole-source minimum guarantee exception (FAR 16.505(b)(2)(i)(D)) as pretext | **MEDIUM** — protestable |
+---
+**Bottom line:** *B-302358* stands for the proposition that the **IDIQ minimum guarantee creates a legally binding obligation at the moment of contract execution** — it must be recorded immediately against a currently available appropriation. Every CO awarding an IDIQ should obligate the minimum on Day 1.
+&gt; **Sources:** GAO B-302358 (Dec. 27, 2004); FAR 16.504(b); 31 U.S.C. § 1501(a)(1); 31 U.S.C. § 1341; 60 Comp. Gen. 219 (1981); KB: `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_16_Contract_Types_Guidance.txt`
+</t>
+        </is>
+      </c>
+      <c r="AS3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW3" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX3" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved)
+RO comparison: Both correctly cover the two core holdings (IDIQ != multiyear, minimum obligation at award). V9 adds: creating vs recording distinction table, ADA analysis with no-year vs annual funds scenario, and cites 2 KB document paths.
+v8 vs v9: SOURCE CITATION IMPROVEMENT -- V8 cited 0 KB document paths (legal_counsel subagent read docs internally but paths were not surfaced). V9 now cites 2 KB paths: FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt and FC_16_Contract_Types_Guidance.txt. This is the direct result of the subagent KB tracking feature (commit f0d5060).
+Tools: v8=[knowledge_search, legal_counsel] | v9=[knowledge_search, legal_counsel]
+Cascade: legal_counsel subagent fetched KB docs in both versions, but V9 now surfaces the paths in the supervisor response.
+Source gap: CLOSED -- V8 had 0 KB paths vs RO's 2; V9 now matches with 2 KB paths.
+KB docs cited: V8=0 | V9=2 (+2 improvement)
+Verdict: Key improvement -- subagent KB document reads now visible. Sources 4-&gt;5.</t>
         </is>
       </c>
     </row>
@@ -4481,6 +4785,175 @@
 Verdict: Equivalent. v7's IT gray zone table is a strong practical addition. Both 20/20.</t>
         </is>
       </c>
+      <c r="AK4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's how the severable/non-severable distinction drives fiscal year funding obligations:
+---
+## Severable vs. Non-Severable: The Fiscal Year Funding Rule
+The entire analysis flows from the **Bona Fide Needs Rule** — 31 U.S.C. § 1502(a) — which requires that an appropriation fund only the needs that arise during its period of availability.
+---
+### Non-Severable Services — Fund Once, from the Year You Award
+A **non-severable** contract is a **single undertaking**: interdependent tasks building toward one end product, where the value derives from complete performance, not from any particular time slice.
+**Rule:** The entire bona fide need arises when the contract is *entered*, so the entire contract value is obligated from the appropriation current at award — even if performance runs into a later fiscal year.
+**Example:** $600K system audit awarded Sept. 15, FY25. Final report due March FY26. → Obligate all $600K from FY25 funds. No incremental funding required.
+**Common examples:** Feasibility studies, program evaluations, audits, custom software development, A/E design, specific litigation support, one-time training programs.
+---
+### Severable Services — Fund Each Year with That Year's Money
+A **severable** contract consists of **recurring, independent units** of service — each period's work has standalone value regardless of other periods.
+**Rule:** Each fiscal year's services are a separate bona fide need of that year. You **cannot** obligate FY25 funds for services performed in FY26. Incremental funding is required.
+**Example:** $1.2M help desk contract (Oct FY25 – Sept FY26, $100K/month):
+- FY25 funds: $300K (Oct–Dec)
+- FY26 funds: $900K (Jan–Sept)
+- ❌ Cannot obligate all $1.2M from FY25
+**Common examples:** Maintenance, janitorial, guard services, systems administration, SaaS subscriptions, ongoing IT support, most O&amp;M contracts.
+---
+### The Short Bridge Exception
+For **severable** services only — if a contract crosses a fiscal year boundary by a **short period** (typically 1–3 months) to avoid a service gap, the entire amount may be funded from the current fiscal year's appropriation.
+**Example:** 3-month systems admin contract, Aug 1 – Oct 31, FY25. → Entire amount may be funded from FY25 funds despite one month of FY26 performance.
+---
+### Multi-Year / No-Year Appropriations — Different Story
+The incremental funding restriction on severable services **applies only to annual (1-year) appropriations**. Per GAO B-317636, if the contract is funded by **multi-year or no-year appropriations**, the 1-year crossing restriction does not apply — the agency may contract for the full period the appropriation allows. (Statutory basis: 41 U.S.C. § 253l for civilian agencies.)
+---
+### Non-Severable + Cost-Reimbursement: Full Obligation at Award
+GAO B-317139 (*FinCEN, BSA Direct*, 2009) is the leading case here. A non-severable cost-reimbursement contract **must be fully obligated at award** — you cannot incrementally fund it via a limitation-of-funds clause. FinCEN obligated only $2M of an $8.98M CPFF contract at award, then charged the remainder to FY05 funds. GAO ruled this violated the bona fide needs rule and required restatement of accounts (and potential Antideficiency Act reporting).
+---
+### Critical Errors to Avoid
+| Common Misconception | Correct Rule |
+|---|---|
+| "All service contracts are severable" | Many are non-severable — studies, audits, specific projects |
+| "If performance crosses FY boundaries, it must be severable" | Non-severable contracts routinely cross FY boundaries |
+| "We can label it non-severable to simplify funding" | Severability is determined by the **nature of services**, not contract language |
+| "Severability is a FAR issue" | It's an **appropriations law** issue (31 U.S.C. § 1502(a)); FAR 37.106 and 32.703-3 implement it |
+---
+### Applicable FAR Provisions
+- **FAR 32.703-2/32.703-3** — Contracts crossing fiscal years, availability of funds
+- **FAR 37.106** — Funding for service contracts by annual appropriations
+- **FAR 52.232-19** — Availability of Funds for the Next Fiscal Year (severable contracts)
+- **FAR 52.232-22** — Limitation of Funds (cost-reimbursement, severable)
+---
+**Sources:**
+- GAO Red Book, Chapter 5 — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- Bona Fide Needs Rule — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- GAO B-317636; GAO B-317139 — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+</t>
+        </is>
+      </c>
+      <c r="AL4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AQ4" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V8 &gt; RO (improved)
+RO comparison: V8 covers all RO content and adds: short bridge exception, multi-year/no-year appropriations (GAO B-317636), non-severable + cost-reimbursement case (GAO B-317139), FAR provisions table. V8 cites 3 specific KB file paths matching RO citation depth.
+V7 vs V8: Same tool (research) and same quality. V8 slightly longer (4652 vs 4446 chars) with richer edge case coverage.
+Tools: v7=research | v8=research (unchanged)
+Cascade effect: Research tool (composite: auto-search + auto-fetch) working correctly -- full document reads producing rich analysis.
+Source gap: CLOSED. V8 cites all 3 relevant KB files (appropriations_law_severable_services.txt, appropriations_law_time_bona_fide_needs.txt, Contract_Obligation_Timing_GAO_Guidance.txt).
+Verdict: Exceptional -- exceeds RO with additional edge cases and GAO case law citations.</t>
+        </is>
+      </c>
+      <c r="AR4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the authoritative breakdown, sourced from GAO Red Book Chapter 5 and confirmed GAO decisions:
+---
+## Severable vs. Non-Severable: Fiscal Year Funding Consequences
+The distinction controls **which fiscal year's appropriation must fund the contract** — it's an appropriations law issue, not a FAR contracting method issue.
+---
+### The Underlying Rule
+**31 U.S.C. § 1502(a) — Bona Fide Needs Rule:** An appropriation is available only for needs that arise during its period of availability. The severable/non-severable determination tells you *when* the need arises.
+---
+### Non-Severable Services — "Single Undertaking"
+**Definition:** A unified effort that cannot be separated into discrete components without losing its essential character or value. The value comes from complete performance, not from incremental portions.
+**Funding Rule:** The entire bona fide need arises **when the contract is entered**. Fund the full contract value from the appropriation current at award — even if performance spans multiple fiscal years.
+**Examples:** Feasibility studies, audits, program evaluations, custom software development, A/E design, specific training courses, litigation support, system integrations.
+&gt; *Concrete example:* $600K system audit, awarded Sept. 15 FY25, final report due March FY26. Obligate the full $600K from FY25 appropriations. ✅
+---
+### Severable Services — "Recurring/Continuing"
+**Definition:** Ongoing or recurring services where each time period's performance has independent value — services can be logically divided by time period.
+**Funding Rule:** Each fiscal year's services are a **separate bona fide need** of that fiscal year. You must fund each year's services with that year's appropriation — incremental funding is required when the contract crosses fiscal years.
+**Examples:** Help desk support, maintenance, guard services, janitorial, systems administration/monitoring, SaaS subscriptions, ongoing IT O&amp;M.
+&gt; *Concrete example:* $1.2M help desk contract, Oct FY25 – Sep FY26. You must fund:
+&gt; - FY25 appropriations: $300K (Oct–Dec FY25, 3 months)
+&gt; - FY26 appropriations: $900K (Jan–Sep FY26, 9 months)
+&gt; Cannot obligate the full $1.2M from FY25 funds. ❌
+---
+### Key Exceptions
+**Short Bridge Exception:** A severable services contract that crosses into the next FY by a short period (typically 1–3 months) may be fully funded from the current year when necessary to avoid a service gap. *(e.g., an Aug 1 – Oct 31 contract funded entirely from FY25 is acceptable.)*
+**Multi-Year / No-Year Appropriations (GAO B-317636):** The 1-year crossing restriction applies only to **annual appropriations**. Agencies using multi-year or no-year funds may contract for severable services for the full period of availability without the incremental funding requirement.
+---
+### The Four-Question Test (GAO Standard)
+&gt; *"Is this essentially a single undertaking, or a series of separate tasks?"*
+| Question | Non-Severable | Severable |
+|---|---|---|
+| Single unified deliverable? | Yes | No |
+| Tasks interdependent? | Yes, build toward unified goal | No, independent and repetitive |
+| Can work be divided by time period? | No | Yes |
+| Value from complete performance? | Yes | Each period has independent value |
+---
+### Common Errors
+| Misconception | Correction |
+|---|---|
+| "All service contracts are severable" | Many are non-severable — studies, audits, specific projects |
+| "If it crosses fiscal years, it must be severable" | Non-severable work routinely spans FYs; duration ≠ severability |
+| "IT contracts are always severable" | Ongoing O&amp;M = severable; specific implementations/migrations = non-severable |
+| "We can make it non-severable by drafting it that way" | Severability is determined by the *nature* of the services — cannot be manufactured through contract language to circumvent the bona fide needs rule |
+---
+### Contract Clauses for Severable Services (Cross-FY)
+- **FAR 52.232-22** — Limitation of Funds (cost-reimbursement)
+- **FAR 52.232-20** — Limitation of Cost (cost-reimbursement)
+- **FAR 52.232-19** — Availability of Funds for Next Fiscal Year
+- **FAR 37.106(a) / 32.703-3** — Contracts crossing fiscal years
+---
+**Bottom line:** If the work is a single undertaking → fully fund at award from the year you enter the contract. If the work is recurring → match each year's funding to that year's services. You cannot manufacture non-severability through contract drafting to avoid this constraint.
+---
+*Sources: GAO Red Book Ch. 5 (GAO-04-261SP) · GAO B-317636 (Apr. 21, 2009) · GAO B-317139 (June 1, 2009) · 31 U.S.C. § 1502(a) · FAR 32.703-3, 37.106*
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/regulatory-policies/appropriations_law_severable_services.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+</t>
+        </is>
+      </c>
+      <c r="AS4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX4" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved)
+RO comparison: V9 covers all RO content (severable/non-severable rules, bona fide needs, GAO legal standard). V9 adds: short bridge exception, multi-year/no-year appropriations, concrete dollar examples, and 4 KB document paths.
+v8 vs v9: Comparable quality. V9 cites 4 KB paths via research subagent tracking.
+Tools: v8=[research] | v9=[research]
+Cascade: Research subagent consistently triggers deep KB fetch.
+Source gap: CLOSED -- V9 matches or exceeds RO source coverage.
+KB docs cited: V8=4 | V9=4 (maintained)
+Verdict: Strong -- maintains V8 quality, research subagent KB tracking stable.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="100.75" customHeight="1">
       <c r="A5" s="5">
@@ -4805,6 +5278,127 @@
 Cascade: CASCADE WORKING -- both fetch full FAR Part 16 text after search. Identical pattern.
 Source gaps: Closed -- full FAR Part 16 text read before answering in both versions.
 Verdict: Equivalent. Both 20/20. Identical cascade behavior.</t>
+        </is>
+      </c>
+      <c r="AK5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **seven exceptions to fair opportunity** under **FAR 16.505(b)(2)(i)** that allow a sole-source task or delivery order under a multiple-award IDIQ contract:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | Exception | Key Requirement |
+|---|-----------|-----------------|
+| **(A)** | **Urgency** | The agency's need is so urgent that providing fair opportunity would result in unacceptable delays. |
+| **(B)** | **Unique/Highly Specialized** | Only one awardee is capable of providing the supplies or services at the level of quality required because they are unique or highly specialized. |
+| **(C)** | **Logical Follow-On** | The order must be issued on a sole-source basis for economy and efficiency because it is a logical follow-on to a prior order, *provided all awardees received fair opportunity on the original order*. |
+| **(D)** | **Minimum Guarantee** | It is necessary to place the order with a particular awardee to satisfy a minimum guarantee under that contract. |
+| **(E)** | **Statutory Authorization** | A statute expressly authorizes or requires the purchase from a specified source *(applies to orders exceeding the SAT)*. |
+| **(F)** | **Small Business Set-Aside** | Per FAR Part 19, the contracting officer may set aside the order for small business concerns — this exception is **not** subject to the J&amp;A, approval, or posting requirements. |
+| **(G)** | **DoD/NASA/Coast Guard — OTFAOC** | For DoD, NASA, and the Coast Guard only: the order satisfies one of the other-than-full-and-open-competition exceptions under FAR Part 6.103 (10 U.S.C. 3406(c)(5)). |
+---
+## Documentation &amp; Approval Requirements
+**Above MPT but ≤ SAT:** Written rationale documenting the basis for the exception (simplified — for logical follow-on, explain why it's "logical").
+**Above SAT:** Full written justification ("Justification for an Exception to Fair Opportunity") including:
+- Description of supplies/services and estimated value
+- Specific exception cited with supporting rationale
+- Price reasonableness determination
+- CO certification and approving official signature
+**Approval thresholds:**
+| Order Value | Approving Official |
+|-------------|-------------------|
+| &gt; SAT – $900K | Contracting Officer's certification suffices |
+| &gt; $900K – $20M | Advocate for Competition (non-delegable) |
+| &gt; $20M – $90M | Head of Procuring Activity (or SES/Flag Officer) |
+| &gt; $90M | Senior Procurement Executive (non-delegable) |
+**Posting:** Within **14 days** of award, post the justification to SAM.gov for a minimum of 30 days — *except* for urgency (Exception A), where posting is allowed within **30 days** after award.
+---
+**Key distinction:** Fair opportunity exceptions under FAR 16.505 are **not subject to FAR Part 6** competition requirements — they operate on a separate, lower statutory authority. Exception (F) (small business set-asides) is explicitly excluded from the J&amp;A/approval/posting requirements.
+&gt; **Source:** FAR Part 16 RFO (HHS Class Deviation 2026-01, effective Nov. 21, 2025) — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="AL5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP5" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AQ5" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V8 &gt; RO (improved)
+RO comparison: Column E contains Q4-relevant content (fair opportunity exceptions), not Q4 (fair opportunity). V8 correctly answers with all 7 FAR 16.505(b)(2)(i) exceptions including small business set-aside (Exception F) and DoD/NASA/Coast Guard OTFAOC (Exception G). Approval thresholds, posting requirements, and key distinction between FAR 16.505 and Part 6 all correct.
+V7 vs V8: Same tools and quality. V8 slightly longer (3164 vs 2902 chars). Both cite specific KB file (FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt).
+Tools: v7=search_far,knowledge_fetch | v8=search_far,knowledge_fetch (unchanged)
+Cascade effect: search_far -&gt; knowledge_fetch cascade working correctly. Full document fetch after search.
+Source gap: CLOSED. V8 cites FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt with full S3 key.
+Verdict: Top score -- comprehensive exception listing with complete approval/posting requirements.</t>
+        </is>
+      </c>
+      <c r="AR5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **seven exceptions to fair opportunity** under **FAR 16.505(b)(2)(i)** that permit a sole-source task or delivery order under a multiple-award IDIQ contract:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | Exception | Key Condition |
+|---|-----------|---------------|
+| **(A)** | **Urgency** | The agency's need is so urgent that providing fair opportunity would result in unacceptable delays |
+| **(B)** | **Unique / Highly Specialized** | Only one awardee is capable of providing the supplies or services at the required quality level because they are unique or highly specialized |
+| **(C)** | **Logical Follow-On** | Economy and efficiency require sole-source award as a logical follow-on to a prior order — *provided all awardees had fair opportunity on the original order* |
+| **(D)** | **Minimum Guarantee** | Necessary to satisfy the contract's minimum guarantee |
+| **(E)** | **Statutory Authorization** | A statute expressly authorizes or requires purchase from a specified source *(applies only to orders above the SAT)* |
+| **(F)** | **Small Business Set-Aside** | Order is set aside for small business concerns under FAR Part 19 — **not subject to** the justification, approval, and posting requirements that apply to (A)–(E) |
+| **(G)** | **DoD/NASA/Coast Guard — OTFAOC** | Order satisfies a FAR Part 6 exception to full and open competition (e.g., only one responsible source, unusual/compelling urgency) — **DoD, NASA, and Coast Guard only** |
+---
+## Documentation &amp; Approval Requirements
+These requirements apply to exceptions **(A)–(E) and (G)** — not to (F) small business set-asides:
+| Order Value | Justification Required | Approval Level |
+|-------------|------------------------|----------------|
+| Above MPT, ≤ SAT ($350K) | Written basis for exception; logical follow-on rationale if (C) | CO certification |
+| Above SAT, ≤ $900K | Formal written J&amp;A (9 required elements) | CO certification |
+| &gt; $900K – $20M | Formal written J&amp;A | Advocate for Competition *(non-delegable)* |
+| &gt; $20M – $90M | Formal written J&amp;A | Head of Procuring Activity (or SES/Flag Officer) |
+| &gt; $90M | Formal written J&amp;A | Senior Procurement Executive *(non-delegable)* |
+**Posting:** Justifications for orders above the SAT must be posted to SAM.gov within **14 days** of award (or **30 days** for urgency exception (A)).
+---
+## Key Distinctions from FAR Part 6
+Fair opportunity under FAR 16.505 is **not** full and open competition under FAR Part 6. The ordering process is exempt from Part 6, Part 14, and Part 15.3 competition requirements. Exception **(F)** (small business set-asides) carries **no J&amp;A or posting requirement** — it's the cleanest path to a single-awardee order when small business participation qualifies.
+---
+**Source:** FAR 16.505(b)(2)(i)(A)–(G) | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="AS5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW5" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX5" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved)
+RO comparison: RO column E contains Q4 content (fair opportunity exceptions), misaligned with Q4 question. V9 correctly answers with all 7 FAR 16.505(b)(2)(i) exceptions, verbatim statutory text, documentation/approval thresholds, and 1 KB path.
+v8 vs v9: Consistent quality. Both cite FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt.
+Tools: v8=[search_far, knowledge_fetch] | v9=[search_far, knowledge_fetch]
+Cascade: search_far -&gt; knowledge_fetch working correctly.
+KB docs cited: V8=1 | V9=1 (maintained)
+Verdict: Stable -- FAR search + fetch cascade reliable for regulatory questions.</t>
         </is>
       </c>
     </row>
@@ -5857,6 +6451,348 @@
 Verdict: Equivalent. Both 20/20. v7 adds web-verified primary sources and SBIR jurisdiction nuance.</t>
         </is>
       </c>
+      <c r="AK6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excellent. I now have all the source material needed. Let me deliver the full analysis.
+---
+# SBIR Elimination + Simultaneous Debriefing Request + Day-8 Protest: Complete Procedural Analysis
+---
+## I. The SBIR-Specific Procedural Context
+SBIR competitions are conducted under **FAR Part 15** (competitive negotiated acquisitions), which is what triggers the debriefing entitlement framework. The elimination of an offeror from a phased SBIR competition (e.g., exclusion from further consideration after Phase I screening, or exclusion from competitive range in Phase II) is functionally equivalent to a **competitive range exclusion** under FAR 15.204-1, making FAR 15.206 (preaward debriefings) and FAR 15.301 (postaward debriefings) directly applicable.
+One important threshold issue: **SBIR is not expressly exempted from Part 15 debriefing requirements**, and GAO has consistently applied the standard protest timeliness rules to SBIR protests. The agency must provide a debriefing when requested within the required timeframe.
+---
+## II. What Triggers the Debriefing Entitlement: Pre-Award vs. Post-Award
+This is the most consequential structural decision, and it must be resolved *before* the procedural sequence can run correctly.
+### Scenario A — Elimination Occurred BEFORE Award (Most Common in SBIR)
+In a phased SBIR competition, if the offeror was **excluded from the competitive range or further phases before any award was made**, the applicable provision is **FAR 15.206-2 (Preaward Debriefing)**.
+**Key rules under FAR 15.206-2:**
+- The excluded offeror must **request the debriefing within 3 days** after receipt of the exclusion notice.
+- The debriefing must be provided "as soon as practicable" — in practice, before award if feasible.
+- The offeror **may elect to delay** the preaward debriefing until after award; if so, it must include all post-award debriefing content (FAR 15.206-2). *Critically: this election may have significant protest timeliness consequences — see Section IV below.*
+- Content is limited: evaluation of significant elements of the offeror's proposal, summary of the rationale for elimination, and responses to procedural questions. **The agency cannot disclose** number/identity of other offerors, their content, rankings, or comparative evaluations.
+### Scenario B — Elimination Occurred AFTER Award (Less Common in SBIR)
+If the offeror was notified of elimination simultaneously with or after award notification, the applicable provision is **FAR 15.301 (Postaward Debriefing)**.
+- Request must be made **within 3 days** of the award notice per FAR 15.301-1.
+- Debriefing must be provided within **5 days** of the written request to the maximum extent practicable.
+- Content is substantially richer: overall evaluated cost/price and technical ratings of both the successful offeror and the debriefed offeror, overall ranking, summary rationale for award, past performance information, and responses to procedural questions.
+---
+## III. The Procedural Sequence for This Fact Pattern
+**Day 0** — Offeror receives written elimination notice (start of all clocks).
+**Day 3** — Deadline for the offeror to request a **preaward debriefing** (FAR 15.206-2) if the exclusion was pre-award, or a **postaward debriefing** (FAR 15.301-1) if elimination was post-award. The request was made (implied by the fact pattern), so the clock under the debriefing exception to GAO's 10-day rule is now engaged.
+**Day 8** — Offeror simultaneously:
+1. **Requests the debriefing** — This is timely if submitted within 3 days, and this fact pattern suggests the request came at Day 8. If the exclusion notice came at Day 0 and the debriefing request wasn't made until Day 8, **the debriefing request is untimely** under FAR 15.206-2/15.301-1.
+2. **Files the protest at GAO** — Submitted via EPDS before 5:30 p.m. Eastern.
+&gt; ⚠️ **Critical ambiguity in the fact pattern:** The question states the offeror "simultaneously requests a debriefing and files a protest on Day 8." If the debriefing request was not made until Day 8 (i.e., no earlier request), the request is **5 days late** under the 3-day requirement. This has cascading effects discussed below.
+---
+## IV. Protest Timeliness Analysis — The 10-Day Rule and the Debriefing Exception
+### The Default Rule
+Under **4 C.F.R. § 21.2(a)(2)** (GAO Bid Protest Regulations), a protest must be filed **not later than 10 calendar days** after the protester knew or should have known of the basis for protest.
+The offeror received the elimination notice on Day 0. By Day 8, the 10-day clock has been running for 8 days. **The protest is facially timely under the default rule** — it was filed within 10 days of when the basis was known (Day 0 elimination notice). Day 10 has not yet passed.
+### The Debriefing Exception
+FAR Part 15 competitive proposals trigger a special timeliness rule under **4 C.F.R. § 21.2(a)(2)** (the "debriefing exception"):
+- **A protest based on grounds known before or from the debriefing shall NOT be filed before the debriefing date offered.**
+- **It shall be filed not later than 10 days after the date on which the debriefing is held.**
+This exception serves two purposes: (1) it prevents premature protests before offerors have meaningful information, and (2) it provides additional time — the clock resets to 10 days from the debriefing date rather than 10 days from the elimination notice.
+**But there is a critical restriction:** The debriefing exception applies only when the debriefing is **timely requested and required.** Under FAR 15.301-1 (postaward): *"Protest deadlines are NOT extended when the Government merely accommodates an untimely request."*
+### The Untimely Request Problem
+If the debriefing request was not made until Day 8 (simultaneously with the protest), and the 3-day window had already passed:
+1. The agency is **not obligated to provide the debriefing** — FAR 15.206-2 and 15.301-1 both state untimely requests "need not" be honored.
+2. The agency **may** accommodate the request as a discretionary matter.
+3. But even if accommodated: **the 10-day protest clock does NOT reset to the debriefing date.** The debriefing exception under 4 C.F.R. § 21.2(a)(2) only extends timeliness for timely-requested, required debriefings — *not* for debriefings provided as a courtesy for late requests. (See FAR 15.301-1: "Protest deadlines are not extended when the Government accommodates an untimely request.")
+**Result under the untimely request scenario:** The Day 8 GAO protest is timely under the default 10-day rule (basis known Day 0, filed Day 8 = within 10 days). But the protester **loses the debriefing exception's benefit** — they cannot wait for the debriefing to file additional grounds and have those additional grounds protected by a new 10-day window from the debriefing date.
+### If the Request Was Timely (Within 3 Days)
+If the debriefing *was* requested within 3 days of the elimination notice (Days 0–3), and the protest filed on Day 8 is treated as filed *before* the debriefing:
+- GAO's rule states a protest **shall not be filed before the debriefing date offered** for grounds that are known from or before the debriefing. Filing at Day 8 without yet receiving the debriefing creates a **premature filing risk** for grounds that will be informed by the debriefing.
+- However, grounds **already fully known** from the elimination notice itself (e.g., improper evaluation criteria, procedural violations evident from the notice) can be protested at any time within the 10-day window — including before the debriefing.
+- For grounds that the protester will first learn from the debriefing, the proper approach is to wait for the debriefing and then file (or file a supplemental/amended protest) within 10 days of the debriefing date.
+**GAO has held** (consistent with *SMS Data Products Group, B-423341*): When an offeror files a timely protest within 10 days of debriefing *delivery*, the protest is not premature even if the offeror had not yet received responses to follow-up questions — provided the follow-up request itself was untimely. The debriefing is "concluded" on delivery when follow-up questions are untimely.
+---
+## V. The CICA Stay — How Debriefing Timing Controls It
+This is where the pre-award vs. post-award distinction becomes operationally critical for the agency.
+### The Statutory Stay Framework
+Under **CICA (31 U.S.C. § 3553)** and **FAR 33.104**, when GAO receives a protest, mandatory stay provisions apply within specific windows:
+**The CICA stay applies when GAO notifies the agency of the protest within:**
+- **10 calendar days after contract award**, OR
+- **5 calendar days after the debriefing date offered to the protester** for any debriefing required under FAR 15.505 or 15.506
+**Whichever is LATER** governs.
+*(Source: NIH Manual 6033-2; NIH Policy Manual 6033-2)*
+### Scenario Analysis: Pre-Award Protest (No Award Has Been Made)
+If the protest is filed at Day 8 and no award has yet been made:
+- The **pre-award CICA stay** applies: the agency must **withhold award** while the protest is pending at GAO.
+- The 10-day/5-day stay windows aren't directly relevant here — the stay is triggered by the pre-award protest notice from GAO, and the agency simply cannot proceed to award without either (a) waiting for GAO's decision or (b) obtaining a D&amp;F override.
+- **Override standard (FAR 33.104(b)):** Requires "urgent and compelling circumstances" that significantly affect U.S. interests AND award is likely within 30 calendar days of the written finding. This requires **HCA execution + DASAMP approval** at NIH/HHS per HHSAR 333.104(b)(1).
+### Scenario Analysis: Post-Award Protest (Award Already Made)
+If award has already been made and GAO notifies the agency:
+**The 10-day window:** GAO notified agency within 10 days of award → **mandatory stay of performance** applies. Agency must suspend contract performance.
+**The 5-day debriefing window (critical for this scenario):**
+- If a debriefing was timely requested and offered, the stay window extends to **5 calendar days after the debriefing date offered** — whichever is later than the 10-day post-award window.
+- If the debriefing hasn't been provided yet when the protest is filed (as here), the agency must calculate: when will/did the agency "offer" a debriefing date? The 5-day clock runs from the **date offered**, not the date held.
+&gt; **Practical consequence:** If the agency delays offering a debriefing date, it effectively extends the window during which a timely post-award protest can still trigger the mandatory stay. This incentivizes agencies to offer debriefings promptly — and is exactly why the FAR Companion Part 33 guidance warns: *"Avoid unnecessarily extending the protest window. Prepare to quickly provide debriefings when requested after award decisions."*
+**Override standard (FAR 33.104(c)):** Performance may continue if HCA determines (and DASAMP approves at NIH/HHS) that:
+- Performance is in the **best interests of the United States**, OR
+- **Urgent and compelling circumstances** will not permit waiting for GAO's decision.
+Full D&amp;F required, routed through IC Director → NIH PCO → HCA → DASAMP/OGC-GLD.
+---
+## VI. The Offeror's Strategic Choice: Pre-Award vs. Post-Award Debriefing Election
+Under FAR 15.206-2, when an offeror is excluded from competitive range **before award**, it can **elect to delay** the preaward debriefing until after award. If delayed, the debriefing must include all postaward content. This election has significant consequences:
+| Factor | Take Pre-Award Debriefing | Delay Until Post-Award |
+|--------|--------------------------|------------------------|
+| **Information received** | Limited (no comparative data) | Full (ratings, rankings, rationale for award) |
+| **Protest stay effect** | Pre-award stay stops award immediately | Post-award stay requires meeting 10/5-day windows |
+| **Protest timeliness** | 10 days from pre-award debriefing date | 10 days from post-award debriefing date |
+| **Protest grounds** | May be narrower (less info) | Broader grounds available (award-specific) |
+| **Risk** | May lock in limited grounds | Award made before protest filed — stay may not apply |
+| **Agency preference** | Faster resolution; award unimpeded | Debriefing stretches protest risk window |
+**The key risk of electing delay:** If award is made before the protester files, the protest becomes a post-award protest. The mandatory stay only applies if GAO notifies the agency within the 10/5-day windows. If the delayed debriefing occurs 30 days after award, for example, the 5-day window from the debriefing date offered would extend the stay window — but the 10-day post-award window would have already closed.
+---
+## VII. The Day 8 Simultaneous Filing — Step-by-Step Procedural Sequence
+Here is the correct procedural sequence for all parties from Day 0:
+| Day | Offeror | Agency/CO | GAO |
+|-----|---------|-----------|-----|
+| **0** | Receives elimination notice; 3-day debriefing request clock starts; 10-day protest clock starts | Issues written notice per FAR 15.206-1(a) | — |
+| **0–3** | **Must request debriefing** to preserve entitlement and debriefing exception to protest timeliness | Receives request; schedules debriefing "as soon as practicable" | — |
+| **8** | Simultaneously requests debriefing (potentially late) + files protest via EPDS (timely under default 10-day rule) | Must notify GAO attorney; assess whether stay applies; begin D&amp;F if override needed | Receives protest; determines filing valid; sends notice to agency |
+| **8–13** | Awaits debriefing; may file supplemental grounds within 10 days of debriefing | Provides debriefing within 5 days of written request (FAR 15.301-1); assess stay obligation | Protest docketed; notice sent to agency |
+| **~13–18** | 10-day window to file supplemental protest grounds from debriefing date (if debriefing timely requested) | Agency report due within **30 days** of GAO notice | 30-day clock for agency report running |
+| **~38** | Comments on agency report due within **10 days** of report filing | Agency report filed | Agency report received |
+| **~108** | — | — | **Decision due within 100 days** of protest filing (or 65 days under express option) |
+---
+## VIII. NIH/HHS-Specific Stay Override Process
+If the agency wishes to proceed notwithstanding the stay:
+**For GAO protests — mandatory routing per NIH Manual 6033-2:**
+1. CO prepares and signs D&amp;F (pre-award: urgent/compelling + award within 30 days; post-award: best interest or urgent/compelling)
+2. Routed through: **IC Director of Acquisitions → NIH Protest Control Officer (PCO) → HCA**
+3. HCA executes (authority **not redelegable**)
+4. Forwarded with request to **DASAMP, OS, DHHS** for approval (via OGC-GLD)
+5. OGC-GLD concurrence → DASAMP approval → OGC-GLD notifies GAO
+6. CO may proceed only upon receipt of notification
+**For agency protests (if protester filed with agency instead):**
+- Pre-award: CO authority after concurrence of activity's protest control officer and OGC-GLD
+- Post-award: HCA approval required
+- Routed: IC Director → NIH PCO → HCA
+---
+## IX. Summary: The Critical Legal Points
+1. **Day 8 GAO filing is timely** under the default rule (4 C.F.R. § 21.2(a)(2)) — filed within 10 days of known basis (Day 0 notice). No timeliness defect on the protest itself.
+2. **If the debriefing request was not made until Day 8**, it is **untimely** under FAR 15.206-2/15.301-1. The agency may accommodate it, but: (a) the debriefing exception's 10-day reset does not apply, and (b) the CICA stay windows are calculated from when a timely debriefing was "offered" — a late-requested, accommodated debriefing does not extend the stay clock.
+3. **If the debriefing request was made within 3 days** (Days 0–3), and the protest was filed at Day 8 *before* the debriefing was held, the protest is not premature for grounds already known — but for grounds that will emerge from the debriefing, the protester should file supplemental grounds within 10 days of the debriefing date.
+4. **Pre-award protest → mandatory stay of award.** Post-award protest → mandatory stay of performance if GAO notifies within 10 days of award OR 5 days of debriefing date offered, whichever is later.
+5. **Override at NIH requires DASAMP approval** — not just HCA execution. This is a hard HHS-specific requirement on top of CICA (HHSAR 333.104(b)(1) and (c)(2)).
+6. **Do not delay offering the debriefing date unnecessarily.** Every day the agency waits to offer a debriefing date after a timely request extends the outer boundary of when a stay-eligible post-award protest can be filed.
+---
+**Sources:**
+- FAR 15.206-2 (Preaward Debriefing), FAR 15.301-1 (Postaward Debriefing) — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Source_Selection_RFO_2025.txt`
+- 4 C.F.R. § 21.2(a)(2) — GAO Timeliness Rules; GAO Bid Protests Essential Guide — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt`
+- FAR 33.104(b) and (c) — CICA Stay Provisions; NIH Manual 6033-2 / NIH Policy Manual 6033-2 — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt`
+- FAR Companion Part 33 — Debriefing best practices — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt`
+- GAO B-423341 (*SMS Data Products*) — Enhanced debriefing timeliness and "concluded" debriefing analysis — `eagle-knowledge-base/approved/legal-counselor/case-law/evaluation/GAO_B-423341_ECP_Misleading_Discussions_Best_Value.txt`
+- 4 C.F.R. § 21.0(g), § 21.3(i) — EPDS filing requirements — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt`
+</t>
+        </is>
+      </c>
+      <c r="AL6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP6" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AQ6" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V8 &gt; RO (improved)
+RO comparison: V8 produces the most comprehensive SBIR protest analysis in the baseline suite (17,853 chars). Covers: SBIR/FAR Part 15 context, pre-award vs post-award debriefing (FAR 15.206-2 / 15.301), protest timeliness (10-day rule + debriefing exception under 4 CFR 21.2(a)(2)), CICA stay mechanics (31 USC 3553 / FAR 33.104), strategic election table, day-by-day procedural sequence, NIH/HHS-specific stay override process (DASAMP approval chain). Cites 6 specific KB file paths.
+V7 vs V8: V7 used 5 tools (including web_search/web_fetch); V8 uses 3 tools but produces longer response (17853 vs 13831 chars). V8 adds day-by-day procedural table and NIH-specific routing chain.
+Tools: v7=search_far,research,knowledge_fetch,web_search,web_fetch | v8=search_far,research,knowledge_fetch
+Cascade effect: Full cascade working -- search_far + research (composite) + knowledge_fetch all engaged.
+Source gap: CLOSED. V8 cites 6 KB files including GAO_Bid_Protests_Essential_Guide_for_COs.txt, NIH_6033_2_Stay_Provisions_Protests.txt, FC_33_Protests_Disputes_Appeals.txt.
+Verdict: Exceptional -- deepest analysis in the suite, exceeds RO with NIH-specific procedural detail.</t>
+        </is>
+      </c>
+      <c r="AR6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I now have comprehensive primary source text from the FAR Part 15 (RFO/FAR 2.0), NIH Manual 6033-2, GAO Bid Protests Essential Guide, and the FAR Companion Part 33. Here is the complete, authoritative analysis:
+---
+# SBIR Competition Elimination: Protest + Debriefing Procedural Analysis
+## The Situation
+- **Day 0:** Offeror receives written elimination notice from SBIR competition (excluded from competitive range or otherwise not selected pre-award)
+- **Day 8:** Offeror simultaneously (a) requests a debriefing and (b) files a GAO protest
+- **Debriefing:** Not yet provided
+There are two entirely distinct legal tracks operating simultaneously, and the interaction between them is the crux of the procedural analysis.
+---
+## TRACK 1: Debriefing Entitlement and Timing
+### Which FAR Provision Applies — 15.505 or 15.506?
+This is the threshold question. The answer controls the stay analysis.
+| Scenario | Applicable Provision |
+|---|---|
+| Offeror **excluded from competitive range** before award | **FAR 15.206-2** (Preaward Debriefing) |
+| Offeror in competitive range, award made to another | **FAR 15.301-1** (Postaward Debriefing) |
+&gt; **Note on FAR 2.0 numbering:** The current RFO/FAR 2.0 class deviation renumbers legacy FAR 15.505 → **15.206-2** (preaward) and FAR 15.506 → **15.301-1** (postaward). The legal content is substantively identical; the CICA statute and 4 C.F.R. § 21.2 still reference the preaward/postaward debriefing framework. Legacy citations (15.505/15.506) remain valid in most filed protests.
+For an **SBIR competition elimination**, the offeror has been cut before award — this is a **preaward debriefing** scenario under FAR 15.206-2 / legacy 15.505.
+### Debriefing Request Timeliness
+**FAR 15.206-2:** Request must be submitted **within 3 days** after receipt of the exclusion notice.
+The offeror requested on **Day 8** — **this is untimely under FAR 15.206-2.** An untimely preaward debriefing request need not be honored. The agency has discretion to decline or accommodate it.
+**Consequences of untimely preaward request:**
+- The offeror is no longer *entitled* to a preaward debriefing as of right
+- FAR 15.206-2 states: "Untimely requests need not be given preaward or postaward debriefing; offerors entitled to no more than one debriefing per proposal"
+- The agency *may* accommodate the request anyway, but any resulting debriefing does **not** extend protest deadlines (FAR 15.301-1: "Protest deadlines NOT extended when Government accommodates untimely request or delayed preaward debriefing")
+**Option to request delay until post-award (FAR 15.206-2):**
+An offeror may request that a preaward debriefing be delayed until after award. If delayed, it must include all information from the postaward debriefing. However, this election *affects protest timeliness* — see Track 2 below.
+---
+## TRACK 2: Protest Timeliness Analysis
+### The Governing Rule — 4 C.F.R. § 21.2(a)(2)
+The baseline: protests must be filed **not later than 10 calendar days** after the basis of protest was known or should have been known.
+**Day 8 filing is therefore timely** as a baseline matter — it falls within the 10-day window from the Day 0 elimination notice. The basis of protest (the elimination decision) was known on Day 0.
+### The Debriefing Exception — The Critical Wrinkle
+GAO's bid protest regulations contain a special rule for procurements conducted on the basis of competitive proposals where a debriefing is **requested and required:**
+&gt; "With respect to any protest basis known or should have been known before or as a result of a debriefing, the initial protest shall NOT be filed before the debriefing date offered, and shall be filed not later than **10 days after the date on which the debriefing is held.**" — 4 C.F.R. § 21.2(a)(2)
+**The purpose:** Encourage meaningful debriefings *before* protest decisions, not after.
+### Does This Exception Apply Here?
+This creates the key procedural tension:
+| Question | Answer |
+|---|---|
+| Was the debriefing *requested*? | Yes — Day 8 |
+| Was a debriefing *required* (i.e., did the agency offer one)? | **TBD** — depends on whether the preaward request was timely |
+| Was the request timely? | **No** — Day 8 exceeds the 3-day window |
+**Because the request was untimely,** the agency is not required to provide the debriefing. When no debriefing is *required* (because entitlement was forfeited by untimely request), the 10-day debriefing exception does not toll the protest deadline. **The protest clock ran from Day 0 on the known basis.**
+**Result:** The Day 8 protest is timely under the baseline 10-day rule (4 C.F.R. § 21.2(a)(2)) — it was filed within 10 days of the elimination notice. It does not benefit from the debriefing exception, but it doesn't need to.
+---
+## TRACK 3: The CICA Automatic Stay — Where the Debriefing Type Becomes Critical
+### The Statutory Stay Framework
+Under CICA (31 U.S.C. § 3553), when GAO receives a timely protest, the agency must generally **suspend award or halt performance.** The critical question is when the "automatic stay" clock runs.
+**Per NIH Manual 6033-2 / FAR 33.104(b):**
+&gt; "CICA stay provisions apply when the agency receives notice of protest from GAO within:
+&gt; - **Ten calendar days after contract award**, OR
+&gt; - **Within five calendar days after the debriefing date offered** to the protester for any debriefing required by FAR 15.505 or 15.506 — **whichever is later**"
+### Applying the Stay Analysis to This Scenario
+#### If the Protest Is PRE-AWARD (Award Not Yet Made):
+The protest was filed **before any award** — this is a pre-award protest. The pre-award stay under FAR 33.104(b)(1) applies:
+- Agency must **withhold award** while protest is pending at GAO
+- To override the stay and proceed with award: the HCA must execute a D&amp;F finding **urgent and compelling circumstances** AND award is likely within 30 days (FAR 33.104(b)(1))
+- At NIH, this D&amp;F must be approved by DASAMP, OS, DHHS (HHSAR 333.104(b)(1)) — **a significant approval burden**
+**This is the most powerful stay outcome for the protester.** No award can be made pending resolution.
+#### If Award Had Already Been Made:
+If award preceded the protest (post-award scenario), the 10-day window controls:
+- Protest on Day 8 → within 10 days of award → **automatic stay of performance applies**
+- Agency must suspend performance unless HCA executes D&amp;F on "best interests" or "urgent and compelling" grounds (FAR 33.104(c))
+#### The 5-Day Debriefing Stay Extension:
+This is where the debriefing election matters most:
+| Debriefing Type | Stay Trigger |
+|---|---|
+| **Preaward debriefing provided (timely)** | Stay window = 5 days after debriefing date offered |
+| **No debriefing (untimely request)** | Stay window = 10 days after award only |
+| **Delayed debriefing (offeror elected to defer to post-award)** | Stay window = 5 days after the deferred debriefing date offered |
+**The practical effect:** If the protester had timely requested a preaward debriefing (within 3 days), the agency would have been obligated to offer one, and the automatic stay trigger would have been *extended* to 5 days after that debriefing date — giving the protester more runway to observe award, receive the debriefing, and then file within a still-open stay window.
+Because the Day 8 request was untimely, the offeror **forfeited the debriefing-triggered stay extension.** The stay is governed solely by the 10-days-post-award clock.
+---
+## TRACK 4: CO's Procedural Obligations Upon Receiving the Protest
+### Immediate Actions Required
+1. **Notify GAO** that protest has been received (within 1 business day of receiving copy from protester, per 4 C.F.R. § 21.1)
+2. **Implement stay** — withhold award or suspend performance (pre- or post-award, as applicable)
+3. **Notify NIH Protest Control Officer (PCO)** — route through IC Director of Acquisitions → NIH PCO
+4. **Litigation hold** — immediately preserve all acquisition records, evaluations, source selection documents, and ESI (NIH Manual 6033-2)
+5. **Prepare Agency Report** — due to GAO within **30 days** of protest notice (4 C.F.R. § 21.3), including:
+   - CO's statement of facts
+   - Memorandum of law
+   - Copies of all relevant acquisition documents
+   - Whether statutory stay is in place
+### On the Debriefing Question
+The CO faces a practical decision: accommodate the untimely Day 8 debriefing request or decline it.
+**Considerations:**
+- Providing the debriefing voluntarily may **reduce protest risk** by giving the protester the factual basis it's seeking — they may withdraw if the debriefing reveals no viable grounds
+- Providing the debriefing does **not** reset protest timelines (FAR 15.301-1 is explicit)
+- Declining preserves the CO's procedural position but provides no information that might lead to early withdrawal
+- Best practice per FC 33.105-3: "Avoid unnecessarily extending protest window. Prepare to quickly provide debriefings when requested."
+**Recommendation:** Accommodate the debriefing — but document clearly that it is being provided as a courtesy, not as an entitlement, and that it does not affect any protest deadline.
+---
+## The Debriefing Type Election: Pre-Award vs. Post-Award — Full Comparison
+| Factor | Preaward Debriefing (FAR 15.206-2) | Delayed/Postaward Debriefing (FAR 15.301-1) |
+|---|---|---|
+| **Request deadline** | Within 3 days of exclusion notice | Within 3 days of award notice |
+| **Agency must provide within** | No specific deadline; "promptly" | 5 days after written request (to maximum extent practicable) |
+| **Content** | Evaluation of significant elements; rationale for elimination; responses to procedure questions | Full content PLUS: overall ratings of both offerors, overall ranking, summary of rationale for award, commercial item info |
+| **Cannot disclose** | Number/identity/content/rankings of other offerors | Point-by-point comparisons; trade secrets; indirect cost rates; names of PP references |
+| **Stay window effect** | 5 days after offered date extends CICA stay trigger | 5 days after offered date extends CICA stay trigger |
+| **Protest timing** | 10 days after debriefing held; cannot file *before* debriefing date offered | 10 days after debriefing held; cannot file *before* debriefing date offered |
+| **Information available** | Less — no awardee comparison data | More — awardee scores, pricing, rankings visible |
+**Strategic note for the protester:** Electing to defer a preaward debriefing until after award (permitted under FAR 15.206-2) gives the offeror *more information* (full postaward content) and *extends the stay window* — at the cost of a longer wait and the risk that meaningful contract performance begins in the interim.
+---
+## Timeline Summary: Day-by-Day
+| Day | Event | Legal Effect |
+|---|---|---|
+| **0** | Elimination notice received | Protest basis known; 10-day GAO clock starts; 3-day debriefing request window opens |
+| **3** | Preaward debriefing request deadline | **Deadline passes** — Day 8 request will be untimely |
+| **8** | Protester requests debriefing AND files GAO protest | Protest is **timely** (within 10 days); debriefing request is **untimely** (beyond 3 days) |
+| **9** | GAO notifies agency of protest | Agency implements stay; CO notifies NIH PCO; litigation hold |
+| **10** | Outer limit for timely protest (baseline) | Day 8 filing safely within window |
+| **38** | Agency Report due at GAO | CO statement, memo of law, documents |
+| **100** | GAO decision deadline (standard) | Or 65 days under express option |
+---
+## SBIR-Specific Considerations
+SBIR competitions are generally conducted under **2 C.F.R. Part 910** and agency-specific SBIR regulations, but the acquisition/protest procedural framework still flows through the FAR when conducted using competitive proposals (FAR Part 15 procedures). A few SBIR-specific notes:
+1. **GAO jurisdiction:** GAO has jurisdiction over SBIR protests to the extent the agency used a competitive proposal process (negotiated acquisition). SBIR sole-source Phase II awards raise different jurisdictional questions (SBA's SBIR Ombudsman may have concurrent jurisdiction).
+2. **"Interested party" standing:** The eliminated offeror has a direct economic interest and qualifies as an interested party under 4 C.F.R. § 21.0(a) — standing is not in question.
+3. **SBA issues are carved out:** If the protest involves size status or SBIR eligibility determinations, those go to SBA, not GAO (4 C.F.R. § 21.5(b)).
+---
+## Key Takeaways
+| Issue | Conclusion |
+|---|---|
+| **Is the Day 8 protest timely?** | ✅ Yes — within 10 calendar days of the known basis (4 C.F.R. § 21.2(a)(2)) |
+| **Is the Day 8 debriefing request timely?** | ❌ No — FAR 15.206-2 requires request within 3 days of exclusion notice |
+| **Is the agency required to provide a debriefing?** | No — untimely request forfeits entitlement; agency may accommodate as courtesy |
+| **Does a courtesy debriefing toll protest deadlines?** | No — FAR 15.301-1 explicitly bars extension for accommodated untimely requests |
+| **Is the automatic CICA stay triggered?** | Depends on whether award has been made: pre-award → stay on award; post-award within 10 days → stay on performance |
+| **Does the untimely debriefing request affect the stay?** | Yes — forfeits the 5-day-post-debriefing stay extension; stay runs on 10-day-post-award clock only |
+| **CO's best action on debriefing?** | Accommodate voluntarily, document as courtesy, no deadline extension |
+| **Override stay (if agency wants to proceed)?** | HCA D&amp;F required; DASAMP approval required (NIH/HHS); urgent and compelling (pre-award) or best interests (post-award) standard |
+---
+**Sources:**
+- FAR 15.206-2 (Preaward Debriefings) / FAR 15.301-1 (Postaward Debriefings) — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Source_Selection_RFO_2025.txt`
+- 4 C.F.R. § 21.2(a)(2) — GAO Bid Protest Regulations (Timeliness)
+- GAO Bid Protests Essential Guide (GAO-18-510SP) — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt`
+- NIH Manual 6033-2 / NIH Policy 6033-2 — Stay Provisions for Protests — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt`
+- FAR Companion Part 33 — `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt`
+- HHSAR 333.104(b)(1), (c)(2) — HCA/DASAMP approval for stay override
+- GAO B-423341 (SMS Data Products) — Enhanced debriefing timeliness precedent
+**Sources:**
+- `eagle-knowledge-base/approved/legal-counselor/case-law/evaluation/GAO_B-423341_ECP_Misleading_Discussions_Best_Value.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt`
+</t>
+        </is>
+      </c>
+      <c r="AS6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW6" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX6" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved)
+RO comparison: Both produce comprehensive SBIR protest analysis. V9 adds: FAR 2.0 numbering (15.206-2), NIH Manual 6033-2 stay provisions, and 6 KB doc paths. RO covers similar ground but V9 is more extensively sourced.
+v8 vs v9: V9 cites 6 KB paths. Tools expanded with web_search and web_fetch.
+Tools: v8=[search_far, research, knowledge_fetch] | v9=[search_far, research, knowledge_fetch, web_search, web_fetch]
+Cascade: Full cascade -- FAR + research + KB fetch + web. Maximum depth.
+Source gap: CLOSED -- V9 covers all RO protest sources plus web references.
+KB docs cited: V8=6 | V9=6 (maintained)
+Verdict: Strongest response in suite -- maintains V8 20/20 with additional web sourcing.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="159" customHeight="1">
       <c r="A7" s="5">
@@ -6135,6 +7071,125 @@
 Verdict: Equivalent. Both 18/20. v7 staged gate model slightly more concrete.</t>
         </is>
       </c>
+      <c r="AK7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a good design tension to name clearly. Let me reflect back what you're describing:
+**The core problem:**
+- Too few questions → documents that need rework (SOW written, then IGCE reveals it's too expensive, now you're backtracking)
+- Too many questions → chatty, theoretical, never gets to the work
+- Multiple valid entry points (quote-first, requirement-first, budget-first) → hard to know when you have "enough" to proceed
+**What you're really asking:** What's the right gate before document generation starts?
+---
+Here's how I'd frame the design decision:
+**The minimum viable context set** — what EAGLE actually needs before touching a document:
+| Field | Why it matters before generation |
+|-------|----------------------------------|
+| **What** | Drives scope, SOW tasks |
+| **How much** | Determines FAR part, workflow, and whether the SOW is even needed |
+| **When** | Period of performance shapes IGCE structure |
+| **Vehicle** | Changes everything — task order vs new contract vs micro-purchase |
+If any of those four are missing or assumed, you get rework.
+---
+**The tradeoff you're describing is really a sequencing problem:**
+```
+Current: SOW → IGCE → [too expensive] → back to SOW
+Better:  Budget check → vehicle check → SOW → IGCE
+```
+The IGCE should be the *second* document, not third or fourth — it's the forcing function that validates scope before you write a full SOW. Or even rougher: a **should-cost estimate** before the SOW is even drafted.
+---
+**Two design approaches worth discussing:**
+**Option A — Lightweight gate (2-3 questions, hard stop)**
+Before *any* document: confirm value, PoP, vehicle. If value unknown, force a rough estimate. Block generation until those 3 fields exist.
+**Option B — Sequence inversion**
+IGCE-first workflow for full acquisitions. Background/objectives → rough cost estimate → *then* SOW. Catches the "too expensive" problem before scope is written.
+---
+Which of those feels closer to the right direction? Or is the real issue more about the "distracted chatting theory forever" side of the old approach?
+</t>
+        </is>
+      </c>
+      <c r="AL7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AM7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP7" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="AQ7" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V8 = RO (comparable)
+RO comparison: Both correctly diagnose the constraint-first vs requirements-first sequencing tension. V8 proposes "minimum viable context set" (What/How much/When/Vehicle); RO frames as "three walls of the box" (budget/timeline/scope). V8 offers two concrete design options (lightweight gate vs sequence inversion). RO proposes 4-step checkpoint with scope summary validation gate.
+V7 vs V8: V8 slightly shorter (2087 vs 2480 chars) but equally actionable. V7 offered a concrete 3-stage gating model.
+Tools: v7=none | v8=none (unchanged -- design discussion, no tools expected)
+Cascade effect: N/A -- design question, no KB research needed.
+Source gap: N/A -- no sources expected for design discussion. Sources scored 3/5 inherently.
+Verdict: Stable, well-framed design discussion with actionable options.</t>
+        </is>
+      </c>
+      <c r="AR7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Good — now I have the full picture of the intake skill. Here's what I'm hearing from you:
+---
+**The core tension you're identifying:**
+| Problem | Old approach | New approach (current) | The gap |
+|---|---|---|---|
+| Too much theory | Background/objectives first → got chatty | SOW fast → clean but shallow | User hits IGCE and has to backtrack |
+| Entry point mismatch | Linear: intake → docs | Multiple real entry points | No sequencing logic for "price before scope" |
+| Scope-price loop | Rare | Common in cloud/IT | System doesn't handle it |
+---
+**The specific failure mode you're naming:**
+User says "buy cloud services" → EAGLE generates SOW → User tries to price it → Too expensive → Now what? The system has no **backward path**. The SOW was built without the pricing constraint that should have shaped it.
+The real workflow for cloud/IT looks like this:
+```
+Rough need → [PRICE CHECK] → Scope calibration → SOW → IGCE → AP
+                 ↑___________________________|
+                 (if too expensive, reshape scope)
+```
+Not:
+```
+Need → SOW → IGCE → (oops, too expensive) → ???
+```
+---
+**What I think you're trying to solve — confirm this:**
+1. **Gate ordering** — Price/budget validation should happen *before* or *concurrent with* scope definition, not after SOW is already drafted
+2. **Entry point awareness** — The system doesn't know if you're coming in scope-first, budget-first, or vendor-quote-first, and it should route differently for each
+3. **Loop handling** — When cost exceeds budget, there needs to be a structured "reshape scope" path, not just "go back to the beginning"
+Is that the problem? And are you thinking about this as a **prompt/workflow change**, a **UI flow change**, or both?
+</t>
+        </is>
+      </c>
+      <c r="AS7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW7" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="AX7" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 = RO (comparable)
+RO comparison: Both correctly identify constraint-first vs requirements-first sequencing tension. V9 uses load_skill for intake context. RO provides similar analysis with 'three walls of the box' framing.
+Tools: v8=N/A (new question) | v9=[load_skill]
+Cascade: N/A -- design discussion, no regulatory content needed.
+KB docs cited: V9=0 (expected for design questions)
+Verdict: Stable -- design reasoning quality consistent.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="20" t="n">
@@ -6153,6 +7208,85 @@
       <c r="D8" s="20" t="inlineStr">
         <is>
           <t>I need to sole-source a $280,000 annual software maintenance contract to Illumina Inc. for our BaseSpace Sequence Hub platform. Only Illumina can maintain this proprietary genomic analysis software. What documents do I need and what's the justification authority?</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>"compliance-strategist/
+302 files
+supervisor-core/checklists/
+302 files
+Good — I can see the J&amp;A template (6.a. Single Source J&amp;A - up to SAT.docx), the NIH checklist, FAR Part 6 guidance, and the J&amp;A Desk Guide. Let me pull all the relevant files simultaneously.
+compliance-strategist/FAR-guidance/FAR_Part_6_Competition_RFO_2025.txt
+6698 chars
+legal-counselor/protest-guidance/JA_Desk_Guide_January_2025_Updated.txt
+57126 chars
+supervisor-core/checklists/OAG_FY25_01_NIH_Acquisition_File_Checklists_MERGED_CORRECTED.txt
+41401 chars
+supervisor-core/core-procedures/HCA_SPE_Approval_Thresholds_Updated.txt
+5440 chars
+Reasoning…
+think
+Good. Now let me check the single-source J&amp;A template and the HHS PMR SAP checklist to round out the picture.
+Reading 6.a. Single Source J&amp;A - up to SAT.docx
+0 blocks
+compliance-strategist/PMR-checklists/HHS_PMR_SAP_Checklist.txt
+2738 chars
+Reasoning…
+think
+Here's the complete picture. One threshold finding changes the whole approach — let me walk through it.
+Sole-Source Analysis: Illumina BaseSpace Sequence Hub Maintenance
+⚠️ First: Threshold Reality Check
+At $280,000, you're below the SAT ($350,000). Per the NIH J&amp;A Desk Guide (updated November 2025), the full FAR Part 6 J&amp;A process does not apply. The right instrument is a Sole Source Justification (SSJ) — NIH's simplified template specifically for acquisitions between $25K–$350K.
+However, this changes if you have option years. The threshold calculation includes all options:
+Structure	Total Value	Instrument Required
+Base year only	$280,000	SSJ (CO signs = approved)
+Base + 1 option	$560,000	Full J&amp;A — CO approval (≤$900K)
+Base + 4 options	$1,400,000	Full J&amp;A — CO approval (≤$900K)
+If you're planning a multi-year contract with options, you need the full J&amp;A template (Justification_and_Approval_Over_350K_Template.docx), not the simplified SSJ. The CO approval authority still applies since the total stays under $900K.
+Justification Authority
+FAR 13.106-1(b)(1)(i) — Contracting officers may solicit from one source if only one source is reasonably available (urgency, exclusive licensing agreements, brand-name, or industrial mobilization).
+This is the right authority. The SSJ template explicitly cites this provision. Your justification narrative needs to demonstrate:
+Illumina is the OEM of proprietary software — only they possess source code, update mechanisms, security patches, and license key management for BaseSpace Sequence Hub
+No third-party maintenance provider can satisfy the requirement because the software architecture and APIs are proprietary and undocumented outside Illumina
+The maintenance requirement is technically inseparable from the original software license
+Critical warning from the template itself: The unique qualifications cannot be based on cost/best value, historical past performance, lack of advance planning, or prior relationships. The justification must rest entirely on technical necessity.
+Required Document Package
+For a single base year at $280,000:
+Document	Template	Notes
+Sole Source Justification (SSJ)	6.a. Single Source J&amp;A - up to SAT.docx	12 sections + PO and CO signatures; CO signature = approval
+Statement of Need (SON)	3.b. SON - Services based on Catalog Pricing.docx	Describes maintenance services scope
+IGCE	4.b. IGE for Services based on Catalog Price.xlsx	Price reasonableness determination
+Market Research Memo	FY26 Streamlined Market Research Report.docx	Documents that no other sources exist
+HHS-653 Small Business Review	HHS-653 form	Required for all actions &gt;MPT ($15K)
+SAM.gov Synopsis	N/A — post to SAM.gov	Required per FAR 5.101; actions &gt;$25K must be announced
+SAM.gov Verification	N/A	Confirm Illumina is registered and not excluded
+Requisition / Funding Document	—	Standard funding cert
+COR Designation Memo	NIH COR Appointment Memorandum.docx	Required for all contracts
+IT Security Checklist	HHSAR_CD_2024_01_OAMS_Security_Checklist_Template.txt	⚠️ See below
+⚠️ IT Clearance — Likely Required
+BaseSpace Sequence Hub is a cloud-based genomics platform. Per HHSAR CD 2024-01 (OAMS Security), IT acquisitions involving cloud-hosted systems require an IT security review and completion of the OAMS Security Checklist before award. This is a frequently missed requirement on software maintenance renewals. Confirm with your IT security officer whether an Authority to Operate (ATO) or updated assessment is required.
+Section 508 compliance documentation should also be addressed — software tools used by NIH staff require 508 conformance review per OAG-FY25-02.
+SSJ Narrative Checklist (12 Required Sections)
+The NIH SSJ template requires all of these in order:
+Agency/contracting activity identification (HHS/NIH/NCI + PO info)
+Nature of action — software maintenance, new or follow-on, FFP contract type
+Description of supplies/services + total estimated value (including all options)
+Statutory authority — check the box: FAR 13.106-1(b)(1)(i)
+Unique qualifications of Illumina — proprietary OEM, no third-party alternative
+Efforts to solicit from other sources + SAM.gov synopsis status
+CO determination that price will be fair and reasonable
+Market research description and results
+Other supporting facts (why competitive technical data package doesn't exist)
+List of sources expressing written interest (likely ""none"")
+Actions to remove barriers to competition in future acquisitions
+PO + PO's supervisor certification; then CO certification = approval
+Bottom Line
+For $280K single year: SSJ + CO signature = done. No Competition Advocate, no HCA, no DAPE routing. Turnaround is typically 1–2 weeks.
+If you're doing multi-year with options: you need the full J&amp;A, but at ≤$900K total, the CO still approves — just using the longer FAR Part 6 template with the additional 12 content elements.
+Want me to draft the SSJ narrative for you? I'd need: (1) is this new or a follow-on to an existing contract, and (2) how many option years are you planning?
+Scroll to bottom
+"</t>
         </is>
       </c>
       <c r="AD8" s="20" t="inlineStr">
@@ -6212,6 +7346,99 @@
 </t>
         </is>
       </c>
+      <c r="AR8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete picture for your Illumina BaseSpace Sequence Hub sole-source acquisition:
+---
+## Illumina BaseSpace — $280,000 Sole-Source Acquisition
+### Justification Authority
+**FAR 13.106-1(b) — Soliciting from a Single Source (Simplified Acquisition Procedures)**
+Since $280,000 is **below the Simplified Acquisition Threshold (SAT) of $350,000**, you use the streamlined SAP authority, not the full FAR Part 6 JOFOC process. The legal basis mirrors FAR 6.302-1(a)(2) — "Only One Responsible Source" — but the procedural requirement is lighter: a Single Source Justification (SSJ) approved by the CO only. No Competition Advocate review required.
+---
+### Required Documents
+| Document | Status | Key Notes |
+|---|---|---|
+| **Single Source Justification (SSJ)** | ✅ Required | FAR 13.106-1(b); CO signature only (no Competition Advocate at this value) |
+| **Purchase Request (PR)** | ✅ Required | With funds certification from Budget Office |
+| **IGCE** | ✅ Required | $280K estimate; HHSAM 307.105-71 |
+| **Market Research Report** | ✅ Required | Confirms no alternative vendors; HHSAM 310.000 |
+| **Price Reasonableness Determination** | ✅ Required | Prior year comparison + vendor quote; FAR 13.106-3(a) |
+| **Required Sources Checklist** | ✅ Required | FAR 8.002; AbilityOne, GSA, NITAAC checked |
+| **HHS-653 Small Business Review** | ✅ Required | OSDBU concurrence needed (Large Business set-aside dissolve) |
+| **IT Security &amp; Privacy Checklist** | ✅ Required | Cloud-based platform; HHSAM 339.101 |
+| **SAM.gov Synopsis** | ✅ Required | Value exceeds $25K; 15-day response period; FAR 5.101(a)(1) |
+| **SAM.gov Registration Verification** | ✅ Required | Active registration + exclusions check at award |
+| **Section 889 Compliance** | ✅ Required | FAR 52.204-25 in contract |
+| **Section 508 Documentation** | ✅ Required | IT acquisition; FAR 39.203 |
+| **NIH Policy 6027 License Review** | ✅ Required | Proprietary software licensing terms review |
+| **COR Designation** | ✅ Required | FAC-COR certified |
+| **FPDS-NG Entry** | ✅ Required | Within 3 days of award |
+---
+### SSJ Core Arguments (What Your Justification Must Establish)
+1. **Proprietary Ownership** — Illumina exclusively owns the BaseSpace Sequence Hub source code, cloud infrastructure, and IP. No third party has legal access to maintain it.
+2. **Technical Impossibility of Third-Party Maintenance** — Maintenance requires direct access to Illumina's private codebase, AWS-hosted infrastructure, version control, and security certificate authorities — all inaccessible to any outside entity.
+3. **No Authorized Third-Party Maintainers** — Illumina has no authorized reseller or maintenance partner program for BSH.
+4. **Integration Lock-In** — BSH is natively integrated with NIH's deployed NovaSeq/NextSeq instruments. Switching platforms would constitute a separate major acquisition and disrupt active research.
+5. **Market Research Confirms Single Source** — No equivalent on GSA Schedule IT 70, SEWP V, NITAAC, or AbilityOne. No open-source alternative (Galaxy, GATK) provides the same integrated SLA-backed environment.
+---
+### Approval Chain
+| Level | Threshold | Who Approves |
+|---|---|---|
+| **This acquisition ($280K)** | ≤ $350K SAT | **Contracting Officer only** |
+| Over $350K – $900K | SAT to $900K | CO + D&amp;F under FAR Part 6 |
+| $900K – $20M | | CO + HCA + Competition Advocate |
+**No Competition Advocate review required here.**
+---
+### Pre-Award Timeline Requirements
+- **SAM.gov sole-source synopsis** → post before award, 15-day response period
+- **Obtain formal Illumina quote** → compare to IGCE; if variance &gt;10%, require cost breakdown
+- **Complete HHS-653 in SBCX system** → before award
+- **IT Security checklist** → before award (cloud genomics platform)
+- **NIH Policy 6027 license review** → flag any unacceptable software license provisions
+---
+### Future Competition Obligations
+The SSJ must document steps to address the sole-source lock-in, specifically:
+- **Platform alternatives assessment** — 12 months before contract expiration
+- **Data portability** — maintain genomic data in open formats (FASTQ, BAM, VCF)
+- **Sources Sought** — post to SAM.gov 12 months before follow-on procurement
+---
+&gt; **Note:** EAGLE found that PKG-2026-0001 already contains a complete SSJ, Purchase Request, Market Research Report, and Price Reasonableness Determination for this exact requirement. Would you like to open those existing documents, generate any missing items, or start a fresh package?
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/purchase_request/v1/Purchase-Request---Illumina-BaseSpace-Sequence-Hub.md`
+</t>
+        </is>
+      </c>
+      <c r="AS8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW8" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX8" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved) [NEW QUESTION]
+RO comparison: Both correctly identify $280K below SAT, requiring SSJ not full JOFOC. V9 adds complete 15-item document checklist table, sole-source rationale language, and 4 KB doc paths. RO provides similar analysis with option year warning.
+Tools: v9=[query_compliance_matrix, research]
+Cascade: Compliance matrix + research subagent -- full cascade.
+KB docs cited: V9=4 (HHS_PMR_Common_Requirements, File_Reviewers_Checklist_FRC, etc.)
+Verdict: Strong -- comprehensive sole-source guidance with actionable checklist.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="20" t="n">
@@ -6230,6 +7457,120 @@
       <c r="D9" s="20" t="inlineStr">
         <is>
           <t>What are the simplified acquisition threshold and micro-purchase threshold under current FAR? Also pull any NIH-specific policies that supplement these thresholds, including local purchase card policies, HCA approval requirements, and NIH procedural steps beyond standard FAR Part 13.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>compliance-strategist/
+302 files
+supervisor-core/
+302 files
+Good — I can see exactly the right files. Let me pull all four simultaneously:
+compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Noncommercial_RFO_2025.txt
+6958 chars
+compliance-strategist/NIH-policies/NIH_FAQ_Simplified_Acquisitions.txt
+24645 chars
+compliance-strategist/NIH-policies/NIH_Purchase_Card_Supplement_Streamlined_2025.txt
+21492 chars
+supervisor-core/core-procedures/HCA_SPE_Approval_Thresholds_Updated.txt
+5440 chars
+Now let me also grab the PMR Threshold Matrix and the GPC Streamlined Guide for the full picture:
+compliance-strategist/PMR-checklists/HHS_PMR_Threshold_Matrix.txt
+2589 chars
+compliance-strategist/SOPs/HHS_GPC_Streamlined_Guide_2025.txt
+24172 chars
+Reasoning…
+think
+Here's the full picture, drawn from five KB sources: FAR_Part_13_Simplified_Noncommercial_RFO_2025.txt, NIH_Purchase_Card_Supplement_Streamlined_2025.txt, HHS_GPC_Streamlined_Guide_2025.txt, HCA_SPE_Approval_Thresholds_Updated.txt, and HHS_PMR_Threshold_Matrix.txt.
+Simplified Acquisition &amp; Micro-Purchase Thresholds — NIH Full Reference
+1. Current Thresholds (FAC 2025-06, Effective October 1, 2025)
+Threshold	Amount	Key Change
+Micro-Purchase Threshold (MPT)	$15,000	↑ from $10,000
+Simplified Acquisition Threshold (SAT)	$350,000	↑ from $250,000
+Service Contract Labor Standards (SCLS) limit (GPC)	$2,500	Unchanged
+Construction / Davis-Bacon limit (GPC)	$2,000	Unchanged
+NIH price reasonableness documentation trigger	$5,000	NIH-specific
+2. FAR Part 13 — Core Requirements
+Hierarchy first: FAR Part 13 (noncommercial) only applies when Part 12 (commercial items) and Part 8 (required sources) cannot satisfy the requirement. Always check those first.
+Competition:
+Above MPT but ≤ SAT: Mandatory small business set-aside (FAR 13.102)
+Single source below SAT requires a written D&amp;F under FAR Subpart 1.5
+Do not split requirements to avoid thresholds — prohibited by FAR 13.003(c)(2)
+Price reasonableness: CO must determine fair and reasonable; base on competitive quotations whenever possible (FAR 13.203(a))
+Clauses:
+Use FAR 52.213-4 (Terms and Conditions—Simplified Acquisitions (Noncommercial)) as the consolidated clause vehicle
+Do not use Part 12 clauses (52.212-1/2/4) in noncommercial simplified acquisitions
+FAR 52.232-39 (Unenforceability of Unauthorized Obligations) automatically applies to every micro-purchase, including GPC transactions
+Post-award: Upon request, provide brief written explanation of award decision to unsuccessful quoters (FAR 13.301)
+3. NIH Purchase Card (GPC) — Micro-Purchase Layer
+Spending Controls
+Transaction Type	GPC Ceiling
+General purchases	$15,000 (MPT)
+SCLS-covered services	$2,500
+Construction (Davis-Bacon)	$2,000
+A&amp;E services (simple, no drawings)	$2,000
+Convenience checks (all other)	$7,500 (half of MPT)
+Convenience checks (SCLS services)	$2,500
+Convenience checks (construction)	$2,000
+Key rule: If a recurring service is expected to exceed $15,000 in the aggregate over 12 months, it must go to the CO — the GPC cannot be used, even if each individual payment is under $15,000. Per HHS_GPC_Streamlined_Guide_2025.txt, Section 7.3
+What a Cardholder Can and Cannot Do
+Cannot sign maintenance or service agreements that bind the Government — must go to a warranted CO for signature
+Cannot make purchases in excess of their Single Purchase Limit (SPL) or Monthly Purchase Limit (MPL)
+Can pay monthly costs under a CO-established agreement if the agreement allows GPC as payment and each payment is within the SPL
+4. NIH-Specific Clearances &amp; Pre-Approvals Beyond FAR Part 13
+These are NIH/HHS procedural requirements that layer on top of FAR — per NIH_Purchase_Card_Supplement_Streamlined_2025.txt:
+Category	NIH-Specific Requirement
+Radioactive materials	RSB clearance number from DRS (301-496-3277) required; authorized user must submit Form 88-1 to Radiation Safety 24 hrs before receipt
+Custom antibodies	Vendor must have active PHS Assurance — verify on OLAW website
+IT products (laptops/desktops)	Use NITAAC → NASA SEWP → GSA (in that priority); CIO waiver required for non-standard configurations
+Construction	GPC limited to $2,000; only by cardholders assigned to Office of Acquisition, ORF, or pre-approved by ORF
+Food / conferences	Must comply with HHS Efficient Spending Policy; NIH Form 827-1 (Non-Delegable Attachment A) required; DDM approval before obligation
+Ergonomic equipment	Free ORS ergonomic evaluation with recommended equipment required before purchase
+Space heaters / fans	ORF must attempt mechanical fix first; written ORF Facility Manager approval required; prohibited in labs/patient care/clinics under any circumstances
+Cellular devices	IC IT department approval required; must comply with Section 889
+Prescription safety glasses	NIH Form 29-2; hand-carry to OMS, Building 10, Room 6C310
+Microsoft software	Must purchase through Microsoft Enterprise Agreement BPA
+Printing devices	Must use FSSI Print Management BPAs or NIH ECS III GWAC; IC EO approval required to deviate
+5. Required Sources — Priority Order (NIH)
+Before any GPC purchase or simplified acquisition, NIH requires checking sources in this sequence:
+Products:
+HHS/OPDIV/IC inventories
+Excess from other agencies (GSA)
+Federal Prison Industries (UNICOR) — mandatory only above $15,000
+AbilityOne Program
+GSA Wholesale Supply
+Category Management BPAs
+GSA Multiple Award Schedules
+HHS preferred sources (IDIQ/BPA) 9a. GSA Commercial Platforms (Amazon Business, Fisher Scientific) — MPT limit only 9b. Open market (small business preference)
+Services: AbilityOne → Category Management BPAs → GSA MAS → HHS preferred sources → open market
+6. HCA/SPE Approval Thresholds (Above SAT)
+These apply once you clear the SAT. Per HCA_SPE_Approval_Thresholds_Updated.txt:
+Justifications &amp; Approvals (J&amp;As) — Updated per FAC 2025-06:
+Value	Approval Level
+≤ $900,000	CO (or as established by OA)
+$900K – $20M	HCA + NIH Competition Advocate
+$20M – $90M	HCA + additional reviews
+&gt; $90M	SPE through HHS/OAP + HHS CA
+⚠️ The old $68M HHS-internal threshold is pending HHS update to align with FAC 2025-06. Use the FAR statutory thresholds above until HHS issues updated guidance.
+Acquisition Plans:
+Value	Approval Level
+SAT – $20M	One level above CO
+$20M – $50M	OA Director (approved by HCA)
+$50M – $150M	HCA-NIH
+&gt; $150M	HHS/OAP
+Route all APs and Acquisition Strategies through AMPSS for HCA signature. Submit supporting docs to DAPE@nih.gov.
+7. Key NIH Procedural Steps Beyond Standard FAR Part 13
+These are NIH-specific procedural requirements that have no direct FAR analog:
+SF-44 is phased out at NIH. Use GPC as the primary micro-purchase mechanism. Convenience checks are last resort only.
+Price reasonableness documentation at $5,000+ — NIH-specific trigger (FAR only requires it generally; NIH sets $5,000 in writing).
+HHS-653 Small Business Review Form required on all purchases above $15,000 (per AA 2023-02 Amendment 3, PMR threshold matrix).
+Receiving must be entered in iProcurement within 5 workdays of acceptance; original paper receiving report filed in contract file.
+Vendor rotation — must rotate equitably among qualified vendors to extent practicable (FAR 13.202; emphasized in NIH policy).
+No acquisition plan required below SAT, but all planning considerations must still be documented in the file. Exception: written AP required for cost-reimbursement or high-risk contracts regardless of value.
+GSA Advantage survey for orders above MPT but ≤ SAT: survey at least 3 contractors (FAR 8.405-1(c)) — this is a survey, not mandatory 3 formal quotes.
+Temporary services cap: individual limited to 120 workdays (extendable to 240 total with written IC justification). Cannot restart with a new vendor to circumvent limit.
+Bottom line on thresholds: MPT is $15,000 and SAT is $350,000 effective October 1, 2025. NIH adds significant procedural layers — particularly around required sources, clearances for specialized purchases, GPC controls on SCLS/construction, and the mandatory HHS-653 form above MPT. The one area to watch: the old HHS $68M J&amp;A threshold hasn't been formally updated to align with FAC 2025-06's $90M FAR ceiling — use the FAR threshold until HHS issues clarifying guidance.
+Chat Message</t>
         </is>
       </c>
       <c r="AD9" s="20" t="inlineStr">
@@ -6400,8 +7741,142 @@
 </t>
         </is>
       </c>
+      <c r="AR9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete picture — FAR thresholds, NIH-specific supplemental policies, and procedural requirements layered on top.
+---
+## Acquisition Thresholds &amp; NIH-Specific Policies
+### Part 1 — Current FAR Thresholds (FAC 2025-06, Effective October 1, 2025)
+| Threshold | Value | Authority |
+|---|---|---|
+| **Micro-Purchase (general)** | **$15,000** | FAR 2.101, 13.201 |
+| Micro-Purchase (construction) | $2,000 | FAR 2.101 |
+| Micro-Purchase (SCA services) | $2,500 | FAR 2.101 |
+| Micro-Purchase (contingency ops) | $25,000 | FAR 2.101 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 2.101, 13.003 |
+| Commercial item simplified test (Part 13.5) | $7,500,000 | FAR 13.500 |
+| SAM.gov synopsis required | $25,000 | FAR 5.101 |
+| Service Contract Labor Standards (SCA) | $2,500 | FAR 22.1003 |
+&gt; ⚠️ **Note:** The MPT increased from $10,000 to $15,000 under FAC 2025-06. FPDS-NG reporting is required for all awards **above** the MPT ($15K+). SAM exclusions check and HHS-653 SB form are also triggered at the MPT.
+---
+### Part 2 — NIH/HHS Supplemental Policies
+#### A. HCA Approval Thresholds (NIH-Specific, Updated November 2025)
+These are **NIH internal thresholds layered on top of FAR**, sourced from the HCA/SPE Approval Thresholds document:
+**Acquisition Plans:**
+| Total Dollar Amount | Approval Level |
+|---|---|
+| SAT → $20M | One level above CO |
+| $20M → &lt;$50M | OA Director (designee approved by HCA) |
+| $50M → $150M | **HCA-NIH** (Director, OALM) |
+| &gt;$150M | HHS/Office of Acquisition Policy (OAP) |
+| High-Risk or Special Interest (any $) | HHS/OAP |
+**Justifications &amp; Approvals (J&amp;As) — Post FAC 2025-06:**
+| Estimated Value (incl. options) | Approval Level | FAR Cite |
+|---|---|---|
+| ≤ $900,000 | Contracting Officer | FAR 6.304(a)(1) |
+| $900K → $20M | HCA + NIH Competition Advocate | FAR 6.304(a)(2)-(3) |
+| $20M → $90M | HCA + additional reviews | FAR 6.304(a)(3) |
+| &gt;$90M | HHS SPE through HHS/OAP &amp; HHS CA | FAR 6.304(a)(4) |
+&gt; 📌 NIH previously used a $68M internal threshold — this is under review and has been superseded by the updated FAR statutory tiers above pending formal HHS update.
+**Acquisition Strategy Approvals:**
+| Lifecycle Cost | Approval Level |
+|---|---|
+| &lt;$50M | OA Director (HCA-approved) |
+| $50M → &lt;$100M | HCA-NIH |
+| $100M → &lt;$150M | Deputy Director for Management, NIH |
+| ≥$150M | HHS/OAP |
+**Submission:** Route all Acquisition Strategies and Acquisition Plans through **AMPSS** for HCA signature. Submit J&amp;As and supporting documentation to **DAPE@nih.gov** per HHS Acquisition Alert 2023-09 and Guide 2023-04.
+---
+#### B. Purchase Card Policies — NIH-Specific (NIH Manual 6307-3)
+The purchase card in NIH has additional requirements **beyond FAR 13.202**:
+1. **Approving Official responsibility:** The Purchase Card Approving Official (cardholder's supervisor or AO) must verify that all required clearances and technical coordination have been obtained **before** the card transaction is processed — applies to *all* card buys regardless of dollar value.
+2. **Required sources check:** Buyers/cardholders must check Appendix 1 of NIH Manual 6307-3 for the commodity type to confirm whether a **Required Source**, **Clearance**, or **Technical Coordination** is needed. Commodity-specific examples:
+   - Audiovisual production services &gt;$5,000 → OCPL clearance required
+   - Telecom services → CIT technical coordination required
+   - Printing → PSC Printing Office is a required source
+   - IT/information security → IC ISSO clearance required
+   - Animals (vertebrates) → DVR required source or IC-ACUC clearance
+3. **Segregation of duties:** The Funds Approver and Contracting Officer (or card approver) must be **different individuals** — a RED finding on NIH's File Reviewer's Checklist (FRC).
+4. **File retention:** Card transaction files must be retained **3 years after final payment** (simplified acquisitions); contract files 6 years 3 months.
+---
+#### C. NIH Procedural Steps Beyond Standard FAR Part 13
+These apply across the FAR 13 range (both MPT and SAP) and are **NIH-specific additions**:
+| Step | Requirement | Authority |
+|---|---|---|
+| **Clearance check** | Search NIH Manual 6307-3 Appendix 1 for commodity — obtain clearance PRIOR to any award vehicle | NIH Manual 6307-3 |
+| **Technical coordination** | Communicate with designated office before submitting PR for 40+ commodity types | NIH Manual 6307-3 |
+| **Required sources** | Check priority sources per FAR 8.002 and NIH-specific required sources (DVR, PSC, Medical Arts, etc.) | FAR 8.002; NIH FRC A2 |
+| **HHS-653 SB form** | Required for all open market actions above the MPT ($15K) — must verify approval in SBCX system | HHS AA 2023-02 Amendment 3 |
+| **BAA/TAA checklist** | Buy American Act/Trade Agreements Act checklist required | HHSAM 325.102-70 |
+| **IT security checklist** | Information Security &amp; Privacy Certification Checklist for any IT-touching acquisition | HHSAM 339.101(c)(1) |
+| **Section 889 compliance** | FAR 52.204-25 required in all solicitations and contracts; documentation required | FAR 4.2105(b) |
+| **DCIS 6M (inherently governmental)** | Required for services contracts &gt;$150K — description of work must be adequate | NIH FRC D2 |
+| **FPAA** | Facility Project Approval Agreement required for equipment &gt;$2M with facility modifications | NIH Manual 6307-3 |
+| **FPDS-NG entry** | Must be completed within 3 business days of award for all actions above MPT | FAR 4.604; NIH FRC D7 |
+---
+#### D. EO 14271 / HHS AA 2026-01 — New SPE Approval Requirement (Effective October 1, 2025)
+This is a **major new overlay** above the SAT:
+- **Trigger:** Any non-commercial product or service above SAT ($350,000)
+- **Requirement:** Written SPE approval **before solicitation release**
+- **Process:** Submit market research report + justification why commercial solution cannot meet need → SPE reviews within 30 days
+- **Timeline impact:** Add 35–45 days to non-commercial acquisitions above SAT
+- **Exclusions:** FSS/GSA Schedule orders, leases, construction, SBIR, and acquisitions at or below SAT are **exempt**
+- **Class approvals** available for recurring non-commercial requirements with identical justification
+---
+### Quick Decision Guide by Dollar Value
+```
+≤$15K (MPT)       → FAR 13.2 micro-purchase; no competition required
+                     NIH adds: clearance check, required sources, card AO verification
+$15K–$25K          → Open market; post to SAM.gov or oral solicitation documented
+                     NIH adds: HHS-653 SB form, clearance check, FPDS-NG
+$25K–$350K (SAT)   → SAP; synopsis on SAM.gov; max practicable competition
+                     NIH adds: HHS-653, clearance, BAA checklist, Section 889
+&gt;$350K             → Full FAR (Part 15 or 8.4); written AP required
+                     NIH adds: HCA approval tiers, EO 14271 SPE approval if non-commercial
+```
+---
+**Sources:**
+- FAR Thresholds: Compliance Matrix (FAC 2025-06, effective October 1, 2025)
+- NIH approval tiers: `HCA_SPE_Approval_Thresholds_Updated.txt`
+- Purchase card &amp; clearance procedures: `NIH_6307_3_Special_Clearance_Procedures.txt` (NIH Manual 6307-3, DSAPS/OAMP)
+- EO 14271 / non-commercial SPE approval: `HHS_AA_2026_01_EO_14271_Non_Commercial_Approval.txt`
+- NIH File Reviewer's Checklist (FRC): OALM Acquisition Compliance Review Standards (updated November 2025)
+- HHS PMR SAP Checklist (updated November 2025)
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Policy_6307_3_Special_Clearance_Procedures_2014.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_SAP_Checklist.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+</t>
+        </is>
+      </c>
+      <c r="AS9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW9" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX9" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved) [NEW QUESTION -- enhanced Q1]
+RO comparison: V9 provides FAR thresholds AND NIH-specific policy layers (HCA approval tiers, J&amp;A thresholds, purchase card limits). RO covers similar FAR thresholds plus NIH FAQ. V9 adds HCA/SPE approval threshold table.
+Tools: v9=[query_compliance_matrix, research]
+Cascade: Compliance matrix + research -- pulls NIH policy overlays.
+KB docs cited: V9=4 (HHS_PMR_SAP_Checklist, Common_Requirements, FRC, NIH_Policy_6307)
+Verdict: Enhanced Q1 answered comprehensively -- NIH layers add value.</t>
+        </is>
+      </c>
     </row>
-    <row r="10">
+    <row r="10" ht="409.5" customHeight="1">
       <c r="A10" s="20" t="n">
         <v>9</v>
       </c>
@@ -6418,6 +7893,52 @@
       <c r="D10" s="20" t="inlineStr">
         <is>
           <t>What did GAO hold in B-302358 regarding IDIQ minimum obligation requirements? Search the knowledge base for the full decision text and cite the specific KB documents you find.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>legal-counselor/
+302 files
+I can see exactly what I need. There's a file at legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt. Let me pull that along with the related IDIQ funding appropriations law file.
+legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt
+28370 chars
+legal-counselor/appropriations-law/appropriations_law_IDIQ_funding.txt
+18283 chars
+Reasoning…
+think
+Here's the full analysis of GAO B-302358 based on the KB decision text.
+GAO B-302358 — Bureau of Customs and Border Protection (Dec. 27, 2004)
+KB Source: legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt Supporting file: legal-counselor/appropriations-law/appropriations_law_IDIQ_funding.txt
+Core Holdings
+GAO issued two holdings in this case:
+Holding 1 — Contract Type: The ACE contract (a 5-year, $5B IDIQ) was not a multiyear contract under 41 U.S.C. § 254c, despite the contract file containing a multiyear Determination &amp; Findings and FAR clause 52.217-2. GAO was blunt: "Customs plainly awarded an IDIQ contract and not a multiyear contract." Contract substance controls over erroneous labels. The two contract types are mutually exclusive — a multiyear contract requires the need to be "reasonably firm and continuing," while an IDIQ contract by definition requires the government to be unable to predetermine quantities above the minimum. You cannot satisfy both simultaneously.
+Holding 2 — Minimum Obligation (the foundational rule): Customs violated the recording statute (31 U.S.C. § 1501(a)) by failing to obligate the $25M IDIQ minimum at contract award on February 11, 2003. GAO's controlling language:
+"When an agency executes an indefinite-quantity contract such as an IDIQ contract, the agency must record an obligation in the amount of the required minimum purchase." "At the time of award, the government has a fixed liability for the minimum amount to which it committed itself." "This is so whether [the agency] ever issues a task order to the contractor or not, and is so immediately upon contract award."
+What Customs Actually Did Wrong
+Date	Required Action	What Customs Did	Violation
+Feb. 11, 2003 (award)	Obligate $25M from FY03 funds	Obligated nothing	Recording statute
+Sep. 28, 2003	N/A	Obligated $45K from FY03	Under-obligated
+Nov. 2003–Sep. 2004	N/A	Obligated $955K from FY04 funds	Wrong fiscal year
+Customs's defense — that the minimum had ultimately been satisfied through task orders — was dismissed. GAO held that timely recording is required to protect the integrity of obligational accounting records regardless of eventual satisfaction.
+The Mechanism: Why the Minimum Triggers Immediate Obligation
+GAO's reasoning rests on FAR clause 52.216-22, which states the government "SHALL ORDER" at least the minimum. That mandatory language creates a legal liability at the instant of contract award. Per the recording statute, legal liability = obligation. The minimum must be charged to the appropriation current in the fiscal year of contract award — FY2003 in this case.
+Subsequent task orders that draw down the minimum require no new obligation. New obligations arise only after the minimum is exhausted, and those are chargeable to the fiscal year in which the task order is placed.
+Multiyear vs. Multiple-Year Terminology — A Specific Warning
+GAO flagged that the entire dispute originated from terminology confusion. Per the KB file:
+"The unfortunate partial homonymy of the terms 'multiyear' and 'multiple year' evidently led to confusion both at Customs and at OIG."
+The KB specifically cites Cibinic &amp; Nash (1996): "'Multiyear' should only be used when referring to the unique arrangements covered in FAR Subpart 17.1." A 5-year IDIQ is a multiple-year contract (descriptive), not a multiyear contract under § 254c (legal term of art requiring head-of-agency determination and advance appropriations commitment).
+Remedial Actions Required
+GAO directed both Customs (Interior SWB) and DOD to:
+Deobligate $955K from FY2004 appropriations
+Obligate $955K from FY2003 appropriations
+Determine whether sufficient FY2003 funds existed — if not, report an Antideficiency Act violation per 31 U.S.C. § 1341(a)
+Practical Takeaway for NIH/NCI
+This is the foundational IDIQ minimum obligation case cited throughout the KB. The operational rules it establishes:
+✅ Obligate the guaranteed minimum at contract award — not at first task order
+✅ Use the fiscal year appropriation current at award — not future-year funds
+✅ Document bona fide need — the companion case, B-321640 (SBA, 2011), held that obligating a minimum without genuine current-year requirements is a "parking funds" violation of the bona fide needs rule
+⚠️ Never label an IDIQ as a "multiyear contract" — the terms are legally incompatible and the mislabeling in this case triggered a multi-year audit and ADA investigation
+Let me know if you want me to pull the companion cases — B-321640 and B-321640's "parking funds" doctrine — or if you're working through a specific IDIQ obligation scenario.</t>
         </is>
       </c>
       <c r="AD10" s="20" t="inlineStr">
@@ -6476,8 +7997,98 @@
 </t>
         </is>
       </c>
+      <c r="AR10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I now have comprehensive sourced information. Here is the full analysis:
+---
+## GAO Decision B-302358 — IDIQ Minimum Obligation Requirements
+**⚠️ KB Note:** B-302358 does not exist as a standalone case file in the EAGLE knowledge base. The analysis below is drawn from:
+1. **FAR Part 16 IDIQ Comprehensive RFO 2025** (`eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`) — the controlling regulation implementing FAR 16.504
+2. **GAO Red Book (Chapter 7)** — cited in the wifcon.com analysis of B-302358
+3. **Wifcon.com** — practitioner analysis citing the full decision text (fetched: https://www.wifcon.com/discussion/index.php?/blogs/entry/166-myth-information-obligating-the-minimum-in-idiq-contracts/)
+4. Direct GAO.gov (blocked via bot protection — decision text not retrievable directly)
+---
+### What GAO Held in B-302358
+**Case:** *Matter of Bureau of Customs and Border Protection — Automated Commercial Environment Contract*
+**Decision:** B-302358 (Comptroller General)
+---
+#### Core Holding
+GAO held that an agency **must record an obligation for the IDIQ contract minimum at the time of contract award** — not at the time individual orders are placed.
+Specifically:
+&gt; The Bureau of Customs and Border Protection awarded an IDIQ contract (the Automated Commercial Environment contract) with a **$25 million minimum guarantee**. Customs did not record the $25 million obligation until **five months after contract award**. GAO held this violated the recording statute, **31 U.S.C. § 1501(a)(1)**, because the legal liability for the minimum arose at the moment the contract was executed.
+---
+#### The Two-Part Legal Analysis
+GAO distinguished between two related but separate concepts:
+| Concept | What It Means | When It Happens |
+|---|---|---|
+| **Creating** an obligation | The Government's legal liability is incurred | At IDIQ contract award (the minimum guarantee binds the Government) |
+| **Recording** an obligation | The accounting entry that evidences the obligation | Must happen contemporaneously with creation |
+GAO held that **awarding an IDIQ contract creates an immediate, fixed obligation for the contract minimum** under the recording statute. The agency's failure to record it promptly does not eliminate the obligation — it just means the agency violated 31 U.S.C. § 1501.
+---
+#### The Recording Statute — 31 U.S.C. § 1501(a)(1)
+GAO grounded its decision in the recording statute's text:
+&gt; *"An amount shall be recorded as an obligation of the United States Government only when supported by documentary evidence of — (1) a binding agreement between an agency and another person (including an agency) that is — (A) in writing, in a way and form, and for a purpose authorized by law; and (B) executed before the end of the period of availability for obligation of the appropriation or fund used for specific goods to be delivered, real property to be bought or leased, or work or service to be provided…"*
+An IDIQ contract satisfies all elements: it is a binding written agreement executed before the appropriation's expiry. The minimum guarantee is thus a **fixed legal liability** — not contingent on future orders.
+---
+#### Practical Implications for IDIQ Contracting
+1. **Obligation at award:** The contract minimum must be charged against a currently available appropriation at the time the IDIQ contract is executed — not when the first delivery order is placed.
+2. **Underrecording = Antideficiency Act risk:** Failing to record a legitimate obligation may result in violating the Antideficiency Act (31 U.S.C. § 1341). The GAO Red Book (Chapter 7, p. 7-6) states: *"The overrecording and the underrecording of obligations are equally improper."*
+3. **Recording does not create the obligation:** Conversely, if the minimum was never recorded but the contract was awarded, the obligation still exists — it is simply unrecorded. The fiscal year charged is the year of award.
+4. **Subsequent orders are separate obligations:** Orders placed above the minimum are recorded as they are issued. The minimum guarantee is the only amount obligated at contract award.
+---
+#### Connection to FAR 16.504
+The KB document (FAR Part 16 IDIQ, at **16.504-1(b)**) directly implements the principle underlying B-302358:
+&gt; *"The contract must require the Government to order and the contractor to furnish at least a stated minimum quantity of supplies or services. To ensure that the contract is binding, the minimum quantity must be **more than a nominal quantity**, but it should not exceed the amount that the Government is fairly certain to order."* — FAR 16.504-1(b) (KB source, at p. 4)
+The "more than a nominal quantity" requirement exists precisely because a purely nominal minimum would fail to create a genuine binding obligation — undermining the enforceability of the contract and the purpose of B-302358's recording requirement.
+---
+### Summary
+| Issue | GAO's Answer |
+|---|---|
+| When does minimum obligation arise? | At IDIQ contract award |
+| When must it be recorded? | Simultaneously with award |
+| Legal basis? | 31 U.S.C. § 1501(a)(1) (recording statute) |
+| Failure to record = ? | Violation of recording statute; Antideficiency Act risk |
+| Does late recording cure the problem? | No — obligation existed regardless; recording merely evidences it |
+| Can you wait for the first order? | **No** — this is the myth B-302358 corrects |
+---
+### Sources
+| Source | Type | Location |
+|---|---|---|
+| FAR Part 16 IDIQ Comprehensive RFO 2025 (§§ 16.504-1, 16.504-2) | KB Regulation | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt` |
+| *Myth-Information: Obligating the Minimum in IDIQ Contracts* (Don Mansfield, WIFCON) — citing GAO B-302358 and GAO Red Book Ch. 7 | Web (fetched) | https://www.wifcon.com/discussion/index.php?/blogs/entry/166-myth-information-obligating-the-minimum-in-idiq-contracts/ |
+| GAO Red Book, Principles of Federal Appropriations Law, Chapter 7 (pp. 7-6, 7-8) | Secondary (cited in KB legal agent definition) | `eagle-knowledge-base/approved/agents/02-legal.txt` |
+| 31 U.S.C. § 1501(a)(1) | Statute | Recording statute — federal appropriations law |
+&gt; **Note:** The GAO.gov URL for B-302358 returned HTTP 403 (bot-blocked). If you need the full Comptroller General decision text, retrieve it directly at: `https://www.gao.gov/decisions/appro/302358.htm` in a browser, or via Westlaw/LexisNexis under B-302358.
+</t>
+        </is>
+      </c>
+      <c r="AS10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW10" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX10" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved) [NEW QUESTION -- enhanced Q2]
+RO comparison: V9 correctly identifies B-302358 not present as standalone KB file, provides transparent sourcing note, draws from FAR Part 16 IDIQ and web. RO had direct KB file access. Both cover core holdings correctly.
+Tools: v9=[knowledge_search, knowledge_fetch, web_search, web_fetch]
+Cascade: Full cascade -- KB search + fetch + web supplementation.
+KB docs cited: V9=3 (FAR_Part_16_IDIQ, agents/02-legal, + web sources)
+Verdict: Strong -- transparent about source limitations, supplements with web.</t>
+        </is>
+      </c>
     </row>
-    <row r="11">
+    <row r="11" ht="409.5" customHeight="1">
       <c r="A11" s="20" t="n">
         <v>10</v>
       </c>
@@ -6494,6 +8105,123 @@
       <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Explain how the bona fide needs rule under 31 U.S.C. 1502(a) interacts with the severable vs. non-severable distinction when funding a service contract that crosses fiscal years. Include both the severable services rules and the time-based bona fide needs rules.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>financial-advisor/
+302 files
+financial-advisor/appropriations-law/appropriations_law_severable_services.txt
+17549 chars
+financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt
+13462 chars
+compliance-strategist/regulatory-policies/appropriations_law_severable_services.txt
+17549 chars
+financial-advisor/appropriations-law/appropriations_law_options.txt
+20401 chars
+financial-advisor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt
+13398 chars
+Reasoning…
+think
+This is a well-layered fiscal law question. Here's a full synthesis drawn from the KB files on bona fide needs, severable services, and option exercise timing — cross-referenced with the Army Deskbook and FAR provisions.
+The Bona Fide Needs Rule and Severable/Non-Severable Services: How They Interact
+I. The Statutory Backbone
+31 U.S.C. § 1502(a) provides:
+"The balance of an appropriation or fund limited for obligation to a definite period is available only for payment of expenses properly incurred during the period of availability or to complete contracts properly made within that period of availability."
+This creates two requirements that must both be satisfied:
+The obligation must occur within the fund's period of availability, AND
+The need the obligation satisfies must be a bona fide need of that same fiscal year.
+The rule prevents "parking" funds, stockpiling, or end-of-year spending on future-year requirements. Congressional control over annual appropriations is the constitutional root (Art. I, § 9).
+II. The Services Performance Rule — The Foundation
+For services, the default bona fide need arises in the fiscal year when performance occurs, not when the contract is awarded. This is the "performance period rule."
+This creates an immediate problem for service contracts that cross fiscal year boundaries (e.g., awarded September 30, performance runs October 1 through the following year). The question becomes: which year's appropriation funds which portion?
+The answer turns entirely on severability.
+III. The Severable/Non-Severable Distinction — The Pivotal Fork
+Per the GAO standard, the test is:
+"Whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."
+Characteristic	Severable	Non-Severable
+Deliverable	Recurring outputs (ongoing value each period)	Single end product or unified result
+Task interdependence	Independent, repetitive tasks	Interdependent, build toward unified goal
+Time divisibility	Can be logically divided by time period	Cannot divide without losing essential character
+Source of value	Each period's services stand alone	Value derives from complete performance
+Examples	Help desk, maintenance, guard services, SaaS subscriptions, sys admin	Studies, audits, system development, litigation support, A/E design, training programs
+Critical rule: Severability is determined by the nature of the services, not by how the contract is written. You cannot draft your way around this. (Per appropriations_law_severable_services.txt, Error #4.)
+IV. The Two Funding Regimes
+A. Severable Services — Incremental Funding Required
+Each fiscal year's services are a separate bona fide need of that year. The performance period rule applies fully. You must match each year's appropriation to that year's performance.
+Worked Example:
+Period	Months	Value	Appropriation
+Oct 2025 – Sep 2026	12 months	$1,200,000 total	—
+Oct–Dec 2025 (FY26 Q1)	3 months	$300,000	FY26 funds
+Jan–Sep 2026 (FY26 Q2–4)	9 months	$900,000	FY26 funds
+If the contract begins mid-FY and crosses into the next FY, you must split the obligation. You cannot cover all 12 months from the year the contract was awarded if those months straddle the October 1 boundary.
+FAR hooks:
+FAR 37.106 — Funding and term of service contracts; confirms severable services must be funded from the appropriation current when services are performed
+FAR 32.703-3 — Contracts crossing fiscal years
+FAR 52.232-19 — Availability of Funds for the Next Fiscal Year (required clause for severable service contracts that cross FY boundaries)
+FAR 52.232-22 — Limitation of Funds (cost-reimbursement)
+B. Non-Severable Services — Full Obligation at Award Authorized
+The entire contract is a single bona fide need of the fiscal year in which the contract is entered. The whole value may be obligated from that year's appropriation even if performance extends into one or more subsequent fiscal years.
+Worked Example:
+Contract awarded September 15, FY25. Scope: Program evaluation with final report. Performance: October 2025 – March 2026. Value: $600,000.
+✅ Obligate entire $600,000 from FY25 funds at award. ✅ Performance extending into FY26 is permissible — no incremental funding needed. Rationale: The study is a single undertaking; the entire effort is the bona fide need of FY25 when the contract was made.
+No incremental funding clauses required. Standard funding clauses are sufficient.
+V. The Short Bridge Exception (Severable Only)
+Even for severable services, agencies may obligate current-year funds for a contract that extends a short distance into the next fiscal year, to avoid a service gap.
+Conditions:
+Bridge into the new year is minimal (typically 1–3 months)
+Operational necessity to avoid a gap in services
+Documented business reason
+Example: Award a 3-month bridge contract August 1, FY25 running through October 31, FY25. Even though October is in FY26, the entire $150,000 may be funded from FY25 appropriations.
+This is an administrative exception — don't stretch it. A contract designed to push 9 months of FY26 services onto FY25 funds under a "bridge" label is a violation.
+VI. The Interaction Matrix — All Three Variables Together
+Contract Type	Crosses FY?	Funding Rule	Common Error
+Non-severable	No	Single FY funds, obligate at award	N/A
+Non-severable	Yes	Still single FY funds — obligate full amount at award from FY when contract entered	Thinking multi-FY performance requires split funding
+Severable	No (same FY)	Single FY funds	N/A
+Severable	Yes	Must split — each FY's services funded with that FY's appropriation	Using award-year funds to cover entire period
+Severable	Short bridge only	Award-year funds for brief overlap permissible	Using "bridge" language for extended FY crossover
+VII. Options — A Third Layer
+Options add a third layer because each option period is a separate bona fide need. Per appropriations_law_options.txt:
+"The bona fide need for an option period arises in the fiscal year when the option period will be performed, not when the base contract was awarded."
+Standard rule: You must fund each option period with the appropriation current when that option period's need arises (i.e., the appropriation for the fiscal year of performance).
+Advance exercise exception: You may exercise an option slightly early (typically 30–90 days) using the prior year's funds IF:
+The contract requires advance notice (e.g., 60-day notice provision)
+Operational necessity is documented
+You are not doing it to consume expiring funds
+⛔ Classic violation: On September 25, with expiring FY25 funds in hand, exercising a FY26 option "to use up the money" — this is a bona fide needs violation even if the contract was awarded in FY25.
+Severability still applies to options: A non-severable option period that spans two fiscal years can still be fully funded from the appropriation current when the option is exercised. A severable option period that spans two fiscal years requires split fiscal year funding.
+VIII. The Time-Based Bona Fide Needs Rules — Special Cases
+The KB also identifies specific timing rules beyond the severable/non-severable distinction:
+Supplies: The bona fide need arises in the fiscal year when delivery is required and accepted — the delivery date controls, not the order date. Exception: Long lead-time items ordered in current FY for future delivery, where normal procurement lead time extends beyond FY end and the need genuinely arises now.
+Construction: Bona fide need arises when the work is actually performed, not when funds are obligated or design is complete. Advance planning/design may be a separate severable bona fide need.
+No-year appropriations: The bona fide needs rule still applies — you need a genuine current requirement; you just aren't constrained by the fiscal year expiration clock.
+Multi-year contracts (FAR 17.1): These are a distinct statutory mechanism (41 U.S.C. § 254c) allowing up to 5 years of requirements to be funded from a current-year appropriation — but require specific statutory authority and a Head of Agency determination. Not to be confused with routine contracts that happen to span multiple years.
+IX. Common Violations and Tells
+Violation	Tell-Tale Sign
+Severable services funded with single-year appropriation	Full 12-month value obligated at award; contract crosses October 1
+End-of-year parking for future needs	Large obligation in late September for services not starting until November+
+Improper advance option exercise	Option exercised 4+ months early with no notice-period justification
+Drafting non-severability to avoid incremental funding	SOW calls services "non-severable" but tasks are clearly recurring and independent
+IDIQ minimum parking	Minimum obligated at award but no task orders issued all year
+X. Required Acquisition Plan Documentation Language
+For Non-Severable:
+"The services required under this acquisition constitute a non-severable undertaking. The contract will produce [specific deliverable] through interdependent tasks that cannot be meaningfully divided into discrete time periods. Accordingly, the entire contract value of $[X] will be obligated from FY [XXXX] appropriations at contract award, even though performance extends into FY [XXXX+1]. This approach complies with the bona fide needs rule under 31 U.S.C. § 1502(a) because the entire undertaking represents a bona fide need of FY [XXXX]."
+For Severable:
+"The services required under this acquisition are severable, consisting of [recurring services] where each period's performance has independent value. Because the contract crosses fiscal year boundaries, funding will be incremented as follows:
+FY [XXXX] appropriations: $[amount] for services from [dates]
+FY [XXXX+1] appropriations: $[amount] for services from [dates] This incremental approach complies with the bona fide needs rule by matching each fiscal year's appropriation to the bona fide need arising in that year."
+XI. Key Citations
+Authority	Citation
+Statutory rule	31 U.S.C. § 1502(a)
+Services performance rule	GAO Red Book, Vol. I, Ch. 5, § B.4
+FAR services crossing FY	FAR 32.703-3; FAR 37.106
+Availability of funds clause	FAR 52.232-19
+Options rule	FAR 17.207; GAO B-329061 (Feb. 25, 2009)
+Severable case law	GAO B-223096 (custodial, severable); GAO B-235580 (language training, non-severable); GAO B-237407 (guard services, severable)
+Constitutional root	Art. I, § 9 (Appropriations Clause)
+Sources: appropriations_law_severable_services.txt, appropriations_law_time_bona_fide_needs.txt, appropriations_law_options.txt, Army_Contract_Attorneys_Deskbook_2025_Chapter_4.txt
+Bottom line: The bona fide needs rule and the severable/non-severable distinction are inseparable concepts. The rule sets the timing requirement; severability determines when the need arises — either at contract formation (non-severable) or incrementally as services are rendered (severable). Getting the severability determination wrong is the most common path to an ADA-implicating obligation. When the determination is close — particularly on hybrid contracts or large-dollar IT efforts — escalate to OGC before obligating.</t>
         </is>
       </c>
       <c r="AD11" s="20" t="inlineStr">
@@ -6613,8 +8341,173 @@
 </t>
         </is>
       </c>
+      <c r="AR11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is a thorough treatment of how the bona fide needs rule under 31 U.S.C. § 1502(a) interacts with the severable/non-severable distinction for service contracts that cross fiscal years.
+---
+# The Bona Fide Needs Rule &amp; Severable vs. Non-Severable Services
+## I. THE STATUTORY FOUNDATION
+**31 U.S.C. § 1502(a)** states:
+&gt; *"The balance of an appropriation or fund limited for obligation to a definite period is available only for payment of expenses properly incurred during the period of availability or to complete contracts properly made within that period of availability."*
+The practical rule derived from this: **an annual appropriation may only fund needs that genuinely arise during that appropriation's period of availability.** It prevents agencies from parking funds, stockpiling, or using current-year money to pre-pay future-year requirements.
+The key variable for service contracts is **when the need arises** — and that question is answered differently depending on whether the services are severable or non-severable.
+---
+## II. THE SERVICES PERFORMANCE PERIOD RULE
+For services (unlike supplies, which use a delivery-date rule), **the bona fide need arises in the fiscal year in which the services are performed.** This is called the **performance period rule**.
+That single sentence drives everything below. The severable/non-severable distinction is the mechanism that determines *which* fiscal year's performance period is the controlling one.
+---
+## III. THE SEVERABLE vs. NON-SEVERABLE DISTINCTION
+### The GAO Legal Standard
+&gt; *"The question is whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."*
+&gt; — GAO Red Book, Chapter 5
+This is a **facts-and-circumstances** test applied to the nature of the services, not to contract language. **You cannot make severable services non-severable by writing the contract differently** — the underlying nature of the work controls.
+### Non-Severable Services — "Single Undertaking"
+Services are **non-severable** when they constitute a **single integrated undertaking** that cannot be broken into discrete, independently valuable increments without losing essential character.
+**Indicators:**
+- Single unified deliverable (a report, an audit opinion, a completed system, a design)
+- Interdependent tasks that build toward one outcome
+- Cannot logically be divided by time period
+- Value derives only from complete performance
+**Examples:** Feasibility study with final report, financial audit, litigation support for a specific case, custom software development for a defined system, A&amp;E design for a facility, a specific training course.
+**Funding consequence:** The **entire contract** is the bona fide need of the **fiscal year in which the contract is entered** — even if performance extends into one or more future fiscal years. You obligate the full amount from the current-year appropriation at award.
+&gt; *Example: A program evaluation contract is awarded September 15, FY25 for $600K. Work begins October 2025; final report is due March 2026. The entire $600K is obligated from FY25 funds. The study is a single undertaking; FY25 is when the need arose.*
+### Severable Services — "Series of Separate Tasks"
+Services are **severable** when they are **recurring or continuing** in nature, where each time period's performance has **independent value** standing alone.
+**Indicators:**
+- Repetitive, discrete units of service (each shift, each day, each month)
+- Each period's services are useful regardless of what happens in other periods
+- Work can be logically divided by time period without losing value
+- No single culminating deliverable
+**Examples:** Help desk support, systems administration, janitorial services, guard services, grounds maintenance, subscription/SaaS services, ongoing IT O&amp;M, security operations center monitoring.
+**Funding consequence:** **Each fiscal year's portion of service is a separate bona fide need of that fiscal year.** You must fund incrementally — current-year appropriation for current-year services, next-year appropriation for next-year services.
+&gt; *Example: A help desk contract runs October 1, FY25 through September 30, FY26 at $100K/month ($1.2M total). You cannot obligate the full $1.2M from FY25 funds. FY25 funds cover October–December 2025 ($300K); FY26 funds must cover January–September 2026 ($900K).*
+---
+## IV. THE INTERACTION: HOW THE BONA FIDE NEEDS RULE OPERATES DIFFERENTLY BY CATEGORY
+| | **Non-Severable** | **Severable** |
+|---|---|---|
+| **When does the need arise?** | Year the contract is entered | Year each increment of service is performed |
+| **Appropriation used** | Single FY appropriation at award | Multiple FYs — each year funds its own services |
+| **Can cross FYs?** | Yes, freely | Yes, but must be incrementally funded |
+| **Incremental funding required?** | No | Yes, if crossing FY boundary |
+| **Risk if funded wrong** | Low (non-severable = full obligation permitted) | High — using FY25 funds for FY26 services is a Bona Fide Needs Rule violation |
+---
+## V. THE SHORT BRIDGE EXCEPTION (SEVERABLE SERVICES)
+For **severable services**, GAO and agency practice recognize a narrow exception when a contract is awarded **near the end of a fiscal year** and spans a short period into the next fiscal year (typically **1–3 months**), provided:
+- The bridge into the next fiscal year is minimal
+- There is operational necessity (avoiding a gap in services)
+- It is not a device to circumvent the annual appropriations process
+&gt; *Example: An IT systems administration contract is awarded August 1, FY25, running through October 31, FY25 (3 months). Even though October is in FY26, the full $150K may be obligated from FY25 funds. The one-month bridge is administratively reasonable.*
+This exception does **not** extend to contracts that run 6–12 months into a new fiscal year. Only a short, operationally necessary bridge qualifies.
+---
+## VI. OPTIONS — EACH OPTION PERIOD IS A SEPARATE BONA FIDE NEED
+Options interacting with the severable/non-severable distinction add another layer:
+- **Each option period** represents a **distinct, separate bona fide need** of the fiscal year in which that option period will be *performed*.
+- Options are **not** obligated at base contract award; they are obligated **when exercised**.
+- You may not exercise an FY26 option using FY25 funds merely to avoid losing FY25 money — that is a bona fide needs violation.
+**Advance exercise exception:** A CO may exercise an option in a prior fiscal year (using prior-year funds) only if:
+- Operational necessity requires advance exercise (e.g., a 60-day notice requirement)
+- The exercise occurs close to the start of the option period (typically within 90 days)
+- There is documented business reason to avoid a service gap
+---
+## VII. APPROPRIATION TYPE MATTERS — NO-YEAR AND MULTI-YEAR FUNDS
+The severable services restriction on crossing fiscal years **applies only to annual (one-year) appropriations.** If the contract is funded with:
+- **No-year (available until expended) appropriations** — The fiscal year matching rule does not apply; severable services can be funded from a single no-year appropriation. The bona fide needs rule still applies (no speculative future needs), but incremental funding across fiscal years is not required.
+- **Multi-year appropriations** — Similarly, a two- or three-year appropriation can fund severable services across the years it covers without the incremental funding constraint.
+- **Annual appropriations** — Full severable services rules apply.
+---
+## VIII. FAR CLAUSES TRIGGERED BY SEVERABILITY DETERMINATION
+| Scenario | Applicable Clause |
+|---|---|
+| Severable services, cost-reimbursement, crossing FYs | **FAR 52.232-22** (Limitation of Funds) |
+| Severable services, fixed-price, crossing FYs | **FAR 52.232-19** (Availability of Funds for the Next Fiscal Year) |
+| Cost-reimbursement, limitation of cost | **FAR 52.232-20** (Limitation of Cost) |
+| Multi-year contracts (statutory authority) | **FAR 17.103** (Multiyear contracting) |
+| Contracts crossing fiscal years (general) | **FAR 32.703-2 / 32.703-3** |
+---
+## IX. GRAY AREAS REQUIRING ANALYSIS
+Several common service types require deliberate analysis rather than automatic classification:
+| Service Type | Analysis Required |
+|---|---|
+| **Agile software development** | If sprints build toward a single defined system → Non-severable. If ongoing enhancement with no defined end state → potentially Severable. |
+| **Project management** | For a specific project with deliverables → Non-severable. For ongoing program management → Severable. |
+| **Technical support** | For a specific implementation/deployment → Non-severable. For ongoing help-desk-style support → Severable. |
+| **Cybersecurity** | SOC monitoring → Severable. Penetration test with report → Non-severable. Incident response for specific incident → Non-severable. |
+| **Consulting** | Defined engagement with end product → Non-severable. Ongoing advisory without defined deliverable → Severable. |
+---
+## X. CRITICAL ERRORS TO AVOID
+| Common Error | Correct Rule |
+|---|---|
+| "All service contracts are severable" | Many service contracts are non-severable (studies, audits, defined projects) |
+| "Crossing fiscal years means the contract is severable" | Severability turns on the nature of the services, not duration |
+| "We can write the contract as non-severable to simplify funding" | Severability is determined by the nature of services, not contract language |
+| "FY25 funds can cover FY26 severable services as long as the contract was awarded in FY25" | No — each FY's services must be funded from that FY's appropriation |
+| "Severability is a FAR issue" | Severability is an **appropriations law** issue; FAR clauses implement it but do not create it |
+---
+## XI. ACQUISITION PLAN DOCUMENTATION REQUIREMENT
+The AP should explicitly document the severability determination:
+**For Non-Severable:**
+&gt; *"The services required under this acquisition constitute a non-severable undertaking. The contract will produce [specific deliverable] through interdependent tasks that cannot be meaningfully divided into discrete time periods. Accordingly, the entire contract value of $[X] will be obligated from FY [XXXX] appropriations, even though performance will extend into FY [XXXX+1]."*
+**For Severable:**
+&gt; *"The services required under this acquisition are severable in nature, consisting of recurring [description] services where each period's performance has independent value. The contract will cross fiscal year boundaries, requiring incremental funding: FY [XXXX] appropriations $[X] for services from [dates]; FY [XXXX+1] appropriations $[X] for services from [dates]."*
+---
+## XII. SUMMARY FLOWCHART
+```
+Service contract crosses fiscal years?
+│
+├─ NO → Fund normally from current-year appropriation
+│
+└─ YES → Is the service SEVERABLE or NON-SEVERABLE?
+          │
+          ├─ NON-SEVERABLE (single undertaking, unified deliverable)
+          │    → Need arises in FY of contract award
+          │    → Obligate full amount from current-year appropriation
+          │    → No incremental funding required
+          │
+          └─ SEVERABLE (recurring, each period independently valuable)
+               → Need arises in each FY of performance
+               → MUST fund incrementally: each FY's services from that FY's funds
+               → Exception: short bridge (1–3 months) for operational necessity
+               → Clauses: FAR 52.232-19 (fixed-price) or 52.232-22 (cost-reimb.)
+```
+---
+**Sources:**
+- *Appropriations Law: Time – Bona Fide Needs Rule* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- *Appropriations Law: Severable vs. Non-Severable Services* (GAO Red Book Ch. 5) — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- *Contract Obligation Timing GAO Guidance* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+- *Appropriations Law: Option Exercise Timing and Funding* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_options.txt`
+- 31 U.S.C. § 1502(a); FAR 32.703-2, 32.703-3, 52.232-19, 52.232-22; GAO Red Book (GAO-04-261SP), Chapter 5
+**Sources:**
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_IDIQ_funding.txt`
+</t>
+        </is>
+      </c>
+      <c r="AS11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW11" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX11" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved) [NEW QUESTION -- enhanced Q3]
+RO comparison: V9 provides the most comprehensive appropriations law response in the suite (12,595 chars). Covers statutory foundation, performance period rule, severable/non-severable, 10 USC 2410a, option exercise, edge cases.
+Tools: v9=[search_far, research]
+Cascade: FAR search + research subagent -- deep appropriations analysis.
+KB docs cited: V9=5 (severable, bona_fide_needs, options, IDIQ_funding, GAO_Guidance)
+Verdict: Exceptional -- most thorough appropriations response with edge cases.</t>
+        </is>
+      </c>
     </row>
-    <row r="12">
+    <row r="12" ht="409.5" customHeight="1">
       <c r="A12" s="20" t="n">
         <v>11</v>
       </c>
@@ -6631,6 +8524,47 @@
       <c r="D12" s="20" t="inlineStr">
         <is>
           <t>List every exception to the fair opportunity requirement for task orders under FAR 16.505(b)(2)(i), including the small business set-aside exception at subparagraph (F). There should be seven exceptions (A through G). Cite the exact FAR paragraph for each.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>compliance-strategist/FAR-guidance/
+302 files
+compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt
+71196 chars
+compliance-strategist/FAR-guidance/FAR_Part_16_Contract_Types_Comprehensive_RFO_2025.txt
+40101 chars
+Reasoning…
+think
+www.acquisition.gov
+1 sources
+FAR 16.505(b)(2)(i) exceptions fair opportunity task orders A through G text 2025
+27 results
+www.acquisition.gov, www.law.cornell.edu
+2 sources
+Reasoning…
+think
+Here are all seven exceptions, verbatim from the codified FAR (48 CFR 16.505(b)(2)(i)), verified against acquisition.gov and eCFR as of today.
+FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+The contracting officer shall give every awardee a fair opportunity to be considered for a delivery order or task order exceeding the micro-purchase threshold unless one of the following statutory exceptions applies:
+(A) — Urgency
+FAR 16.505(b)(2)(i)(A) The agency need for the supplies or services is so urgent that providing a fair opportunity would result in unacceptable delays.
+(B) — Unique/Highly Specialized Capability
+FAR 16.505(b)(2)(i)(B) Only one awardee is capable of providing the supplies or services required at the level of quality required because the supplies or services ordered are unique or highly specialized.
+(C) — Logical Follow-On
+FAR 16.505(b)(2)(i)(C) The order must be issued on a sole-source basis in the interest of economy and efficiency because it is a logical follow-on to an order already issued under the contract, provided that all awardees were given a fair opportunity to be considered for the original order.
+(D) — Minimum Guarantee
+FAR 16.505(b)(2)(i)(D) It is necessary to place an order to satisfy a minimum guarantee.
+(E) — Statutory Authority (Above SAT Only)
+FAR 16.505(b)(2)(i)(E) For orders exceeding the simplified acquisition threshold, a statute expressly authorizes or requires that the purchase be made from a specified source.
+(F) — Small Business Set-Aside (the exception you flagged)
+FAR 16.505(b)(2)(i)(F) In accordance with section 1331 of Public Law 111-240 (15 U.S.C. 644(r)), contracting officers may, at their discretion, set aside orders for any of the small business concerns identified in 19.000(a)(3). When setting aside orders for small business concerns, the specific small business program eligibility requirements identified in part 19 apply.
+(G) — FAR Part 6 Exceptions (DoD / NASA / Coast Guard Only)
+FAR 16.505(b)(2)(i)(G) For DoD, NASA, and the Coast Guard, the order satisfies one of the exceptions permitting the use of other than full and open competition listed in 6.302 (10 U.S.C. 3406(c)(5)). The public interest exception shall not be used unless Congress is notified in accordance with 10 U.S.C. 3204(a)(7).
+Three Practitioner Notes for NIH/HHS
+1. (F) is not a J&amp;A exception. Small business set-asides under (F) are explicitly exempt from the written justification, approval, and 14-day SAM.gov posting requirements at FAR 16.505(b)(2)(ii). Per the regulation, those requirements apply only to exceptions (A)–(E) and (G). An (F) set-aside requires compliance with FAR Part 19 eligibility rules — not a J&amp;A.
+2. (G) does not apply to NIH/HHS. This exception is limited by statute to DoD, NASA, and the Coast Guard (10 U.S.C. 3406(c)(5)). NIH COs cannot invoke it.
+3. HHS RFO structural note. Under HHS Class Deviation 2026-01 (the Revolutionary FAR Overhaul, effective November 21, 2025), this material was renumbered and restructured into FAR 16.507-6. The substance of exceptions (A)–(E) and (G) maps to 16.507-6(b)(1)–(6); the (F) small business carve-out moved to 16.507-6(c) as a separate paragraph rather than a numbered exception. The codified 48 CFR text at 16.505(b)(2)(i) has not yet been updated via rulemaking — both the old and new structural references are currently in circulation. If you're working in FPDS, the system still uses the (A)–(G) reporting codes.</t>
         </is>
       </c>
       <c r="AD12" s="20" t="inlineStr">
@@ -6684,8 +8618,84 @@
 </t>
         </is>
       </c>
+      <c r="AR12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are all **seven exceptions to the fair opportunity requirement** under **FAR 16.505(b)(2)(i)**, with exact paragraph citations. These apply to task and delivery orders placed on a sole-source basis above the micro-purchase threshold under multiple-award IDIQ contracts.
+---
+## Seven Exceptions to Fair Opportunity — FAR 16.505(b)(2)(i)
+| # | Exception | FAR Citation |
+|---|-----------|-------------|
+| A | **Urgency** | FAR 16.505(b)(2)(i)(A) |
+| B | **Unique/Highly Specialized** | FAR 16.505(b)(2)(i)(B) |
+| C | **Logical Follow-On** | FAR 16.505(b)(2)(i)(C) |
+| D | **Minimum Guarantee** | FAR 16.505(b)(2)(i)(D) |
+| E | **Statutory Authorization** | FAR 16.505(b)(2)(i)(E) |
+| F | **Small Business Set-Aside** | FAR 16.505(b)(2)(i)(F) |
+| G | **DoD/NASA/Coast Guard — Other Than Full and Open** | FAR 16.505(b)(2)(i)(G) |
+---
+### Verbatim Text of Each Exception
+**FAR 16.505(b)(2)(i)(A) — Urgency**
+&gt; The agency need for the supplies or services is **so urgent** that providing a fair opportunity would result in unacceptable delays.
+**FAR 16.505(b)(2)(i)(B) — Unique/Highly Specialized**
+&gt; **Only one awardee is capable** of providing the supplies or services required at the level of quality required because the supplies or services ordered are unique or highly specialized.
+**FAR 16.505(b)(2)(i)(C) — Logical Follow-On**
+&gt; The order must be issued on a sole-source basis in the interest of economy and efficiency because it is a **logical follow-on** to an order already issued under the contract, provided that all awardees were given a fair opportunity to be considered for the original order.
+**FAR 16.505(b)(2)(i)(D) — Minimum Guarantee**
+&gt; It is necessary to place an order to **satisfy a minimum guarantee**.
+**FAR 16.505(b)(2)(i)(E) — Statutory Authorization**
+&gt; For orders exceeding the SAT, a **statute expressly authorizes or requires** that the purchase be made from a specified source.
+**FAR 16.505(b)(2)(i)(F) — Small Business Set-Aside**
+&gt; In accordance with **FAR Part 19** and Public Law 111-240 (15 U.S.C. 644(r)), contracting officers may **set aside orders or place orders under reserves for small business concerns**. These actions are **not subject to** the justification, approval, and posting requirements that apply to exceptions (A)–(E) and (G).
+**FAR 16.505(b)(2)(i)(G) — DoD/NASA/Coast Guard Other Than Full and Open**
+&gt; For **DoD, NASA, and the Coast Guard only**, the order satisfies one of the exceptions permitting the use of **other than full and open competition** listed in FAR Part 6 (10 U.S.C. 3406(c)(5)). The public interest exception must not be used unless Congress is notified per 10 U.S.C. 3204(a)(7).
+---
+### Key Distinctions to Note
+| Feature | Exceptions (A)–(E) &amp; (G) | Exception (F) |
+|---|---|---|
+| Written justification required? | **Yes** (above SAT) | **No** |
+| Approval required? | **Yes** (tiered by value) | **No** |
+| GPE posting required (within 14 days)? | **Yes** (above SAT) | **No** |
+| Urgency posting deadline? | 30 days (exception A) | N/A |
+### Approval Thresholds for Exceptions (A)–(E) &amp; (G)
+| Order Value | Approving Official |
+|---|---|
+| Above SAT, ≤ $900K | Contracting Officer (self-certify) |
+| &gt; $900K – $20M | Advocate for Competition |
+| &gt; $20M – $90M | Head of Procuring Activity |
+| &gt; $90M | Senior Procurement Executive |
+*(DoD/NASA/Coast Guard thresholds: $150M for HPA level and SPE level)*
+---
+**Source:** FAR Part 16, Subpart 16.5 — *Ordering: Fair Opportunity and Exceptions* (`eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`), incorporating HHS Class Deviation 2026-01 (RFO). Standard FAR 16.505 numbering used throughout per the cross-reference table in that document.
+</t>
+        </is>
+      </c>
+      <c r="AS12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU12" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW12" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="AX12" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 = RO (comparable) [NEW QUESTION -- enhanced Q4]
+RO comparison: Both list all 7 FAR 16.505(b)(2)(i) exceptions with verbatim text. V9 includes exact paragraph citations and approval dollar thresholds. RO had web-supplemented verification.
+Tools: v9=[search_far, knowledge_fetch]
+Cascade: search_far -&gt; knowledge_fetch -- standard regulatory lookup.
+KB docs cited: V9=1 (FAR_Part_16_IDIQ_Comprehensive_RFO_2025)
+Verdict: Strong regulatory response -- verbatim text adds value. Sources adequate.</t>
+        </is>
+      </c>
     </row>
-    <row r="13">
+    <row r="13" ht="409.5" customHeight="1">
       <c r="A13" s="20" t="n">
         <v>12</v>
       </c>
@@ -6702,6 +8712,152 @@
       <c r="D13" s="20" t="inlineStr">
         <is>
           <t>An offeror eliminated from a SBIR Phase II competition wants to protest at GAO. Search the knowledge base for all relevant protest guidance documents, including GAO bid protest guides, NIH stay provision policies, and debriefing requirements. List each KB document found with its file path before analyzing the protest process.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>legal-counselor/
+302 files
+compliance-strategist/
+302 files
+Good — I've found the full KB structure. Now let me pull all seven protest-relevant documents simultaneously.
+legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt
+17606 chars
+legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt
+22462 chars
+legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt
+17094 chars
+legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt
+14773 chars
+legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt
+5549 chars
+legal-counselor/protest-guidance/JA_Desk_Guide_January_2025_Updated.txt
+57126 chars
+legal-counselor/protest-guidance/GAO_B-409917_Failure_to_Rebut_Agency_Arguments.txt
+26005 chars
+Now let me also pull the two remaining protest files — the timeliness case and the interested party case — plus check the FAR Part 15 debriefing provisions and NIH R&amp;D policy (relevant for SBIR).
+legal-counselor/protest-guidance/GAO_B-419831_PIA_Allegations_Interested_Party.txt
+25651 chars
+legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt
+9796 chars
+compliance-strategist/NIH-policies/NIH_6315_1_RD_Contracts_Part2_Evaluation_Award.txt
+38005 chars
+Reasoning…
+think
+Here is the complete analysis — starting with the KB document inventory, then the SBIR-specific protest process.
+KB Documents Found: Protest-Relevant Files
+Primary Protest Guidance (9 documents in legal-counselor/protest-guidance/)
+#	File Path	What It Covers
+1	legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt	GAO 10th Ed. (GAO-18-510SP) — full procedural guide: jurisdiction, timeliness, filing, agency report, protective orders, decisions
+2	legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt	NIH Manual 6033-2 (EAGLE-annotated) — D&amp;F procedures, routing, approval authority for stay override
+3	legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt	NIH Policy Manual 6033-2 (original 2008 text) — D&amp;F templates, routing slip, DASAMP approval chain
+4	legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt	NIH Manual 6033-1 — format/content of CO's Statement of Facts; submission routing and deadlines
+5	legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt	FAR Companion Part 33 — solicitation clarity, documentation practices, debriefing best practices, ADR
+6	legal-counselor/protest-guidance/GAO_B-409917_Failure_to_Rebut_Agency_Arguments.txt	Gella LLC (NIH LTASC) — failure-to-rebut doctrine; reevaluation consistency; similar experience
+7	legal-counselor/protest-guidance/GAO_B-419831_PIA_Allegations_Interested_Party.txt	Alpine Companies — interested party standing; PIA reporting; clarifications vs. material exceptions
+8	legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt	Optimo IT (NIH CIO-SP4) — EPDS strict deadlines; 5:30 PM cutoff; no email filing when EPDS functional
+9	legal-counselor/protest-guidance/JA_Desk_Guide_January_2025_Updated.txt	J&amp;A Desk Guide — competition requirements, authorities (tangentially relevant to protest grounds)
+Supporting NIH R&amp;D Policy
+#	File Path	What It Covers
+10	compliance-strategist/NIH-policies/NIH_6315_1_RD_Contracts_Part2_Evaluation_Award.txt	NIH Manual 6315-1 Part 2 — R&amp;D SRG evaluation, competitive range, FAR 15.505/15.506 debriefings, source selection documentation
+11	legal-counselor/ethics-integrity/ACQuipedia_Protests_Integrity_Ethics.txt	Procurement integrity / protest ethics (listed in KB index; complements the above)
+SBIR Phase II Protest at GAO: Complete Analysis
+⚠️ Threshold Issue #1 — Is This a Contract or a Grant?
+This is the first question to resolve before anything else. GAO has bid protest jurisdiction only over federal contracts, not grants or cooperative agreements.
+If the SBIR Phase II award is a contract → GAO jurisdiction exists under CICA (31 U.S.C. §§ 3551–3556)
+If it's a grant or cooperative agreement → GAO has no jurisdiction; the offeror's only avenue is agency-level appeal or SBA
+Many NIH SBIR Phase II awards are grants. If this is an NCI SBIR Phase II contract, the full GAO protest process applies. Confirm the award instrument type immediately.
+⚠️ Threshold Issue #2 — Is the Offeror an "Interested Party"?
+Per B-419831 (Alpine Companies) and 4 C.F.R. § 21.0(a)(1):
+An interested party is an actual or prospective offeror whose direct economic interest would be affected, and who would be in line for award if the protest were sustained.
+For SBIR Phase II, eligibility is restricted to Phase I awardees. If the offeror:
+Never completed Phase I, or
+Was found technically unacceptable on its face, or
+Could not receive award even if all protest grounds were sustained
+...then GAO will dismiss for lack of standing. The CO should assess this early and argue it in the agency report if applicable.
+Step-by-Step: The Protest Process
+PHASE 1 — Immediate Actions (Day 0–5)
+When NIH receives notice from GAO that a protest has been filed:
+Action	Authority	Deadline
+Litigation hold — preserve ALL acquisition records, emails, documents	NIH Manual 6033-1	Immediately
+Notify OGC-GLD (Departmental Protest Control Officer)	NIH Manual 6033-1	Day 1
+Notify NIH Protest Control Officer (PCO) at DAPE, OAMP	NIH Manual 6033-1	Day 1
+Determine if statutory stay applies (award within 10 days, or within 5 days of debriefing offered)	FAR 33.104(b)/(c); NIH 6033-2	Day 1
+Transmit protest file (4 copies to DPCO/OGC-GLD, 1 to NIH PCO) — all documents except CO Statement	NIH Manual 6033-1	Day 5
+PHASE 2 — Debriefing (If Not Yet Provided)
+Per FC_33_Protests_Disputes_Appeals.txt and FAR 15.505/15.506:
+Pre-award (competitive range exclusion): FAR 15.505 debriefing — offeror may request before award
+Post-award: FAR 15.506 debriefing — written request required within 3 days of notification
+Critical timing interaction (per GAO Essential Guide, 4 C.F.R. § 21.2):
+If a required debriefing has been offered, the protest timeliness clock does not start until the debriefing date. The protester has 10 calendar days after the debriefing to file at GAO.
+The CICA stay is triggered if GAO notifies NIH of the protest within 10 days of award OR 5 days of the debriefing date offered, whichever is later.
+Per FC_33: Avoid unnecessarily extending the protest window — offer debriefings promptly. Consider including technical evaluation documentation relevant to the requesting vendor. Frame debriefings as learning opportunities, not adversarial events.
+PHASE 3 — Stay Determination (Days 1–5 if needed)
+Per NIH Manual 6033-2 (both versions):
+If the CICA stay is triggered and NIH wants to proceed with award or continue performance anyway, the CO must prepare a Determination &amp; Findings (D&amp;F) stating:
+Situation	Standard Required
+Pre-award protest — proceed with award	(a) Urgent and compelling circumstances, AND (b) award likely within 30 days
+Post-award protest — continue performance	EITHER (a) Performance in best interest of U.S., OR (b) Urgent and compelling circumstances
+NIH-Specific Approval Chain — NOT DELEGABLE:
+CO prepares D&amp;F
+    ↓
+CO's Supervisor
+    ↓
+IC Director, Office of Acquisitions
+    ↓
+NIH Protest Control Officer (DAPE, OAMP)
+    ↓
+HCA (Head of Contracting Activity) — executes D&amp;F [authority NOT redelegable]
+    ↓
+OGC-GLD concurrence
+    ↓
+DASAMP (Deputy Asst. Secretary for Acquisition Mgmt &amp; Policy, HHS) — approves
+    ↓
+OGC-GLD notifies GAO
+SBIR R&amp;D arguments for "best interest" justification might include: patient/research continuity, irreplaceable biological samples, clinical trial participant safety, or fiscal year funding expiration.
+PHASE 4 — CO's Statement of Facts (Day 14)
+Per NIH Manual 6033-1, the CO Statement must follow the recommended 4-section format:
+Section	Content
+1. Background	Purpose of acquisition, brief history, estimated contract value
+2. Chronology	AP date, SAM.gov posting, RFP release, proposal due date, SRG evaluation, competitive range, award date, debriefing dates, protest receipt date
+3. Issues, Findings &amp; Circumstances	Address each allegation individually — both favorable and unfavorable rationale. Separate technical, business, and administrative allegations.
+4. Summary &amp; Recommendations	CO's conclusions supporting agency position
+Mark all sets: "Immediate Action – GAO Protest B-[number]"
+PHASE 5 — Agency Report (Day 30)
+Per the GAO Essential Guide (4 C.F.R. § 21.3), the full agency report must include:
+CO Statement (signed)
+Memorandum of law (prepared by OGC-GLD)
+Protester's proposal
+Evaluation documents (TER, scoring sheets, SRG documentation per NIH 6315-1)
+Source selection documentation
+Solicitation and all amendments
+Abstract of offers
+5 days before report due: File list of documents being released vs. withheld (with reasons). Protester has 2 days to object.
+Early voluntary disclosure encouraged — per GAO Essential Guide, early document production can resolve protests faster and prevents piecemeal supplemental filings.
+PHASE 6 — Comments and Decision
+Milestone	Deadline
+Protester's comments on agency report	10 calendar days after report filed
+Failure to file comments → mandatory dismissal	—
+Standard GAO decision	100 calendar days from protest filing
+Express option (if requested within 5 days)	65 calendar days
+Per Gella LLC (B-409917, NIH): If the agency provides a detailed response and the protester merely states "we stand on our initial protest" without substantively rebutting each argument, GAO will find no basis to sustain — the protest is effectively conceded by the protester's silence.
+SBIR Phase II–Specific Protest Vulnerabilities
+Based on the NIH 6315-1 R&amp;D evaluation framework, the most common protest grounds in a SBIR Phase II competition are:
+Risk	What GAO Reviews	Mitigation
+Improper SRG evaluation	Whether evaluation followed stated criteria in RFP	Document SRG scores, strengths/weaknesses by criterion; no predetermined cutoffs
+Untimely competitive range notification	Whether excluded offeror was notified and offered debriefing	Notify promptly under FAR 15.505
+Unstated evaluation criteria	Whether factors not in RFP were applied	Stick exactly to RFP evaluation criteria; field-specific experience must be "reasonably encompassed" by stated criteria (Gella LLC)
+Misleading discussions	Whether all competitive range offerors received equal opportunity	Document all discussion questions; treat all offerors consistently
+Past performance	No relevant past performance → neutral, not negative per FAR 15.305(a)(2)(iv)	Assign neutral; do not exclude (Alpine Companies)
+PIA allegations	If protester claims source selection info was leaked	Require protester to provide specifics within 14 days; document CO response
+Filing timeliness (against protester)	Whether protest filed within 10 days of known basis	Argue untimeliness if protest basis was knowable before or at debriefing
+⚠️ What the KB Does NOT Cover
+The KB has no SBIR-specific protest guidance. One important external note: Under the Small Business Act (15 U.S.C. § 638(j)(2)(A)), agencies have broad discretion in SBIR Phase II selections based on Phase I performance. GAO has held that SBIR Phase II funding decisions are within agency discretion where the solicitation and evaluation criteria were applied as announced. However, procedural defects (improper evaluation, disparate treatment, failure to follow stated criteria) remain fully protestable.
+Bottom Line for the CO
+Three immediate actions:
+Confirm award instrument (contract vs. grant) — determines GAO jurisdiction
+Assess interested party standing — was protester actually in line for award if sustained?
+Impose litigation hold and notify OGC-GLD today — the 5-day file production deadline is unforgiving</t>
         </is>
       </c>
       <c r="AD13" s="20" t="inlineStr">
@@ -6818,8 +8974,183 @@
 </t>
         </is>
       </c>
+      <c r="AR13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is the complete analysis, organized exactly as requested — KB documents first, then the substantive protest guidance.
+---
+## Knowledge Base Documents Found — SBIR Phase II GAO Protest
+### 📁 Protest Guidance Folder: `eagle-knowledge-base/approved/legal-counselor/protest-guidance/`
+| # | Title | S3 File Path |
+|---|-------|-------------|
+| 1 | **GAO Bid Protests — Essential Guide for Contracting Officers** *(GAO-18-510SP, 10th Ed.)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt` |
+| 2 | **FAR Companion Part 33: Protests, Disputes, and Appeals** *(v2.0, Oct 2025)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt` |
+| 3 | **NIH Manual 6033-2: Stay Provisions for Protests** *(Updated 2008, current HHSAR version)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt` |
+| 4 | **NIH Policy Manual 6033-2: Stay Provisions for Protests** *(2008 policy version)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt` |
+| 5 | **NIH Manual 6033-1: Contracting Officer's Statement of Facts and Circumstances in GAO Protests** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt` |
+| 6 | **GAO Decision B-419956.258: EPDS Filing Timeliness** *(Optimo IT v. NIH/CIO-SP4, June 2023)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt` |
+### 📁 Related Supporting Documents
+| # | Title | S3 File Path |
+|---|-------|-------------|
+| 7 | **ACQuipedia — Protests, Integrity, and Ethics** | `eagle-knowledge-base/approved/legal-counselor/ethics-integrity/ACQuipedia_Protests_Integrity_Ethics.txt` |
+| 8 | **NIH Policy Manual 6035: Broad Agency Announcements** *(Contains SBIR-adjacent debriefing rules)* | `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Policy_6035_Broad_Agency_Announcements_2016.txt` |
+| 9 | **FAR Part 15 — Contracting by Negotiation (RFO 2025)** *(Pre/post-award debriefing requirements)* | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Negotiation_RFO_2025.txt` |
+| 10 | **FAR Part 15 — Source Selection (FAR 2.0/RFO Version)** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Source_Selection_RFO_2025.txt` |
+---
+## Analysis: GAO Protest by Eliminated SBIR Phase II Offeror
+### ⚠️ Threshold Issue — SBIR Is a Special Case
+The KB documents flag this immediately: **NIH Policy Manual 6035 (BAAs) explicitly carves out SBIR** — *"The requirements of this manual chapter do NOT apply to the Small Business Innovation Research (SBIR) program."* SBIR Phase II competitions use a BAA-like process but operate under their own statutory framework (15 U.S.C. § 638). This creates a nuanced jurisdictional landscape for GAO.
+---
+### 1. GAO Jurisdiction Over SBIR Phase II Protests
+**Authority:** Competition in Contracting Act (31 U.S.C. §§ 3551–3556); GAO Bid Protest Regulations, 4 C.F.R. Part 21.
+GAO **can** hear SBIR Phase II protests where the allegation is that the **agency failed to follow the stated evaluation criteria or applicable regulations** — not broad programmatic decisions. GAO does **not** address:
+- Which company's proposal was scientifically superior
+- Programmatic management decisions
+- SBA SBIR policy decisions (SBA jurisdiction)
+The offeror must qualify as an **"interested party"** — an actual offeror with a direct economic interest, meaning it would be in line for award if the protest were sustained (4 C.F.R. § 21.0(a)).
+---
+### 2. Debriefing Requirements — Critical Threshold Step
+**Source: NIH Policy Manual 6035 (BAA/SBIR-adjacent); FAR 15.506**
+For **FAR-based** SBIR Phase II awards, the eliminated offeror is entitled to a **post-award debriefing** if it:
+- Submits a **written request within 3 days** of receiving notice that its proposal was not selected
+NIH must then:
+- Provide the debriefing **within 5 days** of receiving the written request (to the maximum extent practicable)
+**Mandatory debriefing content (from NIH Policy 6035):**
+| ✅ Must Include | ❌ Must NOT Include |
+|----------------|-------------------|
+| Evaluation of significant proposal elements | Number of other proposals submitted |
+| Rationale summary for non-selection | Identity or content of other proposals |
+| Responses to procedural compliance questions | Ranking or evaluation of other proposals |
+| | Point-by-point comparisons with other proposals |
+| | Trade secrets or privileged commercial/financial data |
+&gt; **Why this matters for protest strategy:** The debriefing date controls the protest deadline. Per the GAO Essential Guide, where a debriefing is required by FAR 15.505/15.506, the protest **shall not be filed before the debriefing date offered** and must be filed **no later than 10 calendar days after the debriefing is held.**
+---
+### 3. Filing the GAO Protest — Timeliness Is Everything
+**Source: GAO Essential Guide (4 C.F.R. § 21.2); GAO Decision B-419956.258**
+&gt; ⚠️ **The most common reason GAO dismisses protests is timeliness.** This is strictly enforced with no grace periods.
+| Scenario | Deadline |
+|----------|----------|
+| Protest ground known before or during debriefing | **10 calendar days after debriefing held** — do NOT file before debriefing |
+| Protest ground known independent of debriefing | **10 calendar days from when basis known or should have been known** |
+| After agency-level protest: GAO follow-on | **10 calendar days from adverse agency action** |
+**Days are calendar days.** If the last day falls on a Saturday, Sunday, or Federal holiday, the deadline extends to the next business day.
+**The offeror must diligently pursue information** — including requesting prompt debriefings. Waiting passively does not toll the 10-day clock.
+---
+### 4. Filing Mechanics — EPDS Requirements
+**Source: GAO Decision B-419956.258 (Optimo IT v. NIH, June 2023)**
+This NIH-specific GAO case is directly on point. Key rules:
+- All protests **must be filed in EPDS** (epds.gao.gov) by **5:30 PM Eastern Time** on the deadline day
+- A document is "filed" only when received in EPDS — email to protests@gao.gov does **not** count when EPDS is functioning normally
+- **10 minutes late = dismissal.** No exceptions for user-side technical issues
+- Alternative email filing is **only** permitted when EPDS has a confirmed system-wide failure — and only after contacting GAO to confirm the outage
+**Best practice:** File at least 1–2 business days early; never plan to file on the deadline day.
+**Required protest content (4 C.F.R. § 21.1):**
+1. Protester name, address, email, phone (attorney if represented)
+2. Electronic signature
+3. Agency name and solicitation/contract number
+4. **Detailed statement of legal and factual grounds** (with copies of relevant documents)
+5. Statement establishing interested party status
+6. Statement establishing timeliness
+7. Specific request for ruling by Comptroller General
+8. Form of relief requested
+A copy must also be furnished to the CO (or designated protest recipient) **no later than 1 day after filing with GAO.**
+---
+### 5. Automatic Stay of Performance (CICA Stay)
+**Source: NIH Manual 6033-2; NIH Policy 6033-2 (2008); FAR 33.104**
+When a GAO protest is filed, an **automatic stay** suspends award or performance **if** the protest is filed within:
+- **10 calendar days after contract award**, OR
+- **5 calendar days after the debriefing date offered** to the protester
+- *Whichever is later*
+**Override — To Proceed Despite a Stay (GAO Protest):**
+NIH must prepare a written **Determination and Findings (D&amp;F)** and navigate a multi-level approval chain — the highest in the federal acquisition system:
+```
+CO prepares D&amp;F
+     ↓
+IC Director, Office of Acquisitions
+     ↓
+NIH Protest Control Officer (DAPE/OAMP)
+     ↓
+Head of Contracting Activity (HCA) — executes (NOT delegable)
+     ↓
+Deputy Assistant Secretary for Acquisition Management
+and Policy (DASAMP), OS, DHHS — final approval
+```
+**Standard for pre-award protests:** Urgent and compelling circumstances + award likely within 30 days.
+**Standard for post-award protests:** Contract performance in the best interest of the United States, **OR** urgent and compelling circumstances.
+---
+### 6. Agency Response Process
+**Source: NIH Manual 6033-1; GAO Essential Guide (4 C.F.R. § 21.3)**
+Once GAO notifies NIH of the protest, internal NIH deadlines are:
+| Deadline | Action |
+|----------|--------|
+| **5 calendar days** from receipt | Complete protest file (all documents except CO Statement) → OGC-GLD (4 copies) + NIH PCO (1 copy) |
+| **14 calendar days** from receipt | CO's Statement of Facts and Circumstances due |
+| **30 calendar days** from receipt | OGC-GLD submits complete Agency Report to GAO |
+The CO Statement (NIH Manual 6033-1) must include:
+- **Section 1 – Background:** Acquisition overview, contract value estimate
+- **Section 2 – Chronology of Events:** From AP through award through protest receipt
+- **Section 3 – Issues, Findings, Circumstances:** Each allegation addressed individually
+- **Section 4 – Summary/Recommendations**
+**⚠️ Litigation Hold:** Upon receipt of protest, ALL relevant records (including email and ESI) must be immediately preserved. The litigation hold overrides any normal records retention schedule.
+**Key contacts:**
+- **NIH PCO:** DAPE/OAMP/OALM, 6100 Executive Blvd., Room 6C01, (301) 496-6014
+- **Departmental PCO (OGC-GLD):** 200 Independence Ave. SW, Room 713-F, (202) 619-0150
+---
+### 7. GAO Decision Timeline and Outcomes
+**Source: GAO Essential Guide (4 C.F.R. § 21.9)**
+| Track | Decision Issued |
+|-------|----------------|
+| Standard | Within **100 calendar days** of filing |
+| Express Option | Within **65 calendar days** (request within 5 days of filing) |
+Three possible outcomes:
+1. **Dismiss** — procedural/substantive defects (timeliness most common)
+2. **Deny** — agency complied with regulations, or violation caused no prejudice
+3. **Sustain** — agency violated statute/regulation and protester was prejudiced
+**If sustained:** GAO may recommend recompete, new source selection, or award consistent with applicable rules. GAO also typically recommends reimbursement of the protester's protest costs (filing fees, reasonable attorney's fees, expert witness fees) — but never lost profits.
+---
+### Summary Checklist for the SBIR Phase II Offeror
+```
+□ 1. Request debriefing in writing within 3 days of notice of non-selection
+□ 2. Attend debriefing — this starts the 10-day protest clock
+□ 3. Identify protest grounds (evaluation criteria not followed? Procedural error?)
+□ 4. File protest in EPDS no later than 10 calendar days after debriefing
+□ 5. File before 5:30 PM Eastern — plan to file 1-2 days early
+□ 6. Serve copy on CO within 1 day of GAO filing
+□ 7. Include all required EPDS content (detailed legal/factual grounds)
+□ 8. Request protective order if proprietary info likely to be at issue
+□ 9. File comments on Agency Report within 10 calendar days of report
+□ 10. Consider requesting Express Option (65-day track) within 5 days of filing
+```
+&gt; **Bottom line:** The debriefing is the strategic pivot point — it locks in the protest deadline, defines the protest grounds, and triggers the stay window. An SBIR Phase II offeror should request the debriefing immediately upon receiving rejection notice and use it to identify any deviations from the stated evaluation criteria before the 10-day clock runs.
+</t>
+        </is>
+      </c>
+      <c r="AS13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AT13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW13" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX13" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &gt; RO (improved) [NEW QUESTION -- enhanced Q5/SBIR protest]
+RO comparison: V9 provides KB document inventory FIRST (11 documents with full S3 paths), then substantive protest analysis. RO pulls similar docs but V9's format is more transparent and reproducible.
+Tools: v9=[knowledge_search, knowledge_fetch]
+Cascade: KB search -&gt; fetch -- deep retrieval (11 unique KB paths). Highest source count in entire baseline suite.
+KB docs cited: V9=11 (GAO Essential Guide, FC_33, NIH 6033-2, NIH 6033-1, etc.)
+Verdict: Exceptional -- transparent KB inventory + comprehensive analysis.</t>
+        </is>
+      </c>
     </row>
-    <row r="14">
+    <row r="14" ht="409.5" customHeight="1">
       <c r="A14" s="20" t="n">
         <v>13</v>
       </c>
@@ -6838,9 +9169,75 @@
           <t>Generate a Statement of Work for a $200,000 annual IT help desk support contract for the NCI Center for Biomedical Informatics and Information Technology (CBIIT). Requirements: 5 FTEs providing Tier 1-3 support, 24/7 coverage, SLA of 15-minute response for Tier 1. Before generating, identify which SOW template from the knowledge base you will use and show its full S3 path in your reasoning.</t>
         </is>
       </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>supervisor-core/essential-templates/
+302 files
+supervisor-core/
+302 files
+Two SOW templates exist in the KB. Let me discover both to determine which is better suited for an IT services contract, and also pull the HHSAR security checklist guidance since this is IT work at NCI.
+Reading statement-of-work-template-eagle-v2.docx
+0 blocks
+Reading statement-of-work-template-eagle.docx
+0 blocks
+compliance-strategist/HHSAR-guidance/HHSAR_CD_2024_01_OAMS_Security_Checklist_Guide.txt
+13910 chars
+Reasoning…
+think
+Good. I have everything I need. Here's my reasoning before generating:
+Template Selected: s3://rh-eagle/supervisor-core/essential-templates/statement-of-work-template-eagle-v2.docx
+I found two SOW templates in the KB:
+statement-of-work-template-eagle.docx (v1) — space-separated placeholders
+statement-of-work-template-eagle-v2.docx (v2) — underscore-separated placeholders, newer formatting
+v2 is the correct choice — it's the current version with updated placeholder syntax.
+HHSAR CD 2024-01 mapping for this IT services contract: Per HHSAR_CD_2024_01_OAMS_Security_Checklist_Guide.txt, this aligns with Scenario B (IT Managed Services with Government Data Access), triggering: HHSAR 352.204-71, 352.204-72, 352.204-73, 352.239-71/72, 352.239-74, 352.239-78/79.
+Now generating the filled SOW:
+Filling statement-of-work-template-eagle-v2.docx
+1 warnings
+Reasoning…
+think
+Several sections didn't take in the first pass due to multi-paragraph text keys and HTML encoding differences. Executing a complete index-based replacement pass now:
+Filling statement-of-work-template-eagle-v2.docx
+1 warnings
+Reasoning…
+think
+The index-based replacement isn't firing (the tool appears to process these from the original template each time, and certain paragraph styles resist both approaches). Let me do a targeted final pass with exact single-paragraph text keys for all remaining sections:</t>
+        </is>
+      </c>
       <c r="AD14" s="20" t="inlineStr">
         <is>
           <t>[RERUN] Tools: create_document | Response: Generated a draft sow document. You can open it from the document card. | ISSUE: Agent generated SOW correctly but did NOT show template name or S3 path before generating. This confirms EAGLE-77 is still open.</t>
+        </is>
+      </c>
+      <c r="AR14" s="20" t="inlineStr">
+        <is>
+          <t>Generated a draft sow document. You can open it from the document card.
+**Template:** Using template: Statement of Work (SOW) Template - Eagle v2 (eagle-knowledge-base/approved/supervisor-core/essential-templates/statement-of-work-template-eagle-v2.docx)</t>
+        </is>
+      </c>
+      <c r="AS14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AT14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW14" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="AX14" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V9 &lt; RO (regression) [NEW QUESTION -- SOW generation]
+RO comparison: RO provides 1,907 chars of context about the generated SOW including key sections, scope elements, and contract details. V9 returns only 255 chars saying 'Generated a draft sow document.' The actual SOW exists as a document artifact, but the chat response lacks summary or preview.
+Tools: v9=[create_document]
+Cascade: Document generation uses correct template (SOW Template Eagle v2).
+KB docs cited: V9=1 (template path only)
+Verdict: Document generated correctly but chat response too terse. User must navigate to document card. create_document should echo key sections back.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add RO vs EAGLE search comparison doc, update Jira QA memo, baseline Excel
- New: RO vs EAGLE search pipeline comparison documenting path-first vs
  AI-ranking-first discovery strategies and the hybrid fix
- Update Jira QA EAGLE-70-77 resolution memo
- Excel: baseline question responses from path-search testing

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Use Case List.xlsx
+++ b/Use Case List.xlsx
@@ -89,7 +89,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +144,12 @@
         <bgColor rgb="002E7D32"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+        <bgColor rgb="001565C0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -172,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -237,6 +243,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3168,7 +3177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX14"/>
+  <dimension ref="A1:BT14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.26953125" defaultRowHeight="70" customHeight="1"/>
   <cols>
     <col width="9.26953125" customWidth="1" style="5" min="1" max="3"/>
@@ -3203,6 +3212,28 @@
     <col width="14" customWidth="1" min="48" max="48"/>
     <col width="14" customWidth="1" min="49" max="49"/>
     <col width="100" customWidth="1" min="50" max="50"/>
+    <col width="100" customWidth="1" min="51" max="51"/>
+    <col width="14" customWidth="1" min="52" max="52"/>
+    <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="56" max="56"/>
+    <col width="100" customWidth="1" min="57" max="57"/>
+    <col width="100" customWidth="1" min="58" max="58"/>
+    <col width="14" customWidth="1" min="59" max="59"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
+    <col width="14" customWidth="1" min="61" max="61"/>
+    <col width="14" customWidth="1" min="62" max="62"/>
+    <col width="14" customWidth="1" min="63" max="63"/>
+    <col width="100" customWidth="1" min="64" max="64"/>
+    <col width="100" customWidth="1" min="65" max="65"/>
+    <col width="100" customWidth="1" min="66" max="66"/>
+    <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="14" customWidth="1" min="68" max="68"/>
+    <col width="14" customWidth="1" min="69" max="69"/>
+    <col width="14" customWidth="1" min="70" max="70"/>
+    <col width="14" customWidth="1" min="71" max="71"/>
+    <col width="100" customWidth="1" min="72" max="72"/>
   </cols>
   <sheetData>
     <row r="1" ht="70" customFormat="1" customHeight="1" s="2">
@@ -3454,6 +3485,116 @@
       <c r="AX1" s="23" t="inlineStr">
         <is>
           <t>V9 vs RO + V8 Comparative Judgment</t>
+        </is>
+      </c>
+      <c r="AY1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V10 Response (2026-04-07)</t>
+        </is>
+      </c>
+      <c r="AZ1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V10 Accuracy (0-5)</t>
+        </is>
+      </c>
+      <c r="BA1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V10 Completeness (0-5)</t>
+        </is>
+      </c>
+      <c r="BB1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V10 Sources (0-5)</t>
+        </is>
+      </c>
+      <c r="BC1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V10 Actionability (0-5)</t>
+        </is>
+      </c>
+      <c r="BD1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V10 Total (0-20)</t>
+        </is>
+      </c>
+      <c r="BE1" s="23" t="inlineStr">
+        <is>
+          <t>V10 vs RO + V9 Comparative Judgment</t>
+        </is>
+      </c>
+      <c r="BF1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V11 Response (2026-04-07)</t>
+        </is>
+      </c>
+      <c r="BG1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V11 Accuracy (0-5)</t>
+        </is>
+      </c>
+      <c r="BH1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V11 Completeness (0-5)</t>
+        </is>
+      </c>
+      <c r="BI1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V11 Sources (0-5)</t>
+        </is>
+      </c>
+      <c r="BJ1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V11 Actionability (0-5)</t>
+        </is>
+      </c>
+      <c r="BK1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V11 Total (0-20)</t>
+        </is>
+      </c>
+      <c r="BL1" s="23" t="inlineStr">
+        <is>
+          <t>V11 vs RO + V10 Comparative Judgment</t>
+        </is>
+      </c>
+      <c r="BM1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Response (2026-04-07)</t>
+        </is>
+      </c>
+      <c r="BN1" s="23" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Response (2026-04-07)</t>
+        </is>
+      </c>
+      <c r="BO1" s="24" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Accuracy (0-5)</t>
+        </is>
+      </c>
+      <c r="BP1" s="24" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Completeness (0-5)</t>
+        </is>
+      </c>
+      <c r="BQ1" s="24" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Sources (0-5)</t>
+        </is>
+      </c>
+      <c r="BR1" s="24" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Actionability (0-5)</t>
+        </is>
+      </c>
+      <c r="BS1" s="24" t="inlineStr">
+        <is>
+          <t>EAGLE V12 Total (0-20)</t>
+        </is>
+      </c>
+      <c r="BT1" s="24" t="inlineStr">
+        <is>
+          <t>V12 vs RO + V11 Comparative Judgment</t>
         </is>
       </c>
     </row>
@@ -3793,6 +3934,192 @@
 Cascade: N/A -- threshold lookup, no KB cascade needed.
 KB docs cited: V8=0 | V9=0 (unchanged, expected for compliance_matrix queries)
 Verdict: Stable -- compliance matrix tool delivers accurate threshold data.</t>
+        </is>
+      </c>
+      <c r="AY2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Based on the official HHS and NIH guidance effective October 1, 2025 (FAC 2025-06):
+## Current Acquisition Thresholds
+**Micro-Purchase Threshold (MPT): $15,000** (increased from $10,000)
+**Simplified Acquisition Threshold (SAT): $350,000** (increased from $250,000)
+### Threshold Variations by Category
+**Micro-Purchase Threshold Exceptions:**
+- Construction (Davis-Bacon Act): **$2,000**
+- Service Contract Labor Standards: **$2,500**
+- Contingency Operations (inside U.S.): **$25,000**
+- Contingency Operations (outside U.S.): **$40,000**
+**Simplified Acquisition Threshold Exceptions:**
+- Contingency Operations (inside U.S.): **$1,000,000**
+- Contingency Operations (outside U.S.): **$2,000,000**
+- Humanitarian/Peacekeeping Operations (outside U.S.): **$650,000**
+- Commercial Items Simplified Procedures (FAR 13.500): **$9,000,000**
+### Key Triggered Requirements
+**Above $15,000 MPT:**
+- Small business set-aside consideration required
+- HHS-653 Small Business Review Form required
+**Above $25,000:**
+- Synopsis required or exception documented
+**Above $350,000 SAT:**
+- Full Acquisition Plan required (FAR 7.105)
+- Market Research Report required
+- J&amp;A required for sole source
+- Enhanced competition procedures
+- CPARS evaluations required
+---
+**Sources:**
+- HHS PMR Threshold-Based Requirements Matrix (FAC 2025-06) - eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_Threshold_Matrix.txt
+- NIH Acquisition Glossary (November 2025 Update) - eagle-knowledge-base/approved/supervisor-core/core-procedures/NIH_Acquisition_Glossary.txt
+- NIH Purchase Card Supplement (2025) - eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Purchase_Card_Supplement_Streamlined_2025.txt
+**Sources:**
+- `eagle-knowledge-base/approved/supervisor-core/core-procedures/HCA_SPE_Approval_Thresholds_Updated.txt`
+</t>
+        </is>
+      </c>
+      <c r="AZ2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD2" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE2" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: Both correctly cite $15K MPT, $350K SAT under FAC 2025-06. V10 now uses the research tool instead of query_compliance_matrix, reading 4 KB documents: HHS_PMR_Threshold_Matrix, NIH_Acquisition_Glossary, NIH_Purchase_Card_Supplement, HCA_SPE_Approval_Thresholds. Adds all MPT exceptions (construction, SCA, contingency inside/outside U.S.) and SAT exceptions (contingency, humanitarian, commercial FAR 13.500).
+v9 vs v10: MAJOR IMPROVEMENT -- V9 used query_compliance_matrix (0 KB docs). V10 uses research tool, reading 4 KB docs. Response grew 790-&gt;1,854 chars. Sources score improves from 4-&gt;5.
+Tools: v9=[query_compliance_matrix] | v10=[research]
+KB docs cited: V9=0 | V10=4 (+4 improvement)
+Verdict: Research tool upgrade delivers threshold data WITH policy context.</t>
+        </is>
+      </c>
+      <c r="BF2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under **FAC 2025-06** (effective October 1, 2025), the two key thresholds are:
+---
+### Micro-Purchase Threshold (MPT) — FAR 13.2
+| Category | Threshold |
+|---|---|
+| **General (supplies/services)** | **$15,000** |
+| Services subject to the Service Contract Act | $2,500 |
+| Construction (Davis-Bacon Act) | $2,000 |
+| Contingency/overseas operations | $25,000 |
+At or below $15,000 (general): no competition required, no synopsis, no formal acquisition plan.
+---
+### Simplified Acquisition Threshold (SAT) — FAR 13.5
+| Category | Threshold |
+|---|---|
+| **Standard SAT** | **$350,000** |
+| Commercial items (test program) | $7.5M |
+| Certain commercial items | $15M |
+Between $15K–$350,000: simplified acquisition procedures apply (FAR Part 13). Above $350,000: full competition and formal acquisition planning requirements kick in.
+---
+**Other thresholds worth knowing in this range:**
+- **$25,000** — SAM.gov synopsis required (FAR 5.101)
+- **$150,000** — VETS 4212 affirmative action plan applies
+- **$750,000** — Small business subcontracting plan required (large business primes)
+</t>
+        </is>
+      </c>
+      <c r="BG2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI2" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK2" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="BL2" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 = RO (comparable)
+RO comparison: Both correctly cite $15K MPT, $350K SAT under FAC 2025-06. V11 used only query_compliance_matrix (no research tool). Response is shorter (1,093 vs V10's 1,854 chars) but accurate — includes MPT exceptions table, SAT tiers, and additional thresholds ($25K synopsis, $150K VETS, $750K subcontracting).
+v10 vs v11: REGRESSION in tool choice -- V10 used research (4 KB docs, 1,854 chars). V11 used only query_compliance_matrix (0 KB docs, 1,093 chars). Shorter but still accurate. Sources score drops 5-&gt;4 because no KB documents fetched.
+Tools: v10=[research] | v11=[query_compliance_matrix]
+KB docs cited: V10=4 | V11=0 (-4 regression)
+Verdict: Accurate but thinner -- compliance matrix alone is sufficient for thresholds but misses the policy context research provides.</t>
+        </is>
+      </c>
+      <c r="BM2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under **FAC 2025-06** (effective October 1, 2025), the two key thresholds are:
+---
+### Micro-Purchase Threshold (MPT) — FAR 2.101 / FAR 13.2
+| Category | Threshold |
+|---|---|
+| **General (supplies/services)** | **$15,000** |
+| Construction | $2,000 |
+| Services subject to the Service Contract Act | $2,500 |
+| Contingency operations | $25,000 |
+At or below the MPT, competition is **not required** and purchases may be made with minimal documentation (e.g., purchase card).
+---
+### Simplified Acquisition Threshold (SAT) — FAR 2.101 / FAR Part 13
+| Category | Threshold |
+|---|---|
+| **Standard SAT** | **$350,000** |
+| Commercial items (test program) | $7.5M |
+| Certain commercial items | $15M |
+Above the SAT, full and open competition is required and simplified acquisition procedures no longer apply.
+---
+**Key practical implications:**
+- **Under $15K** → FAR 13.2 micro-purchase; no competition required; purchase card eligible
+- **$15K–$350K** → FAR 13.5 simplified acquisition; competition required; streamlined procedures apply
+- **Above $350K** → FAR Part 15 or 8.4 full competition procedures
+Need threshold-specific document requirements or compliance rules for a particular acquisition?
+</t>
+        </is>
+      </c>
+      <c r="BN2" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under **FAC 2025-06** (effective October 1, 2025):
+| Threshold | Amount | FAR Reference |
+|---|---|---|
+| **Micro-Purchase Threshold (MPT)** | **$15,000** | FAR 2.101 / FAR 13.2 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 2.101 / FAR 13.3 |
+**Key notes:**
+- **Micro-Purchase ($0–$15K):** No competition required (FAR 13.202(a)). Purchase card or micro-purchase order. No formal SOW, IGCE, or Acquisition Plan needed.
+- **Simplified Acquisition ($15K–$350K):** FAR Part 13.5 procedures apply. Competition required unless justified. Streamlined AP, market research, and SOW needed.
+- **MPT exceptions:** Lower thresholds apply for construction ($2,000 — Davis-Bacon Act) and services subject to the Service Contract Act ($2,500).
+- **Commercial item simplified test:** Extends SAP procedures up to $7.5M for commercial items (FAR 13.500).
+</t>
+        </is>
+      </c>
+      <c r="BO2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP2" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ2" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BR2" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS2" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="BT2" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 = RO (comparable)
+RO comparison: Both correctly cite $15K MPT, $350K SAT under FAC 2025-06. V12 uses query_compliance_matrix (correct tool). Response is concise (864 chars) with clean threshold table. Missing construction/SCA sub-thresholds that V11 had.
+v11 vs v12: V12 shorter (864 vs 1,211 chars V11). Drops sub-threshold detail (construction $2K, SCA $2.5K) that V11 included. Comp score 4 vs 5.
+Tools: v11=[query_compliance_matrix] | v12=[query_compliance_matrix]
+KB docs cited: V11=0 | V12=0 (expected for threshold lookup)
+Verdict: Correct but slightly less complete than V11 on sub-thresholds.</t>
         </is>
       </c>
     </row>
@@ -4278,6 +4605,277 @@
 Source gap: CLOSED -- V8 had 0 KB paths vs RO's 2; V9 now matches with 2 KB paths.
 KB docs cited: V8=0 | V9=2 (+2 improvement)
 Verdict: Key improvement -- subagent KB document reads now visible. Sources 4-&gt;5.</t>
+        </is>
+      </c>
+      <c r="AY3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## GAO B-302358: IDIQ Minimum Obligation Requirements
+**Case**: Bureau of Customs and Border Protection - Automated Commercial Environment Contract  
+**Date**: December 27, 2004
+### Core Holdings
+**1. Obligation Timing**
+Agencies **must record an obligation for the guaranteed minimum amount at the time of IDIQ contract award**, not when task orders are issued.
+**2. Legal Basis**
+- The government incurs a **fixed legal liability** for the minimum amount at contract execution
+- FAR Clause 52.216-22 states: "The Government **SHALL ORDER** at least the quantity... designated as the 'minimum'"
+- "Shall order" = mandatory commitment = legal liability = obligation
+**3. Recording Statute Violation**
+Customs violated 31 U.S.C. § 1501(a) by:
+- Failing to obligate the $25M minimum at February 11, 2003 contract award
+- Obligating only $45K from FY 2003 funds (5 months after award)
+- Obligating $955K from **FY 2004 funds** instead of FY 2003 funds
+- Should have obligated entire $25M from FY 2003 appropriations on award date
+**4. Risk Created**
+Failure to timely record obligations:
+- Violates the recording statute
+- Creates risk of Antideficiency Act violations
+- Compromises integrity of obligational accounting records
+- May result in using wrong fiscal year appropriations
+### What Agencies Must Do
+**At Contract Award:**
+✓ Record obligation for the **full guaranteed minimum amount**  
+✓ Use appropriations from **fiscal year of contract award**  
+✓ Record obligation **immediately upon contract execution**
+**Task Orders:**
+- Task orders that draw down the minimum: **No new obligation** (already obligated at award)
+- Once minimum exhausted: Obligate additional task orders from fiscal year when order is placed
+### Required Account Adjustments
+GAO directed Customs and DOD to:
+1. **Deobligate** $955K from FY 2004 appropriations
+2. **Obligate** $955K from FY 2003 appropriations
+3. **Determine** if Antideficiency Act violation occurred (insufficient FY 2003 funds available)
+4. **Report** any deficiency per Antideficiency Act
+### IDIQ vs. Multiyear Contracts (Key Distinction)
+GAO held the contract was **IDIQ, NOT multiyear** under 41 U.S.C. § 254c:
+**Multiyear Contracts (§ 254c):**
+- Buy more than one year's **firm requirements**
+- Need is "reasonably firm and continuing"
+- Obligate all years at award
+- Require head of agency determination
+**IDIQ Contracts:**
+- Government **cannot predetermine** precise quantities above minimum
+- Only minimum obligated at award
+- Additional obligations as task orders placed
+- NOT governed by § 254c
+GAO: *"A single contract cannot satisfy these wholly inconsistent sets of statutory and regulatory requirements."*
+### Practical Guidance
+**IDIQ Contract Award Checklist:**
+- [ ] Guaranteed minimum identified in contract
+- [ ] Budget office certified funds available for minimum
+- [ ] Funds are from fiscal year of contract award
+- [ ] Obligation will be recorded at contract execution
+- [ ] FAR Clause 52.216-22 included
+- [ ] For interagency agreements: both agencies will obligate appropriately
+**Customs's Excuse Rejected:**
+Customs argued the minimum had been "fulfilled" through subsequent task orders, so no harm occurred. GAO held this **irrelevant** - the recording statute requires **timely recording** to ensure accounting integrity and prevent Antideficiency Act violations.
+---
+**Sources:**
+- GAO Decision B-302358 (December 27, 2004) - Full text retrieved from eagle-knowledge-base/approved/legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt
+</t>
+        </is>
+      </c>
+      <c r="AZ3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD3" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE3" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: Both correctly cover the two core holdings (IDIQ != multiyear, minimum obligation at award). V10 adds: remedial actions required, IDIQ vs multiyear distinction table, practical guidance checklist.
+v9 vs v10: V10 goes direct (knowledge_search + knowledge_fetch) instead of using legal_counsel subagent. Faster (38s vs 171s) with same quality. Cites GAO_B-302358_IDIQ_Min_Fund.txt directly.
+Tools: v9=[knowledge_search, legal_counsel] | v10=[knowledge_search, knowledge_fetch]
+KB docs cited: V9=2 | V10=1 (direct fetch, no subagent overhead)
+Verdict: Faster path to same quality -- direct fetch vs subagent delegation.</t>
+        </is>
+      </c>
+      <c r="BF3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The legal counsel agent returned the full authentic analysis. Here's the summary:
+---
+## GAO B-302358 — *Bureau of Customs and Border Protection / ACE Contract*
+**December 27, 2004 | 31 U.S.C. § 3529 Legal Decision**
+This was not a bid protest — CBP and DHS OIG jointly requested a legal opinion from GAO's General Counsel on two questions arising from the Automated Commercial Environment (ACE) IDIQ contract awarded to IBM Global Services ($25M minimum / $5B maximum).
+---
+### Two Core Holdings
+**HOLDING 1: An IDIQ Contract Cannot Be a Multiyear Contract**
+GAO held the two contract types are legally incompatible and mutually exclusive:
+| Feature | IDIQ | Multiyear (41 U.S.C. § 254c) |
+|---|---|---|
+| Quantity | Not specified | Reasonably firm and continuing |
+| Government obligation | Only the minimum | Entire multi-year amount |
+| Funding trigger | Each task order | Award year + termination costs |
+Customs had erroneously included FAR **52.217-2** (Cancellation Under Multiyear Contracts) in the IDIQ. GAO held that a mislabeled or mistakenly included clause does **not** transform the contract's legal character — substance controls over label.
+---
+**HOLDING 2: The IDIQ Minimum Must Be Obligated at Contract Award**
+&gt; *"When an agency executes an indefinite-quantity contract such as an IDIQ contract, the agency must record an obligation in the amount of the required minimum purchase."*
+The legal mechanics:
+1. **The minimum quantity clause creates a fixed legal liability at the moment of contract award** — not when task orders are placed.
+2. **31 U.S.C. § 1501(a)(1)** (the recording statute) requires obligation recording upon incurrence of legal liability.
+3. Customs violated this rule by waiting five months to obligate the $25M minimum. GAO did **not** find a formal Antideficiency Act violation only because no-year appropriations were used and adequate funds existed — but issued a strong compliance directive.
+Subsequent task orders create separate, additional obligations charged to the **fiscal year in which the order is placed**, per 60 Comp. Gen. 219 (1981).
+---
+### Practical Compliance Takeaways
+| Issue | Rule |
+|---|---|
+| Minimum obligation timing | Must be obligated **at contract award** |
+| Task order obligations | Charged to **FY of order issuance** |
+| Minimum size | Must be **more than nominal** (FAR 16.504(b)) |
+| Erroneous multiyear clauses | Do not transform IDIQ character |
+| Multiple-award IDIQs | Each awardee gets their own minimum, obligated individually |
+---
+### Why It Still Matters
+B-302358 is foundational fiscal law. It directly governs:
+- **GWAC/IDIQ awards** (NITAAC CIO-SP4, Alliant, etc.) — each awardee's minimum must be obligated at award
+- **Minimum guarantee sole-source exception** (FAR 16.505(b)(2)(i)(D)) — only valid if the minimum was properly stated *and* obligated at award
+- **Antideficiency Act exposure** — agencies using annual appropriations face bona fide needs rule complications if the minimum isn't satisfied within the period of availability
+---
+**Sources:**
+- GAO B-302358 (Dec. 27, 2004) — full analysis via legal counsel KB
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+- FAR 16.504; 31 U.S.C. §§ 1341, 1501(a)(1), 1502(a)
+Need the compliance checklist or application to a specific acquisition?
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_16_Contract_Types_Guidance.txt`
+</t>
+        </is>
+      </c>
+      <c r="BG3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI3" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK3" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="BL3" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 = RO (comparable)
+RO comparison: Both correctly cover two core holdings (IDIQ != multiyear, minimum obligation at award). V11 adds detailed comparison table, quotes statutory text, identifies specific FAR clauses (52.216-22, 52.217-2).
+v10 vs v11: V11 used legal_counsel subagent (173.9s vs V10's 38.3s). Quality comparable but 4.5x slower. Sources score drops because legal_counsel subagent KB reads are less transparent than direct fetch.
+Tools: v10=[knowledge_search, knowledge_fetch] | v11=[knowledge_search, legal_counsel]
+KB docs cited: V10=1 | V11=1 (via subagent, less transparent)
+Verdict: Same quality, much slower -- subagent delegation adds latency without improving depth.</t>
+        </is>
+      </c>
+      <c r="BM3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## GAO B-302358 — Bureau of Customs and Border Protection (ACE Contract)
+**Decided: December 27, 2004**
+---
+### Two Core Holdings
+**1. IDIQ ≠ Multiyear Contract Under 41 U.S.C. § 254c**
+GAO held that the ACE contract (awarded to IBM Global Services, $25M min / $5B max) was an IDIQ contract — **not** a multiyear contract subject to 41 U.S.C. § 254c (now § 3903). The statutory requirements are mutually exclusive:
+- **IDIQ**: Government commits only to a minimum; future orders are discretionary
+- **Multiyear (§ 254c)**: Government binds itself to a known requirement for future years in advance of appropriations
+Critically, GAO held that a contract's **legal character is determined by the rights bargained for — not its label**. CBP had erroneously included FAR 52.217-2 (Cancellation Under Multiyear Contracts) in the IDIQ contract, but GAO refused to let that mislabeling change the contract's nature, citing *Crown Laundry v. United States*, 29 Fed. Cl. 506 (1993).
+---
+**2. The Minimum Guarantee Must Be Obligated at Contract Award**
+This is the decision's most widely cited holding. Under **31 U.S.C. § 1501(a)(1)** (the Recording Statute), GAO held:
+&gt; *"At the time of award, the government has a fixed liability for the minimum amount to which it committed itself."*
+CBP awarded the ACE contract on April 27, 2001 but did not obligate the $25M minimum until **five months later** when task orders were finally issued. GAO found this violated the Recording Statute's requirement to record an obligation when a legal liability is incurred.
+The rule in plain terms:
+| Event | Obligation Required? |
+|---|---|
+| IDIQ contract execution | ✅ YES — minimum guarantee, immediately |
+| Each subsequent task order | ✅ YES — at the time the order is placed |
+| Contract award (amounts above minimum) | ❌ No — only as orders are placed |
+CBP escaped an Anti-Deficiency Act finding solely because it used **no-year appropriations** — funds that don't expire. Agencies using **annual O&amp;M or procurement funds** have no such cushion.
+---
+### Practical Takeaways for NIH Contracting
+1. **Obligate the minimum at award** — not at first order, not when performance begins. Document it in your financial system concurrently with contract execution.
+2. **Nominal minimums are legally defective** — FAR 16.504(b) requires the minimum be "more than a nominal quantity." A $1 minimum lacks consideration and can be challenged.
+3. **Annual fund IDIQ awards near September 30 are high-risk** — if the minimum can't be obligated before funds expire, the contract cannot be legally awarded.
+4. **Don't include FAR 52.217-2 in an IDIQ** — it creates confusion and audit exposure, even if it doesn't change the contract's legal character.
+5. **Task orders are separately obligated** in the fiscal year they are placed — this is a distinct rule from the minimum obligation requirement.
+---
+**Sources:**
+- GAO B-302358, Dec. 27, 2004 (CBP ACE Contract)
+- FAR 16.504 (Indefinite-Quantity Contracts)
+- 31 U.S.C. § 1501(a)(1) (Recording Statute)
+- *GAO Red Book*, Vol. II, Ch. 7 (Variable Quantity Contract Obligations)
+- KB: `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_16_Contract_Types_Guidance.txt`
+</t>
+        </is>
+      </c>
+      <c r="BN3" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## GAO B-302358 — *Bureau of Customs and Border Protection*
+**Decided: December 27, 2004**
+---
+### Two Holdings
+**Holding 1 — Contract Classification**
+The ACE contract was an IDIQ under FAR 16.504, not a multiyear contract under 41 U.S.C. § 254c. GAO held that contract type is determined by **substantive terms and actual administration** — not labels. CBP had mistakenly included FAR 52.217-2 (the multiyear cancellation clause), but GAO refused to let an inadvertently included clause transform an IDIQ into a multiyear contract.
+---
+**Holding 2 — The Core IDIQ Minimum Obligation Rule**
+&gt; *"Upon award of the ACE contract, Customs should have obligated the contract minimum of $25 million in accordance with 31 U.S.C. § 1501(a), the recording statute."*
+At IDIQ execution, the Government incurs a **fixed legal liability** for the minimum guaranteed quantity. That obligation must be recorded **on the day of award** — not when the first task order is issued.
+CBP waited five months before recording the $25M minimum. GAO rejected the "inadvertent delay" defense entirely.
+---
+### Why It Matters
+| Event | Required Action |
+|---|---|
+| **IDIQ contract award** | Obligate full minimum guarantee immediately — charged to appropriation current at award |
+| **Each subsequent task/delivery order** | Obligate order amount — charged to appropriation current **at time of order** |
+The key citations underlying the holding:
+- **31 U.S.C. § 1501(a)(1)** — Recording statute: obligation attaches when a binding written agreement is executed
+- **FAR 16.504(a)(1)** — Government commits to purchase only the stated minimum
+- **65 Comp. Gen. 4, 6 (1985)** — Agencies must record obligations when legal liability is incurred
+---
+### Practical Bottom Line
+1. **Obligate the minimum at award** — no exceptions, no waiting for task orders
+2. **Use the right clauses** — 52.216-22 for IDIQ; 52.217-2 only for true § 254c multiyear contracts
+3. **Subsequent orders use then-current appropriations** — you cannot retroactively charge orders to an expired appropriation used at award
+Failure to record the minimum at award is a near-certain ADA violation exposure and a standard OIG audit finding. B-302358 is settled law on this point.
+---
+*Sources: GAO B-302358 (Dec. 27, 2004); FAR § 16.504; 31 U.S.C. § 1501(a)(1); 65 Comp. Gen. 4 (1985)*
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_16_Contract_Types_Guidance.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR3" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS3" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT3" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: Both correctly cover two core holdings (IDIQ != multiyear, minimum obligation at award). V12 adds Crown Laundry citation, 65 Comp. Gen. 4, practical bottom-line section, and detailed obligation workflow table.
+v11 vs v12: V12 uses legal_counsel (same as V11) but produces cleaner output (2,576 vs 3,341 chars). More concise with same depth. Sources score improves because V12 cites 2 specific KB docs with full S3 paths.
+Tools: v11=[legal_counsel] | v12=[legal_counsel]
+KB docs cited: V11=1 | V12=2 (improved transparency)
+Verdict: Tighter, better-sourced case law analysis.</t>
         </is>
       </c>
     </row>
@@ -4954,6 +5552,377 @@
 Verdict: Strong -- maintains V8 quality, research subagent KB tracking stable.</t>
         </is>
       </c>
+      <c r="AY4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## Answer
+Based on the appropriations law guidance (31 U.S.C. § 1502(a) and GAO Red Book Chapter 5), the **severable vs. non-severable distinction determines which fiscal year's appropriation must fund a contract** under the bona fide needs rule:
+---
+## The Core Rule
+**The bona fide need for services arises in the fiscal year when the services are performed.**
+---
+## Non-Severable Services (Single Undertaking)
+### Funding Rule
+✓ **Entire contract can be funded from the fiscal year appropriation when the contract is entered**  
+✓ Performance can span multiple fiscal years without additional funding  
+✓ No incremental funding required
+### Why
+Non-severable services constitute a single, unified undertaking that cannot be separated into components without losing essential value. The entire effort represents a bona fide need of the fiscal year when the contract is awarded.
+### Examples
+- Feasibility study producing a final report
+- System audit with single audit opinion
+- Architectural design for a specific facility
+- Legal representation in specific litigation
+- Software development for a defined system
+### Funding Example
+**Contract:** October 1, 2025 – March 31, 2026 (spans FY26 and FY27)  
+**Value:** $600,000  
+**Service:** System audit with final report (non-severable)
+**Funding Approach:**  
+✓ Obligate entire $600,000 from **FY 2026** appropriations  
+✓ No incremental funding needed even though performance extends into FY27  
+✓ Rationale: The audit is a single undertaking; entire effort is a bona fide need of FY26 when contract is entered
+---
+## Severable Services (Recurring/Continuing)
+### Funding Rule
+✗ **Cannot fund future fiscal year services with current-year appropriation**  
+✓ **Must fund incrementally:** Each fiscal year's services funded with that fiscal year's appropriation  
+✓ Requires FAR 52.232-22 (Limitation of Funds) or FAR 52.232-19 (Availability of Funds)
+### Why
+Severable services are recurring or continuing services where each unit has independent value. Each fiscal year's portion represents a separate bona fide need of that fiscal year.
+### Examples
+- Help desk support
+- Maintenance and repair services
+- Janitorial services
+- Security guard services
+- Systems administration and monitoring
+- Software-as-a-Service subscriptions
+- Most ongoing IT operations
+### Funding Example
+**Contract:** October 1, 2025 – September 30, 2026 (spans FY26 and FY27)  
+**Value:** $1,200,000 ($100,000/month)  
+**Service:** IT help desk support (severable)
+**Funding Approach:**  
+✓ **Increment 1:** $300,000 from **FY 2026** funds for Oct–Dec 2025 services (3 months in FY26)  
+✓ **Increment 2:** $900,000 from **FY 2027** funds for Jan–Sep 2026 services (9 months in FY27)  
+✗ **Cannot** obligate entire $1,200,000 from FY26 funds  
+✓ Rationale: Each month's services are independent bona fide need of that fiscal year
+---
+## Key Decision Factors
+### Non-Severable Indicators
+- Single final deliverable or unified outcome
+- Interdependent tasks building toward one goal
+- Cannot divide by time periods without losing value
+- Value derives from complete performance
+### Severable Indicators
+- Recurring outputs with independent value each period
+- Discrete, identifiable units of service
+- Each time period's services stand alone
+- Services can be logically divided by time
+---
+## Common Errors
+**Error #1:** "All service contracts are severable"  
+**Truth:** Studies, audits, and specific projects are non-severable
+**Error #2:** "If performance crosses fiscal years, it must be severable"  
+**Truth:** Non-severable services can cross fiscal years; severability depends on the nature of services, not duration
+**Error #3:** "We can make any contract non-severable by writing it that way"  
+**Truth:** Severability is determined by the actual nature of services, not contract language. Cannot manipulate structure to circumvent bona fide needs rule.
+---
+## Short Bridge Exception
+For severable services, a **short bridge across the fiscal year boundary** (typically 1–3 months) may be funded entirely with the prior fiscal year's appropriation when:
+- Necessary to avoid gap in services
+- Bridge period is minimal
+- Agency documents operational necessity
+**Example:** 3-month contract August 1, 2025 – October 31, 2025. Even though October is in FY26, entire contract may be funded with FY25 appropriations as a short bridge.
+---
+## Bottom Line
+The severability determination **directly controls which fiscal year's funds you use**:
+- **Non-severable:** One fiscal year's appropriation funds the entire effort (year of contract award)
+- **Severable:** Must match each fiscal year's services to that fiscal year's appropriation (incremental funding required)
+This isn't just a FAR contracting issue—it's an **appropriations law requirement** under 31 U.S.C. § 1502(a).
+---
+### Sources
+- **Appropriations Law: Severable vs Non-Severable Services** (eagle-knowledge-base/approved/compliance-strategist/regulatory-policies/appropriations_law_severable_services.txt)
+- **Appropriations Law: Time - Bona Fide Needs Rule** (eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt)
+- **Appropriations Law: Incremental Funding** (eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_incremental_funding.txt)
+</t>
+        </is>
+      </c>
+      <c r="AZ4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE4" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: V10 covers all RO content (severable/non-severable rules, bona fide needs, short bridge exception). Adds multi-year/no-year appropriations, concrete examples, and 3 KB document paths.
+v9 vs v10: Comparable quality. V10 cites 3 KB docs via research tool.
+Tools: v9=[research] | v10=[research]
+KB docs cited: V9=4 | V10=3 (slight reduction, different ranking)
+Verdict: Stable -- research tool delivers consistent appropriations analysis.</t>
+        </is>
+      </c>
+      <c r="BF4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete picture on severable vs. non-severable and fiscal year funding:
+---
+## Severable vs. Non-Severable Services: Fiscal Year Funding Rules
+### The Governing Statute
+**31 U.S.C. § 1502(a)** — the Bona Fide Needs Rule: An appropriation is available only for needs that arise during its period of availability. FY 2025 funds pay for FY 2025 needs; you cannot use them for FY 2026 needs.
+The severable/non-severable distinction is how this rule plays out for service contracts that cross fiscal year boundaries.
+---
+### Non-Severable Services — Full Funding at Award
+A contract is **non-severable** when it constitutes a **single undertaking** — one that cannot be divided into components without losing its essential character or value. The deliverable is a unified end product.
+**Fiscal year rule:** The *entire contract* is a bona fide need of the fiscal year in which the contract is entered. You obligate the **full amount from the appropriation current at award**, even if performance runs into the next fiscal year.
+**Examples:** Program evaluations/studies with a final report, financial audits, custom software development, architectural/engineering design for a specific facility, litigation support for a specific case, a defined training course.
+**Funding example:**
+&gt; Contract awarded Sept. 15, 2025 for a $600K system audit. Work runs Oct. 2025–Mar. 2026.
+&gt; → Obligate **$600K from FY 2025 funds**. No incremental funding required.
+&gt; **Key point:** Cannot incrementally fund a non-severable contract. GAO B-317139 (FinCEN/BSA Direct): An agency that obligated only $2M of an $8.9M non-severable cost-reimbursement contract at award, intending to fund the rest in future fiscal years, violated the bona fide needs rule and faced a potential Antideficiency Act violation.
+---
+### Severable Services — Incremental Funding Required
+A contract is **severable** when it consists of **recurring or continuing services** where each time period's performance has independent value — you could stop after any period and still have gotten something useful.
+**Fiscal year rule:** Each fiscal year's portion is a **separate bona fide need** of that fiscal year. You must fund each year's services with **that year's appropriation**. Cannot use FY 2025 funds to pay for FY 2026 services.
+**Examples:** Help desk support, maintenance and repair, janitorial/guard services, systems administration and monitoring, SaaS/database subscriptions, ongoing IT O&amp;M.
+**Funding example:**
+&gt; Help desk contract, Oct. 1, 2025–Sept. 30, 2026, $1.2M ($100K/month)
+&gt; → **FY 2025 funds:** $300K (Oct.–Dec. 2025)
+&gt; → **FY 2026 funds:** $900K (Jan.–Sept. 2026)
+&gt; → Cannot obligate the full $1.2M from FY 2025.
+**Relevant FAR clauses for incrementally funded contracts:**
+- FAR 52.232-22 — Limitation of Funds (cost-reimbursement)
+- FAR 52.232-19 — Availability of Funds for the Next Fiscal Year
+- FAR 37.106(a) — Contracts for services funded by annual appropriations
+---
+### The Short Bridge Exception
+For severable services, agencies may obligate current-year funds for a contract that crosses briefly into the next fiscal year, when:
+- Necessary to avoid a gap in services
+- The bridge period is minimal (typically 1–3 months)
+- Operational necessity is documented
+**Example:** 3-month bridge contract Aug. 1–Oct. 31, 2025 for systems administration. The single month of FY 2026 performance (October) can be funded entirely from FY 2025 funds.
+---
+### Statutory Exception for Annual Appropriations (41 U.S.C. § 253l)
+GAO B-317636 confirmed this exception applies **only to annual (1-year) appropriations.** If a contract is funded by **multi-year or no-year appropriations**, the fiscal-year crossing restriction does not apply — the agency can contract for severable services for the full period of availability of those funds without incremental funding.
+---
+### The GAO Legal Standard
+&gt; *"The question is whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."*
+&gt; — GAO Red Book, Chapter 5
+**Severability is determined by the nature of the services — not by how the contract is written.** You cannot draft your way around this rule.
+---
+### Gray Areas Worth Noting
+| Scenario | Analysis Required |
+|---|---|
+| Agile software development | Non-severable if sprints build toward a defined system; may be severable if open-ended ongoing enhancement |
+| Project management | Non-severable if tied to a specific deliverable; severable if ongoing program management |
+| Penetration test | Non-severable (single report) |
+| SOC monitoring | Severable (recurring daily operations) |
+| Cybersecurity incident response | Non-severable for a specific incident |
+---
+### Documentation
+Your acquisition plan must include a written severability determination. The language needs to either justify full funding at award (non-severable) or show the incremental funding plan by fiscal year (severable). This is a contract file requirement — not optional.
+---
+**Sources:**
+- GAO Red Book, Ch. 5 — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- Bona Fide Needs Rule — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- GAO B-317139 (FinCEN), B-317636, B-318046 — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+- 31 U.S.C. § 1502(a); 41 U.S.C. § 253l; FAR 32.703-2, 37.106(a)
+</t>
+        </is>
+      </c>
+      <c r="BG4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL4" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 covers all RO content (severable/non-severable rules, bona fide needs, funding examples). Adds GAO B-317139 FinCEN case citation, explicit funding examples with dollar amounts, and the 12-month severable ceiling.
+v10 vs v11: Comparable quality. Both use research tool, both produce ~5,500 chars.
+Tools: v10=[research] | v11=[research]
+KB docs cited: V10=3 | V11=3+ (research auto-fetches)
+Verdict: Stable -- research tool delivers consistent appropriations analysis.</t>
+        </is>
+      </c>
+      <c r="BM4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a core appropriations law question with clear rules. Here's the full picture:
+---
+## Severable vs. Non-Severable: Fiscal Year Funding Rules
+The distinction controls everything about **which year's appropriation** must fund a contract. The governing statute is **31 U.S.C. § 1502(a)** (the Bona Fide Needs Rule): an appropriation is available only for needs that arise during its period of availability.
+---
+### The Core Rule by Service Type
+| | **Non-Severable** | **Severable** |
+|---|---|---|
+| **What it is** | A single undertaking — tasks are interdependent and produce one unified end product | Recurring/continuing services — each period's performance has independent value |
+| **When the need arises** | When the contract is **entered into** | When the services are **performed** |
+| **Funding rule** | Fund the **entire contract** from the appropriation current **at award**, even if performance crosses into a future FY | Fund **each fiscal year's services** from **that FY's appropriation** — incremental funding required if crossing FY boundary |
+| **Incremental funding** | Not required (optional) | **Required** when crossing fiscal years |
+---
+### Non-Severable: Full Funding at Award
+**Examples:** Studies, audits, program evaluations, architectural design, custom software development, litigation support, training courses with completion certificates.
+**The rule:** Because the entire effort is a single undertaking, it is a bona fide need of the fiscal year the contract is entered into. You **can** obligate the full contract value from FY25 funds even if performance runs through March FY26.
+&gt; *Example: $600K system audit awarded Oct 1, FY25, final report due March FY26 → Entire $600K obligated from FY25 funds. Correct.*
+**Key trap:** You cannot incrementally fund a non-severable contract by choice to avoid the obligation — GAO Decision **B-317139** (*FinCEN BSA Direct*, June 1, 2009) held that a cost-reimbursement contract for a non-severable system (defined end product) must be **fully obligated at award**. FinCEN's attempt to fund only $2M of an $8.98M non-severable contract was a bona fide needs violation.
+---
+### Severable: Match Each FY's Services to That FY's Funds
+**Examples:** Help desk, maintenance, janitorial, guard services, systems administration, SaaS subscriptions, ongoing IT O&amp;M.
+**The rule:** Each month (or period) of recurring service is its own bona fide need. FY25 funds cannot pay for FY26 services.
+&gt; *Example: $1.2M help desk contract, Oct FY25 – Sep FY26:*
+&gt; - *FY25 funds: $300K (Oct–Dec FY25, 3 months)*
+&gt; - *FY26 funds: $900K (Jan–Sep FY26, 9 months)*
+&gt; - *Cannot obligate all $1.2M from FY25 funds.*
+**Required FAR clauses:**
+- **FAR 52.232-22** — Limitation of Funds (cost-reimbursement) — contractor notifies CO at 75% of funded amount
+- **FAR 52.232-19** — Availability of Funds for Next Fiscal Year (fixed-price severable services)
+---
+### The Short Bridge Exception (Severable)
+For severable services, you may fund a short overlap into the next FY from the current FY's appropriation when necessary to avoid a service gap — typically **1–3 months**. *(e.g., a 3-month contract running Aug–Oct can be fully funded from FY25 funds.)*
+---
+### The Statutory Exception for Crossing FY Boundaries (Severable Only)
+**41 U.S.C. § 253l** (civilian agencies) and **10 U.S.C. § 2410a** (DoD) authorize agencies to enter into severable services contracts that begin in one FY and end **no more than 12 months later** in the next FY, charged entirely to the first FY's appropriation. This is an **exception to the bona fide needs rule** for annual appropriations — it does **not** apply to multi-year or no-year appropriations, which carry no 12-month crossing restriction (GAO **B-317636**, Apr. 21, 2009).
+---
+### Special Situations
+**Options:** Each option period is a **separate bona fide need** — must be funded from the FY when that option period is performed. FY25 funds cannot exercise a FY26 option merely to avoid losing end-of-year money, except under the documented advance exercise exception (operational necessity, typically ≤90 days prior to option start). *(FAR 17.207)*
+**IT/Agile contracts:**
+- Sprint-based work toward a defined system → generally **non-severable** (fund fully at award)
+- Ongoing O&amp;M, help desk, monitoring → **severable** (incremental funding required)
+- Penetration test with final report → **non-severable**; ongoing vulnerability management → **severable**
+**The "you can't write your way out" rule:** Severability is determined by the **nature of the services**, not the contract language. You cannot label a recurring service "non-severable" in the SOW to avoid incremental funding. GAO will look at what was actually acquired.
+---
+### Acquisition Plan Documentation
+For the record, your AP should include an explicit severability determination:
+&gt; **Non-severable:** *"The services constitute a non-severable undertaking producing [specific deliverable] through interdependent tasks. Accordingly, the entire $[X] is obligated from FY[XXXX] appropriations, consistent with the bona fide needs rule."*
+&gt; **Severable:** *"Services are severable and recurring. The contract will cross fiscal year boundaries requiring incremental funding: FY[XXXX] appropriations ($[X]) for [dates]; FY[XXXX+1] appropriations ($[X]) for [dates]."*
+---
+**Sources:**
+- *Appropriations Law: Severable vs. Non-Severable Services* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- *Appropriations Law: Time — Bona Fide Needs Rule* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- *Contract Obligation Timing GAO Guidance (B-317139, B-317636, B-318046)* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+- *Appropriations Law: Incremental Funding* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_incremental_funding.txt`
+- Statutory authority: **31 U.S.C. § 1502(a)**; **41 U.S.C. § 253l**; **FAR 32.703-2**, **FAR 32.703-3**, **FAR 37.106**
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_IDIQ_funding.txt`
+- `eagle-knowledge-base/approved/legal-counselor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt`
+</t>
+        </is>
+      </c>
+      <c r="BN4" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the full picture on severable vs. non-severable and fiscal year funding:
+---
+## Severable vs. Non-Severable: The Fiscal Year Funding Rules
+The distinction drives **which appropriation pays** and **whether incremental funding is required**. It is an appropriations law issue (31 U.S.C. § 1502(a)), not a FAR contract structure issue.
+---
+### The Foundational Rule: Bona Fide Needs (31 U.S.C. § 1502(a))
+An appropriation is available only for needs that arise **during its period of availability**. The severable/non-severable determination controls *when* the need arises.
+---
+### Non-Severable Services — Fund from the Year You Award
+**Definition:** A single undertaking — tasks are interdependent, value comes from complete performance, and the contract produces one end product or result.
+**Funding rule:** The entire bona fide need arises when the contract is entered. You obligate the **full amount from the fiscal year of award**, even if performance spans multiple fiscal years.
+&gt; **Example:** $600K system audit awarded Sept 15, FY25 — final report due March FY26.
+&gt; ✅ Obligate full $600K from FY25 funds. No incremental funding needed.
+**Typical examples:** feasibility studies, program evaluations, audits, architectural/engineering design, specific litigation support, custom software development for a defined system, one-time training programs.
+---
+### Severable Services — Fund the Year the Work is Performed
+**Definition:** Recurring or continuing services where each period's performance has independent value — you could stop after any increment and still have received value.
+**Funding rule:** Each fiscal year's services are a **separate bona fide need of that fiscal year**. You must fund incrementally, matching each year's appropriation to that year's services.
+&gt; **Example:** $1.2M help desk contract, Oct FY25 – Sep FY26 ($100K/month).
+&gt; ✅ FY25 funds: $300K (Oct–Dec, 3 months)
+&gt; ✅ FY26 funds: $900K (Jan–Sep, 9 months)
+&gt; ❌ Cannot obligate the full $1.2M from FY25 funds.
+**Typical examples:** maintenance, janitorial, guard services, systems administration, IT help desk, subscriptions/SaaS licenses, ongoing program management.
+---
+### The Short Bridge Exception
+For severable services, if a contract crosses into the *next* fiscal year by a **short period (typically 1–3 months)** to avoid a service gap, the entire amount may be obligated from the current-year appropriation.
+&gt; **Example:** 3-month contract Aug 1 – Oct 31, FY25. One month (October) falls in FY26.
+&gt; ✅ May fund entire amount from FY25 funds — minimal bridge, operational necessity.
+---
+### The Statutory Bridge Exception (41 U.S.C. § 253l / 10 U.S.C. § 2410a)
+For **annual appropriations only**, these statutes authorize agencies to enter severable services contracts that begin in one fiscal year and end **no more than 12 months later**, obligating the full amount to the first year's appropriation. This is a statutory exception to the bona fide needs rule — it does *not* apply to multi-year or no-year appropriations (per GAO B-317636, Apr. 21, 2009).
+---
+### The Critical Error to Avoid
+You **cannot manipulate contract language** to make severable services appear non-severable. Severability is determined by the *nature* of the services, not how the SOW is written. Attempting to circumvent this is a bona fide needs rule violation and potential Antideficiency Act issue.
+---
+### Gray Areas
+| Scenario | Determination |
+|---|---|
+| Project management for a specific deliverable | Non-severable |
+| Project management for ongoing operations | Severable |
+| Agile dev toward a defined system | Generally non-severable |
+| Agile dev — ongoing enhancement without defined end | May be severable |
+| Security O&amp;M (SOC monitoring, patching) | Severable |
+| Penetration test with final report | Non-severable |
+| One-time system migration/integration | Non-severable |
+| Managed services (ongoing) | Severable |
+---
+### Relevant FAR Clauses for Severable/Incrementally Funded Contracts
+- **FAR 52.232-22** — Limitation of Funds (cost-reimbursement, mandatory)
+- **FAR 52.232-19** — Availability of Funds for Next Fiscal Year (fixed-price severable)
+- **FAR 32.703-2** — Contracts crossing fiscal years
+- **FAR 37.106(a)** — Severable services funded by annual appropriations
+---
+### Options Follow the Same Rule
+Each option period is a **separate bona fide need** requiring that future year's appropriation. You cannot use FY25 funds to exercise an FY26 option period — except where advance exercise is operationally necessary (e.g., 60-day notice requirement), in which case the advance period must be minimal and documented.
+---
+**Bottom line:** If your contract crosses a fiscal year boundary, the first question is always: *Is this a single undertaking or recurring services?* That answer determines whether you need one appropriation or two.
+---
+**Sources:**
+- *Appropriations Law: Severable vs. Non-Severable Services* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- *Bona Fide Needs Rule* — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- *Contract Obligation Timing GAO Guidance* (incl. GAO B-317636, B-317139) — `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+- *Army Contract Attorneys Deskbook 2025, Ch. 4* — 31 U.S.C. §§ 1301, 1341, 1502(a)
+- `eagle-knowledge-base/approved/compliance-strategist/regulatory-policies/appropriations_law_incremental_funding.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_IDIQ_funding.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_incremental_funding.txt`
+- `eagle-knowledge-base/approved/legal-counselor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS4" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT4" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 covers all RO content (severable/non-severable rules, bona fide needs, funding examples). Adds gray area table (agile, PM, pen test), short bridge exception, statutory exception (41 USC 253l), options rule, and FAR clause list.
+v11 vs v12: Uses research (same as V11). Comparable depth (5,983 vs 6,451 chars). Both cite 7-8 KB documents with full S3 paths.
+Tools: v11=[research] | v12=[research]
+KB docs cited: V11=3+ | V12=8 (research auto-fetches)
+Verdict: Stable -- research tool delivers consistent appropriations analysis.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="100.75" customHeight="1">
       <c r="A5" s="5">
@@ -5399,6 +6368,207 @@
 Cascade: search_far -&gt; knowledge_fetch working correctly.
 KB docs cited: V8=1 | V9=1 (maintained)
 Verdict: Stable -- FAR search + fetch cascade reliable for regulatory questions.</t>
+        </is>
+      </c>
+      <c r="AY5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **seven exceptions to fair opportunity** under **FAR 16.505(b)(2)(i)** that allow a sole-source task/delivery order under a multiple-award IDIQ:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | Exception | Key Requirement |
+|---|-----------|-----------------|
+| **(A)** | **Urgency** | Agency need is so urgent that providing fair opportunity would result in unacceptable delays |
+| **(B)** | **Unique / Highly Specialized** | Only one awardee is capable of providing the supplies/services at the required level of quality because they are unique or highly specialized |
+| **(C)** | **Logical Follow-On** | Order must be issued to the same contractor in the interest of economy and efficiency because it is a logical follow-on to an order already issued — *provided all awardees had fair opportunity on the original order* |
+| **(D)** | **Minimum Guarantee** | Necessary to satisfy the contract's minimum guarantee |
+| **(E)** | **Statutory Authorization** | A statute expressly authorizes or requires purchase from a specified source *(applies only above the SAT)* |
+| **(F)** | **Small Business Set-Aside** | Order is set aside for small business concerns under FAR Part 19 / 15 U.S.C. 644(r) — *not subject to J&amp;A, approval, or posting requirements* |
+| **(G)** | **DoD/NASA/Coast Guard OTFAOC** | For DoD, NASA, and Coast Guard only — order satisfies one of the FAR Part 6 exceptions to full and open competition (10 U.S.C. 3406(c)(5)) |
+---
+## Documentation &amp; Approval Requirements
+| Order Value | Justification Required | Approval Level |
+|-------------|----------------------|----------------|
+| Above MPT but ≤ SAT ($350K) | Brief written documentation of basis | CO certification |
+| Above SAT but ≤ $900K | Full written J&amp;A with required elements | CO certification |
+| $900K – $20M | Full written J&amp;A | Advocate for Competition (not delegable) |
+| $20M – $90M | Full written J&amp;A | Head of Procuring Activity (or GO/SES designee) |
+| Above $90M | Full written J&amp;A | Senior Procurement Executive (not delegable) |
+*(DoD/NASA/Coast Guard thresholds are $150M for the top tier.)*
+---
+## Posting Requirement
+- Post J&amp;A on SAM.gov **within 14 days** of award for most exceptions.
+- **Urgency exception (A):** post within **30 days** after award.
+- Exception (F) (small business set-asides) is **exempt** from posting.
+---
+## Key Distinctions from FAR Part 6
+Fair opportunity is **not** full and open competition under FAR Part 6. The exceptions here are specific to ordering against existing multiple-award IDIQs — not new contract awards. The J&amp;A format is a "Justification for an Exception to Fair Opportunity," distinct from a JOFOC.
+&gt; **Source:** FAR 16.505(b)(2)(i)(A)–(G) | HHS Class Deviation 2026-01, § 16.507-6 | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="AZ5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD5" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE5" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: V10 correctly answers with all 7 FAR 16.505(b)(2)(i) exceptions, verbatim statutory text, documentation/approval thresholds, posting requirements, and key distinctions from FAR Part 6.
+v9 vs v10: Consistent quality. Both cite FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt.
+Tools: v9=[search_far, knowledge_fetch] | v10=[search_far, knowledge_fetch]
+KB docs cited: V9=1 | V10=1 (maintained)
+Verdict: Stable -- FAR search + fetch cascade reliable.</t>
+        </is>
+      </c>
+      <c r="BF5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **seven exceptions to fair opportunity** under **FAR 16.505(b)(2)(i)** that allow a sole-source task or delivery order under a multiple-award IDIQ contract:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | Exception | Trigger Condition |
+|---|-----------|-------------------|
+| **(A)** | **Urgency** | The agency need is so urgent that providing fair opportunity would result in unacceptable delays. |
+| **(B)** | **Unique / Highly Specialized** | Only one awardee is capable of performing at the required quality level because the supplies or services are unique or highly specialized. |
+| **(C)** | **Logical Follow-On** | Economy and efficiency require award to the same contractor — the order is a logical follow-on to a prior order (all awardees must have had fair opportunity on the original order). |
+| **(D)** | **Minimum Guarantee** | The order is necessary to satisfy the contract's minimum guarantee. |
+| **(E)** | **Statutory Authorization** | A statute expressly authorizes or requires purchase from a specified source *(applies to orders above the SAT)*. |
+| **(F)** | **Small Business Set-Aside** | Per FAR Part 19, the order is set aside for small business concerns — **not subject to** the J&amp;A/approval/posting requirements that apply to (A)–(E). |
+| **(G)** | **DoD/NASA/Coast Guard OTFAOC** | For those agencies only — an order placed on a sole-source basis when it satisfies one of the FAR Part 6.103 exceptions permitting other than full and open competition. |
+---
+## Documentation &amp; Approval Requirements
+| Order Value | Justification Required | Approval Level |
+|-------------|----------------------|----------------|
+| Above MPT ($15K), at or below SAT ($350K) | Brief written basis for exception | CO certification |
+| Above SAT – $900K | Full written J&amp;A | CO certification (unless agency requires higher) |
+| $900K – $20M | Full J&amp;A | Advocate for Competition |
+| $20M – $90M | Full J&amp;A | Head of Procuring Activity (or SES/GO/FO designee) |
+| Above $90M | Full J&amp;A | Senior Procurement Executive |
+&gt; **DoD/NASA/Coast Guard thresholds differ:** $150M replaces $90M; Advocate threshold at $20M–$150M.
+---
+## Posting Requirement
+- J&amp;As for orders **above the SAT** must be posted to SAM.gov **within 14 days** of award (or **30 days** for urgency exception (A)).
+- Exception **(F) small business set-asides** are exempt from J&amp;A, approval, and posting requirements.
+---
+## Key Points for NIH
+- Fair opportunity is **not** full and open competition under FAR Part 6 — Part 6 procedures and J&amp;A requirements **do not apply** to task orders.
+- The logical follow-on exception **(C)** is frequently used but requires documented rationale explaining *why* the follow-on relationship is logical (scope, PoP, or value).
+- Brand-name justifications at the order level follow a parallel process under FAR 16.505(b)(2)(ii) and require posting for orders &gt;$40K.
+**Source:** FAR Part 16, Subpart 16.5 (HHS Class Deviation 2026-01, effective Nov. 21, 2025) — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="BG5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK5" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL5" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 correctly lists all 7 FAR 16.505(b)(2)(i) exceptions with verbatim statutory text, plus documentation/approval thresholds table by dollar value. RO only listed 6 exceptions (missed the RFO update).
+v10 vs v11: Consistent quality. Both cite FAR Part 16.
+Tools: v10=[search_far, knowledge_fetch] | v11=[search_far, knowledge_fetch]
+KB docs cited: V10=1 | V11=1 (maintained)
+Verdict: Stable -- FAR search + fetch cascade reliable.</t>
+        </is>
+      </c>
+      <c r="BM5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **seven exceptions to fair opportunity** under **FAR 16.505(b)(2)(i)(A)–(G)** that permit a sole-source or single-awardee task order under a multiple-award IDIQ:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | Exception | Basis |
+|---|-----------|-------|
+| **(A)** | **Urgency** | The agency need is so urgent that providing fair opportunity would result in unacceptable delays |
+| **(B)** | **Unique / Highly Specialized** | Only one awardee is capable of providing the supplies or services at the required quality level because they are unique or highly specialized |
+| **(C)** | **Logical Follow-On** | The order must be issued on a sole-source basis in the interest of economy and efficiency as a logical follow-on to an order already issued under the contract |
+| **(D)** | **Minimum Guarantee** | It is necessary to place the order with a particular awardee to satisfy a minimum guarantee |
+| **(E)** | **Statutory Authorization** | A statute expressly authorizes or requires the purchase from a specified source |
+| **(F)** | **Small Business Set-Aside** | Per FAR Part 19, the contracting officer sets aside the order for small business concerns under the multiple-award contract |
+| **(G)** | **DoD/NASA/Coast Guard OTFAOC** | *(Agency-specific)* An order placed on a sole-source basis as a follow-on to a prior order, other than full and open competition — limited to DoD, NASA, and Coast Guard |
+---
+## Key Compliance Points
+**Documentation threshold:** For civilian agencies (including NIH/HHS), orders **exceeding $7M** that use an exception require a written justification. For DoD the threshold is $15M.
+**Fair opportunity ≠ Full &amp; Open Competition:** These exceptions are distinct from FAR Part 6 competition requirements. Fair opportunity is an ordering-level procedure, not a contract award procedure — no Justification &amp; Approval (J&amp;A) under FAR 6.303 is required; instead, the CO documents the specific 16.505 exception basis.
+**Most common at NIH:** Exceptions **(B) Unique/Specialized** and **(C) Logical Follow-On** are the most frequently cited for NIH task orders. Exception **(A) Urgency** is available but requires documented mission impact from delay.
+**Exception (F) note:** A small business set-aside under (F) is not a "sole source" — it restricts competition to small business awardees on the contract, not a single firm.
+---
+*Source: FAR 16.505(b)(2)(i)(A)–(G) | HHS Class Deviation 2026-01 (RFO) effective November 21, 2025*
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="BN5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are the **7 exceptions to fair opportunity** under **FAR 16.505(b)(2)(i)** that permit placing a task order on a single-award (sole-source) basis:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | Exception | Basis |
+|---|-----------|-------|
+| **(A)** | **Urgency** | The agency need is so urgent that providing fair opportunity would result in unacceptable delays |
+| **(B)** | **Unique / Highly Specialized** | Only one awardee is capable of providing the supplies or services at the required quality level because they are unique or highly specialized |
+| **(C)** | **Logical Follow-On** | The order must be placed on a sole-source basis in the interest of economy and efficiency because it is a logical follow-on to an order already issued under the contract |
+| **(D)** | **Minimum Guarantee** | Necessary to place the order with a particular awardee to satisfy a minimum quantity guarantee |
+| **(E)** | **Statutory Authorization** | A statute expressly authorizes or requires the purchase to be made from a specified source |
+| **(F)** | **Small Business Set-Aside** | Per FAR Part 19, the contracting officer sets aside the order for small business concerns under a multiple-award contract |
+| **(G)** | **DoD/NASA/Coast Guard OTFOC** | *(DoD, NASA, Coast Guard only)* An order placed on a sole-source basis as a follow-on to an order already placed under the contract (other than full and open competition) |
+---
+## Key Compliance Points
+**J&amp;A Threshold:** Orders exceeding **$7.5M** (civilian) or **$15M** (DoD) require a written Justification &amp; Approval (J&amp;A) documenting the applicable exception. Below those thresholds, the CO must document the rationale in the contract file but a formal J&amp;A is not required.
+**Not the same as FAR Part 6:** Fair opportunity under 16.505 is a *separate* requirement from full and open competition under FAR Part 6. FAR Part 6 J&amp;As are not required for task orders under multiple-award IDIQs — only the 16.505 documentation is needed.
+**Brand-Name:** If the requirement is brand-name only, a separate brand-name justification is required under FAR 16.505(b)(2)(ii) (formerly cited as 16.507-7 under HHS RFO deviation numbering).
+---
+Need help drafting a J&amp;A or sole-source justification using one of these exceptions?
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR5" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS5" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT5" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 lists all 7 FAR 16.505(b)(2)(i) exceptions with full citation format (A-G), J&amp;A threshold ($7.5M civilian / $15M DoD), brand-name justification note, and NIH-specific common exceptions. Matches RO on all substantive points.
+v11 vs v12: Uses search_far (same as V11). Slightly shorter (2,423 vs 2,629 chars) but equally complete. search_far auto-fetch working -- fetched FAR Part 16 doc.
+Tools: v11=[search_far] | v12=[search_far]
+KB docs cited: V11=1 | V12=1 (maintained)
+Verdict: Stable -- auto-fetch eliminates cascade violation risk.</t>
         </is>
       </c>
     </row>
@@ -6793,6 +7963,538 @@
 Verdict: Strongest response in suite -- maintains V8 20/20 with additional web sourcing.</t>
         </is>
       </c>
+      <c r="AY6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a rich, multi-layered procedural question. Here is a comprehensive breakdown — all rules cited are from verified primary sources.
+---
+# SBIR Elimination + Simultaneous Debriefing Request + Day-8 GAO Protest: Procedural Analysis
+---
+## I. Threshold Classification: Pre-Award or Post-Award Debriefing?
+This is the dispositive question — everything else flows from it.
+**An SBIR "elimination" can occur at two procedurally distinct moments:**
+| Event | FAR Provision | Debriefing Type |
+|---|---|---|
+| Excluded from competitive range (pre-award) | FAR 15.206-2 | **Pre-award debriefing** |
+| Not selected for award (post-award) | FAR 15.301-1 | **Post-award debriefing** |
+The term "elimination notice" in your scenario is ambiguous. A competitive range cut letter triggers pre-award debriefing rights. An unsuccessful offeror notice after award triggers post-award debriefing rights. The procedural rules below address **both tracks**, because the choice between them — which the offeror can influence by how it frames its request — dramatically changes the protest timeline and automatic stay.
+---
+## II. Debriefing Request Timeliness (Day 8)
+### Pre-Award Track (FAR 15.206-2)
+- Request must be made **within 3 days** after receipt of the exclusion notice.
+- **Day 8 is untimely.** The agency is under no obligation to provide the debriefing.
+- However, the agency *may* accommodate an untimely request at CO discretion.
+- **Critical rule:** If the CO accommodates an untimely preaward debriefing request, it does **not** extend the protest clock. FAR 15.301-1 makes this explicit: "Protest deadlines are NOT extended when the Government accommodates an untimely request."
+### Post-Award Track (FAR 15.301-1)
+- Request must be made **within 3 days** after receipt of the award notice.
+- Same outcome: Day 8 is untimely. Agency may accommodate but is not required to.
+- Same rule: accommodating an untimely request does not extend the protest deadline.
+**Bottom line:** The debriefing request on Day 8 is untimely under either track. The CO has discretion to honor it, but must understand that doing so creates no additional protest rights or timeline extensions.
+---
+## III. Protest Timeliness Analysis (the Day-8 Filing)
+### Baseline Rule — 4 C.F.R. § 21.2(a)(2)
+All protests based on grounds "known or should have been known" must be filed **within 10 calendar days** of that knowledge. GAO strictly enforces this — it is the most common grounds for dismissal.
+### The Debriefing Exception — 4 C.F.R. § 21.2(a)(2)
+There is a specific exception for competitive proposals where a debriefing was **requested and is required**:
+&gt; "An initial protest shall **not** be filed before the debriefing date offered to the protester, and shall be filed **not later than 10 days** after the date on which the debriefing is held."
+This exception **tolls** the 10-day clock until after the debriefing — but **only when the debriefing was timely requested and is required by regulation**.
+### How the Day-8 Protest Interacts with the Exception
+| Scenario | Debriefing Status | Protest Timeliness Result |
+|---|---|---|
+| Timely request (≤3 days), pre-award | Required — clock tolled | Protest not premature if filed within 10 days of debriefing date *offered* |
+| Timely request (≤3 days), post-award | Required — clock tolled | Same — 10 days from debriefing date offered |
+| **Untimely request (Day 8), pre or post** | **Not required** | **Debriefing exception does NOT apply — base 10-day rule governs from date basis of protest known** |
+**In this scenario:** The debriefing request was made on Day 8. It was untimely. Therefore:
+- The debriefing exception is **unavailable**.
+- The protest must be filed **within 10 calendar days** of when the basis of protest was known — which is the date of the elimination notice (Day 0).
+- Day 8 is still within the 10-day window. **The protest is timely** under the baseline rule.
+- However, the protester cannot hold the protest open waiting for the (untimely-requested) debriefing to occur. The protest clock runs from the elimination notice, not from any future debriefing date.
+&gt; Compare: *SMS Data Products Group, Inc.* (GAO B-423341, May 29, 2025) — where the protester submitted enhanced debriefing questions one day late, GAO held that the debriefing was "concluded" on the delivery date, not when questions were answered, because the untimely questions did not invoke the tolling provision. The protester correctly filed within 10 days of debriefing delivery. Same logic applies here: untimely requests don't trigger the exception.
+---
+## IV. The Automatic Stay — CICA Rules
+This is where the pre-award vs. post-award distinction becomes most consequential.
+### Pre-Award Protest (Competitive Range Cut — No Contract Awarded Yet)
+- CICA **automatically prohibits award** when GAO receives a protest before award.
+- FAR 33.104(b): Agency may not award while protest is pending unless it makes a written D&amp;F of urgent and compelling circumstances.
+- **Stay trigger:** Automatic upon filing. No time window conditions apply — the agency simply cannot award.
+- To override: Requires HCA D&amp;F + DASAMP (OS/DHHS) approval per HHSAR 333.104(b)(1) and NIH Manual 6033-2.
+### Post-Award Protest (Contract Already Awarded)
+- CICA's automatic **suspension of performance** applies **only if** GAO receives the protest within:
+  - **10 calendar days** after contract award, **OR**
+  - **5 calendar days** after the debriefing date *offered* to the protester (for any debriefing required under FAR 15.505 or 15.506) — **whichever is later**
+- FAR 33.104(c); NIH Manual 6033-2.
+**The 5-calendar-day window off the debriefing date offered is the critical lever:**
+| Debriefing Request | Stay Analysis |
+|---|---|
+| Timely request made → agency offers debriefing date | **5-day window opens from the date offered.** If protest filed within 5 days of that date (and within 10 days of award), automatic stay applies. |
+| Untimely request (Day 8) → agency *may* accommodate | Accommodation of an untimely request **does not create a required debriefing** — so the 5-day window off debriefing does **not** apply. Only the 10-day post-award window applies. |
+| No debriefing requested | Only 10-day post-award window. |
+**In this scenario:** If this is a post-award context, the Day-8 protest must still be evaluated against the 10-day post-award award date. If the contract was awarded and the protest was filed within 10 days of award — the stay is automatic. If the award was more than 10 days ago, no automatic stay attaches, and the agency may continue performance unless the CO voluntarily suspends.
+---
+## V. The Correct Procedural Sequence
+```
+DAY 0:    Offeror receives elimination notice.
+           |
+           ├─ PRE-AWARD TRACK (competitive range cut):
+           |   • Debriefing request deadline: Day 3
+           |   • Automatic stay: In effect the moment GAO protest filed
+           |     (no award may be made while protest pending at GAO)
+           |
+           └─ POST-AWARD TRACK (unsuccessful after award):
+               • Debriefing request deadline: Day 3
+               • Award notice triggers post-award stay window:
+                 10 days from award OR 5 days from debriefing date offered,
+                 whichever is later
+DAY 3:    Debriefing request deadline. Offeror misses it.
+DAY 8:    Offeror simultaneously files:
+           (a) Debriefing request — untimely; CO has discretion to accommodate
+           (b) GAO protest via EPDS by 5:30 PM Eastern — timely under base rule
+               (Day 8 &lt; Day 10 from notice)
+           CO Action upon receiving GAO notice:
+           └─ PRE-AWARD: Stop all award activity. Notify OGC.
+              Prepare litigation hold. Contact NIH PCO.
+              If urgent and compelling reasons exist to proceed with award:
+                → Prepare D&amp;F (FAR 33.104(b)(1))
+                → Route: CO → IC Acquisitions Director → NIH PCO → HCA
+                → HCA executes (not delegable) → DASAMP approval required
+              Agency report due to GAO: 30 days from GAO notice
+              Comments due from protester: 10 days after agency report
+              GAO decision: 100 days standard / 65 days express option
+           └─ POST-AWARD: Automatic stay of performance attaches
+              IF protest filed within 10 days of award (or 5 days of
+              debriefing date offered, whichever is later).
+              If stay attaches — CO cannot direct continued performance unless:
+                → D&amp;F prepared (FAR 33.104(c)(1)/(2))
+                → "Best interests of U.S." or "urgent and compelling" finding
+                → Same routing/approval chain as pre-award
+DAY 8+:   CO decides whether to accommodate untimely debriefing request.
+           If accommodated:
+           • Protest timeline is NOT extended — protest already filed
+           • Debriefing content may give protester basis to supplement protest
+             (supplemental grounds must be filed within 10 days of debriefing)
+           • CO should coordinate with OGC before debriefing given active protest
+DAY 30+:  Agency report due (or Day 20 under express option).
+           5 days before report: File document production list with GAO.
+           2 days after list: Parties may object to scope of disclosure.
+DAY 40+:  Protester comments due (10 days after agency report).
+           CRITICAL: Must be filed in EPDS by 5:30 PM Eastern.
+           Failure to file = mandatory dismissal. No exceptions.
+           (See B-419956.258, Optimo IT LLC — 10-minute late filing dismissed.)
+DAY 65:   GAO decision (express option, if elected within 5 days of filing)
+DAY 100:  GAO decision (standard track)
+```
+---
+## VI. SBIR-Specific Considerations
+SBIR competitions are governed by the Small Business Innovation Research Program under 15 U.S.C. § 638. Key nuances:
+1. **GAO jurisdiction:** GAO generally has jurisdiction over SBIR protests involving competitive range cuts and evaluation improprieties, as these are competitive negotiated acquisitions under FAR Part 15 procedures.
+2. **SBA jurisdiction carve-outs:** GAO will **not** review size standard challenges or 8(a) eligibility determinations — those go to SBA. But improper evaluation, failure to follow solicitation criteria, and procedural violations are reviewable by GAO.
+3. **"Required" debriefing:** FAR 15.505 (pre-award) and 15.506 (post-award) apply to SBIR competitions conducted as competitive proposals — so the debriefing *is* required when timely requested, and the 5-day stay window applies accordingly. Untimely requests, as analyzed above, do not trigger that protection.
+---
+## VII. Summary: The Three Pivotal Decision Points
+| Decision Point | Rule | Consequence of Getting It Wrong |
+|---|---|---|
+| **Was the debriefing request timely (≤3 days)?** | FAR 15.206-2 / 15.301-1 | Untimely = debriefing exception unavailable; 10-day base rule governs; no stay extension off debriefing date |
+| **Is this pre-award or post-award?** | FAR 33.104(b) vs. (c) | Pre-award = automatic prohibition on award. Post-award = automatic stay only within 10/5-day window. Different D&amp;F standards apply. |
+| **Does the protest arrive at GAO in time to trigger the stay?** | CICA / 31 U.S.C. § 3553 | Outside the window = no automatic stay; agency may proceed; CO's only obligation is to report and respond |
+---
+**Sources:**
+- `GAO_Bid_Protests_Essential_Guide_for_COs.txt` — 4 C.F.R. §§ 21.2, 21.3, 21.9
+- `NIH_6033_2_Stay_Provisions_Protests.txt` — FAR 33.104(b)/(c), HHSAR 333.104, NIH stay D&amp;F procedures
+- `FAR_Part_15_Source_Selection_RFO_2025.txt` — FAR 15.206-2, 15.301-1 debriefing rules
+- `FC_33_Protests_Disputes_Appeals.txt` — Debriefing timing and stay window strategy
+- *SMS Data Products Group, Inc.*, GAO B-423341 (May 29, 2025) — untimely enhanced debriefing questions; debriefing concluded on delivery date
+- *Optimo Information Technology, LLC*, GAO B-419956.258 (June 21, 2023) — strict EPDS comment filing deadline enforcement
+**Sources:**
+- `eagle-knowledge-base/approved/legal-counselor/case-law/evaluation/GAO_B-423341_ECP_Misleading_Discussions_Best_Value.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt`
+</t>
+        </is>
+      </c>
+      <c r="AZ6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD6" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE6" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: Both produce comprehensive SBIR protest analysis. V10 uses search_far + research + knowledge_fetch. Covers threshold classification, debriefing timeliness, protest timeline, automatic stay, SBIR-specific considerations. Cites 8 document references including GAO Guide, NIH 6033-2, FAR Part 15, FC 33, and 2 GAO case citations.
+v9 vs v10: V10 drops web_search/web_fetch but maintains quality. Faster (91s vs 134s).
+Tools: v9=[search_far, research, knowledge_fetch, web_search, web_fetch] | v10=[search_far, research, knowledge_fetch]
+KB docs cited: V9=6 | V10=8 (includes case law citations)
+Verdict: Strong -- maintains depth without web dependency.</t>
+        </is>
+      </c>
+      <c r="BF6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a rich body of primary source material. Here's the full legal analysis:
+---
+# SBIR Elimination: Concurrent Debriefing Request + Protest on Day 8 — Procedural &amp; Legal Analysis
+---
+## I. The Situation, Mapped to Governing Law
+The fact pattern involves three intersecting legal regimes:
+| Issue | Governing Authority |
+|---|---|
+| Pre-award debriefing entitlement | FAR 15.505 (10 U.S.C. 3305; 41 U.S.C. 3705) |
+| Post-award debriefing entitlement | FAR 15.506 |
+| Protest timeliness | 4 CFR § 21.2 (GAO Bid Protest Regulations) |
+| CICA automatic stay (pre-award) | FAR 33.104(b); 31 U.S.C. § 3553 |
+| CICA automatic stay (post-award) | FAR 33.104(c) |
+| Stay override | FAR 33.104(b)/(c); HHSAR 333.104; NIH Manual 6033-2 |
+**Important SBIR threshold note:** SBIR competitions are conducted as competitive proposal acquisitions under FAR Part 15 procedures. Debriefing rights under FAR 15.505/15.506 apply fully. The competition's SBIR designation does not create a special debriefing exemption.
+---
+## II. The Debriefing Request — What the Regulations Require
+### A. Pre-Award Debriefing (FAR 15.505)
+The elimination notice triggers the debriefing clock immediately:
+&gt; *"The offeror may request a preaward debriefing by submitting a written request for debriefing to the contracting officer **within 3 days** after receipt of the notice of exclusion from the competition."* — FAR 15.505(a)(1)
+**The offeror here submitted the request on Day 8 — 5 days late.**
+This has two serious consequences:
+1. **The offeror has forfeited the right to a debriefing** under FAR 15.505(a)(3): *"If the offeror does not submit a timely request, the offeror need not be given either a preaward or a postaward debriefing. Offerors are entitled to no more than one debriefing for each proposal."*
+2. **The CO may accommodate the untimely request** — FAR 15.506(a)(4)(i) permits accommodation of untimely debriefing requests, but critically: *"Government accommodation of a request for delayed debriefing… does not automatically extend the deadlines for filing protests."* — FAR 15.506(a)(4)(ii)
+### B. Offeror's Option to Delay Until After Award (FAR 15.505(a)(2))
+Separately, even if a timely request had been made, the offeror could have elected to delay the debriefing until after award. In that case:
+- The debriefing becomes a **post-award debriefing** and must include all post-award information under FAR 15.506(d)
+- Per FAR 15.505(a)(2): *"Debriefings delayed pursuant to this paragraph could affect the timeliness of any protest filed subsequent to the debriefing"* — a direct regulatory warning that this strategy carries protest risk
+---
+## III. The Protest Filed on Day 8 — Timeliness Analysis
+### The General Rule: 4 CFR § 21.2(a)(2)
+&gt; *"Protests other than those covered by paragraph (a)(1) shall be filed not later than **10 days after the basis of protest is known or should have been known**."*
+The basis of protest here is the elimination itself, which the offeror knew on **Day 0** (receipt of notice). The 10-day window runs from Day 0. A Day 8 protest is therefore **facially timely** under the standard rule — 8 days &lt; 10 days.
+### The Debriefing Exception: 4 CFR § 21.2(a)(2), Second Sentence
+The debriefing exception modifies the standard rule for competitive proposals:
+&gt; *"…with the exception of protests challenging a procurement conducted on the basis of competitive proposals under which a debriefing is requested and, when requested, is required. In such cases… the initial protest shall **not be filed before** the debriefing date offered to the protester, but shall be filed **not later than 10 days after the date on which the debriefing is held**."*
+**This exception does two things:**
+1. **Extends** the deadline — the 10-day window runs from the debriefing date, not the elimination date
+2. **Restricts premature filing** — GAO will dismiss a protest as **premature** if filed before the debriefing in cases where a debriefing was requested and is required
+### Does the Exception Apply Here?
+This is the pivotal question:
+**The exception applies when a debriefing is "requested AND, when requested, is required."** Because the request here was untimely (Day 8 vs. 3-day requirement), the CO is **not required** to provide the debriefing. If the CO declines to provide it, the exception arguably does not apply — there is no "required" debriefing — and the protest falls back under the standard 10-day rule from Day 0.
+**Three scenarios play out:**
+| Scenario | Debriefing Status | Effect on Protest |
+|---|---|---|
+| **A** — CO declines untimely request | No debriefing required | Day 8 protest governed by standard 10-day rule; facially timely (Day 8 &lt; Day 10) |
+| **B** — CO accommodates untimely request, debriefing scheduled pre-award | Debriefing provided (voluntary) | FAR 15.506(a)(4)(ii) expressly says accommodation does not extend protest deadlines; Day 8 protest remains measured from Day 0 |
+| **C** — CO accommodates and debriefing is provided post-award | Post-award debriefing (treated as FAR 15.506) | CICA stay window: protest must have been filed within 10 days of award or 5 days post-debriefing, whichever is **later** |
+**Key risk in Scenario A/B:** GAO has held that protesters must **diligently pursue** information that forms protest grounds, including requesting prompt debriefings. An untimely debriefing request can undercut a protester's argument that the 4 CFR § 21.2(a)(2) extended window applies to them.
+---
+## IV. The Simultaneous Protest — Procedural Complications
+The offeror filed the protest on Day 8 **while the debriefing has not yet been provided**. Under 4 CFR § 21.2(a)(2), if the debriefing exception applies, filing **before** the debriefing is held renders the protest **premature** — a basis for dismissal.
+**However**, because the debriefing request was untimely (no mandatory debriefing), the exception's "not before debriefing" restriction likely does not apply, and the Day 8 filing stands as timely under the standard rule.
+This creates a practical paradox for the offeror:
+- If they argue the debriefing exception applies (to get the extended 10-days-post-debriefing window), they simultaneously render their Day 8 protest premature
+- If they forgo that argument, their Day 8 protest is timely — but they must ensure all protest grounds are grounded in information they already possessed
+**Best practice for the offeror's counsel:** File the protest on Day 8 based on known grounds (information in the elimination notice itself). If the debriefing is subsequently provided and reveals new grounds, file a supplemental/amended protest within 10 days of the debriefing. GAO will endeavor to resolve supplemental protests within the 100-day window of the initial protest (FAR 33.104(f)).
+---
+## V. The CICA Automatic Stay — Pre-Award vs. Post-Award
+### A. Pre-Award Stay (FAR 33.104(b))
+Since **no award has been made yet**, the protest falls under the **pre-award stay** regime:
+&gt; *"When the agency has received notice from the GAO of a protest filed directly with the GAO, a contract **may not be awarded** unless authorized, in accordance with agency procedures, by the head of the contracting activity…"* — FAR 33.104(b)(1)
+**Effect:** Receipt of GAO notice automatically **freezes award**. No D&amp;F or override needed to impose the stay — it is automatic. The CO must:
+1. Immediately halt award proceedings
+2. Notify other offerors with reasonable award prospects
+3. Extend offer acceptance periods if needed (FAR 33.104(b)(3))
+### B. Post-Award Stay (FAR 33.104(c))
+If award occurs before the protest notice reaches the agency, the post-award regime applies:
+&gt; *"When the agency receives notice of a protest from the GAO within **10 days after contract award** or within **5 days after a debriefing date offered** to the protester for any debriefing that is required by 15.505 or 15.506, whichever is later, the contracting officer shall immediately suspend performance or terminate the awarded contract…"* — FAR 33.104(c)(1)
+**The CICA stay window is tied directly to the debriefing:**
+| Trigger Event | Stay Window Deadline |
+|---|---|
+| Contract award | 10 calendar days after award |
+| Debriefing date offered (if required) | 5 calendar days after debriefing |
+| Controlling rule | **Whichever is later** |
+This means: if the CO offers a debriefing on Day 20 post-award, a protest filed on Day 22 (within 5 days of the debriefing) **still triggers the automatic stay** — even though it's outside the 10-day award window. This is the strategic value of securing a timely debriefing request.
+### C. How Debriefing Choice Controls the Stay Timeline
+| Offeror Choice | CICA Stay Window |
+|---|---|
+| No debriefing requested (or untimely request, CO declines) | 10 days from award only |
+| Pre-award debriefing (timely, FAR 15.505) | After award: 5 days from debriefing date offered, if later than day 10 |
+| Post-award debriefing (FAR 15.506 or delayed per 15.505(a)(2)) | 5 days from debriefing date offered, if later than day 10 |
+**Critical strategic point:** An offeror who timely requests a debriefing that is delayed by the agency until after award is not penalized — the stay window extends to 5 days post-debriefing. But an offeror who **failed to make a timely request** cannot claim the debriefing-linked stay extension, because no debriefing is "required" in their case.
+---
+## VI. Stay Override — NIH-Specific Procedures
+If the agency wants to proceed with award (pre-award) or continue performance (post-award) despite the protest, the override path is:
+### For GAO Protests (NIH Manual 6033-2; FAR 33.104(b)/(c)):
+**Pre-Award Override** requires:
+- Written D&amp;F: (1) urgent and compelling circumstances, AND (2) award likely within 30 days — FAR 33.104(b)(1)(i)-(ii)
+- Executed by: **NIH HCA** (not delegable)
+- Approved by: **DASAMP, OS, DHHS**
+- Routing: CO → IC Director, Office of Acquisitions → NIH PCO → HCA → OGC-GLD → DASAMP
+**Post-Award Override** requires:
+- Written D&amp;F: performance in best interests of U.S., OR urgent and compelling circumstances — FAR 33.104(c)(2)(i)-(ii)
+- Same HCA execution + DASAMP approval chain
+---
+## VII. Agency Response Obligations — CO Action Timeline
+Once GAO notifies the agency of the protest (not when filed — when GAO notifies):
+| Deadline | Action Required |
+|---|---|
+| Immediately | Implement pre-award stay; notify prospective awardees; begin compiling report; impose litigation hold on all relevant records |
+| Within 1 day | Confirm complete copy of protest received from protester (FAR 33.104(a)(1)) |
+| Within 5 calendar days | Protest file (all docs except CO Statement) to OGC-GLD (4 copies) and NIH PCO (1 copy) — NIH Manual 6033-1 |
+| Within 14 calendar days | CO's Statement of Facts and Circumstances due — NIH Manual 6033-1 |
+| 5 days before report | File document release/withhold list with GAO and parties — FAR 33.104(a)(3)(iii) |
+| Within 30 calendar days | Complete agency report to GAO — FAR 33.104(a)(3)(i) |
+| Protester comments | Due 10 days after report (5 days under express option) — FAR 33.104(a)(6) |
+| GAO decision | Within 100 days (or 65 days under express option) — FAR 33.104(f) |
+---
+## VIII. Decision Tree Summary
+```
+Day 0: Elimination notice received
+       ↓
+       Was debriefing requested within 3 days? (FAR 15.505(a)(1))
+       │
+       NO (request came Day 8)
+       │
+       ├─► CO may decline debriefing entirely — no entitlement
+       │    └─► No required debriefing → 4 CFR 21.2(a)(2) exception does NOT apply
+       │         Day 8 protest → standard 10-day rule from Day 0 → TIMELY
+       │         CICA stay window: 10 days from award only (no debriefing extension)
+       │
+       └─► CO may accommodate voluntarily (FAR 15.506(a)(4)(i))
+            └─► Accommodation does NOT extend protest deadlines (FAR 15.506(a)(4)(ii))
+                 Day 8 protest → still measured from Day 0 → TIMELY
+                 But: if protest was filed before debriefing AND exception argued → PREMATURE risk
+                 CICA stay: voluntary debriefing is not a "required" debriefing
+                 → Does NOT extend the stay window beyond 10 days from award
+Day 8 Protest filed simultaneously with debriefing request
+       ↓
+       Protest is FACIALLY TIMELY under standard rule (Day 8 &lt; Day 10 from Day 0)
+       ↓
+       CO must NOT award contract upon GAO notification (pre-award stay automatic)
+       ↓
+       If award needed anyway → HCA D&amp;F + DASAMP approval required
+```
+---
+## IX. Bottom Line for the CO
+1. **Day 8 protest is facially timely** under the standard 10-day rule (4 CFR § 21.2(a)(2)) — but GAO will scrutinize whether all grounds were reasonably known, and timeliness must be established in the protest itself.
+2. **The debriefing request is untimely** (FAR 15.505(a)(1) requires 3 days; offeror waited 8). The CO is not required to provide it, but may accommodate. Either way, accommodation does not extend protest deadlines or the CICA stay window.
+3. **If no timely debriefing request was made, the 4 CFR § 21.2(a)(2) debriefing exception likely does not apply** — the protest should not be dismissed as premature, and the stay runs from award date only (not debriefing date).
+4. **The pre-award stay is automatic** upon GAO notification. The CO must halt award immediately. No D&amp;F needed to impose it; a D&amp;F is only needed to override it.
+5. **Override requires HCA execution and DASAMP approval at HHS level** — this path is not delegable and requires several days of routing. Mission criticality for SBIR research should be documented in the acquisition plan prospectively.
+6. **Litigation hold attaches immediately** to all records related to the protest, overriding normal disposition schedules (NIH Manual 6033-2).
+---
+**Sources:**
+- FAR 15.505 (Preaward Debriefings), FAR 15.506 (Postaward Debriefings), acquisition.gov (FAC 2026-01)
+- FAR 33.104 (Protests to GAO), acquisition.gov (FAC 2026-01)
+- 4 CFR § 21.2 (Time for Filing), eCFR as of 4/03/2026
+- GAO Bid Protests Essential Guide for COs (GAO-18-510SP), `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt`
+- NIH Policy Manual 6033-2: Stay Provisions for Protests, `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt`
+- NIH Manual 6033-2 (Legal Counselor Reference), `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt`
+- NIH Manual 6033-1: CO's Statement of Facts and Circumstances, `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt`
+</t>
+        </is>
+      </c>
+      <c r="BG6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK6" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL6" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 produces comprehensive SBIR protest analysis with 3 intersecting legal regimes mapped to specific FAR/CFR provisions. Covers debriefing timeliness, protest timeline, automatic stay, SBIR-specific analysis. Cites FAR 15.505, 15.506, 4 CFR 21.2, FAR 33.104, HHSAR 333.104, NIH 6033-2.
+v10 vs v11: V11 uses 5 tools (search_far, knowledge_search, knowledge_fetch, web_search, web_fetch). Produces 14,708 chars (largest in suite). V10 used 3 tools for 12,309 chars.
+Tools: v10=[search_far, research, knowledge_fetch] | v11=[search_far, knowledge_search, knowledge_fetch, web_search, web_fetch]
+KB docs cited: V10=8 | V11=10+ (includes web sources)
+Verdict: Strong -- deepest protest analysis in suite, thorough multi-source research.</t>
+        </is>
+      </c>
+      <c r="BM6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ERROR: </t>
+        </is>
+      </c>
+      <c r="BN6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is the complete procedural and legal analysis:
+---
+# SBIR Elimination + Simultaneous Debriefing Request + Day-8 Protest: Full Procedural Analysis
+## Threshold Framing: What Kind of Debriefing Applies?
+This is the foundational question that drives everything else. An offeror **eliminated from a SBIR competition** — not from the competitive range — triggers **FAR 15.505 (pre-award debriefing)**, not FAR 15.506 (post-award). Here's why it matters:
+&gt; **SBIR elimination = removal from competitive range or declination to proceed.** No award has been made. The relevant debriefing provision is **FAR 15.505**, governing pre-award debriefings of offerors not in the competitive range (or otherwise excluded before award).
+This single determination reshapes every downstream deadline.
+---
+## Part I: The Two Debriefing Regimes Compared
+| | **FAR 15.505 — Pre-Award** | **FAR 15.506 — Post-Award** |
+|---|---|---|
+| **Trigger** | Offeror excluded before award (e.g., eliminated from SBIR competition) | Unsuccessful offeror after award is made |
+| **Request deadline** | Within 3 days of notice of exclusion | Within 3 days of receiving notice of award |
+| **Agency response deadline** | Before award if practicable; otherwise as soon as practicable | Within 5 days of request |
+| **Minimum content** | Weaknesses or deficiencies in proposal; overall evaluated cost/price; ranking; rationale | Awardee's unit cost/price; past performance rating; strengths/weaknesses of unsuccessful offeror |
+| **CICA stay trigger?** | **Yes** — FAR 15.505 is expressly listed | **Yes** — FAR 15.506 is expressly listed |
+| **Protest timing anchor** | 10 days from date debriefing held | 10 days from date debriefing held |
+Both provisions are called out in the CICA statute and in **NIH Manual 6033-2**, which defines the stay window as: *"ten calendar days after contract award OR within five calendar days after the debriefing date offered to the protester for any debriefing required by FAR 15.505 or 15.506 — whichever is later."*
+---
+## Part II: The Day-by-Day Procedural Sequence
+### Day 0 — Elimination Notice Received
+The offeror receives written notice of elimination from the SBIR competition. The clocks start running simultaneously on two tracks:
+**Track A — Debriefing Request:**
+Offeror has **3 days** to request a debriefing under **FAR 15.505** (if pre-award, i.e., no award yet). A timely request entitles the offeror to a debriefing.
+**Track B — Protest Timeliness:**
+The general GAO rule (4 C.F.R. § 21.2(a)(2)) requires protest within **10 calendar days** of when the basis is known or should have been known — *unless* the debriefing exception applies.
+---
+### Day 3 (or within 3 days) — Simultaneous Debriefing Request
+The offeror requests a debriefing. This is timely and triggers the agency's obligation under FAR 15.505.
+---
+### Day 8 — Protest Filed at GAO
+The offeror files the GAO protest. The debriefing has not yet been provided.
+**Is the Day-8 protest timely?**
+Under the general 10-day rule: **Yes** — Day 8 is within 10 calendar days.
+Under the debriefing exception: **Also yes, and more importantly, not premature.**
+GAO's rules under 4 C.F.R. § 21.2(a)(2) include a specific carve-out for competitive proposals with required debriefings:
+&gt; *"A protest that challenges a procurement conducted on the basis of competitive proposals under which a debriefing is requested and, when requested, is required — the protest shall not be filed before the debriefing date offered, and shall be filed not later than 10 days after the date on which the debriefing is held."*
+**Critical implication:** Filing on Day 8 **before the debriefing** is technically premature under the debriefing exception — GAO's regulations contemplate that the protester should wait until after the debriefing. However, since the debriefing has not been "offered" yet (the agency has not scheduled or provided it), the 10-day clock tied to the debriefing has not begun. The Day-8 filing is therefore:
+- **Timely under the general 10-day rule** (Day 8 &lt; Day 10)
+- **Potentially premature** under the debriefing exception if GAO interprets the "offered debriefing date" as still pending
+- **Not dismissed for untimeliness** — GAO generally considers a protest filed before the debriefing as "early" rather than fatally premature, as confirmed in *SMS Data Products Group, Inc.*, B-423341 (May 29, 2025) and *Anika Systems, Inc.*, B-422681 (April 8, 2025): protests filed within 10 days of debriefing delivery but before receiving enhanced debriefing question responses were found **not premature**
+The protective approach is to file after the debriefing to lock in the full 10 days from that date — but filing before is generally preserved as long as it falls within the outer 10-day general limit.
+---
+### After Day 8 — Agency Must Still Provide the Debriefing
+The protest filing does not extinguish the debriefing obligation. **FAR 15.505 requires the agency to provide the debriefing** because the request was timely. The agency must still conduct it.
+**What happens to the protest timeliness window when the debriefing is eventually provided?**
+If the debriefing reveals new grounds for protest beyond what the offeror already knew, the protester may file a **supplemental protest** within 10 days of the debriefing. The initial Day-8 protest remains on the docket; supplemental grounds must independently satisfy timeliness.
+---
+## Part III: The CICA Automatic Stay — How the Debriefing Choice Changes Everything
+This is where the pre-award/post-award distinction has its sharpest operational consequence for the agency.
+### The CICA Stay Trigger Window (NIH Manual 6033-2 / FAR 33.104)
+CICA's automatic stay provisions apply when GAO receives a protest within the later of:
+1. **10 calendar days after contract award**, OR
+2. **5 calendar days after the debriefing date offered** (for debriefings required under FAR 15.505 or 15.506)
+### Scenario A: Pre-Award Debriefing (FAR 15.505) — No Award Yet
+**The protest is filed on Day 8. No award has been made.**
+- There is **no post-award automatic stay** because there is no contract to stay.
+- The operative stay issue is whether the agency can **proceed to award** notwithstanding the pending GAO protest.
+- Under **FAR 33.104(b)** and **NIH Manual 6033-2**, the agency **may still make award** if the Head of Contracting Activity (HCA) executes a written D&amp;F finding:
+  - **(i)** Urgent and compelling circumstances significantly affecting U.S. interests will not permit awaiting GAO's decision, **AND**
+  - **(ii)** Award is likely within 30 calendar days of the finding
+- At NIH, this D&amp;F requires: HCA execution (non-delegable) + **DASAMP (DHHS) approval**, routed through IC Director → NIH PCO → OGC-GLD → HCA → DASAMP
+- **Without that D&amp;F**: The agency should hold award pending the GAO protest resolution (up to 100 days standard, 65 days express)
+**Timeline impact:** If the agency hasn't awarded yet and doesn't override the stay, the competition is frozen until GAO decides or the protest is withdrawn.
+---
+### Scenario B: If Award Had Already Been Made (Post-Award) — FAR 15.506 Context
+For contrast, if award had already occurred and the debriefing were a **FAR 15.506 post-award debriefing**:
+- CICA's automatic **post-award stay** kicks in when GAO notifies the agency of the protest within **10 days of award** *or* **5 days of the offered debriefing date**, whichever is later
+- **The agency must suspend performance** immediately upon GAO notification (FAR 33.104(c)(1))
+- To **override the stay** and continue performance, the HCA must execute a D&amp;F under FAR 33.104(c)(2) finding either:
+  - Performance is in the **best interests of the United States**, OR
+  - **Urgent and compelling circumstances** won't permit waiting
+- Same NIH routing applies: HCA (non-delegable) + DASAMP approval
+**Key strategic point:** The offered debriefing date — not when it's actually conducted — is what triggers the 5-day CICA window. If the agency delays scheduling the debriefing, it can inadvertently extend the window during which a timely-filed protest carries automatic stay effect.
+---
+## Part IV: The "Offered Date" vs. "Held Date" Distinction
+The CICA/FAR language turns on the **"debriefing date offered"** — not the date the debriefing is held. This is operationally significant:
+- If the agency offers a debriefing date on Day 10 (10 days after notice) → the 5-day CICA clock runs from Day 10, meaning a protest filed through Day 15 triggers the automatic stay
+- If the agency delays offering until Day 20 → any protest filed by Day 25 carries automatic stay force
+**FAR Companion Part 33 guidance** is explicit: *"Avoid unnecessarily extending the protest window. Prepare to quickly provide debriefings when requested after award decisions and notifying unsuccessful offerors."* Delay is not neutral — it extends exposure.
+Conversely, offering a prompt debriefing date (e.g., Day 3 or Day 4) shrinks the stay-trigger window to its minimum, reducing the period during which the agency faces automatic stay risk.
+---
+## Part V: Complete Timeline Summary
+```
+Day 0    — Elimination notice issued; debriefing request + protest clocks begin
+Day 0-3  — Offeror timely requests FAR 15.505 debriefing
+Day 8    — Offeror files GAO protest (timely under general 10-day rule)
+           → No award made: no post-award CICA stay triggered yet
+           → Agency must hold award absent urgent/compelling D&amp;F (FAR 33.104(b))
+           → Agency still obligated to conduct debriefing
+[Agency schedules debriefing — say Day 12]
+Day 12   — Debriefing conducted
+           → New 10-day window opens for supplemental protest grounds
+           → CICA pre-award stay clock: if protest filed within 5 days of Day 12
+             (i.e., through Day 17), automatic stay on award applies
+Day 22   — Outer limit for supplemental grounds from Day 12 debriefing
+Day ~108 — Standard GAO decision deadline (100 days from Day 8 filing)
+Day ~73  — Express option deadline (65 days, if agency or GAO invokes it)
+```
+---
+## Part VI: NIH-Specific Approval Chain for Override
+If NIH decides to proceed with award despite the pending protest (**FAR 33.104(b)** override):
+| Step | Action | Official |
+|---|---|---|
+| 1 | CO prepares D&amp;F with background, protest grounds, urgency justification | Contracting Officer |
+| 2 | Routes through IC Director, Office of Acquisitions | IC Director |
+| 3 | NIH Protest Control Officer (PCO) review | NIH PCO |
+| 4 | D&amp;F executed | HCA / OALM Director *(non-delegable)* |
+| 5 | HCA transmits with approval request to DASAMP via OGC-GLD | OGC-GLD forwards |
+| 6 | DASAMP, OS, DHHS approves | DASAMP |
+| 7 | OGC-GLD notifies GAO; NIH PCO notifies CO | OGC-GLD / NIH PCO |
+*Authority: NIH Manual 6033-2; HHSAR 333.104(b)(1)*
+---
+## Summary of Key Rules
+| Issue | Rule | Authority |
+|---|---|---|
+| Debriefing type for SBIR elimination (pre-award) | FAR 15.505 | FAR 15.505 |
+| Debriefing request window | 3 days from notice | FAR 15.505(a) |
+| Day-8 protest timeliness | Timely under general 10-day rule | 4 C.F.R. § 21.2(a)(2) |
+| Pre-debriefing filing: premature? | Generally no, if within 10-day outer limit | *SMS Data Products*, B-423341 |
+| Supplemental grounds after debriefing | New 10-day window from debriefing date | 4 C.F.R. § 21.2(a)(2) |
+| CICA stay window | 10 days post-award OR 5 days post-offered debriefing, whichever later | FAR 33.104; NIH Manual 6033-2 |
+| Override pre-award stay | D&amp;F: urgent/compelling + award within 30 days | FAR 33.104(b); HHSAR 333.104(b)(1) |
+| Override post-award stay | D&amp;F: best interest OR urgent/compelling | FAR 33.104(c)(2) |
+| NIH approval authority (GAO protest) | HCA (non-delegable) + DASAMP | HHSAR 333.104(b)(1); NIH Manual 6033-2 |
+| GAO decision deadline | 100 days standard / 65 days express | 4 C.F.R. § 21.9 |
+---
+**Bottom line for the CO:** The Day-8 filing is timely. The debriefing obligation survives the protest. NIH cannot proceed to award without an HCA/DASAMP D&amp;F. Schedule the debriefing promptly — delay extends the CICA window, not shortens it. Once the debriefing is held, monitor for supplemental grounds within 10 days.
+---
+*Sources: NIH Manual 6033-2 (Stay Provisions for Protests); NIH Policy Manual 6033-2 (2008); GAO Bid Protests — Essential Guide for COs (GAO-18-510SP); FAR Companion Part 33; GAO B-423341 (SMS Data Products, May 2025); GAO B-422681 (Anika Systems, April 2025); 4 C.F.R. Part 21; FAR 15.505, 15.506, 33.103, 33.104; HHSAR 333.104*
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_19_Small_Business_Programs.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_5_Publicizing_RFO_2025.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_9_Responsibility_OCIs_CTAs.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_6315_1_RD_Contracts_Part1_Presolicitation.txt`
+- `eagle-knowledge-base/approved/legal-counselor/case-law/evaluation/GAO_B-422681_Disparate_Evaluation_Price_Realism_Discretion.txt`
+- `eagle-knowledge-base/approved/legal-counselor/case-law/evaluation/GAO_B-423341_ECP_Misleading_Discussions_Best_Value.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR6" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS6" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT6" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 produces comprehensive SBIR protest analysis (13,935 chars) with 6-part structure: debriefing regime comparison, day-by-day timeline, CICA stay analysis, offered vs held date distinction, NIH approval chain, and procedural summary. Cites FAR 15.505, 15.506, 4 CFR 21.2, FAR 33.104, NIH 6033-2, 2 recent GAO cases.
+v11 vs v12: V12 uses search_far + research (vs V11's search_far + knowledge_search + knowledge_fetch + web_search + web_fetch). Simplified tool surface works -- same depth with fewer tool calls. 13,935 chars (vs V11's 14,708).
+Tools: v11=[search_far, knowledge_search, knowledge_fetch, web_search, web_fetch] | v12=[search_far, research]
+KB docs cited: V11=10+ | V12=12 (includes recent GAO cases B-423341, B-422681)
+Verdict: STRONGEST validation of tool simplification -- same quality, 2 tools vs 5.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="159" customHeight="1">
       <c r="A7" s="5">
@@ -7188,6 +8890,163 @@
 Cascade: N/A -- design discussion, no regulatory content needed.
 KB docs cited: V9=0 (expected for design questions)
 Verdict: Stable -- design reasoning quality consistent.</t>
+        </is>
+      </c>
+      <c r="AY7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a really good design tension you're identifying. Let me make sure I understand the core problem:
+**The failure modes you're seeing:**
+1. **Too fast / too thin** — Eagle jumps straight to SOW generation with minimal questions, produces something that looks complete but falls apart when you try to price it (IGCE reveals the scope was wrong, cost is out of budget, now you're walking back)
+2. **Too slow / too chatty** — The background-and-objectives approach was more thorough but could spiral into theory discussions instead of moving toward a work product
+**The real underlying problem:**
+The document workflow has dependencies that run in both directions. Budget constrains scope. Scope drives cost. Cost validates budget. If you generate the SOW first without anchoring to a realistic cost range, you've built on sand.
+---
+**What are you actually trying to solve?**
+A few different directions this could go:
+**Option A — Intake sequencing:** Force a minimum set of budget/scope anchors *before* SOW generation even starts. Not a lot of questions, but the right blocking questions.
+**Option B — Parallel tracks:** Generate SOW and rough IGCE simultaneously from intake data, so the user sees scope and cost together and can reconcile before committing to either.
+**Option C — Checkpoint gates:** Let Eagle generate quickly, but insert a specific "cost reasonableness check" step before the document is marked complete — so going backwards is a designed step, not a failure.
+**Option D — Scope banding:** During intake, establish a cost band ("under $500K, around $1M, over $5M") that constrains what kind of SOW Eagle will write — simple vs. full, T&amp;M vs. FFP, etc.
+Which of those resonates, or is the actual problem something different than what I'm describing?
+</t>
+        </is>
+      </c>
+      <c r="AZ7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD7" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="BE7" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 = RO (comparable)
+RO comparison: Both correctly identify the design tension between fast/thin and slow/chatty document generation. V10 offers 4 concrete solution options (A-D): intake sequencing, parallel tracks, checkpoint gates, scope banding. RO uses 'three walls of the box' framing.
+v9 vs v10: V10 uses no tools (V9 used load_skill). Both produce good design analysis. V10's 4-option structure is slightly more actionable.
+Tools: v9=[load_skill] | v10=[]
+KB docs cited: V10=0 (expected for design questions)
+Verdict: Stable -- design reasoning quality consistent.</t>
+        </is>
+      </c>
+      <c r="BF7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is the core design tension you're describing — and it's a real one:
+**The problem with "shoot first" (current behavior):**
+- Fast and feels responsive
+- But creates rework loops — generate SOW → price it → too expensive → restructure scope → redo SOW
+- No checkpoint before committing to an approach
+**The problem with "gather everything first" (old behavior):**
+- Thorough background and objectives phase
+- But it would theorize indefinitely — "let me explain acquisition strategy options..." — and never produce anything
+- Users would bail before getting to documents
+What you're really describing is a **balance point** — enough upfront validation to avoid expensive rework, without getting stuck in analysis paralysis.
+A few directions worth talking through:
+---
+**Option 1: Lightweight Feasibility Gate**
+Before generating the first document, Eagle runs a 2-3 question "will this work" check:
+- Estimated budget?
+- Existing vehicle or new?
+- Any known constraints (sole source, incumbent, timeline)?
+If the numbers don't support the scope, say so before drafting.
+---
+**Option 2: Progressive Document Sequence**
+Generate documents in dependency order with explicit checkpoints:
+`IGCE first → "Does this budget work?" → Yes → SOW → AP`
+Forces pricing validation before scope commitment.
+---
+**Option 3: Structured Entry Points by Role**
+Different entry workflows based on who's asking:
+- Requestor → starts with IGCE/budget validation
+- COR → starts with scope/objectives
+- CO → starts with strategy and vehicle
+---
+The question I'd push back to you: **where does the rework actually happen most often in your users' reality?** Is it:
+- Scope too broad for budget?
+- Wrong vehicle chosen?
+- Approval threshold surprises?
+That determines which gate matters most.
+</t>
+        </is>
+      </c>
+      <c r="BG7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK7" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="BL7" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 = RO (comparable)
+RO comparison: Both correctly identify the design tension between fast/thin and slow/chatty document generation. V11 offers 3 concrete solution options with pros/cons. RO uses 'three walls of the box' framing.
+v10 vs v11: Both use no tools (expected for design questions). V11 response slightly shorter (1,786 vs 1,787 chars). Quality equivalent.
+Tools: v10=[] | v11=[]
+KB docs cited: V11=0 (expected for design questions)
+Verdict: Stable -- design reasoning quality consistent.</t>
+        </is>
+      </c>
+      <c r="BM7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ERROR: </t>
+        </is>
+      </c>
+      <c r="BN7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is a real tension in the intake design. Let me make sure I understand the core problem:
+**The failure modes you're seeing:**
+1. **Too fast** — Eagle takes a few inputs and generates a SOW before the acquisition strategy is sound. Then the IGCE comes back too expensive and you're walking backwards through decisions that should have been made first.
+2. **Too slow** — The old background/objectives approach was thorough but could spiral into theory-chatting forever without producing anything.
+**The underlying issue:** Document generation and acquisition strategy are two different phases, but Eagle treats them as one. A SOW is only useful if the strategy behind it is locked — contract type, vehicle, competition approach, rough price range. If any of those are wrong, the SOW is wrong.
+**A few approaches worth discussing:**
+**Option A: Strategy gate before documents**
+Force a lightweight strategy checkpoint before any document generation — not a full intake interview, but 4-5 specific decisions logged and confirmed. SOW only generates after those are green.
+**Option B: IGCE-first sequencing**
+Flip the order. Price the requirement before drafting the SOW. If it's too expensive, you reshape scope before you've written anything.
+**Option C: Progressive commitment**
+Generate a short-form strategy memo first (1 page: what, how, how much, who). User confirms. *Then* full document generation unlocks.
+**What's your instinct?** Is the problem more about sequencing (wrong order), or gating (missing checkpoints), or scope discipline (Eagle agrees with whatever the user says)?
+</t>
+        </is>
+      </c>
+      <c r="BO7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR7" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS7" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="BT7" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 = RO (comparable)
+RO comparison: Both correctly identify the design tension between fast/thin and slow/chatty document generation. V12 offers 3 concrete solution options (strategy gate, IGCE-first, progressive commitment). RO uses 'three walls' framing.
+v11 vs v12: Both use no tools (expected for design questions). V12 slightly shorter (1,599 vs 1,786 chars V11). Quality equivalent.
+Tools: v11=[] | v12=[]
+KB docs cited: V12=0 (expected for design questions)
+Verdict: Stable -- design reasoning quality consistent across versions.</t>
         </is>
       </c>
     </row>
@@ -7437,6 +9296,325 @@
 Cascade: Compliance matrix + research subagent -- full cascade.
 KB docs cited: V9=4 (HHS_PMR_Common_Requirements, File_Reviewers_Checklist_FRC, etc.)
 Verdict: Strong -- comprehensive sole-source guidance with actionable checklist.</t>
+        </is>
+      </c>
+      <c r="AY8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete picture for your $280,000 Illumina BaseSpace Sequence Hub sole-source — and good news: EAGLE already has documents generated for this exact scenario in package **PKG-2026-0001**.
+---
+## Justification Authority
+**FAR 13.106-1(b) — Soliciting from a Single Source (Simplified Acquisition)**
+At $280,000 (below the $350,000 SAT), this is NOT a formal J&amp;A under FAR 6.302 — it's a **Single Source Justification (SSJ)**, a lighter document requiring only CO signature. No Competition Advocate review required.
+The conceptual authority mirrors **FAR 6.302-1(a)(2)** — "Only One Responsible Source" — because Illumina exclusively owns and operates BaseSpace Sequence Hub. No third party has access to the codebase, cloud infrastructure, or legal authority to maintain it.
+---
+## Required Documents — Complete Package
+| # | Document | Status | Notes |
+|---|----------|--------|-------|
+| 1 | **Single Source Justification (SSJ)** | ✅ Generated | FAR 13.106-1(b); CO signature only |
+| 2 | **Market Research Report (MRR)** | ✅ Generated | Confirms no alternative vendors or authorized maintainers exist |
+| 3 | **Purchase Request (PR)** | ✅ Generated | Includes CLIN structure ($280K base + 3 options) |
+| 4 | **IGCE** | ✅ Generated | $280K validated via 18–22% industry benchmark |
+| 5 | **Price Reasonableness Determination** | ✅ Generated | FAR 13.106-3(a); requires Illumina quote comparison |
+| 6 | **SAM.gov Sole-Source Synopsis** | ⬜ Action Required | Required before award — value exceeds $25K threshold (FAR 5.101) |
+| 7 | **HHS-653 Small Business Review** | ⬜ Action Required | CO must complete in SBCX; no SB set-aside feasible |
+| 8 | **IT Security &amp; Privacy Checklist** | ⬜ Action Required | Cloud-hosted platform (HHSAM 339.101) |
+| 9 | **Section 889 Compliance** | ⬜ Action Required | FAR 52.204-25 in contract |
+| 10 | **COR Designation** | ⬜ Action Required | FAC-COR certified COR required before award |
+---
+## Key Facts
+- **Approval level:** CO only — no Competition Advocate, no higher HCA review (acquisition is below SAT per FAR 6.304(a)(1))
+- **Contract type:** Firm-Fixed-Price (FAR 16.202) — appropriate for annual maintenance with known scope
+- **SAM.gov synopsis:** Required before award (15-day response period; no responses expected given proprietary nature)
+- **Small business:** Set-aside not applicable — Illumina is a large business with no authorized third-party maintainers
+- **IT review:** Required — BSH is a cloud-hosted SaaS platform with FedRAMP/FISMA implications
+- **License review:** Required per NIH Policy 6027 before award (check for indemnification/IP/liability provisions)
+---
+## Total Package Value Note
+If you're planning option years (3 × ~4% escalation), total estimated value is **$1,189,010**. That's above the $900,000 CO approval threshold under the updated FAC 2025-06 thresholds — **but each option year is exercised independently with current-year funds (severable services per FAR 32.703-3(b))**, so the base year award at $280K remains within CO authority.
+---
+## Immediate Next Steps
+1. **CO obtains Illumina's formal written quote** — compare to $280K IGCE; if variance &gt;10%, request cost breakdown
+2. **Post SAM.gov sole-source synopsis** — 15-day notice before award
+3. **Complete HHS-653** in SBCX with OSDBU coordination
+4. **Complete IT Security Checklist** (HHSAM 339.101) for cloud platform
+5. **Review Illumina EULA** per NIH Policy 6027 before award
+Want me to generate any of the pending compliance documents, or do you need the existing package documents (SSJ, MRR, PR, IGCE) opened for review?
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/market_research/v1/Market-Research-Report---Illumina-BaseSpace-Sequen.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/purchase_request/v1/Purchase-Request---Illumina-BaseSpace-Sequence-Hub.md`
+</t>
+        </is>
+      </c>
+      <c r="AZ8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD8" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE8" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: Both correctly identify $280K below SAT, requiring SSJ not full JOFOC. V10 adds complete document package with status tracking, references existing PKG-2026-0001 documents, and provides immediate next steps.
+v9 vs v10: V10 references 8 document files including templates and checklists.
+Tools: v9=[query_compliance_matrix, research] | v10=[query_compliance_matrix, research]
+KB docs cited: V9=4 | V10=8 (+4 improvement)
+Verdict: Strong -- comprehensive sole-source guidance with document tracking.</t>
+        </is>
+      </c>
+      <c r="BF8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete picture for your Illumina BaseSpace Sequence Hub sole-source acquisition:
+---
+## Justification Authority
+**FAR 13.106-1(b) — Soliciting from a Single Source**
+At $280,000, this falls **below the Simplified Acquisition Threshold (SAT) of $350,000**. You do **not** need a formal FAR Part 6 J&amp;A. Instead, you use a **Single Source Justification (SSJ)** — a simpler instrument requiring only Contracting Officer (CO) signature. No Competition Advocate review required.
+The conceptual basis mirrors **FAR 6.302-1(a)(2)** — "Only One Responsible Source" — but the procedural requirements at the SAP level are significantly lighter.
+---
+## Document Package Required
+| # | Document | Status | Key Requirement |
+|---|----------|--------|-----------------|
+| 1 | **Single Source Justification (SSJ)** | ✅ Required | FAR 13.106-1(b); CO signature only |
+| 2 | **Purchase Request (PR)** | ✅ Required | Fund certification by Budget Office |
+| 3 | **Market Research Report** | ✅ Required | Confirm no alternative vendors or authorized third-party maintainers |
+| 4 | **IGCE** | ✅ Required | $280K estimate via 18–22% OEM benchmark; HHSAM 307.105-71 |
+| 5 | **Price Reasonableness Determination** | ✅ Required | Compare Illumina quote to IGCE; &gt;10% variance triggers cost breakdown |
+| 6 | **Statement of Work (SOW)** | ✅ Required | SLAs, security patches, iCredits, support tiers |
+| 7 | **SAM.gov Sole-Source Synopsis** | ✅ Required | FAR 5.101(a)(1) — $280K exceeds $25K threshold; 15-day posting |
+| 8 | **HHS-653 Small Business Review Form** | ✅ Required | Document SB set-aside not feasible; OSDBU coordination |
+| 9 | **IT Security &amp; Privacy Checklist** | ✅ Required | Cloud-based platform; HHSAM 339.101 |
+| 10 | **Required Sources Checklist** | ✅ Required | FAR 8.002 — AbilityOne, GSA MAS, SEWP V, NITAAC all checked/inapplicable |
+| 11 | **NIH Policy 6027 License Review** | ✅ Required | Review Illumina EULA for unacceptable provisions before award |
+| 12 | **Section 508 Documentation** | ✅ Required | IT acquisition; FAR 39.203 |
+---
+## Why Your Justification Is Strong
+Illumina is the **exclusive developer and proprietor** of BaseSpace Sequence Hub. Your SSJ rests on four legs:
+1. **Proprietary codebase** — source code, APIs, and cloud infrastructure exclusively Illumina-controlled
+2. **No authorized third-party maintainers** — Illumina grants no maintenance licenses to third parties
+3. **Instrument-native integration** — BSH is the only platform with direct data transfer from NIH's NovaSeq/NextSeq instruments
+4. **No alternatives on required sources** — GSA MAS, SEWP V, AbilityOne, and NITAAC have no coverage for BSH maintenance
+---
+## Approval Level
+**CO only.** No Competition Advocate review, no HCA concurrence. The $280K value is below the $350K SAT, so FAR 6.304(a)(1)'s tiered approval structure does not apply. This is the simplest sole-source pathway available.
+---
+## Contract Structure Recommendation
+- **Type:** Firm-Fixed-Price (FFP) per FAR 16.202 — scope is well-defined, Illumina provides fixed annual pricing
+- **Base year + up to 3 one-year options** (estimate OY1–OY3 at ~4% escalation = $1.19M total if all exercised)
+- **Severable services** — fund each year with current-year appropriations per FAR 32.703-3(b)
+---
+## Key Pre-Award Actions
+1. Post SAM.gov sole-source synopsis (**before award**, 15-day waiting period)
+2. Obtain Illumina's formal written quote; compare to $280K IGCE
+3. Complete HHS-653 in SBCX system (OSDBU coordination)
+4. Complete IT Security &amp; Privacy Checklist (HHSAM 339.101) — cloud genomics platform
+5. Review Illumina EULA per NIH Policy 6027
+---
+I already have all five core documents (SSJ, Market Research, Purchase Request, IGCE, Price Reasonableness) drafted in package **PKG-2026-0001**. Want me to generate the remaining items (SOW, IT Security Checklist, Section 508), or would you like to review/finalize the existing package first?
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/market_research/v1/Market-Research-Report---Illumina-BaseSpace-Sequen.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/purchase_request/v1/Purchase-Request---Illumina-BaseSpace-Sequence-Hub.md`
+</t>
+        </is>
+      </c>
+      <c r="BG8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK8" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL8" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 adds complete document package with 12+ items, each with status and key requirements. Includes SSJ template path, SAM.gov posting requirement, HHS-653 small business review, IT security checklist.
+v10 vs v11: Comparable quality. Both use query_compliance_matrix + research. V11 slightly longer (4,735 vs 4,389 chars) with more detailed document table.
+Tools: v10=[query_compliance_matrix, research] | v11=[query_compliance_matrix, research]
+KB docs cited: V10=8 | V11=8+ (research auto-fetches)
+Verdict: Strong -- comprehensive sole-source guidance maintained.</t>
+        </is>
+      </c>
+      <c r="BM8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's a complete breakdown for your $280,000 sole-source Illumina BaseSpace Sequence Hub maintenance contract:
+---
+## Justification Authority
+**FAR 13.106-1(b) — Soliciting from a Single Source (Simplified Acquisition Procedures)**
+At $280,000, this acquisition is **below the $350,000 SAT**, so you do **not** use the full FAR Part 6 J&amp;A process. Instead, you use the simplified authority — a Single Source Justification (SSJ) — based on the same conceptual rationale as **FAR 6.302-1(a)(2): Only One Responsible Source**.
+Your justification argument is strong and well-supported:
+- Illumina exclusively owns the BSH source code, cloud infrastructure, and API architecture
+- No third-party vendors are authorized or technically capable of maintaining BSH
+- NIH's Illumina sequencing instruments (NovaSeq, NextSeq) are natively integrated — switching platforms would be a separate major acquisition
+- Market research confirms no GSA Schedule, SEWP V, NITAAC, or other vehicle covers BSH maintenance
+---
+## Required Documents
+| # | Document | Status | Notes |
+|---|----------|--------|-------|
+| 1 | **Single Source Justification (SSJ)** | ✅ Required | FAR 13.106-1(b); CO approval only — no Competition Advocate review needed below SAT |
+| 2 | **Statement of Work (SOW)** | ✅ Required | Defines SLAs, security requirements, deliverables |
+| 3 | **IGCE** | ✅ Required | $280,000 validated via 3 methods: industry benchmark (18-22% of platform value), component build-up, market comparables |
+| 4 | **Market Research Report** | ✅ Required | Confirms Illumina-only sourcing; checks GSA, SEWP V, NITAAC — all negative |
+| 5 | **Price Reasonableness Determination** | ✅ Required | FAR 13.106-3(a); obtain Illumina's formal quote, compare to IGCE (10% variance threshold) |
+| 6 | **Purchase Request w/ Funds Certification** | ✅ Required | FAR 4.803(a)(1); Budget Office provides accounting string |
+| 7 | **SAM.gov Sole-Source Synopsis** | ✅ Required | FAR 5.101(a) — $280K exceeds $25K threshold; post prior to award |
+| 8 | **HHS-653 Small Business Review** | ✅ Required | OSDBU coordination; large business sole source — no SB set-aside feasible |
+| 9 | **Required &amp; Priority Sources Checklist** | ✅ Required | FAR 8.002 — AbilityOne, GSA Schedule, BPA, NITAAC all checked and cleared |
+| 10 | **IT Security &amp; Privacy Certification** | ✅ Required | HHSAM 339.101 — cloud-based genomic platform triggers this |
+| 11 | **Section 508 Compliance Documentation** | ✅ Required | FAR 39.203 — IT acquisition |
+| 12 | **Section 889 Compliance** | ✅ Required | FAR 52.204-25 in contract |
+| 13 | **NIH Policy 6027 License Review** | ✅ Required | Review Illumina's EULA for unacceptable provisions (indemnification, unilateral termination, etc.) |
+| 14 | **SAM.gov Registration Verification** | ✅ Required | Verify active + no exclusions at time of award |
+| 15 | **DCIS 6M (Inherently Governmental Cert)** | ✅ Required | Services &gt;$150K |
+| 16 | **COR Designation Letter** | ✅ Required | FAC-COR certified COR required before award |
+**Formal Acquisition Plan:** ❌ Not required — below the $350,000 SAT.
+---
+## Approval Level
+**Contracting Officer only.** Since $280,000 is below the $350,000 SAT, there is no Competition Advocate or HCA approval requirement per FAR 6.304(a)(1). This is a significant advantage of staying under the SAT.
+---
+## Key Compliance Items to Watch
+1. **SAM.gov Synopsis first** — post the sole-source notice before award; the 15-day response window gives you time to confirm no other sources emerge
+2. **Get Illumina's formal written quote** before finalizing the price reasonableness determination — if it exceeds the $280K IGCE by &gt;10%, a cost breakdown from Illumina is required
+3. **Option year pricing** — if you're including 3 option years (est. $1.189M total), document each option exercise separately with updated price reasonableness
+4. **Total estimated value with options = ~$1.189M** — still below the $900K J&amp;A HCA approval threshold *per option period*, but note the cumulative value for file documentation purposes
+5. **NIH Policy 6027** — Illumina's standard EULA often contains indemnification provisions that are unacceptable under federal law; CO must review before award
+---
+## Documents Already in Your Package (PKG-2026-0001)
+Good news — EAGLE found a complete set of pre-drafted documents for exactly this acquisition:
+- ✅ SSJ (FAR 13.106-1(b)) — `PKG-2026-0001/justification/v1/`
+- ✅ Market Research Report — `PKG-2026-0001/market_research/v1/`
+- ✅ Purchase Request — `PKG-2026-0001/purchase_request/v1/`
+- ✅ Price Reasonableness Determination — `PKG-2026-0001/price_reasonableness/v1/`
+- ✅ SOW — `PKG-2026-0001/sow/v1/`
+- ✅ QASP — `PKG-2026-0001/qasp/v1/`
+Want me to generate any missing documents (IT Security Checklist, Section 508, HHS-653 SB Review), or would you like to review and finalize the existing package?
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/JA_Desk_Guide_January_2025_Updated.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/market_research/v1/Market-Research-Report---Illumina-BaseSpace-Sequen.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/price_reasonableness/v1/Price-Reasonableness-Determination-Illumina-BaseSp.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/purchase_request/v1/Purchase-Request---Illumina-BaseSpace-Sequence-Hub.md`
+</t>
+        </is>
+      </c>
+      <c r="BN8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Good — I have everything I need from the research. Here's your complete picture:
+---
+## Illumina BaseSpace Sequence Hub — Sole Source Acquisition
+### Justification Authority
+**FAR 13.106-1(b) — Soliciting from a Single Source (Simplified Acquisition Procedures)**
+At $280,000, this falls *below* the $350,000 SAT, so you use the **simplified** sole-source path — not the full FAR Part 6 J&amp;A. The legal basis mirrors **FAR 6.302-1 / 41 U.S.C. 3304(a)(1)** ("Only One Responsible Source"), but the procedural vehicle is a **Single Source Justification (SSJ)** rather than a formal Justification &amp; Approval (JOFOC).
+**Approval level:** Contracting Officer only — no Competition Advocate or HCA review required below the $350K SAT per FAR 6.304(a)(1).
+---
+### Required Documents
+| # | Document | Status | Authority |
+|---|----------|--------|-----------|
+| 1 | **Single Source Justification (SSJ)** | ✅ Required | FAR 13.106-1(b) |
+| 2 | **Statement of Work (SOW)** | ✅ Required | FAR 37.6 |
+| 3 | **Independent Government Cost Estimate (IGCE)** | ✅ Required | HHSAM 307.105-71 |
+| 4 | **Streamlined Market Research Report** | ✅ Required | HHSAM 310.000 |
+| 5 | **Purchase Request w/ Funds Certification** | ✅ Required | FAR 4.803(a)(1) |
+| 6 | **Price Reasonableness Determination** | ✅ Required | FAR 13.106-3(a) |
+| 7 | **Required &amp; Priority Sources Checklist** | ✅ Required | FAR 8.002 |
+| 8 | **HHS-653 Small Business Review Form** | ✅ Required | AA 2023-02 |
+| 9 | **SAM.gov Sole-Source Synopsis** | ✅ Required | FAR 5.101(a)(1) — exceeds $25K |
+| 10 | **IT Security &amp; Privacy Certification** | ✅ Required | HHSAM 339.101 — cloud-hosted platform |
+| 11 | **NIH Policy 6027 License Review** | ✅ Required | NIH Policy 6027 — proprietary software |
+| 12 | **Section 889 Compliance Documentation** | ✅ Required | FAR 52.204-25 |
+| 13 | **QASP** | ✅ Required | FAR 46 — performance-based services |
+| 14 | **COR Designation Letter** | ✅ Required | FAC-COR certification |
+| 15 | **FPDS-NG Report** | ✅ Required (post-award) | FAR 4.604 — within 3 business days |
+&gt; **No Formal Written Acquisition Plan required** — AP is not mandatory below the $350K SAT.
+---
+### Key SSJ Talking Points (What Makes This Sole-Source)
+Your SSJ must establish these four facts:
+1. **Proprietary ownership** — Illumina exclusively owns the BaseSpace Sequence Hub source code, APIs, cloud infrastructure, and security keys. No third party has access.
+2. **Technical impossibility of third-party maintenance** — Maintenance requires direct access to Illumina's codebase, AWS-hosted infrastructure, and version control systems — inaccessible to any other entity.
+3. **No authorized third-party maintainers** — Illumina does not license, certify, or permit outside vendors to maintain BSH. Confirmed via SAM.gov, GSA eLibrary, SEWP V, and NITAAC review.
+4. **Integration dependency** — BSH is natively integrated with NIH's Illumina NovaSeq/NextSeq sequencing instruments. Platform migration would require a separate major acquisition and would disrupt active research operations.
+---
+### Contract Recommendation
+**Firm-Fixed-Price (FFP)** per FAR 16.202 — annual subscription model with defined service levels. Recommend base year + 3 one-year options with **severable services** structure, funded year-by-year with current-year appropriations per FAR 32.703-3(b).
+---
+### One Critical Compliance Note
+Since your estimated total with options would be ~$1.19M, **file the SSJ for the base year ($280K)**. Each option year requires its own price reasonableness documentation at exercise time — do not roll the full multi-year value into the SSJ justification. The CO approval authority is valid because each individual year is below the $350K SAT.
+---
+### Pre-Award Actions Checklist
+- [ ] Post sole-source synopsis to SAM.gov (15-day response period — watch for any responsive competitors before award)
+- [ ] Obtain Illumina's formal written quote; compare to IGCE (flag if &gt;10% variance)
+- [ ] Complete HHS-653 in SBCX system with OSDBU concurrence
+- [ ] Verify Illumina SAM.gov active registration + exclusions check
+- [ ] Review Illumina EULA for unacceptable provisions per NIH Policy 6027 (flag indemnification, unilateral termination, IP ownership clauses)
+- [ ] Designate COR with valid FAC-COR certification
+---
+Want me to generate any of these documents? I already have a complete SSJ, SOW, IGCE, Market Research Report, Purchase Request, and Price Reasonableness Determination on file for this exact acquisition (PKG-2026-0001). I can open any of them for your review or draft additional documents you need.
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/JA_Desk_Guide_January_2025_Updated.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx`
+- `eagle/dev-tenant/packages/PKG-2026-0001/justification/v1/Single-Source-Justification---Illumina-BaseSpace-S.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/market_research/v1/Market-Research-Report---Illumina-BaseSpace-Sequen.docx.content.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/price_reasonableness/v1/Price-Reasonableness-Determination-Illumina-BaseSp.md`
+- `eagle/dev-tenant/packages/PKG-2026-0001/purchase_request/v1/Purchase-Request---Illumina-BaseSpace-Sequence-Hub.md`
+</t>
+        </is>
+      </c>
+      <c r="BO8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR8" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS8" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT8" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 adds complete document package with 15 items including status, authority, and key requirements. Includes SSJ talking points, contract recommendation (FFP severable), compliance note on option year pricing, and pre-award checklist.
+v11 vs v12: Uses query_compliance_matrix + research (same as V11). V12 slightly shorter (5,751 vs 6,014 chars V11) but includes the same comprehensive package list and references existing PKG-2026-0001 documents.
+Tools: v11=[query_compliance_matrix, research] | v12=[query_compliance_matrix, research]
+KB docs cited: V11=8+ | V12=10 (research auto-fetches)
+Verdict: Strong -- comprehensive sole-source guidance maintained.</t>
         </is>
       </c>
     </row>
@@ -7875,6 +10053,607 @@
 Verdict: Enhanced Q1 answered comprehensively -- NIH layers add value.</t>
         </is>
       </c>
+      <c r="AY9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is the comprehensive reference covering both the current FAR thresholds and all NIH/HHS-specific supplemental policies:
+---
+## FAR Thresholds + NIH/HHS Supplemental Policies
+**Current as of FAC 2025-06 (Effective October 1, 2025)**
+---
+### PART 1: STATUTORY THRESHOLDS (Standard FAR)
+| Threshold | Dollar Value | Authority | Key Trigger |
+|-----------|-------------|-----------|-------------|
+| **Micro-Purchase (MPT)** | **$15,000** | FAR 2.101 / 41 U.S.C. 1902 | No competition required; purchase card or simplified purchase order |
+| MPT – Services Subject to SCA | $2,500 | FAR 22.1003-2 | Service Contract Labor Standards apply above this |
+| MPT – Construction | $2,000 | FAR 22.403-1 | Davis-Bacon Act applies above this |
+| MPT – Contingency Operations | $25,000 | FAR 13.201(g) | Elevated MPT in contingency |
+| **Synopsis Required** | **$25,000** | FAR 5.101 | SAM.gov posting mandatory |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 2.101 / 41 U.S.C. 1908 | Full competition required above; written AP required above |
+| Commercial Simplified (Test Program) | $7.5M / $15M | FAR 13.500 | Simplified procedures permitted for commercial items |
+| Subcontracting Plan | $750,000 ($1.5M construction) | FAR 19.702 | Required for large business primes |
+| VETS 4212 | $150,000 | FAR 22.1302 | Affirmative action plan for veterans |
+| TINA / Certified Cost Data | $2,500,000 | FAR 15.403-4 | Truth in Negotiations Act triggers |
+| 8(a) Sole Source – Services | $4,500,000 | FAR 19.805-1(a) | Competitive 8(a) required above |
+| 8(a) Sole Source – Manufacturing | $7,000,000 | FAR 19.805-1(a) | Competitive 8(a) required above |
+---
+### PART 2: NIH / HHS SUPPLEMENTAL POLICIES
+---
+#### A. HCA (Head of Contracting Activity) at NIH
+**Who is the HCA?** Per NIH Policy Manual 6307-3: the Director, Office of Acquisition and Logistics Management (OALM), OD/OM.
+**HCA approval is required for:**
+- Contracts with current Federal employees (HHSAR 303.602) — coordinate through IC channels
+- Facility Project Approval Agreements (FPAA, HHS Form 300) required before award when:
+  - Facility construction **&gt; $1M**
+  - Equipment/instrument installation with facility modifications **&gt; $2M**
+  - Repair projects **&gt; $5M**
+- Inter-agency funds transfers (approved by cognizant Chief Contracting Officer)
+---
+#### B. SPE (Senior Procurement Executive) — New Requirement
+**HHS Acquisition Alert 2026-01 / Executive Order 14271 (effective October 1, 2025):**
+&gt; **All non-commercial products/services ABOVE SAT ($350,000) require written SPE approval BEFORE solicitation release.**
+- Apply via HHS Acquisition Portal (HHSAP) Document Review page
+- Application must include: (1) description of procurement, (2) specific reasons commercial solution cannot meet needs, (3) complete market research report
+- **SPE review timeline: 30 days** from application receipt
+- **Total acquisition delay: 35–45 days** (prep + adjudication)
+- Class approvals available for recurring same-type requirements
+**Exclusions from SPE approval:**
+- Acquisitions ≤ SAT ($350,000)
+- FSS orders/BPAs (Schedule contracts are commercial by definition)
+- Leases, construction (including A-E under Brooks Act), SBIR
+- Assisted acquisitions where requesting agency already provided EO 14271 approval
+---
+#### C. NIH Special Clearance Procedures — NIH Manual 6307-3
+**Key Rule:** All clearances must be obtained **PRIOR TO award** of any purchase order, delivery order, BPA call, purchase card order, or contract.
+**Three types of requirements:**
+| Type | What It Means |
+|------|--------------|
+| **Clearance** | Formal written approval from clearance office required before ordering. Clearance office has **5 working days** to approve/disapprove. |
+| **Technical Coordination** | Requester must communicate and coordinate with specified office *before* submitting procurement request. Document: office contacted, individual, date, summary. |
+| **Required Source** | Must procure through the designated NIH office (not open market). |
+**Selected commodity clearance requirements (Appendix 1):**
+| Commodity | Clearance | Tech Coord | Required Source | Office |
+|-----------|-----------|-----------|----------------|--------|
+| Animals – non-approved source | ✓ | | | IC Animal Program Director |
+| Animals – live vertebrate procedures | ✓ | | | IC-ACUC |
+| Custom antibodies (animal origin) | ✓ | ✓ | ✓ | IC AO + OACU |
+| Audiovisual production services &gt; $5,000 | ✓ | | | OCPL News Media Branch |
+| Biological Safety Cabinets | ✓ | ✓ | | DOHS |
+| Compressed gases (hazardous) | | ✓ | | DOHS |
+| Contracts with current federal employees | ✓ | | | DAPE/HCA |
+| Major scientific equipment (facility impact) | | ✓ | | ORFDO Facility Manager |
+| Foreign acquisition | ✓ | | | Fogarty International Center |
+| Furniture/systems furniture | | ✓ | | ORFDO |
+| Human subjects | ✓ | | | See NIH Manual 7410 |
+| IT/information security | ✓ | | | IC ISSO; FedRAMP for cloud |
+| Printing (above threshold) | | | ✓ | PSC Printing Office |
+| Public affairs/communications &gt; $5,000 | ✓ | | | OCPL |
+| Radioactive materials | ✓ | | | Division of Radiation Safety (NIH 88-1) |
+| Security devices | ✓ | ✓ | | Office of Security and Emergency Response |
+| Space (leased/renovations) | | | ✓ | ORFDO |
+| Stem cells / fetal specimens | ✓ | | | Per NIH Guidelines |
+| Surveys (≥10 public respondents) | ✓ | | | Project Clearance Officer (PRA) |
+| Telecommunications | | ✓ | | CIT Division of Network Systems |
+| Vertebrate animals – approved source | | | ✓ | DVR/CAPS |
+**Retention:** Clearance documentation retained 3 years (simplified acquisitions) or 6 years 3 months (contracts) after final payment.
+---
+#### D. NIH Purchase Card Policies (Supplemental to FAR 13.2)
+Per NIH Manual 6307-3 roles and responsibilities:
+- **Purchase Cardholder** is responsible for obtaining required clearances and disseminating information copies per Appendix 1 *before* charging the card.
+- **Purchase Card Approving Official** (cardholder's immediate supervisor or AO) is responsible for verifying:
+  - All required clearances/technical coordination obtained
+  - Required sources used where appropriate
+- Applies to all purchase card buys regardless of dollar value
+- Purchase card orders are explicitly listed as NIH acquisition vehicles requiring pre-award clearances
+&gt; **Note:** NIH IC-specific card policies may impose more stringent single-purchase limits or additional approvals. Check your IC's internal policy for local limits below the governmentwide $15,000 MPT.
+---
+#### E. HHS PMR &amp; NIH FRC — Procedural Steps Beyond Standard FAR
+**HHS PMR checklist adds these NIH-specific steps (SAP ≤ $350K):**
+| Step | Requirement | Authority |
+|------|------------|-----------|
+| HHS-653 | Small Business Review Form required for all purchases **&gt; MPT ($15K)** | HHS AA 2023-02 Amendment 3 |
+| Mandatory Sources Check | IT, Professional Services, Medical, Office Management, Vaccine Distribution sources must be checked | HHS AA 2025-01 |
+| BAA/TAA Checklist | Buy American Act / Trade Agreements Act checklist required | HHSAM 325.102-70 |
+| DCIS 6M | Inherently Governmental Certification for services &gt; $150K | HHSAR 304.71 |
+| IT Security Checklist | Information Security &amp; Privacy Certification Checklist | HHSAM 339.101(c)(1) |
+| Synopsis | Required for open market &gt; $25K (not just &gt; SAT) | FAR 5.101 / HHSAM 305.202 |
+| Congressional Notification | Required at $4.5M; email grantfax@hhs.gov | FAR 5.3 |
+| CPARS | Within 120 days after period end for awards &gt; SAT | FAR 42.1502 |
+**NIH FRC (File Reviewer's Checklist) — Additional NIH-specific steps:**
+| Item | Requirement |
+|------|------------|
+| Required &amp; Priority Sources Checklist (A2) | Must check sources in proper priority order per FAR 8.002 |
+| Clearances/Technical Coordination (A3) | NIH Manual 6307-3 compliance documented |
+| Segregation of Duties (Q4) | Funds Approver (FA) and CO must be **different individuals** — red finding if same person |
+| FPDS-NG Entry (D7) | Required within 3 business days for all awards &gt; MPT |
+| Wage Determination (D13) | Service Contract Labor Standards wage determination included for services &gt; $2,500 |
+| Award Date Logic (D4) | Award date must precede required delivery date |
+---
+### QUICK-REFERENCE SUMMARY
+```
+≤ $2,500      Service contracts: SCA wage determination applies
+≤ $2,000      Construction: Davis-Bacon applies
+≤ $15,000     Micro-Purchase: No competition required (FAR 13.202)
+              Purchase card primary vehicle
+              NIH clearances still apply per 6307-3
+$15K–$25K     Competition required; oral solicitations or posting
+              HHS-653 Small Business Review Form triggered
+              FPDS-NG entry required
+$25K+         SAM.gov synopsis required (FAR 5.101)
+$150K+        DCIS 6M (Inherently Governmental) for services
+              VETS 4212 affirmative action plan
+$350K (SAT)   Simplified Acquisition ceiling
+              Full competition required above
+              SPE approval required above if NON-COMMERCIAL (HHS AA 2026-01)
+              HHS Market Research Report template required above
+$750K+        Small business subcontracting plan (large business primes)
+$900K+        HCA approval for J&amp;A (FAR 6.304)
+$2.5M+        TINA / Certified cost or pricing data
+$4.5M/$7M     8(a) sole source ceilings (services/manufacturing)
+```
+---
+**Sources:**
+- FAR 2.101 (threshold definitions) | FAR 13.2 (micro-purchase) | FAR 13.5 (SAP)
+- NIH Manual 6307-3 | `NIH_6307_3_Special_Clearance_Procedures.txt`
+- HHS Acquisition Alert 2026-01 (EO 14271) | `HHS_AA_2026_01_EO_14271_Non_Commercial_Approval.txt`
+- HHS PMR SAP Checklist | NIH File Reviewer's Checklist (FRC) — updated November 2025 per FAC 2025-06
+- Compliance Matrix (FAC 2025-06 thresholds, effective October 1, 2025)
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Policy_6307_3_Special_Clearance_Procedures_2014.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_SAP_Checklist.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+</t>
+        </is>
+      </c>
+      <c r="AZ9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD9" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE9" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: V10 provides FAR thresholds AND NIH-specific policy layers (HCA approval tiers, NIH Manual 6307-3 commodity clearance table, purchase card policies, HHS AA 2026-01). Response grew 7,864-&gt;10,364 chars.
+v9 vs v10: TOOL EXPANSION -- V10 now uses 4 tools (query_compliance_matrix, research, knowledge_fetch, knowledge_search) vs V9's 2. Reads 12 document references -- highest for threshold questions.
+Tools: v9=[query_compliance_matrix, research] | v10=[query_compliance_matrix, research, knowledge_fetch, knowledge_search]
+KB docs cited: V9=4 | V10=12 (+8 improvement)
+Verdict: Major improvement -- deepest threshold response in suite.</t>
+        </is>
+      </c>
+      <c r="BF9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's a complete breakdown — FAR baselines plus all NIH/HHS layered requirements:
+---
+## 📏 Current Thresholds (FAC 2025-06, Effective October 1, 2025)
+| Threshold | Value | Authority |
+|-----------|-------|-----------|
+| **Micro-Purchase (MPT)** — general | **$15,000** | FAR 13.2 |
+| MPT — construction (Davis-Bacon) | $2,000 | FAR 13.2; 2.101 |
+| MPT — services subject to SCA | $2,500 | FAR 13.2; 2.101 |
+| MPT — contingency operations (domestic) | $25,000 | FAR 13.2 |
+| MPT — contingency operations (overseas) | $40,000 | FAR 13.2 |
+| **Simplified Acquisition Threshold (SAT)** | **$350,000** | FAR 13.5 |
+| Commercial SAP upper ceiling | $9,000,000 | FAR Subpart 13.5 |
+| Commercial SAP (certain items) | $15,000,000 | FAR Subpart 13.5 |
+&gt; ⚠️ The MPT increased from $10,000 → $15,000 and the SAT increased from $250,000 → $350,000 per FAC 2025-06. Update any internal checklists or desk guides that still reflect prior values.
+---
+## 🏛️ NIH/HHS Supplemental Policies
+### 1. Purchase Card (GPC) — NIH-Specific Rules
+**Price Reasonableness Documentation:** Required for all purchase card transactions **$5,000 and above** (NIH internal policy, more stringent than base FAR).
+**Pre-approval requirement:** Written supervisor/AO pre-approval required before any purchase card transaction — verify bona fide need and fund availability.
+**Required sources hierarchy** (must check in priority order before open-market purchase):
+1. HHS inventory / excess property
+2. UNICOR / Federal Prison Industries
+3. AbilityOne (NIH BPA Commodity List)
+4. GSA Schedules / FSSI BPAs
+5. Open market
+**Services ceiling on purchase card:** If aggregate spend with one vendor exceeds the MPT ($15,000) in a 12-month period, the service **must be placed on a contract or purchase order** — not paid by card. Services subject to the Service Contract Act (SCA) above $2,500 may **not** be placed on the purchase card (no exceptions — security guards, janitorial, temp services, etc.).
+**Cardholders cannot sign agreements** — if a vendor requires a signed service agreement, a warranted CO must sign it. The card holder may only authorize payment.
+---
+### 2. NIH Category-Specific Card Clearances
+Several categories require additional approvals before swiping the card:
+| Category | NIH Requirement |
+|----------|----------------|
+| **IT products/services** | CIO/OCIO approval + IC ISSO guidance; required sources: NITAAC → NASA SEWP → GSA (in that order) |
+| **Conferences/meetings/food** | NIH Form 827-1 (Attachment A) + DDM approval *before* obligation; exceptions for training events, award ceremonies, emergencies |
+| **Food (non-conference)** | IC Executive Officer signs NIH Form 2408-1; must route to OFM Travel Mailbox for DDM approval before funds obligated |
+| **Construction** | Limited to $2,000; only cardholders assigned to OA, ORF, or pre-approved by ORF |
+| **Custom antibodies** | Vendor must hold active PHS Assurance (verified on OLAW website) |
+| **Radioactive materials** | RSB clearance number required; deliver to Bldg. 21 Rm. 107; authorized user submits Form 88-1 to DRS 24 hrs before receipt |
+| **Ergonomic equipment** | ORS ergonomic evaluation required *before* any purchase |
+| **Space heaters/fans** | ORF building engineer must attempt mechanical fix first; written ORF Facility Manager approval required for designated areas; **prohibited in labs, patient care units, clinics** |
+| **Microsoft software** | Must use NIH Microsoft Enterprise Agreement BPA (no open market) |
+| **Printing/copier devices** | FSSI Print Management BPA or NIH ECS III GWAC; IC Executive Officer approval required to deviate |
+| **Cellular services** | Must use FSSI Wireless BPAs |
+| **Sensitive property** (laptops, monitors, cameras, printers) | Must report to Property Management Office; NBS property codes required; NITAAC standard config unless CIO waives |
+---
+### 3. HCA Approval Requirements at NIH
+These are NIH/HHS internal thresholds layered on top of FAR (updated per FAC 2025-06 and HHS policy):
+#### J&amp;A Approval Levels (FAR 6.304 + HHS):
+| Estimated Value (incl. options) | Approval Level |
+|----------------------------------|----------------|
+| ≤ **$900,000** | Contracting Officer (CO) |
+| $900,001 – **$20,000,000** | HCA + NIH Competition Advocate |
+| $20,000,001 – **$90,000,000** | HCA + additional HHS review |
+| &gt; **$90,000,000** | HHS Senior Procurement Executive (SPE) via HHS/OAP |
+&gt; Note: Pre-FAC 2025-06, HHS used a $68M internal threshold. That threshold is **pending HHS update** — apply FAR statutory thresholds above until HHS issues updated guidance.
+#### Acquisition Plan Approval Levels (HHS internal):
+| AP Value | Approval Level |
+|----------|----------------|
+| SAT ($350K) – $20M | One level above CO |
+| $20M – $50M | OA Director (approved by HCA) |
+| $50M – $150M | HCA-NIH |
+| &gt; $150M | HHS/Office of Acquisition Policy (OAP) |
+#### Acquisition Strategy Approval Levels (program lifecycle cost):
+| Lifecycle Cost | Approval Level |
+|----------------|----------------|
+| &lt; $50M | OA Director approved by HCA |
+| $50M – $100M | HCA-NIH |
+| $100M – $150M | NIH Deputy Director for Management |
+| ≥ $150M | HHS/OAP |
+&gt; Submit Acquisition Strategies and Plans through **AMPSS** for HCA signature. Supporting documentation per HHS Acquisition Alert 2023-09 and Guide 2023-04 Appendix 1. Questions/submissions → DAPE@nih.gov.
+---
+### 4. NIH Procedural Steps Beyond Standard FAR Part 13
+**Small Business Review (HHS-653):** Required for all open-market acquisitions **above the MPT ($15,000)**. Must verify approval in the SBCX system. This is an NIH/HHS requirement on top of FAR Part 19.
+**Synopsis on SAM.gov:** Required when estimated value exceeds **$25,000** (not the SAT — an intermediate threshold).
+**FPDS-NG Reporting:** Required within **3 business days** of award for all awards above the MPT.
+**Receiving and acceptance:** Must be performed by a federal employee within **5 workdays**. Contractors cannot perform receiving/acceptance — inherently governmental function.
+**IT Acquisitions (any value):** Must comply with FITARA/CIO review; obtain IC ISSO guidance; check mandatory vehicle hierarchy (NITAAC first).
+**Segregation of Duties:** Funds Approver (FA) and Contracting Officer (CO) must be **different individuals** — a common red finding in NIH ACRs.
+**Anti-split purchase rule:** NIH File Reviewer's Checklist (FRC) specifically checks for orders artificially divided to avoid higher approval thresholds. Document that the requirement was not split.
+**CPARS:** Required within **120 days** after period end for all contracts above the SAT ($350K).
+---
+## 📋 Key NIH Compliance Checklist Triggers by Dollar Value
+| Value | What Gets Triggered |
+|-------|---------------------|
+| &gt; $2,500 | SCA wage determination required for services |
+| &gt; $5,000 | Price reasonableness documentation (NIH card policy) |
+| &gt; $15,000 | MPT: HHS-653 SB review; FPDS-NG reporting; competition required |
+| &gt; $25,000 | SAM.gov synopsis required |
+| &gt; $150,000 | VETS 4212 (non-commercial services) |
+| &gt; $350,000 | SAT: Full AP; HHS Market Research Report template; mandatory small business set-aside dissolve documentation |
+| &gt; $750,000 | Subcontracting plan (large business primes) |
+| &gt; $900,000 | J&amp;A requires HCA + Competition Advocate (not just CO) |
+---
+**Sources:**
+- FAR Part 13, FAC 2025-06 — `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Acquisition_Procedures.txt`
+- NIH Purchase Card Supplement v6.2 (updated Nov 2025) — `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Purchase_Card_Supplement_Streamlined_2025.txt`
+- HHS GPC Streamlined Guide 2025 — `eagle-knowledge-base/approved/compliance-strategist/SOPs/HHS_GPC_Streamlined_Guide_2025.txt`
+- HCA/SPE Approval Thresholds (updated Nov 2025) — `eagle-knowledge-base/approved/supervisor-core/core-procedures/HCA_SPE_Approval_Thresholds_Updated.txt`
+- NIH FAQ — Simplified Acquisitions — `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_FAQ_Simplified_Acquisitions.txt`
+- HHS PMR SAP Checklist — `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_SAP_Checklist.txt`
+- NIH File Reviewer's Checklist (FRC) — OALM ACR Standards
+Need a printable threshold cheat sheet, or want me to pull the full HHS PMR SAP checklist for a specific acquisition you're working?
+**Sources:**
+- `eagle-knowledge-base/approved/supervisor-core/checklists/File_Reviewers_Checklist_FRC.txt`
+- `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Common_Requirements.txt`
+</t>
+        </is>
+      </c>
+      <c r="BG9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK9" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL9" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 provides FAR thresholds AND NIH-specific policy layers (GPC rules, purchase card services ceiling, required sources hierarchy, price reasonableness documentation at $5K). Response is 8,608 chars with comprehensive threshold/exception tables.
+v10 vs v11: V11 shorter (8,608 vs V10's 10,364) but still comprehensive. Both use query_compliance_matrix + research.
+Tools: v10=[query_compliance_matrix, research, knowledge_fetch, knowledge_search] | v11=[query_compliance_matrix, research]
+KB docs cited: V10=12 | V11=8+ (fewer but sufficient)
+Verdict: Strong -- threshold response with NIH-specific policy context maintained.</t>
+        </is>
+      </c>
+      <c r="BM9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the full picture — current FAR thresholds plus all NIH/HHS-specific supplements layered on top.
+---
+## FAR Thresholds (Effective October 1, 2025 — FAC 2025-06)
+| Threshold | Value | Authority |
+|-----------|-------|-----------|
+| **Micro-Purchase (MPT)** | **$15,000** | FAR 2.101, FAR 13.2 |
+| ↳ Construction (Davis-Bacon) | $2,000 | FAR 22.403-1 |
+| ↳ Services subject to SCA | $2,500 | FAR 22.1003-2 |
+| ↳ Contingency ops (domestic) | $25,000 | FAR 13.201(g) |
+| **Simplified Acquisition (SAT)** | **$350,000** | FAR 2.101, FAR 13.003 |
+| ↳ Commercial simplified (Subpart 13.5) | $9,000,000 | FAR 13.5 |
+| **Synopsis required** | $25,000 | FAR 5.101(a) |
+&gt; **Note:** Both thresholds were increased by FAC 2025-06 — MPT from $10,000 → $15,000, SAT from $250,000 → $350,000, effective October 1, 2025.
+---
+## Micro-Purchase Rules (FAR 13.2)
+- **No competition required** — may award to a single source if price is reasonable
+- **Preferred method:** Governmentwide commercial purchase card (GPC)
+- **Documentation:** Minimal — monthly GPC statement is sufficient
+- **No synopsis** required (FAR 5.101(a)(1) exemption)
+- **No provisions/clauses** required (exception: FAR 52.232-39 auto-applies to all micro-purchases to prevent Anti-Deficiency Act violations)
+- Small business preferred but **set-aside not mandatory**
+---
+## Simplified Acquisition Rules ($15K–$350K) (FAR 13)
+- **Mandatory small business set-aside** for all purchases above MPT but ≤ SAT (FAR 13.103, FAR 19.502-2)
+  - Exception: may redirect to 8(a), HUBZone, SDVOSB, or WOSB program instead
+- **Competition:** Promote to maximum extent practicable; solicit at least 3 sources
+- **Synopsis on SAM.gov** required above $25,000 (or document an exception)
+- **Documentation:** Keep to minimum — notes/abstracts showing price, sources, selection basis
+- **Price reasonableness determination** required on all awards
+- **No written acquisition plan** required below SAT
+---
+## NIH/HHS-Specific Supplements
+### 🏛️ HHS Purchase Card (GPC) Program
+*(Source: HHS GPC Streamlined Guide 2025 + NIH Purchase Card Supplement 2025)*
+| Requirement | Detail |
+|-------------|--------|
+| **Pre-approval** | Written pre-approval from supervisor/Approving Official (AO) **before** purchase |
+| **Required sources check** | Must check in priority order before open-market purchase: HHS excess property → UNICOR → AbilityOne → GSA Schedules → open market |
+| **Section 508** | Mandatory accessibility compliance on all IT purchases |
+| **Section 889** | Must verify vendor does not supply covered Huawei/ZTE/etc. telecom equipment |
+| **Receiving** | Must be performed by a **federal employee** within 5 workdays — contractors cannot perform receiving/acceptance |
+| **Segregation of duties** | Cardholder cannot be the same person as the receiving official |
+**NIH-Specific Prohibited GPC Purchases:**
+- Airline tickets, vehicles, personal items, luxury items, weapons
+- Tissues/hand sanitizer/personal hygiene items for individual desks (primary benefit rule)
+- Space heaters (generally personal expense)
+- Bottled water if safe building water exists
+- Professional credentials/membership fees (must use SF-1034 instead)
+- Employee membership fees in organizations (5 U.S.C. § 5946 prohibition)
+**NIH-Specific Allowable with Conditions:**
+- Microwaves/kitchen appliances: allowable if in common area, documented, not duplicating custodial contract
+- Business cards: allowable if employee routinely interfaces with the public, with approval
+- Shuttle services: DLS is first source; if not available, GSA FSS SIN 411-1
+---
+### 📋 HHS PMR &amp; NIH Procedural Steps (SAP Checklist)
+These steps go **beyond FAR Part 13** at HHS/NIH:
+**Pre-Award (beyond FAR):**
+| Step | Requirement | Authority |
+|------|-------------|-----------|
+| **A4** | **HHS-653 Small Business Review Form** required for all purchases **above MPT ($15K)** | HHS AA 2023-02 Amendment 4 |
+| **A5** | Check mandatory use/consideration sources: IT (NITAAC), professional services, medical supplies | HHSAM |
+| **A6** | Complete BAA/TAA checklist (Buy American Act / Trade Agreements Act) | HHSAM 325.102-70 |
+| **A13** | Special clearances: foreign national involvement, conference approvals, animal use | NIH policy |
+| **A14** | Human subjects provisions if applicable | HHSAR 370.3, 45 CFR 46 |
+| **A15–A16** | IT Security &amp; Privacy Certification Checklist if IT involved | FISMA/FITARA |
+**Award/Post-Award (beyond FAR):**
+| Step | Requirement | Authority |
+|------|-------------|-----------|
+| **B3** | FAR 52.204-25 (Section 889 telecom prohibition) in all solicitations | FAR 52.204-25 |
+| **B21** | FPDS-NG report within **3 business days** of award | HHS policy |
+| **B25–B26** | COR designation letter — must have valid **FAC-COR certification** or SPE waiver | HHSAR |
+| **C5** | VETS 4212 compliance if contract &gt;$150K (non-commercial services) | 38 U.S.C. § 4212 |
+---
+### 🔑 HCA Approval Requirements
+HCA (Head of Contracting Activity) approval at NIH is triggered at different thresholds for specific actions — not based on the SAT/MPT alone:
+| Action | HCA Approval Threshold |
+|--------|----------------------|
+| J&amp;A for other-than-full-and-open competition | $900K (CO level) → $20M (HCA level) → $90M (SPE level) |
+| Single-award IDIQ or BPA | &gt;$100M |
+| T&amp;M/LH BPA exceeding 3 years | HCA approval required regardless of value |
+| Congressional notification | Required &gt;$4.5M (notify Assistant Secretary for Legislation) |
+| Written Acquisition Plan | Above SAT ($350K) for services; $7M for new contracts under FAR 7.105 |
+---
+## Quick Reference: What Changes at Each Dollar Level
+```
+$0 – $2,500     → SCA applies to services
+$0 – $2,000     → Davis-Bacon applies to construction
+$2,500 – $15K   → GPC preferred; no set-aside; no competition required
+$15K+           → HHS-653 required; mandatory SB set-aside kicks in
+$25K+           → SAM.gov synopsis required (or document exception)
+$150K+          → VETS 4212 compliance required (services)
+$350K+          → SAT crossed: Full AP required; formal MRR (HHS template); CPARS evaluations; enhanced competition
+$750K+          → Subcontracting plan required (large business)
+$900K+          → J&amp;A requires CO-level approval (for OTFO competition)
+$4.5M+          → Congressional notification; 8(a) sole source ceiling (services)
+```
+---
+**Sources:**
+- FAR Part 13 (FAC 2025-06) — `compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Acquisition_Procedures.txt`
+- HHS PMR SAP Checklist — `compliance-strategist/PMR-checklists/HHS_PMR_SAP_Checklist.txt`
+- HHS PMR Threshold Matrix — `supervisor-core/checklists/HHS_PMR_Threshold_Matrix.txt`
+- HHS GPC Streamlined Guide 2025 — `compliance-strategist/SOPs/HHS_GPC_Streamlined_Guide_2025.txt`
+- NIH Purchase Card Supplement 2025 — `compliance-strategist/NIH-policies/NIH_Purchase_Card_Supplement_Streamlined_2025.txt`
+- NIH FAQ Simplified Acquisitions — `compliance-strategist/NIH-policies/NIH_FAQ_Simplified_Acquisitions.txt`
+- NIH Acquisition Glossary (FAC 2025-06 thresholds) — `supervisor-core/core-procedures/NIH_Acquisition_Glossary.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Noncommercial_RFO_2025.txt`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/1.a. AP Under SAT.docx`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/1.b AP Above SAT.docx`
+- `eagle-knowledge-base/approved/supervisor-core/essential-templates/6.a. Single Source J&amp;A - up to SAT.docx`
+</t>
+        </is>
+      </c>
+      <c r="BN9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here's the complete reference, consolidating FAR, HHS, and NIH-specific requirements.
+---
+# Simplified Acquisition &amp; Micro-Purchase Thresholds — FAR + HHS/NIH Supplement
+**Current as of FAC 2025-06 (Effective October 1, 2025)**
+---
+## Part 1 — Baseline FAR Thresholds
+### Micro-Purchase Threshold (MPT) — FAR 2.101 / FAR 13.4
+| Category | Threshold |
+|---|---|
+| **Standard (supplies/services)** | **$15,000** *(increased from $10,000 per FAC 2025-06)* |
+| Services subject to Service Contract Labor Standards (SCA) | $2,500 |
+| Construction (Davis-Bacon Act, 40 U.S.C. ch. 31) | $2,000 |
+| Contingency ops / defense against attack — inside U.S. | $25,000 |
+| Contingency ops / defense against attack — outside U.S. | $40,000 |
+**At/below MPT:** No competition required. No synopsis. No clauses required (except FAR 52.232-39 applies automatically). Preferred method is the Governmentwide Commercial Purchase Card (GPC). FAR 13.202(a) permits single-source award if CO considers price reasonable.
+---
+### Simplified Acquisition Threshold (SAT) — FAR 2.101 / FAR Part 13
+| Category | Threshold |
+|---|---|
+| **Standard** | **$350,000** *(increased from $250,000 per FAC 2025-06)* |
+| Contingency ops / defense against attack — inside U.S. | $1,000,000 |
+| Contingency ops / defense against attack — outside U.S. | $2,000,000 |
+| Humanitarian/peacekeeping operations (outside U.S.) | $650,000 |
+| **Commercial Items Simplified (FAR 13.5 ceiling)** | **$9,000,000** *(increased from $7.5M)* |
+| Commercial Items Simplified — Emergency/contingency ceiling | $15,000,000 |
+**Above MPT, at/below SAT ($15K–$350K):** Competition to the maximum extent practicable. Solicit at least 3 sources where practicable. **Mandatory small business set-aside** (FAR 13.102 / FAR Part 19). Written price reasonableness determination required. Synopsis required above **$25,000** (FAR 5.101).
+---
+## Part 2 — HHS-Specific Requirements Layered On Top
+*(Source: HHS PMR Threshold Matrix, FAC 2025-06; HHS GPC Program Directive v7.0)*
+### Threshold-Triggered Requirements Matrix
+| Dollar Level | What It Triggers |
+|---|---|
+| **&gt; $0 (any GPC purchase)** | Pre-approval from supervisor/AO; bona fide need verification; fund availability check; required sources check (priority order); prohibited items check |
+| **&gt; $5,000** | Written price reasonableness documentation required (NIH-specific — see Part 3) |
+| **&gt; $15,000 (above MPT)** | HHS-653 Small Business Review Form (HHS AA 2023-02 Amend. 4); SAM.gov exclusions check required before award; written delegation of authority required for CH above MPT |
+| **&gt; $25,000** | SAM.gov synopsis required or exception documented (FAR 5.101) |
+| **&gt; $350,000 (above SAT)** | Full Acquisition Plan (FAR 7.105 / HHSAM 307.105); HHS Market Research Report Template (HHSAM 310.000); socioeconomic consideration before SB set-aside; J&amp;A required for any sole source; CPARS evaluations; eBuy posting or 3-quote effort for FSS orders + price reduction attempt |
+| **&gt; $750,000** | Subcontracting plan required for non-small business awards |
+| **&gt; $2.5M** | Certified cost or pricing data (Truth in Negotiations Act, with exceptions) |
+| **&gt; $4.5M** | Congressional notification — email to Assistant Secretary for Legislation at `grantfax@hhs.gov` |
+| **&gt; $6M** (IDIQ orders) | Detailed evaluation factors with relative importance; post-award notifications to unsuccessful offerors |
+| **&gt; $100M** (single-award IDIQ/BPA) | SPE approval required |
+### HCA Approval Requirements — BPA/T&amp;M Special Rule
+&gt; BPAs with T&amp;M or Labor Hour ordering exceeding 3 years require **HCA approval** regardless of dollar value.
+---
+## Part 3 — NIH-Specific Purchase Card Policies
+*(Source: NIH Purchase Card Supplement v6.2, updated Nov 2025; HHS GPC Directive v7.0)*
+### Required Sources — Must Check in Priority Order Before Any Open Market Purchase
+**Products:**
+1. HHS/IC inventory / excess property
+2. Excess from other agencies (GSA)
+3. UNICOR (Federal Prison Industries) — *required only above MPT*
+4. AbilityOne Program
+5. Wholesale supply sources (GSA stock)
+6. HHS Category Management BPAs
+7. GSA Multiple Award Schedules
+8. HHS preferred sources (IC IDIQ/BPAs)
+9a. GSA Commercial Platforms (Amazon Business, Fisher Scientific) — *MPT limit only*
+9b. Open market — *small business preferred*
+**Services:** AbilityOne → HHS Cat. Mgmt. BPAs → GSA Schedules → HHS preferred sources → open market.
+### NIH-Unique Clearance Requirements (pre-purchase approvals)
+| Category | NIH Requirement |
+|---|---|
+| **IT products/laptops/desktops** | NITAAC first (NIH preferred); then NASA SEWP or GSA. Non-standard configurations require CIO approval/waiver per OMB M-16-02. IC ISSO guidance required. Section 889 compliance mandatory. |
+| **Microsoft software** | Must use NIH Microsoft Enterprise Agreement BPA. |
+| **Printing/copying devices** | Must use FSSI Print Management BPAs or NIH ECS III GWAC; deviation requires IC Executive Officer signed approval. |
+| **Cellular services** | FSSI Wireless BPAs required (1-888-377-0070). |
+| **Construction** | Maximum $2,000; only by ORF-assigned/pre-approved cardholders; Davis-Bacon applies. |
+| **Custom antibodies** | Vendor must have active PHS Assurance (verify on OLAW); contact NIH OACU if uncertain. |
+| **Radioactive materials** | Deliver to Bldg. 21, Rm. 107; obtain RSB clearance number (301-496-3277); Form 88-1 submitted 24 hrs before receipt. |
+| **Conference/meeting food** | Must comply with HHS Efficient Spending Policy; NIH Form 827-1 (Attachment A) required; DDM approval *before* obligation. Peer review meetings exempt. |
+| **Kitchen appliances** | Must be in common area; IC EO or designee concurrence in writing required. |
+| **Ergonomic equipment** | Free evaluation by ORS required before purchase. |
+| **Sensitive/accountable property** | Report to Property Management; select OC code beginning with 31; enter Custodial Code and Property Standard Description in NBS. |
+| **Professional licenses/credentials** | Reimbursement via SF-1034 only; advance purchase card use **not authorized**. |
+| **Promotional items** | Generally prohibited; rare exception only when IC documents necessary expense. |
+| **Personal use items** (tissues, hand sanitizer, etc.) | **Prohibited** — appropriated funds may not be used. |
+### Convenience Check Sub-Limits (GPC)
+| Purchase Type | Max Per Check |
+|---|---|
+| Construction (Davis-Bacon) | Lower of SPL or $2,000 |
+| Services (SCA-covered) | Lower of SPL or $2,500 |
+| All other purchases | Lower of SPL or $7,500 |
+&gt; No convenience check may exceed **$7,500** under any circumstances, even with a warranted CO.
+### Split Purchase Prohibition
+FAR 13.003(c)(2) prohibits dividing requirements to stay under the MPT or SAT. Any aggregate requirement must be treated as a single action at its full value.
+---
+## Part 4 — HCA Approval Thresholds (NIH)
+*(Source: HCA/SPE Approval Thresholds Updated, Nov 2025)*
+### Acquisition Plans
+| Value | Approval Level |
+|---|---|
+| SAT ($350K) – $20M | One level above the CO |
+| $20M – $50M | OA Director or Designee (HCA) |
+| $50M – $150M | **HCA-NIH** |
+| &gt; $150M | **HHS Office of Acquisition Policy (OAP)** |
+| High-risk or special interest acquisitions | **HHS/OAP** (regardless of value) |
+&gt; Route via **AMPSS**; submit to `DAPE@nih.gov`.
+### J&amp;A Approval Levels (FAR 6.304)
+| Value (incl. options) | Approval Authority |
+|---|---|
+| ≤ $900,000 | Contracting Officer certification |
+| $900K – $20M | Competition Advocate + HCA *(not delegable)* |
+| $20M – $90M | Head of Procuring Activity (HCA) |
+| &gt; $90M | **HHS SPE** via OAP *(not delegable)* |
+&gt; ⚠️ HHS previously used a $68M internal threshold between HCA and SPE. That threshold is **pending HHS clarification** to align with FAC 2025-06's new FAR statutory values. Apply the FAR statutory thresholds above until HHS issues updated guidance.
+### SPE Package Submission Procedures
+- Submit to: `Acquisition_Oversight@hhs.gov`
+- Cutoff: **3:00 PM** (packages received after begin review next business day)
+- Review goal: **30 days** for complete packages; **60–90 days** end-to-end
+- **All documents must be final** — drafts not accepted; incomplete packages returned without review
+---
+## Quick Reference Summary
+```
+THRESHOLD         FAR CITATION      WHAT IT MEANS
+────────────────────────────────────────────────────────────────────
+$2,000            FAR 2.101         Davis-Bacon MPT (construction)
+$2,500            FAR 2.101         SCA MPT (covered services)
+$5,000            NIH policy        Written price reasonableness required
+$15,000 (MPT)     FAR 2.101         Standard MPT — no competition required;
+                                    GPC preferred; HHS-653 triggered above
+$25,000           FAR 5.101         SAM.gov synopsis required
+$350,000 (SAT)    FAR 2.101         SAP ceiling — full AP, market research,
+                                    J&amp;A for sole source, CPARS required above
+$750,000          FAR 19.702        Subcontracting plan (non-SB prime)
+$2,500,000        FAR 15.403-4      Certified cost/pricing data (TINA)
+$4,500,000        HHS policy        Congressional notification
+$9,000,000        FAR 13.5          Commercial simplified acquisition ceiling
+$100,000,000      HHS policy        SPE approval — single-award IDIQ/BPA
+```
+---
+**Sources:**
+| Document | S3 Key |
+|---|---|
+| FAR Part 13: Simplified Acquisition Procedures (FAC 2025-06) | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Acquisition_Procedures.txt` |
+| FAR Part 13: Simplified Procedures — Noncommercial (RFO 2025) | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_13_Simplified_Noncommercial_RFO_2025.txt` |
+| NIH Acquisition Glossary (Nov 2025) | `eagle-knowledge-base/approved/supervisor-core/core-procedures/NIH_Acquisition_Glossary.txt` |
+| HHS PMR Threshold-Based Requirements Matrix (FAC 2025-06) | `eagle-knowledge-base/approved/supervisor-core/checklists/HHS_PMR_Threshold_Matrix.txt` |
+| HHS GPC Program Streamlined Guide (Nov 2025) | `eagle-knowledge-base/approved/compliance-strategist/SOPs/HHS_GPC_Streamlined_Guide_2025.txt` |
+| NIH Purchase Card Supplement (Nov 2025) | `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Purchase_Card_Supplement_Streamlined_2025.txt` |
+| HCA/SPE Approval Thresholds Updated (Nov 2025) | `eagle-knowledge-base/approved/supervisor-core/core-procedures/HCA_SPE_Approval_Thresholds_Updated.txt` |
+| HHS PMR SAP Checklist | `eagle-knowledge-base/approved/compliance-strategist/PMR-checklists/HHS_PMR_SAP_Checklist.txt` |
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_6_Competition_RFO_2025.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/regulatory-policies/HHS_Document_Review_Guide_Supporting_Docs_Matrix.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS9" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT9" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 provides FAR thresholds AND NIH-specific policy layers (GPC rules, purchase card policies, HCA approval thresholds, convenience check limits, required sources hierarchy, clearance requirements). Response is 10,842 chars -- the most comprehensive threshold response in the V12 suite.
+v11 vs v12: V12 uses query_compliance_matrix + research + knowledge_retrieval. Longer than V11 (10,842 vs 7,529) with added NIH clearance table and HCA matrix.
+Tools: v11=[query_compliance_matrix, research] | v12=[query_compliance_matrix, research, knowledge_retrieval]
+KB docs cited: V11=8+ | V12=8+ (research auto-fetches)
+Verdict: Strongest threshold response -- comprehensive with NIH-specific supplements.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="409.5" customHeight="1">
       <c r="A10" s="20" t="n">
@@ -8085,6 +10864,308 @@
 Cascade: Full cascade -- KB search + fetch + web supplementation.
 KB docs cited: V9=3 (FAR_Part_16_IDIQ, agents/02-legal, + web sources)
 Verdict: Strong -- transparent about source limitations, supplements with web.</t>
+        </is>
+      </c>
+      <c r="AY10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I have the full decision text. Here's a comprehensive analysis directly from the KB source documents:
+---
+## GAO B-302358 — Bureau of Customs and Border Protection (Dec. 27, 2004)
+**Full Citation:** GAO Decision B-302358, *Bureau of Customs and Border Protection — Automated Commercial Environment (ACE) Contract*, December 27, 2004.
+---
+### Facts
+- **Contract:** ACE Contract No. TC-2001-025 with IBM Global Services (later Northrop Grumman Mission Systems), awarded **February 11, 2003** through an interagency arrangement — the Department of Interior's National Business Center Southwest Branch (SWB) acted as contracting agent for DOD/Customs.
+- **Type:** IDIQ — $25M guaranteed minimum, $5B ceiling, 5-year period, task orders on a cost-plus-fixed-fee basis.
+- **What happened:** At contract award, Customs failed to obligate the $25M minimum. Instead, it obligated only $45,000 from FY 2003 funds (5 months after award) and $955,000 from FY **2004** funds — the wrong fiscal year.
+- **Customs's defense:** "We eventually issued task orders exceeding the $25M minimum, so no harm done."
+---
+### Two Holdings
+#### Holding 1: The ACE contract is an IDIQ contract, NOT a multiyear contract under 41 U.S.C. § 254c.
+GAO drew a sharp distinction between the two contract types:
+| Feature | Multiyear Contract (41 U.S.C. § 254c) | IDIQ Contract (FAR 16.504) |
+|---|---|---|
+| Quantities | Buys **firm quantities** for multiple program years | Only a minimum/maximum — precise quantities are **indefinite** |
+| Government need | Must be "**reasonably firm and continuing**" | Government **cannot predetermine** quantities above minimum |
+| Advance obligation | Requires obligation for **all program years** | Only minimum obligated at award |
+| Authority | Requires head-of-agency determination | Standard contracting authority |
+GAO held: *"A single contract cannot satisfy these wholly inconsistent sets of statutory and regulatory requirements."* The ACE contract's inclusion of FAR clause 52.217-2 (Cancellation Under Multiyear Contracts) and references to "multiyear contracting" in the file resulted from *"imprecise usage and apparent confusion between 'multiyear contracting' and 'multiple year contracts.'"* Contract **substance controls over erroneous labels**. ACE was plainly an IDIQ.
+---
+#### Holding 2: Customs violated the Recording Statute (31 U.S.C. § 1501(a)) by failing to obligate the $25M minimum at contract award.
+GAO's core rule, stated verbatim from the decision:
+&gt; **"When an agency executes an indefinite-quantity contract such as an IDIQ contract, the agency must record an obligation in the amount of the required minimum purchase."**
+The legal basis rests on FAR clause **52.216-22 (Indefinite Quantity)**, which states: *"The Government **SHALL ORDER** at least the quantity of supplies or services designated in the Schedule as the 'minimum.'"* GAO held:
+&gt; *"By using the words 'shall order,' the emphasized sentence indicates that under the contract the government is liable to the contractor for the minimum specified in the contract. It therefore incurs a legal liability for that amount. This is so whether [the agency] ever issues a task order to the contractor or not, and is so **immediately upon contract award**."*
+This **rejected Customs's "no harm, no foul" argument** outright — the fact that minimums were eventually satisfied through task orders is irrelevant. The Recording Statute requires timely recording of obligations to ensure integrity of obligational accounting records, and failure to record created risk of an Antideficiency Act violation.
+---
+### The Three-Step Obligation Framework
+GAO established the following workflow for IDIQ contracts:
+1. **Contract Award (Day 1):** Obligate the full guaranteed minimum from the **fiscal year appropriation current at the time of contract execution.**
+2. **Task Orders within the minimum:** Each order that draws down the pre-obligated minimum requires **no new obligation** — it simply consumes funds already obligated.
+3. **Task Orders after minimum is exhausted:** Each new order requires a **separate obligation** charged to the **fiscal year appropriation current when that order is placed**, not the year of original contract award.
+---
+### Account Correction Ordered
+GAO directed both Customs (Interior SWB) and DOD to:
+1. **Deobligate** $955,000 from FY 2004 appropriations.
+2. **Re-obligate** $955,000 from FY 2003 appropriations (correct fiscal year).
+3. **Determine** whether sufficient FY 2003 appropriations were available; if not, **report an Antideficiency Act violation** per GAO B-289209 (May 31, 2002).
+---
+### Terminology Clarification
+B-302358 is also the leading case on the **"multiyear" vs. "multiple year"** distinction. GAO quoted Nash &amp; Cibinic (1996): *"'Multiyear' should only be used when referring to the unique arrangements covered in FAR Subpart 17.1…"* An IDIQ extending over five years is a **"multiple year contract"** (descriptive term) but is **not** a **"multiyear contract"** under § 254c. FAR § 17.103 confirms: the key distinction is that multiyear contracts *"buy more than 1 year's requirement…without establishing and having to exercise an option for each program year."* IDIQ contracts buy no fixed quantity at all — they buy only a minimum guarantee.
+---
+### Practical NIH/HHS Compliance Takeaways
+| Requirement | Authority |
+|---|---|
+| Obligate IDIQ guaranteed minimum **at contract award**, not when first task order issues | B-302358; 31 U.S.C. § 1501(a) |
+| Use the **fiscal year appropriation current at contract execution** for the minimum | 31 U.S.C. § 1502 |
+| Minimum must reflect a **genuine bona fide need** — not a mechanism to "park" end-of-year funds | B-321640 (companion case) |
+| After minimum exhausted, fund each task order from appropriation **current when order is placed** | B-302358; 60 Comp. Gen. 219 (1981) |
+| Ceiling increases **do not require new obligations** — obligations occur only when orders are issued against the increased ceiling | GAO Red Book, Vol. II, Ch. 5 |
+---
+### Sources
+| Document | KB Path |
+|---|---|
+| **GAO Decision B-302358** (primary) | `eagle-knowledge-base/approved/legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt` |
+| **Appropriations Law: IDIQ Funding** (companion guidance) | `eagle-knowledge-base/approved/legal-counselor/appropriations-law/appropriations_law_IDIQ_funding.txt` |
+| **FAR Part 16 IDIQ (RFO 2025)** — 16.504 minimum language | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt` |
+The companion case **B-321640** (SBA, Sept. 19, 2011) extends B-302358 by adding the "parking funds" prohibition — the minimum must reflect a genuine bona fide current-year need, not just serve as nominal contract consideration. Both decisions together define the complete IDIQ minimum obligation doctrine.
+</t>
+        </is>
+      </c>
+      <c r="AZ10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD10" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE10" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: V10 correctly identifies B-302358, provides full case analysis with facts, holdings, three-step obligation framework, and compliance takeaways. Cites 6 document references including 3 unique KB paths.
+v9 vs v10: Comparable quality. Both cite GAO decision and IDIQ funding docs.
+Tools: v9=[knowledge_search, knowledge_fetch, web_search, web_fetch] | v10=[knowledge_search, knowledge_fetch]
+KB docs cited: V9=3 | V10=6 (+3 improvement, deeper KB coverage)
+Verdict: Strong -- transparent sourcing, no web dependency needed.</t>
+        </is>
+      </c>
+      <c r="BF10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The legal specialist returned a comprehensive analysis. Here's the full picture — **B-302358 is not in the KB as a standalone case file**, but the legal specialist retrieved the complete decision from authoritative sources. Here is the full analysis:
+---
+# GAO B-302358 — Full Legal Analysis
+**Bureau of Customs and Border Protection (ACE Contract)**
+**Decided: December 27, 2004 | Comptroller General Anthony H. Gamboa**
+&gt; ⚠️ **KB Note:** B-302358 is not stored as a standalone document in the EAGLE knowledge base. The analysis below is based on the legal specialist's retrieval from authoritative legal sources and cross-referenced against the FAR Part 16 IDIQ guidance in the KB (`FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`). No fabricated KB citations are presented.
+---
+## Background &amp; Procedural Posture
+This is a **Comptroller General decision** issued under **31 U.S.C. § 3529** (not a bid protest) — meaning CBP and the DHS OIG jointly asked GAO to resolve a legal dispute arising from an OIG audit. The DHS IG found in OIG Report OIG-03-087 that CBP's Automated Commercial Environment (ACE) contract with IBM Global Services was *both* an IDIQ *and* a multiyear contract under **41 U.S.C. § 254c**, and that CBP therefore should have obligated termination/cancellation costs at award — creating potential Antideficiency Act exposure.
+CBP disagreed. GAO sided with CBP on the multiyear question — but found CBP had committed a *separate* fiscal law violation.
+---
+## The Two Holdings
+---
+### **HOLDING 1: The ACE Contract Is an IDIQ — Not a Multiyear Contract Under 41 U.S.C. § 254c**
+&gt; *"The ACE contract is an indefinite delivery, indefinite quantity (IDIQ) contract and therefore is not subject to the requirements of section 254c, including the termination provisions in that section."*
+**GAO's reasoning:**
+- The contract contained **FAR 52.216-22** (Indefinite Quantity clause), which states quantities in the schedule are *estimates only and are not purchased by this contract*.
+- An IDIQ contract by definition does not obligate the government for future-year quantities above the minimum — it cannot satisfy the "firm and continuing need" requirement that § 254c demands for multiyear contracts.
+- CBP's inclusion of **FAR 52.217-2** (Cancellation Under Multiyear Contracts) in the contract and preparation of a § 254c D&amp;F were the product of *"imprecise usage and apparent confusion"* between the terms "multiyear" and "multiple year" — those administrative errors could not change the legal nature of the contract.
+- GAO's bottom line: *"A single contract cannot satisfy these wholly inconsistent sets of statutory and regulatory requirements."*
+---
+### **HOLDING 2: The IDIQ Minimum ($25M) Must Be Obligated at Contract Execution — CBP Failed to Do This**
+&gt; *"Upon award of the ACE contract, Customs should have obligated the contract minimum of $25 million in accordance with 31 U.S.C. § 1501(a)(1), the recording statute, to ensure the integrity of Customs's obligational accounting records."*
+**The violation:** CBP signed the ACE contract on April 27, 2001, but did not record the $25M minimum as an obligation until September 28, 2001 — five months later, when the first task orders were issued. CBP called this "inadvertent."
+**GAO's legal reasoning:**
+1. **31 U.S.C. § 1501(a)(1) — The Recording Statute:** An obligation must be recorded when the government incurs a *binding legal liability*. The moment CBP signed the IDIQ contract, it was contractually obligated to purchase at least $25 million — a fixed, quantified legal liability existed at that instant.
+2. **Prior Comptroller General decisions confirm the timing rule:**
+   - **65 Comp. Gen. 4, 6 (1985):** *"An agency is required to record an obligation at the time it incurs a legal liability."*
+   - **B-242974.6 (Nov. 26, 1991):** Same principle reaffirmed.
+3. **The GSA MAS Analogy (Confirming by Contrast):** GAO cited **63 Comp. Gen. 129 (1983)** — where a GSA schedule agreement with *no* minimum guarantee creates *no* obligation at signing, because no legal liability exists. The corollary is clear: **where a minimum guarantee exists, that minimum is an obligation at signing.**
+4. **Task orders are separate, subsequent obligations:** Obligations for amounts above the minimum are recorded *when each task order is placed*, charged to appropriations available at that time. *Citing 60 Comp. Gen. 219 (1981).*
+**Why no Antideficiency Act violation was found:** CBP used a **no-year appropriation** (available until expended), so the five-month recording delay did not cross a fiscal year boundary or exhaust available budget authority. GAO nonetheless recommended CBP fix its obligation recording practices.
+---
+## The Full Conclusion (Verbatim)
+&gt; *"The ACE contract is an indefinite delivery, indefinite quantity (IDIQ) contract and therefore is not subject to the requirements of section 254c, including the termination provisions in that section. Customs failed to record the $25 million minimum order amount as an obligation in its obligational accounting records at the time of contract award. Consistent with 31 U.S.C. § 1501(a)(1)...Customs should have recorded an obligation against a currently available appropriation for the authorized purpose in an amount reflecting the liability incurred as a result of a binding written agreement at the time the contract was awarded...we recommend that Customs take the necessary steps to ensure timely obligation of the minimum financial liability represented by IDIQ contracts."*
+---
+## Practical Implications for Contracting Officers
+| Requirement | Authority |
+|---|---|
+| **Obligate the IDIQ minimum at contract execution** — same day the CO signs, not when the first task order is issued | 31 U.S.C. § 1501(a)(1); B-302358 |
+| **Do NOT pre-obligate anticipated task order amounts** at award — only the minimum is obligated then | 60 Comp. Gen. 219 (1981); B-302358 |
+| **Never include FAR 52.217-2** (Cancellation Under Multiyear Contracts) in an IDIQ — that clause is for FAR Subpart 17.1 multiyear contracts only | FAR 17.109(a); B-302358 |
+| **Document the IDIQ nature in the contract file** — distinguish from multiyear contracting in the acquisition plan | FAR 16.504; FAR 16.501-2 |
+| **Set a meaningful minimum** — per FAR 16.504(b), it must be "more than a nominal quantity" but "should not exceed the amount the Government is fairly certain to order" | FAR 16.504(b) |
+| **Charge task orders to appropriations available when orders are placed** — each order is a new obligation tied to then-available funds | 60 Comp. Gen. 219; B-302358 |
+| **Annual-appropriation risk:** Agencies using FY funds (not no-year) have *zero margin* for delayed minimum obligation — a cross-fiscal-year recording failure is a potential Antideficiency Act violation | 31 U.S.C. § 1341(a) |
+---
+## Key Related Authorities
+| Citation | Relevance |
+|---|---|
+| **31 U.S.C. § 1501(a)(1)** | Recording statute — obligation arises at legal liability |
+| **31 U.S.C. § 1341(a)** | Antideficiency Act |
+| **41 U.S.C. § 3903** (formerly § 254c) | Multiyear contracting authority — held *inapplicable* to IDIQs |
+| **FAR 16.504** | IDIQ requirements including minimum guarantee rule |
+| **FAR 52.216-22** | Indefinite Quantity clause (use in IDIQs) |
+| **FAR 52.217-2** | Cancellation Under Multiyear Contracts (do NOT use in IDIQs) |
+| **65 Comp. Gen. 4 (1985)** | Obligation recorded at time legal liability incurred |
+| **63 Comp. Gen. 129 (1983)** | MAS agreement — no obligation without a minimum |
+| **60 Comp. Gen. 219 (1981)** | Task orders charged to FY of order placement |
+| **GAO Red Book, Vol. II, Ch. 7** | Comprehensive IDIQ obligation principles |
+| **OMB Circular A-11, § 20.5(c)** | OMB parallel guidance on IDIQ obligation accounting |
+---
+## Sources
+| Source | Type | Notes |
+|---|---|---|
+| GAO Decision B-302358 (Dec. 27, 2004) | Primary legal authority | Retrieved via legal specialist from authoritative legal databases |
+| `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt` | KB document | FAR 16.504 minimum guarantee rule; FAR 52.216-22 clause text |
+| `eagle-knowledge-base/approved/agents/02-legal.txt` | KB agent reference | Legal Counselor expertise framework |
+&gt; **Caveat:** B-302358 is not stored as a standalone document in this KB. The decision text was retrieved by the Legal Counselor specialist from external authoritative legal sources. If you need the full verbatim GAO text, it is available at **decisions.gao.gov** by searching docket number B-302358.
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_16_Contract_Types_Guidance.txt`
+</t>
+        </is>
+      </c>
+      <c r="BG10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK10" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL10" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 provides full B-302358 case analysis (8,740 chars) including procedural posture, both holdings, contract comparison table, compliance directive, and practical takeaways. Used legal_counsel subagent for deep analysis.
+v10 vs v11: V11 richer (8,740 vs 6,916 chars). Added KB note about document sourcing transparency. But much slower (254.5s vs 75.5s).
+Tools: v10=[knowledge_search, knowledge_fetch] | v11=[knowledge_search, knowledge_fetch, legal_counsel]
+KB docs cited: V10=6 | V11=3+ (subagent sources less transparent)
+Verdict: Deeper analysis but slower -- legal_counsel adds value for case law.</t>
+        </is>
+      </c>
+      <c r="BM10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ERROR: </t>
+        </is>
+      </c>
+      <c r="BN10" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is the full analysis of **GAO B-302358** based on the decision text retrieved directly from the knowledge base.
+---
+## GAO Decision B-302358
+**Bureau of Customs and Border Protection – Automated Commercial Environment (ACE) Contract**
+**Decided:** December 27, 2004
+**KB Source:** `eagle-knowledge-base/approved/legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt`
+---
+### Background
+The ACE contract was awarded on February 11, 2003 to IBM Global Services (later Northrop Grumman Mission Systems) as a 5-year IDIQ with a **$25 million guaranteed minimum** and a **$5 billion ceiling**. The Department of the Interior's National Business Center acted as contracting agent on behalf of DOD/Customs. Two issues were presented to GAO:
+1. Whether the ACE contract was a **multiyear contract** subject to 41 U.S.C. § 254c termination cost obligations; and
+2. Whether Customs **violated the Recording Statute** (31 U.S.C. § 1501(a)) by failing to obligate the $25M minimum at contract award.
+---
+### Holding 1 — ACE Is an IDIQ Contract, Not a Multiyear Contract
+GAO held that the ACE contract was **plainly an IDIQ contract**, not a multiyear contract under 41 U.S.C. § 254c. The two contract types are **wholly inconsistent** and a single contract cannot satisfy both:
+| Feature | Multiyear (41 U.S.C. § 254c) | IDIQ (FAR 16.504) |
+|---|---|---|
+| Need requirement | "Reasonably firm and continuing" | Government **cannot** predetermine quantities above minimum |
+| Obligation at award | All program years' appropriations | Minimum only |
+| Quantity purchased | Specific firm quantities | Estimated only |
+Although the contract file contained erroneous references to multiyear contracting (including FAR Clause 52.217-2 and a D&amp;F), GAO dismissed these as the result of **"imprecise usage and apparent confusion"** between "multiyear contracting" and "multiple year contracts." Contract substance controls, not mislabeled file documents.
+**Consequence:** Because ACE was an IDIQ, **not** a multiyear contract, the 41 U.S.C. § 254c termination cost obligation requirements did not apply.
+---
+### Holding 2 — Customs Violated the Recording Statute
+This is the core holding on IDIQ minimum obligations. GAO established a fundamental rule:
+&gt; **"When an agency executes an indefinite-quantity contract such as an IDIQ contract, the agency must record an obligation in the amount of the required minimum purchase."**
+#### Legal Basis
+The obligation arises from FAR Clause 52.216-22 (Indefinite Quantity), which states:
+&gt; **"The Government *shall* order at least the quantity of supplies or services designated in the Schedule as the 'minimum.'"**
+GAO reasoned: *"By using the words 'shall order,' the contract indicates that under the contract the government is liable to the contractor for the minimum specified. It therefore incurs a legal liability for that amount. This is so whether the agency ever issues a task order to the contractor or not, and is so **immediately upon contract award**."*
+This legal liability triggers the Recording Statute (31 U.S.C. § 1501(a)), which requires agencies to record obligations when legal liability is incurred — i.e., **at contract award, not when task orders are placed**.
+#### What Customs Did Wrong
+| Date | What Should Have Happened | What Actually Happened |
+|---|---|---|
+| Feb. 11, 2003 (award) | Obligate $25,000,000 from FY 2003 funds | **No obligation recorded** |
+| Sept. 28, 2003 | Draw from pre-obligated minimum | Obligated only $45,000 from FY 2003 (far short) |
+| Nov. 2003–Sept. 2004 | Additional orders draw from FY 2003 obligation | Obligated $955,000 from **FY 2004** funds — **wrong fiscal year** |
+Customs's defense — that it had ultimately issued task orders exceeding the $25M minimum — was rejected by GAO as **irrelevant**:
+&gt; *"It is irrelevant that the minimum has been satisfied. The Recording Statute requires timely recording of obligations to ensure the integrity of obligational accounting records."*
+#### Consequences
+- The $955,000 charged to FY 2004 was charged to the **wrong fiscal year** (should have been FY 2003), violating 31 U.S.C. § 1502.
+- GAO directed Customs and DOD to **deobligate** $955,000 from FY 2004 and **re-obligate** it from FY 2003.
+- If insufficient FY 2003 funds were available, an **Antideficiency Act violation** (31 U.S.C. § 1341) would need to be reported.
+---
+### The Correct IDIQ Obligation Workflow (Per B-302358)
+```
+CONTRACT AWARD (Day 1):
+  → Obligate FULL minimum guarantee from fiscal year of award
+  → Legal liability exists regardless of whether any task orders are placed
+TASK ORDERS (Subsequent):
+  → Orders drawing down the minimum = no new obligation (already obligated)
+  → Once minimum is exhausted → each additional task order obligated
+    from the fiscal year the order is placed
+```
+---
+### Practical Takeaways for NIH Acquisitions
+1. **Obligate the minimum at award.** Do not wait for task orders to be finalized. The legal liability exists the moment the contract is signed.
+2. **Use the correct fiscal year.** The minimum must come from appropriations current at the time of contract award — not next year's funds.
+3. **Nominal minimums create real obligations.** Even a small guaranteed minimum (e.g., $250 on a GWAC like CIO-SP3) creates a recording statute obligation at award.
+4. **File content matters.** Mislabeled clauses (e.g., Clause 52.217-2 in an IDIQ file) do not change the legal character of the contract — substance controls.
+---
+### Related KB Document Also Retrieved
+**GAO B-321640** (`eagle-knowledge-base/approved/legal-counselor/appropriations-law/GAO_B-321640_ADA_Bonafide_Need_IDIQ.txt`) builds on B-302358 and adds a second requirement: the IDIQ minimum must not only be obligated at award — it must also reflect a **genuine bona fide need** at the time of obligation. SBA violated this in B-321640 by obligating $1.3M and $1.9M at fiscal year-end without issuing any task orders until the following year ("parking" funds).
+---
+### Sources
+| Document | S3 Key |
+|---|---|
+| **GAO B-302358** (primary) | `eagle-knowledge-base/approved/legal-counselor/appropriations-law/GAO_B-302358_IDIQ_Min_Fund.txt` |
+| **GAO B-321640** (companion) | `eagle-knowledge-base/approved/legal-counselor/appropriations-law/GAO_B-321640_ADA_Bonafide_Need_IDIQ.txt` |
+| **FAR 16.504** (IDIQ minimum requirement) | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt` |
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/proposal-guidance/GAO_B-413104.36_CTA_Accounting_System_Verification.txt`
+- `eagle-knowledge-base/approved/legal-counselor/case-law/consolidation/GAO_B-409528_Consolidation_Small_Business_Analysis_2014.txt`
+- `eagle-knowledge-base/approved/legal-counselor/case-law/consolidation/GAO_B-410074_Task_Order_Consolidation_Analysis.txt`
+- `eagle-knowledge-base/approved/legal-counselor/case-law/consolidation/GAO_B-417500_BPA_Consolidation_Analysis.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-409917_Failure_to_Rebut_Agency_Arguments.txt`
+- `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419831_PIA_Allegations_Interested_Party.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS10" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT10" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 provides full B-302358 case analysis (7,253 chars) including background, both holdings with detailed tables, the obligation workflow diagram, companion case B-321640, and practical NIH takeaways. Uses search_far + research instead of V11's legal_counsel subagent -- faster (59s vs 254.5s V11).
+v11 vs v12: Major improvement. V12 uses search_far + research (59s) vs V11's knowledge_search + knowledge_fetch + legal_counsel (254.5s). Same depth, 4.3x faster.
+Tools: v11=[knowledge_search, knowledge_fetch, legal_counsel] | v12=[search_far, research]
+KB docs cited: V11=3+ | V12=3 (direct KB access, fully transparent)
+Verdict: Tool simplification win -- same quality, much faster, transparent sources.</t>
         </is>
       </c>
     </row>
@@ -8506,6 +11587,464 @@
 Verdict: Exceptional -- most thorough appropriations response with edge cases.</t>
         </is>
       </c>
+      <c r="AY11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is a comprehensive breakdown of how the bona fide needs rule under **31 U.S.C. § 1502(a)** interacts with the severable/non-severable distinction for service contracts that cross fiscal years.
+---
+# The Bona Fide Needs Rule &amp; Severable vs. Non-Severable Services
+## I. The Statutory Foundation
+**31 U.S.C. § 1502(a)** states:
+&gt; *"The balance of an appropriation or fund limited for obligation to a definite period is available only for payment of expenses properly incurred during the period of availability or to complete contracts properly made within that period of availability."*
+The operative principle: an annual appropriation is available **only** for bona fide needs that arise **during** its period of availability (October 1 – September 30 for a given fiscal year). You cannot use FY 2025 funds for needs that arise in FY 2026, and vice versa.
+The bona fide needs rule is a **timing rule**. It controls both:
+1. **When** the obligation is recorded, and
+2. **Whether** a genuine need exists in that fiscal year.
+---
+## II. The Performance Period Rule for Services
+For supplies, the controlling event is the **delivery date**. For services, a different rule applies:
+&gt; **The bona fide need for services arises in the fiscal year in which the services are *performed*.**
+This is where the severable/non-severable distinction becomes the central analytical question.
+---
+## III. The Severable vs. Non-Severable Distinction
+The GAO's governing standard (GAO Red Book, Chapter 5):
+&gt; *"The question is whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."*
+### Non-Severable Services
+**Definition:** A single undertaking that cannot be feasibly separated into components without losing its essential character or value.
+**Key indicators:**
+- Produces a single end product or result
+- Tasks are interdependent and build toward a unified outcome
+- Cannot be logically divided by time period
+- Value derives only from complete performance
+**Examples:** Program evaluation with final report, system audit, architectural design, custom software development for a specific system, litigation representation, one-time training course, penetration test with report.
+**Funding consequence under § 1502(a):**
+The entire contract is the bona fide need of the **fiscal year in which the contract is entered**, regardless of how long performance takes. You may obligate the **full amount from one appropriation** even if performance extends into the following fiscal year.
+&gt; *Example: A $600,000 system audit contract awarded September 15, FY 2025, with final report due March 2026 — entire $600,000 obligated from FY 2025 funds. Permissible.*
+### Severable Services
+**Definition:** Recurring or continuing services where each unit (or time period) of service has independent value regardless of what comes before or after it.
+**Key indicators:**
+- Discrete, identifiable units of service
+- Each time period's output has standalone value
+- Services can be logically divided by time period
+- Performance in one period does not depend on another
+**Examples:** Help desk support, maintenance, guard services, grounds maintenance, systems administration, managed services, SaaS/database subscriptions, most ongoing IT O&amp;M.
+**Funding consequence under § 1502(a):**
+Each fiscal year's services are a **separate bona fide need** of that fiscal year. A single-year appropriation **cannot** fund services that fall in a different fiscal year. Incremental funding is **required** when the contract crosses a fiscal year boundary.
+&gt; *Example: A $1,200,000/year help desk contract ($100K/month) awarded October 1, FY 2025 through September 30, FY 2026 — must use FY 2025 funds for Oct–Dec 2025 ($300K) and FY 2026 funds for Jan–Sep 2026 ($900K). Funding the full 12 months from FY 2025 alone violates § 1502(a).*
+---
+## IV. The Interaction Matrix
+| Scenario | Severable? | § 1502(a) Rule | Funding Approach |
+|---|---|---|---|
+| Audit contract, Oct–Mar, awarded Sep | No | Need arises at award | Full obligation from award-year appropriation |
+| Help desk, Oct–Sep, awarded Oct | Yes | Need arises each month | Incremental: FY25 for Oct–Dec, FY26 for Jan–Sep |
+| Custom software build, Oct–Jun | No | Need arises at award | Full obligation from award-year appropriation |
+| Systems admin, Aug–Oct (bridge) | Yes | Short bridge exception | Full obligation from FY25 (1-month bridge) |
+| Option Year 2 services | N/A | Need arises in option year | Option exercised with funds current at exercise |
+| Agile dev to defined end state | No | Need arises at award | Full obligation from award-year appropriation |
+| Agile dev with no defined end | Yes | Need arises each period | Incremental funding required |
+---
+## V. The Short Bridge Exception (Severable Services Only)
+For severable services, an exception exists when a contract is awarded **near the end of a fiscal year** and performance extends a short period (typically **1–3 months**) into the next fiscal year — where the crossing is operationally necessary to avoid a gap in services.
+&gt; *Example: Contract for systems administration, August 1 – October 31, FY 2025/2026. The one-month October overlap into FY 2026 is a permissible short bridge. The full $150,000 may be obligated from FY 2025 funds.*
+The exception is narrow. It does not permit funding an entire base year or option year from a prior fiscal year's appropriation.
+---
+## VI. Option Years — A Critical Overlay
+Options are a distinct bona fide needs issue that sits on top of the severable/non-severable analysis:
+**Fundamental rule:** Each option period is a **separate bona fide need** of the fiscal year in which that option period falls.
+- Option Year 1 (Oct 2026–Sep 2027) → FY 2026 funds at exercise
+- Cannot exercise an FY 2026 option with FY 2025 funds simply to avoid losing FY 2025 money
+**Advance exercise exception:** A CO may exercise an option in the prior fiscal year using prior-year funds **if**:
+- Operational necessity requires advance notice (e.g., contractual 60-day notice requirement)
+- Exercise occurs close to the start of the option period (typically within ~90 days)
+- The purpose is not to circumvent the bona fide needs rule
+---
+## VII. Special Cases
+### Multiyear Contracts (FAR 17.1 / 41 U.S.C. § 254c)
+Not to be confused with multi-year performance contracts. Multiyear contracts are a **specific statutory authority** allowing obligation of up to 5 years of requirements from a current-year appropriation. They require:
+- Specific statutory authorization
+- Head of agency determination
+- A cancellation ceiling for termination liability
+These are the *exception*, not the rule.
+### No-Year / Multi-Year Appropriations
+When funded with **no-year funds** (available until expended) or **multi-year appropriations**, severable services contracts crossing fiscal years are **not subject to the one-year crossing restriction** — because the appropriation itself is not limited to a single fiscal year. The bona fide needs rule still applies (no speculative future needs), but incremental annual funding is not required.
+### Cost-Reimbursement Contracts
+Adding funds to a cost-reimbursement contract post-award has additional rules layered on top. The appropriation that funds an increase depends on whether the increase is:
+- **Antecedent liability** (cost overrun from original scope) → funded from original appropriation year
+- **Discretionary increase** (new or expanded work) → funded from the appropriation current at the time of modification
+---
+## VIII. Common Violations
+| Violation | What Went Wrong |
+|---|---|
+| FY25 funds obligated for FY26 recurring services | Severable services not incrementally funded |
+| Full-year SaaS subscription obligated from last month of FY25 | Severable subscription extends well into FY26 |
+| FY25 IDIQ minimum obligated, no task orders issued | "Parking" funds — no genuine bona fide need |
+| Option Year 2 exercised in prior FY to "use up" expiring funds | Circumvents bona fide needs rule |
+| Contract re-labeled "non-severable" to allow full-year funding | Severability is determined by the **nature of services**, not contract language |
+That last point bears emphasis: **you cannot manufacture non-severability through drafting.** GAO looks past the label to the actual character of the services.
+---
+## IX. Documentation Requirements
+The acquisition plan and contract file should explicitly address severability:
+**For non-severable services:**
+&gt; *"The services required under this acquisition constitute a non-severable undertaking. The contract will produce [specific deliverable] through interdependent tasks that cannot be meaningfully divided into discrete time periods. The entire contract value is obligated from FY [XXXX] appropriations in compliance with 31 U.S.C. § 1502(a)."*
+**For severable services:**
+&gt; *"The services required are severable, consisting of [recurring services] where each period's performance has independent value. Incremental funding will be applied: FY [XXXX] appropriations ($X) for services from [dates]; FY [XXXX+1] appropriations ($X) for services from [dates]."*
+---
+## X. The Five-Question Severability Checklist
+Before funding any service contract that crosses a fiscal year:
+1. **What is the primary deliverable?** Single product/report → likely non-severable. Ongoing outputs → likely severable.
+2. **Can the work be logically divided by time period?** If yes, severable.
+3. **Are the tasks interdependent?** If all tasks build toward one unified goal, non-severable.
+4. **Does each period's performance have standalone value?** If yes, severable.
+5. **What is the contract's purpose?** Accomplish a specific objective (non-severable) vs. provide ongoing capability (severable).
+---
+**Sources:**
+- 31 U.S.C. § 1502(a) — Period of availability (statutory authority)
+- GAO Red Book, Chapter 5: Availability of Appropriations: Time | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- Appropriations Law: Severable vs. Non-Severable Services (GAO Red Book Ch. 5) | `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- 2025 Contract Attorneys Deskbook, Chapter 4 (TJAGLCS) | `eagle-knowledge-base/approved/legal-counselor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt`
+- FAR 32.703-2, FAR 32.703-3, FAR 17.103 (FAR framework provisions)
+</t>
+        </is>
+      </c>
+      <c r="AZ11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD11" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE11" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: V10 provides comprehensive appropriations law response covering 10 sections: statutory foundation, performance period rule, severable/non-severable distinction, interaction matrix, short bridge, options, special cases, common violations, documentation requirements with template language, and five-question severability checklist.
+v9 vs v10: Comparable quality. Both use search_far + research.
+Tools: v9=[search_far, research] | v10=[search_far, research]
+KB docs cited: V9=5 | V10=6 (+1)
+Verdict: Stable -- comprehensive appropriations response maintained.</t>
+        </is>
+      </c>
+      <c r="BF11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is a thorough explanation of how the bona fide needs rule interacts with the severable/non-severable distinction for service contracts that cross fiscal years.
+---
+# The Bona Fide Needs Rule &amp; Severable vs. Non-Severable Services
+## I. The Statutory Foundation — 31 U.S.C. § 1502(a)
+The **bona fide needs rule** derives from the period of availability statute:
+&gt; *"The balance of an appropriation or fund limited for obligation to a definite period is available only for payment of expenses properly incurred during the period of availability or to complete contracts properly made within that period of availability."*
+In plain terms: **FY 2025 appropriations may only fund FY 2025 needs.** You cannot obligate current-year funds for requirements that genuinely arise in a future year, nor use future-year funds for requirements that arose in the current year.
+The rule exists to enforce congressional control over the appropriations process — it prevents agencies from "parking" funds, stockpiling, or circumventing annual appropriations cycles.
+---
+## II. The Central Question for Service Contracts: *When Does the Need Arise?*
+For **supplies**, the rule is relatively simple: the need arises in the fiscal year in which delivery is required (the *delivery date rule*).
+For **services**, it is more complex. The need arises in the fiscal year in which services are *performed* — but what "fiscal year's services" means depends entirely on whether the services are **severable or non-severable**. This distinction is the pivotal appropriations law question for any service contract that crosses a fiscal year boundary.
+---
+## III. The Severable/Non-Severable Distinction
+### Non-Severable Services — The "Single Undertaking" Rule
+**Definition:** Services that constitute a *single undertaking* — the tasks are interdependent, build toward a unified outcome, and cannot be meaningfully divided into discrete time periods without losing essential character or value.
+**GAO Standard:** *"The question is whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."*
+**Indicators of non-severability:**
+- Single end product or deliverable (report, audit opinion, completed system)
+- Tasks in early phases are prerequisites for later phases
+- Value derives only from complete performance, not from incremental portions
+- Time periods are arbitrary scheduling milestones, not independent scopes
+**Common examples:** feasibility studies, financial audits, litigation support, custom software development toward a defined system, A/E design for a specific project, a specific training course.
+**Appropriations law consequence:** The *entire* contract is the bona fide need of the fiscal year in which the contract is *entered*. You may fully obligate the contract from the appropriation current at award, even if performance extends well into a subsequent fiscal year.
+&gt; **Example:** A $600,000 program evaluation contract is awarded September 15, FY2025. Work begins October 1, FY2025; the final report is due March 31, FY2026. → Obligate the full $600,000 from FY2025 funds. The entire study is a single undertaking and a bona fide FY2025 need. No incremental funding required.
+---
+### Severable Services — The "Performance Period" Rule
+**Definition:** Services that are *recurring or continuing* in nature, where each unit of service (day, week, month) has independent value regardless of other periods' performance.
+**Indicators of severability:**
+- Discrete, repetitive tasks that repeat on a regular schedule
+- Each time period's services stand alone — the value of October's services is not diminished by canceling November's
+- The work could logically be divided and awarded to different contractors for different periods
+- There is no single unified end product
+**Common examples:** help desk support, facilities maintenance, janitorial services, security guard coverage, systems administration/monitoring, subscriptions/SaaS licenses, ongoing IT O&amp;M.
+**Appropriations law consequence:** Each fiscal year's services are a *separate* bona fide need of that fiscal year. You **cannot** fund FY2026 services with FY2025 funds. If the contract crosses fiscal years, it must be **incrementally funded** — each year's appropriation funds that year's services.
+&gt; **Example:** A $1,200,000 help desk support contract runs October 1, FY2025 – September 30, FY2026 (12 months, $100,000/month). The contract is awarded September 15, FY2025.
+&gt; - **FY2025 funds:** $300,000 for October–December 2025 (3 months)
+&gt; - **FY2026 funds:** $900,000 for January–September 2026 (9 months)
+&gt; - Cannot obligate the full $1,200,000 from FY2025 appropriations. To do so would improperly fund FY2026 bona fide needs with FY2025 money.
+---
+## IV. The Time-Based Rules: How the Calendar Interacts
+### Rule 1 — The Standard Performance Period Rule
+Each fiscal year's services are a separate bona fide need. Fund proportionally. This is the default for all severable services crossing fiscal years.
+### Rule 2 — The Short Bridge Exception
+An agency may obligate funds near the *end* of a fiscal year for a severable services contract that crosses into the next fiscal year by a **short period** (typically 1–3 months), provided:
+- The bridge is necessary to avoid a gap in service delivery
+- The crossing period is minimal (not the majority of performance)
+- Operational necessity is documented
+&gt; **Example:** A 3-month bridge contract runs August 1 – October 31, FY2025/FY2026. Even though one month falls in FY2026, the entire $150,000 may be funded from FY2025 appropriations. The 1-month bridge is an acceptable, administratively reasonable exception.
+### Rule 3 — The Lead Time Exception (Supplies, Applies by Analogy)
+For supplies with long procurement lead times extending beyond fiscal year end, current-year funds may be obligated if the need genuinely arises in the current year even though delivery falls in a future year. This applies to service contracts in limited circumstances where set-up or mobilization time makes advance contracting necessary.
+### Rule 4 — Option Year Rule
+Each option period is a **separate bona fide need** funded from the appropriation current when that option period is performed — not from the base year appropriation.
+- Base year → FY2025 funds
+- Option Year 1 (FY2026 performance) → FY2026 funds when exercised
+- Cannot use FY2025 funds to exercise FY2026 options merely to avoid losing year-end money
+**Advance exercise exception:** A CO may exercise an option period using prior-year funds if *operational necessity* requires advance notice (e.g., 60-day contract notice requirement), the exercise occurs close to the option start (typically within 90 days), and the advance exercise is documented and not motivated by fund expiration.
+---
+## V. Critical Interaction: Severability Is Determined by *Nature*, Not Contract Language
+A recurring and dangerous error: **you cannot write a severable service contract into a non-severable one to simplify funding.** Severability is an appropriations law determination based on the actual character of the services, not on how the SOW is drafted or what the parties call it. GAO will look through the label to the substance.
+Similarly, crossing fiscal years does not *make* a contract severable. A non-severable study contract lasting 18 months is still properly funded entirely from the appropriation current at award.
+---
+## VI. Practical Funding Matrix
+| Scenario | Severable? | Cross FY? | Funding Rule |
+|---|---|---|---|
+| Program evaluation, 9-month PoP, single report | No | Yes | Full obligation at award from FY of award |
+| Help desk support, 12-month PoP | Yes | Yes | Incremental: each FY funds its own services |
+| 3-month bridge contract, 1 month in next FY | Yes | Yes (briefly) | Full obligation from current FY (short bridge exception) |
+| Option Year 1 exercise for IT O&amp;M | Yes | New FY | Must use new FY appropriation when exercised |
+| Custom software development, 18-month PoP | No | Yes | Full obligation at award from FY of award |
+| SOC monitoring, 12-month contract | Yes | Yes | Incremental by FY |
+| Penetration test with final report | No | Maybe | Full obligation at award |
+| Agile dev sprints toward defined system | No | Likely | Full obligation at award (single undertaking) |
+| Ongoing SaaS subscription, annual renewal | Yes | No* | Fund each renewal with current FY appropriation |
+---
+## VII. Contract Structure and Required FAR Clauses
+**For non-severable services** crossing fiscal years:
+- Standard funding clauses are sufficient
+- No incremental funding clause required
+- Acquisition plan should document the non-severability rationale
+**For severable services** crossing fiscal years, include:
+- **FAR 52.232-19** — Availability of Funds for the Next Fiscal Year *(used in fixed-price severable service contracts that cross FY)*
+- **FAR 52.232-22** — Limitation of Funds *(cost-reimbursement, incrementally funded)*
+- **FAR 52.232-20** — Limitation of Cost *(fully funded cost-reimbursement)*
+- **FAR 32.703-2** — general authority for contracts crossing fiscal years
+---
+## VIII. Required Acquisition Plan Documentation
+**For non-severable services:**
+&gt; *"The services under this acquisition constitute a non-severable undertaking. The contract will produce [specific deliverable] through interdependent tasks that cannot be meaningfully divided into discrete time periods. The entire contract value of $[X] will be obligated from FY[XXXX] appropriations. Performance extending into FY[XXXX+1] is permissible because the entire undertaking represents a bona fide need of FY[XXXX] when the contract is entered."*
+**For severable services:**
+&gt; *"The services under this acquisition are severable in nature — recurring [type of services] where each period's performance has independent value. The contract crosses fiscal year boundaries and will be incrementally funded: FY[XXXX] appropriations $[amount] for services [dates]; FY[XXXX+1] appropriations $[amount] for services [dates]. This approach matches each fiscal year's appropriation to that year's bona fide needs per 31 U.S.C. § 1502(a)."*
+---
+## IX. Common Violations to Avoid
+| Violation | What Happens | Prevention |
+|---|---|---|
+| Using FY25 funds for full 12-month severable contract when 9 months fall in FY26 | Antideficiency Act exposure; improper obligation | Incremental funding; proportional split |
+| Characterizing severable services as non-severable in SOW language | GAO looks through the label to the substance | Honest severability analysis |
+| Exercising FY26 option with FY25 funds to avoid year-end fund expiration | Bona fide needs violation | Use FY26 funds; advance exercise only for operational necessity |
+| IDIQ minimum "parked" in September with no current-year task orders planned | Parking funds violation per GAO B-321640 | Award IDIQ only when genuine current-year need exists |
+| End-of-year award of severable 12-month contract entirely funded from expiring appropriation | Bona fide needs violation for months falling in next FY | Short bridge exception applies to 1–3 months only |
+---
+## X. The No-Year / Multi-Year Appropriation Exception
+If the contract is funded by a **no-year appropriation** (available until expended) or a **multi-year appropriation** (available for a defined period longer than one year, per 41 U.S.C. § 254c), the fiscal-year crossing restriction on severable services does not apply in the same way — the single appropriation is already available for the full performance period. The bona fide needs rule still applies (cannot obligate for speculative future needs), but the annual fiscal year matching requirement is relaxed.
+---
+**Sources:**
+- 31 U.S.C. § 1502(a) — Period of Availability Statute
+- GAO Red Book, Chapter 5: Availability of Appropriations: Time (GAO-04-261SP)
+- GAO Decision B-321640 (Sep. 19, 2011) — SBA IDIQ parking violation
+- GAO Decision B-329061 (Feb. 25, 2009) — Bona fide needs general principles
+- FAR 32.703-2 — Contracts Crossing Fiscal Years
+- FAR 52.232-19, 52.232-20, 52.232-22
+- KB: `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- KB: `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+**Sources:**
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_IDIQ_funding.txt`
+</t>
+        </is>
+      </c>
+      <c r="BG11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK11" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL11" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 provides comprehensive bona fide needs analysis (12,541 chars) covering statutory foundation, severable/non-severable distinction, GAO standards, interaction rules, special cases, and practical checklists. Longest appropriations response in suite.
+v10 vs v11: V11 richer (12,541 vs 10,588 chars). Both use search_far + research.
+Tools: v10=[search_far, research] | v11=[search_far, research]
+KB docs cited: V10=6 | V11=6+ (research + search_far auto-fetch)
+Verdict: Strongest appropriations response in suite -- comprehensive and actionable.</t>
+        </is>
+      </c>
+      <c r="BM11" s="20" t="inlineStr">
+        <is>
+          <t>ERROR: All connection attempts failed</t>
+        </is>
+      </c>
+      <c r="BN11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here is a comprehensive, authoritative breakdown of how the bona fide needs rule under **31 U.S.C. § 1502(a)** interacts with the severable/non-severable distinction for service contracts crossing fiscal years.
+---
+# The Bona Fide Needs Rule and Severable vs. Non-Severable Services
+## I. THE STATUTORY ANCHOR: 31 U.S.C. § 1502(a)
+&gt; *"The balance of an appropriation or fund limited for obligation to a definite period is available only for payment of expenses properly incurred during the period of availability or to complete contracts properly made within that period of availability."*
+This is the **time dimension** of appropriations law. It works alongside:
+- **31 U.S.C. § 1301** (Purpose Statute — *what* funds can pay for)
+- **31 U.S.C. §§ 1341–1342** (Antideficiency Act — *how much*)
+The bona fide needs rule is the practical expression of § 1502(a): an agency may only obligate a current-year appropriation for needs that **genuinely arise** during that appropriation's period of availability. It prevents "parking" funds, stockpiling, and circumventing Congress's annual control over the purse.
+&gt; ⚠️ **Critical threshold point:** § 1502(a) applies *only* to appropriations **limited to a definite period** (annual appropriations). It does not apply to no-year or multi-year appropriations — a point that drives the statutory exceptions discussed below.
+---
+## II. HOW THE NEED "ARISES" FOR SERVICES
+For services, the bona fide need arises **when the services are performed**, not when the contract is awarded. This is the **performance period rule**.
+But this rule bifurcates entirely based on whether the services are **severable or non-severable**. These two categories carry fundamentally different obligation rules.
+---
+## III. THE SEVERABLE / NON-SEVERABLE DISTINCTION
+### A. Non-Severable Services — The "Single Undertaking" Doctrine
+**Legal Standard (GAO):**
+&gt; *"The question is whether the contract is essentially for a single undertaking or job, or whether it may reasonably be said to envision a series of separate tasks."*
+Non-severable services produce a **single end product** through interdependent tasks that cannot be meaningfully divided into discrete time periods. The **value derives from complete performance**, not from any individual increment.
+**Hallmarks:**
+| Factor | Non-Severable Indicator |
+|---|---|
+| Primary deliverable | Single report, system, audit opinion, or outcome |
+| Task interdependence | Phases build toward unified result |
+| Time divisibility | Cannot logically split by period without losing value |
+| Purpose | Accomplish specific objective |
+**Common examples:** feasibility studies, system audits, custom software development, litigation support for a specific case, program evaluations, A/E design for a specific facility, specific training courses.
+**Funding rule for non-severable services crossing fiscal years:**
+The entire contract is a **bona fide need of the fiscal year in which the contract is entered**. You **may** obligate the full contract value from the appropriation current at award, even if performance extends well into the next fiscal year.
+&gt; ✅ **Example:** Study contract awarded September 15, 2025 (FY25) for $500K. Work begins October 2025; final report due March 2026.
+&gt; → Obligate entire $500K from FY25 appropriations. Performance spanning FY26 is permissible. The single undertaking is the bona fide need of FY25.
+**GAO precedent — B-317139 (FinCEN, June 1, 2009):** FinCEN's BSA Direct system development contract was non-severable because it called for delivery of a defined end-product system that "could not feasibly be subdivided for separate performance by fiscal year." The agency was required to obligate the full estimated cost of **$8,982,985** at FY04 award — not incrementally across fiscal years. By obligating only $2M at award, FinCEN violated the bona fide needs rule.
+&gt; ⛔ **Critical error to avoid:** You **cannot** incrementally fund a non-severable contract merely because you lack current-year funds. For cost-reimbursement non-severable contracts, FAR 16.301-1 requires establishing an obligation equal to the estimated total cost ceiling at award.
+---
+### B. Severable Services — The Fiscal Year Matching Rule
+Severable services are **recurring or continuing** in nature. Each period's services have **independent value** — the services in October stand alone from those in November. Performance in one period does not depend on another.
+**Hallmarks:**
+| Factor | Severable Indicator |
+|---|---|
+| Primary deliverable | Ongoing services or recurring outputs |
+| Task interdependence | Independent, repetitive tasks |
+| Time divisibility | Can logically divide by time periods |
+| Purpose | Provide ongoing capability |
+**Common examples:** help desk support, maintenance services, janitorial/guard services, systems administration, SOC monitoring, database subscriptions/SaaS licenses, administrative support.
+**Funding rule for severable services crossing fiscal years:**
+Each fiscal year's services are a **separate bona fide need** of that fiscal year. You **must** fund each year's services with that year's appropriation. You **cannot** use FY25 funds to pay for FY26 services.
+&gt; ✅ **Example:** IT help desk contract, October 1, 2025 – September 30, 2026, at $100K/month ($1.2M total).
+&gt; - FY25 funds: $300K (October–December 2025 = 3 months in FY25)
+&gt; - FY26 funds: $900K (January–September 2026 = 9 months in FY26)
+&gt; → **Cannot** obligate the full $1.2M from FY25 appropriations.
+This **incremental funding** requirement for severable services is mandatory when the contract crosses fiscal year boundaries — it is not optional.
+---
+## IV. THE STATUTORY EXCEPTION FOR SEVERABLE SERVICES — 41 U.S.C. § 253l (Civilian) / 10 U.S.C. § 2410a (DoD)
+Congress recognized that the strict fiscal-year-matching rule created enormous administrative burdens (COs had to modify every service contract at FY end to add new-year funding). These statutes create a **limited exception**:
+&gt; An agency may enter into a severable services contract that **begins in one fiscal year and ends no more than 12 months later**, and **obligate the total contract amount to the first fiscal year's appropriation** — even though performance crosses into the next fiscal year.
+**Key conditions:**
+- The crossing cannot exceed 12 months total contract performance
+- This is a **statutory exception to the bona fide needs rule** — it permits FY25 funds to be used for services that technically constitute a FY26 need, but only within the 12-month window
+- **FAR 37.106(a)** and **FAR 32.703-3(a)** implement these statutes, and both expressly state they apply only to contracts "funded by annual appropriations"
+**GAO B-317636 (April 21, 2009)** is the controlling decision: no-year and multi-year appropriations are **not** subject to the 12-month restriction. Agencies using those fund types may contract for the full period of availability the statute allows, because § 1502(a) simply doesn't apply to open-ended appropriations.
+&gt; ✅ **Practical use of the exception:** Award a 12-month IT support contract starting August 1, 2025 (ending July 31, 2026) and fund the entire amount from FY25 appropriations under the statutory exception — even though 10 months of performance falls in FY26.
+---
+## V. THE SHORT BRIDGE EXCEPTION (Administrative)
+Separate from the statutory exception above, GAO has recognized a narrower **short bridge** principle: an agency may fund a brief bridge period of severable services crossing into the next fiscal year (typically 1–3 months) entirely with the prior year's appropriation, provided:
+- The bridge is necessary to avoid a gap in critical services
+- The bridge period is minimal
+- Operational necessity is documented
+&gt; ✅ **Example:** Award a 3-month bridge contract on August 1, 2025 for systems administration through October 31, 2025 (one month in FY26). Entire $150K may be funded from FY25 appropriations.
+This is a **narrower** administrative exception and does not substitute for the statutory 12-month exception above.
+---
+## VI. THE TIME-BASED BONA FIDE NEEDS RULES SUMMARIZED
+| Acquisition Type | When Need Arises | Crosses FY? | Funding Rule |
+|---|---|---|---|
+| **Supplies** | Delivery date | N/A | Fund from FY when delivery occurs (lead-time exception for long-lead items) |
+| **Non-severable services** | When contract entered | Yes — permitted | Fully fund from FY of award; no incremental funding required or permitted for the base obligation |
+| **Severable services (annual funds)** | When services performed | Yes — incremental funding required | Each FY's services funded with that FY's appropriation |
+| **Severable services (§ 253l/2410a exception)** | FY of contract start | Yes — up to 12 months | May fully fund from start-year appropriation |
+| **Severable services (no-year / multi-year funds)** | N/A (§ 1502(a) inapplicable) | Yes — no restriction | Fund from available appropriation for full performance period |
+| **Construction** | When work performed | Yes — often incremental | Multi-year appropriations or incremental funding typically required |
+---
+## VII. OPTIONS — THE RECURRING BONA FIDE NEEDS TRAP
+Option periods interact with this framework in a way that catches many agencies:
+- **Each option period is a separate bona fide need** requiring funding from the fiscal year when that option period will be performed.
+- Options are **not** obligated at base award; obligation occurs when the option is exercised.
+- You **cannot** use FY25 funds to exercise an FY26 option merely to avoid losing FY25 money. Doing so is a bona fide needs violation.
+**Advance exercise exception:** You *may* exercise an FY26 option in FY25 (using FY25 funds) if:
+- Operational necessity requires advance notice (e.g., a 60-day notice clause)
+- The exercise occurs close to the start of the option period (typically within 90 days)
+- It is not a pretext to park expiring funds
+&gt; ✅ **Example:** 60-day notice clause on an IT support contract. Option period begins October 1, 2026. CO may exercise in late July 2026 using FY26 funds to avoid a gap — this is proper. Exercising in June 2025 using FY25 funds to "use them up" is a violation.
+---
+## VIII. COMMON VIOLATIONS
+| Violation | What Happened | Why It's Wrong |
+|---|---|---|
+| FY25 funds for FY26 severable services | Help desk contract FY-year funded entirely from FY25 | Each FY's services are a separate bona fide need |
+| Non-severable contract incrementally funded | Study contract funded in pieces across 3 FYs | Entire undertaking is FY of award's bona fide need; must fully obligate at award |
+| IDIQ minimum "parking" | $1.9M minimum obligated FY10, no task orders until FY11 (SBA, B-321640) | No genuine current-year need at time of obligation |
+| Advance option exercise to park funds | FY26 option exercised in August 2025 to use expiring FY25 funds | No operational necessity; circumvents annual appropriations process |
+| Contract language creating false non-severability | SOW drafted to appear non-severable for ongoing O&amp;M services | Severability is determined by the nature of services, not contract language |
+---
+## IX. FAR CLAUSES THAT IMPLEMENT THESE RULES
+| Clause | Context |
+|---|---|
+| **FAR 52.232-22** (Limitation of Funds) | Required for incrementally funded cost-reimbursement contracts; contractor notifies CO at 75% of funded amount |
+| **FAR 52.232-20** (Limitation of Cost) | Fully funded cost-reimbursement ceiling |
+| **FAR 52.232-19** (Availability of Funds for Next FY) | Fixed-price severable services crossing FY |
+| **FAR 37.106(a)** | Implements 41 U.S.C. § 253l — severable services crossing FY with annual funds, up to 12 months |
+| **FAR 32.703-3** | Contracts crossing fiscal years — applicability to annual appropriations only |
+| **FAR 17.207** | Option exercise — CO must determine continued need, performance acceptability, and fund availability |
+---
+## X. DOCUMENTATION REQUIREMENT
+Every acquisition plan for a cross-FY service contract must include a severability determination. Standard language:
+**Non-severable:**
+&gt; *"The services constitute a non-severable undertaking. The contract will produce [specific deliverable] through interdependent tasks that cannot be meaningfully divided into discrete time periods. The entire contract value of $[X] will be obligated from FY [XXXX] appropriations. This complies with the bona fide needs rule because the entire undertaking is a bona fide need of FY [XXXX]."*
+**Severable:**
+&gt; *"The services are severable, consisting of recurring [service type] where each period's performance has independent value. Incremental funding is required: FY[XXXX] appropriations: $[amount] for services [dates]; FY[XXXX+1] appropriations: $[amount] for services [dates]. This matches each fiscal year's appropriation to that year's services."*
+---
+### Sources
+- **31 U.S.C. § 1502(a)** — Period of availability (time statute)
+- **41 U.S.C. § 253l / 10 U.S.C. § 2410a** — Severable services statutory exception
+- **GAO Red Book, Chapter 5** — Availability of Appropriations: Time (GAO-04-261SP)
+- **GAO B-317636** (Apr. 21, 2009) — Severable services / no-year appropriations
+- **GAO B-317139** (June 1, 2009) — FinCEN non-severable contract incremental funding violation
+- **GAO B-321640** (Sep. 19, 2011) — SBA IDIQ parking funds violation
+- **2025 Contract Attorneys Deskbook, Chapter 4** — JAG School, TJAGLCS
+- **FAR 37.106, 32.703-3, 17.207, 52.232-22**
+- KB: `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_time_bona_fide_needs.txt`
+- KB: `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_severable_services.txt`
+- KB: `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Contract_Obligation_Timing_GAO_Guidance.txt`
+**Sources:**
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_IDIQ_funding.txt`
+- `eagle-knowledge-base/approved/financial-advisor/appropriations-law/appropriations_law_incremental_funding.txt`
+- `eagle-knowledge-base/approved/legal-counselor/appropriations-law/Army_Contract_Attorneys_Deskbook_2025_Chapter_4_Appropriations_Law_Summary.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR11" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS11" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT11" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 provides comprehensive bona fide needs analysis (14,393 chars) covering statutory foundation, severable/non-severable distinction with detailed tables, statutory exception (41 USC 253l), short bridge exception, options trap, common violations table, FAR clauses, and documentation templates.
+v11 vs v12: V12 longer (14,393 vs 12,541 chars V11). Uses search_far + research (same pattern). Adds violation examples table and required AP language templates.
+Tools: v11=[search_far, research] | v12=[search_far, research]
+KB docs cited: V11=6+ | V12=4+ (research + search_far auto-fetch)
+Verdict: Strongest appropriations response in V12 suite -- comprehensive and actionable.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="409.5" customHeight="1">
       <c r="A12" s="20" t="n">
@@ -8692,6 +12231,207 @@
 Cascade: search_far -&gt; knowledge_fetch -- standard regulatory lookup.
 KB docs cited: V9=1 (FAR_Part_16_IDIQ_Comprehensive_RFO_2025)
 Verdict: Strong regulatory response -- verbatim text adds value. Sources adequate.</t>
+        </is>
+      </c>
+      <c r="AY12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are all **seven exceptions to the fair opportunity requirement** under **FAR 16.505(b)(2)(i)**, cited exactly from the authoritative source text:
+---
+## Exceptions to Fair Opportunity — FAR 16.505(b)(2)(i)(A)–(G)
+&gt; **Basis:** For multiple-award IDIQ contracts, a contracting officer must provide each awardee a fair opportunity to be considered for each order exceeding the micro-purchase threshold — **unless one of the following seven exceptions applies.** These exceptions permit sole-source placement of an order or BPA. Orders exceeding the SAT require a written justification; approval thresholds apply at $900K / $20M / $90M.
+---
+### **(A) — Urgency** | FAR 16.505(b)(2)(i)(A)
+The agency need for the supplies or services is **so urgent** that providing a fair opportunity would result in **unacceptable delays**.
+&gt; *Note: For urgency orders, the J&amp;A must be posted within **30 days** after award (rather than the standard 14 days).*
+---
+### **(B) — Unique or Highly Specialized** | FAR 16.505(b)(2)(i)(B)
+**Only one awardee is capable** of providing the supplies or services required at the level of quality required because the supplies or services ordered are **unique or highly specialized**.
+---
+### **(C) — Logical Follow-On** | FAR 16.505(b)(2)(i)(C)
+The order must be issued on a sole-source basis in the interest of **economy and efficiency** because it is a **logical follow-on** to an order already issued under the contract, provided that all awardees were given a fair opportunity to be considered for the original order.
+&gt; *Note: The justification must describe why the relationship between the initial order and the follow-on is logical — in terms of scope, period of performance, or value.*
+---
+### **(D) — Minimum Guarantee** | FAR 16.505(b)(2)(i)(D)
+It is necessary to place an order to **satisfy a minimum guarantee** under the contract.
+---
+### **(E) — Statutory Authorization** | FAR 16.505(b)(2)(i)(E)
+For orders **exceeding the SAT**, a **statute expressly authorizes or requires** that the purchase be made from a specified source.
+---
+### **(F) — Small Business Set-Asides** | FAR 16.505(b)(2)(i)(F)
+Under **FAR Part 19** and **Public Law 111-240 (15 U.S.C. 644(r))**, a contracting officer may **set aside orders for small business concerns** under multiple-award contracts, or place orders under reserves established for small businesses.
+&gt; **Critical distinction:** This exception is **not subject to** the justification, approval, and posting requirements that apply to exceptions (A)–(E) and (G). Small business set-asides and reserves operate under Part 19 authority, not as a traditional sole-source justification.
+---
+### **(G) — DoD/NASA/Coast Guard OTFAOC** | FAR 16.505(b)(2)(i)(G)
+Applicable **only to DoD, NASA, and the Coast Guard**: the order satisfies one of the exceptions permitting the use of **other than full and open competition** listed in **FAR Part 6** (10 U.S.C. 3406(c)(5)).
+&gt; *Note: The public interest exception under this subparagraph may not be used unless Congress is notified in accordance with 10 U.S.C. 3204(a)(7).*
+---
+## Approval Levels for Exceptions (A)–(E) and (G)
+| Order Value | Approval Authority |
+|---|---|
+| Above SAT, ≤ $900K | Contracting Officer certification |
+| &gt; $900K – $20M | Advocate for Competition (non-delegable) |
+| &gt; $20M – $90M | Head of Procuring Activity (or SES/flag officer) |
+| &gt; $90M | Senior Procurement Executive (non-delegable) |
+*(DoD/NASA/Coast Guard thresholds: $150M substitutes for $90M at the top tier.)*
+---
+**Source:** FAR Part 16, Subpart 16.5 — *FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt* (HHS Class Deviation 2026-01, effective November 21, 2025 for HHS). All seven exceptions cited to standard FAR 16.505(b)(2)(i)(A)–(G) numbering per the RFO-to-standard-FAR cross-reference table in the same document.
+</t>
+        </is>
+      </c>
+      <c r="AZ12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB12" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BC12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD12" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="BE12" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 = RO (comparable)
+RO comparison: Both list all 7 FAR 16.505(b)(2)(i) exceptions with verbatim text and exact paragraph citations. V10 includes approval levels table.
+v9 vs v10: Comparable. V10 cites 1 KB path (FAR_Part_16_IDIQ) -- same as V9.
+Tools: v9=[search_far, knowledge_fetch] | v10=[search_far, knowledge_fetch]
+KB docs cited: V9=1 | V10=1 (maintained)
+Source gap: RO cites FAR_Part_16_Contract_Types_Comprehensive -- V10 does not.
+Verdict: Strong regulatory response -- verbatim text accurate.</t>
+        </is>
+      </c>
+      <c r="BF12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are all **seven exceptions** to the fair opportunity requirement for task and delivery orders under multiple-award IDIQ contracts, per **FAR 16.505(b)(2)(i)(A)–(G)**:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity
+| # | FAR Citation | Exception | Key Notes |
+|---|---|---|---|
+| A | **FAR 16.505(b)(2)(i)(A)** | **Urgency** | The agency need is so urgent that providing fair opportunity would result in unacceptable delays. |
+| B | **FAR 16.505(b)(2)(i)(B)** | **Unique / Highly Specialized** | Only one awardee is capable of providing the supplies or services at the level of quality required because they are unique or highly specialized. |
+| C | **FAR 16.505(b)(2)(i)(C)** | **Logical Follow-On** | The order must be placed sole-source in the interest of economy and efficiency because it is a logical follow-on to an order already issued under the contract — provided all awardees had fair opportunity on the original order. |
+| D | **FAR 16.505(b)(2)(i)(D)** | **Minimum Guarantee** | It is necessary to place the order with a particular awardee to satisfy the contract's minimum guarantee. |
+| E | **FAR 16.505(b)(2)(i)(E)** | **Statutory Authorization** | For orders exceeding the SAT, a statute expressly authorizes or requires the purchase from a specified source. |
+| F | **FAR 16.505(b)(2)(i)(F)** | **Small Business Set-Aside** | Per FAR Part 19 and Pub. L. 111-240 (15 U.S.C. 644(r)), the contracting officer may set aside orders for small business concerns under multiple-award contracts. **Not subject** to the justification, approval, and posting requirements that apply to exceptions A–E and G. |
+| G | **FAR 16.505(b)(2)(i)(G)** | **DoD / NASA / Coast Guard — Other Than Full and Open Competition (OTFAOC)** | Applies only to DoD, NASA, and Coast Guard. The order satisfies one of the exceptions permitting other than full and open competition listed in FAR Part 6.103 (10 U.S.C. 3406(c)(5)). The public interest exception under this authority requires Congressional notification per 10 U.S.C. 3204(a)(7). |
+---
+## Key Procedural Points
+**Justification &amp; Approval (J&amp;A) thresholds** for exceptions A–E and G (sole source orders above the SAT):
+| Order Value | Approval Authority |
+|---|---|
+| Above MPT, at or below SAT | CO documents basis in file; no formal J&amp;A required |
+| Above SAT – $900K | CO certification sufficient (no separate approver required) |
+| $900K – $20M | Advocate for Competition (non-delegable) |
+| $20M – $90M ($150M DoD) | Head of Procuring Activity or SES/General Officer |
+| Above $90M ($150M DoD) | Senior Procurement Executive (non-delegable) |
+**Posting:** Within **14 days** of award (30 days for urgency exception A), post the justification to SAM.gov for a minimum of 30 days.
+**Exception F is categorically different:** Small business set-aside orders under FAR 19 and 15 U.S.C. 644(r) are **not subject** to the J&amp;A, approval, or posting requirements. This is why Exception (F) appears as a separate provision in the regulation rather than in the numbered list — it is a policy authorization, not a sole-source exception.
+---
+**Source:** FAR Part 16, Subpart 16.5 — *Ordering: Fair Opportunity and Exceptions* (`eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`), incorporating HHS Class Deviation 2026-01 / RFO cross-reference table confirming 7 exceptions at FAR 16.505(b)(2)(i)(A)–(G).
+</t>
+        </is>
+      </c>
+      <c r="BG12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK12" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL12" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 lists all 7 FAR 16.505(b)(2)(i) exceptions with full citation format (A-G), verbatim statutory text, and documentation/approval requirements table by dollar threshold. Includes DoD/NASA/Coast Guard OTFAOC exception.
+v10 vs v11: Comparable quality. V11 slightly shorter (3,430 vs 3,851) but equally complete.
+Tools: v10=[search_far, knowledge_fetch] | v11=[search_far, knowledge_fetch]
+KB docs cited: V10=1 | V11=1 (maintained)
+Verdict: Stable -- verbatim FAR text with approval thresholds.</t>
+        </is>
+      </c>
+      <c r="BM12" s="20" t="inlineStr">
+        <is>
+          <t>ERROR: All connection attempts failed</t>
+        </is>
+      </c>
+      <c r="BN12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Here are all **seven exceptions to the fair opportunity requirement** under **FAR 16.505(b)(2)(i)**, subparagraphs **(A) through (G)**:
+---
+## FAR 16.505(b)(2)(i) — Exceptions to Fair Opportunity for Task/Delivery Orders
+&gt; Applies to orders placed against multiple-award IDIQ contracts exceeding the micro-purchase threshold.
+---
+### (A) — Urgency | FAR 16.505(b)(2)(i)(A)
+The agency need is **so urgent** that providing fair opportunity would result in unacceptable delays. The contracting officer must document that the urgency was not the result of a lack of advance planning.
+---
+### (B) — Unique / Highly Specialized Capability | FAR 16.505(b)(2)(i)(B)
+**Only one awardee** is capable of providing the supplies or services at the level of quality required because the supplies or services are **unique or highly specialized**. The CO must document why no other contract holder can meet the need.
+---
+### (C) — Logical Follow-On | FAR 16.505(b)(2)(i)(C)
+The order must be issued on a sole-source basis in the **interest of economy and efficiency** because it is a **logical follow-on to an order already issued** under the contract — provided that all awardees were given a fair opportunity to be considered for the original order.
+---
+### (D) — Minimum Guarantee | FAR 16.505(b)(2)(i)(D)
+It is **necessary to place the order with a particular awardee** to satisfy the **minimum guarantee** quantity established at contract award.
+---
+### (E) — Statutory Authorization | FAR 16.505(b)(2)(i)(E)
+A **statute expressly authorizes or requires** that the purchase be made from a specified source (e.g., mandatory sources under FAR Part 8, AbilityOne, etc.).
+---
+### (F) — Small Business Set-Aside | FAR 16.505(b)(2)(i)(F)
+In accordance with **FAR Part 19**, the contracting officer may **set aside orders for small business concerns** (including specific socioeconomic categories: 8(a), HUBZone, SDVOSB, WOSB) under multiple-award contracts. This exception permits bypassing fair opportunity among all awardees when the order is reserved for small business participants.
+---
+### (G) — DoD/NASA/Coast Guard OTFAOC | FAR 16.505(b)(2)(i)(G)
+**Limited to DoD, NASA, and the Coast Guard only.** An order may be placed on a sole-source basis when the order would otherwise be placed using **other than full and open competition** procedures — i.e., when circumstances warranting a sole-source determination exist beyond those covered by exceptions (A)–(E).
+---
+## Documentation Requirements
+| Order Value | Documentation Required |
+|---|---|
+| ≤ $7M (civilian) / ≤ $15M (DoD) | Written D&amp;F signed by contracting officer |
+| &gt; $7M (civilian) / &gt; $15M (DoD) | J&amp;A approved at higher level (see FAR 16.505(b)(2)(ii)) |
+---
+## Key Distinctions
+- **Fair opportunity ≠ Full and Open Competition.** Fair opportunity is a FAR Part 16 ordering procedure, not a FAR Part 6 competition requirement. Exceptions here are governed by 16.505, not 6.302.
+- **Exception (F)** is structurally distinct — it authorizes narrowing competition *to* a set-aside pool, not eliminating competition entirely.
+- **Exception (G)** is agency-limited (DoD/NASA/Coast Guard); civilian agencies (including NIH/HHS) do **not** have access to this exception.
+**Source:** FAR 16.505(b)(2)(i)(A)–(G) | *FAR Part 16 IDIQ Comprehensive Guidance (HHS Class Deviation 2026-01, effective November 21, 2025)*
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_16_IDIQ_Comprehensive_RFO_2025.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR12" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS12" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT12" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 lists all 7 FAR 16.505(b)(2)(i) exceptions with full citation format (A-G), verbatim statutory text, documentation threshold table ($7M civilian / $15M DoD), and key distinctions section (fair opp vs full &amp; open, Exception F structural note, Exception G agency limitation).
+v11 vs v12: V12 uses search_far (same as V11). Slightly longer (3,511 vs 3,430 V11) with expanded descriptions per exception.
+Tools: v11=[search_far, knowledge_fetch] | v12=[search_far]
+KB docs cited: V11=1 | V12=1 (maintained)
+Verdict: Stable -- verbatim FAR text with approval thresholds.</t>
         </is>
       </c>
     </row>
@@ -9149,6 +12889,547 @@
 Verdict: Exceptional -- transparent KB inventory + comprehensive analysis.</t>
         </is>
       </c>
+      <c r="AY13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excellent — all six core documents fully fetched. Here is the complete analysis:
+---
+## Knowledge Base Documents Found — Protest Guidance Inventory
+Below are **all relevant KB documents** identified, with their file paths:
+| # | Title | KB File Path |
+|---|-------|-------------|
+| 1 | **GAO Bid Protests – Essential Guide for Contracting Officers** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt` |
+| 2 | **FAR Companion Part 33: Protests, Disputes, and Appeals** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt` |
+| 3 | **NIH Manual 6033-2: Stay Provisions for Protests** (Reference Version) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt` |
+| 4 | **NIH Policy Manual 6033-2: Stay Provisions for Protests** (Policy Version, 2008) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt` |
+| 5 | **NIH Manual 6033-1: CO's Statement of Facts and Circumstances in GAO Protests** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt` |
+| 6 | **GAO Decision B-419956.258: Optimo IT – EPDS Filing Timeliness** (NIH CIO-SP4 case) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt` |
+| 7 | **GAO Decision B-409917.11: Gella LLC – Failure to Rebut Agency Arguments** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-409917_Failure_to_Rebut_Agency_Arguments.txt` |
+| 8 | **ACQuipedia – Protests, Integrity, and Ethics** | `eagle-knowledge-base/approved/legal-counselor/ethics-integrity/ACQuipedia_Protests_Integrity_Ethics.txt` |
+| 9 | **FAR Part 15 Negotiation – RFO 2025** (debriefing requirements at FAR 15.505/506) | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Negotiation_RFO_2025.txt` |
+| 10 | **ACQuipedia Source Selection and Evaluation Guide** (debriefing + protest context) | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/ACQuipedia_Source_Selection_Evaluation.txt` |
+---
+## Analysis: GAO Protest Process for an Eliminated SBIR Phase II Offeror
+### ⚠️ Threshold Issue: SBIR Jurisdiction at GAO
+This is the **first question to answer**, and it is dispositive. GAO's jurisdiction under 4 C.F.R. § 21.5 has important carve-outs. SBIR Phase II competitions are procurements conducted under the Small Business Innovation Research program — GAO **does** generally have jurisdiction over SBIR Phase II awards as procurement actions, because they result in contracts for services or R&amp;D. However, the offeror must verify the award was made under a competitive solicitation subject to CICA and FAR Part 33, not an agency-internal program funding decision. Assuming standard SBIR Phase II competitive evaluation, GAO jurisdiction attaches.
+---
+### 1. Interested Party Standing — 4 C.F.R. § 21.0(a)
+The offeror must be an **actual or prospective offeror with a direct economic interest** in the procurement. For a Phase II elimination, this means the offeror must show it would be **next in line for award** if the protest is sustained. If only one award was planned and the protester was eliminated from competition (not merely ranked lower), it must demonstrate it would be a viable awardee upon a re-evaluation or resolicitation. This is a threshold standing requirement GAO will assess immediately.
+---
+### 2. Debriefing — The Critical First Step
+**Before filing at GAO**, the eliminated offeror should request a debriefing. This is strategically and procedurally important:
+#### Pre-Award (FAR 15.505)
+- If eliminated from the competitive range, the offeror may request a **preaward debriefing**
+- Must request it within **3 days** of receipt of notice of exclusion
+- Agency may delay debriefing until after award, but must provide it
+#### Post-Award (FAR 15.506)
+- If eliminated at award stage, the offeror may request a **postaward debriefing**
+- Must request within **3 days** of notification of award
+- Agency must debrief within **5 days** of the request
+- Debriefing must include: evaluation ratings, strengths/weaknesses, overall ranking, and a summary of the rationale for award
+#### Why This Matters for the Protest Clock
+Per 4 C.F.R. § 21.2 and FAR Companion FC 33.105-3:
+&gt; *"The initial protest shall NOT be filed before the debriefing date offered, and shall be filed not later than 10 days after the date on which the debriefing was held."*
+The **CICA stay** provisions also tie to the debriefing date: the automatic stay triggers if GAO receives protest notice within **10 calendar days after award OR 5 calendar days after the debriefing date offered, whichever is later.** This means requesting a debriefing can actually **extend the protest window** and the stay trigger period.
+---
+### 3. Timeliness — The #1 Reason for Dismissal
+Timeliness is strictly enforced. GAO has zero tolerance (see *Optimo IT, B-419956.258* — 10 minutes late = dismissed).
+| Scenario | Deadline |
+|----------|----------|
+| Solicitation defects apparent before proposals due | Before closing date |
+| All other grounds (including award/evaluation challenges) | **10 calendar days** after basis known or should have been known |
+| With required debriefing | **10 calendar days** after debriefing held |
+| After adverse agency-level protest decision | **10 calendar days** after knowledge of adverse action |
+**Calendar days** are used. The day the basis becomes known is **not counted**. If day 10 falls on a weekend/federal holiday, it rolls to the next business day.
+**Practical trap:** If the offeror learns the basis for protest from the debriefing, the 10-day clock runs from the **debriefing date**, not the award date. The offeror cannot sit on known grounds and wait.
+---
+### 4. Filing Requirements — EPDS (4 C.F.R. § 21.1)
+All protests must be filed in GAO's **Electronic Protest Docketing System (EPDS)** at `epds.gao.gov`. Per *Optimo IT (B-419956.258)* — an NIH case — email to protests@gao.gov is **not a valid filing** unless EPDS is confirmed system-wide unavailable after contacting GAO.
+**Deadline:** Filed (received in EPDS) by **5:30 PM Eastern Time** on the deadline day.
+**Minimum content required:**
+1. Name, address, phone, email of protester or representative
+2. Electronic signature
+3. Agency name, solicitation/contract number
+4. **Detailed statement of legal AND factual grounds** (copies of relevant documents)
+5. Statement establishing interested party status
+6. Statement establishing timeliness
+7. Specific request for Comptroller General ruling
+8. Form of relief requested
+**Same day (within 1 business day):** Complete copy must be furnished to the CO or location designated in the solicitation.
+Optional but advisable:
+- Request for **protective order** (especially to access awardee's proposal)
+- Request for specific documents (with relevance explanation)
+- Request for hearing
+---
+### 5. The Automatic Stay — CICA Suspension
+Once GAO receives the protest and notifies the agency, **CICA automatically suspends** award or performance if notice is received within:
+- **10 calendar days** after contract award, **OR**
+- **5 calendar days** after the debriefing date offered to the protester (whichever is later)
+This stay is powerful — NIH **cannot proceed with award or continue performance** without a formal override.
+#### NIH's Stay Override Procedure (NIH Manual 6033-2)
+If NIH wants to override the CICA stay, the process is extremely burdensome:
+| Step | Who | Action |
+|------|-----|--------|
+| 1 | CO | Prepares signed Determination &amp; Findings (D&amp;F) |
+| 2 | IC Director, Office of Acquisitions | Reviews and forwards |
+| 3 | NIH Protest Control Officer (PCO), DAPE/OAMP | Reviews and routes |
+| 4 | Head of Contracting Activity (HCA) | **Executes** (non-delegable) |
+| 5 | OGC – General Law Division | Concurrence; forwards to HHS |
+| 6 | DASAMP, OS, DHHS | **Final approval** (non-delegable) |
+**Pre-award override** requires: (a) urgent and compelling circumstances + (b) award likely within 30 calendar days.
+**Post-award override** requires: (a) performance in **best interests of the United States**, OR (b) urgent and compelling circumstances.
+Because this chain runs to the HHS Deputy Assistant Secretary level, NIH cannot quickly override the stay — which gives the protester significant leverage in a meritorious case.
+---
+### 6. Agency Report — 30-Day Response (4 C.F.R. § 21.3 / NIH Manual 6033-1)
+Once GAO notifies NIH of the protest:
+| Deadline | Requirement |
+|----------|-------------|
+| **5 calendar days** | CO delivers complete protest file (all docs except CO Statement) to OGC-GLD (4 copies) and NIH PCO (1 copy), marked "Immediate Action – GAO Protest B-[number]" |
+| **14 calendar days** | CO's Statement of Facts and Circumstances due |
+| **30 calendar days** | OGC-GLD submits complete Agency Report to GAO |
+The CO's Statement must include:
+- **Section 1:** Background and contract value estimate
+- **Section 2:** Chronology of events (AP date, SAM.gov posting, solicitation, proposals, competitive range, negotiations, source selection, debriefing, protest receipt)
+- **Section 3:** Response to each allegation individually, with rationale
+- **Section 4:** Summary of recommendations
+**Litigation Hold:** Immediately upon receipt of protest, NIH must preserve **all** relevant records including emails. Litigation hold overrides any retention/disposal schedule.
+---
+### 7. Protester's Comments — 10 Days After Agency Report
+The protester receives the agency report and has **10 calendar days** to file written comments in EPDS. **Failure to file = mandatory dismissal** (no discretion). Per *Gella LLC (B-409917.11)*: failure to **substantively rebut** agency arguments on specific grounds = those grounds deemed **abandoned**. Generic disagreement is insufficient.
+---
+### 8. GAO Decision Timeline
+| Track | Timeline |
+|-------|----------|
+| Standard | Decision within **100 days** of filing |
+| Express Option | Decision within **65 days** (request within 5 days of filing; agency report due 20 days; comments due 5 days) |
+**Three possible outcomes:**
+1. **Dismiss** — procedural or substantive defect
+2. **Deny** — no violation, or violation did not prejudice protester
+3. **Sustain** — violation found and prejudiced protester
+If sustained, GAO may recommend: terminate contract, recompete, issue new solicitation, award to protester, or other corrective action. GAO also typically recommends **reimbursement of protest costs** (filing fees, reasonable attorneys' fees) — with costs capped by statute except for small businesses.
+---
+### 9. Alternative Venues
+| Venue | Notes |
+|-------|-------|
+| **Agency-level protest** | Must be filed before or simultaneously with GAO; provides inexpensive, informal resolution; if adverse, 10-day clock runs to file at GAO |
+| **U.S. Court of Federal Claims (COFC)** | More expensive; handles pre-award protests; temporary restraining order/preliminary injunction must be sought |
+| **ADR** | GAO offers negotiation assistance and outcome prediction; FAR 33.214 |
+---
+### 10. Key Risk Flags for the SBIR Phase II Protester
+1. **SBIR-specific evaluation criteria** — Phase II awards often involve both technical merit and commercialization potential; protester should clearly identify which evaluation criterion was misapplied
+2. **Interested party standing** — If multiple firms competed and were not eliminated, protester must show it would be next in line for award
+3. **Timeliness trap** — If any protest ground was apparent from the solicitation or pre-award notice, that ground must be filed before or at the debriefing, not 10 days later
+4. **Protective order** — Should be requested immediately if the awardee's proposal is needed to substantiate disparate evaluation claims
+5. **EPDS filing** — File early; never rely on email as a substitute; build in technical buffer time per *Optimo IT*
+---
+**Sources:**
+- `GAO_Bid_Protests_Essential_Guide_for_COs.txt` — GAO-18-510SP, 4 C.F.R. Part 21
+- `NIH_6033_1_GAO_Protest_CO_Statement.txt` — NIH Manual Chapter 6033-1 (8/21/2008)
+- `NIH_6033_2_Stay_Provisions_Protests.txt` / `NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt` — NIH Manual Chapter 6033-2, FAR 33.103–33.104, HHSAR 333.104
+- `FC_33_Protests_Disputes_Appeals.txt` — FAR Companion Part 33 (v2.0, Oct 2025)
+- `GAO_B-419956.258_EPDS_Filing_Timeliness.txt` — *Optimo Information Technology, LLC*, B-419956.258 (June 21, 2023)
+- `GAO_B-409917_Failure_to_Rebut_Agency_Arguments.txt` — *Gella LLC*, B-409917.11
+- `ACQuipedia_Protests_Integrity_Ethics.txt` — DAU ACQuipedia (2024/2025)
+</t>
+        </is>
+      </c>
+      <c r="AZ13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BA13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD13" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BE13" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &gt; RO (improved)
+RO comparison: V10 provides KB document inventory (10 docs with full S3 paths), then comprehensive protest analysis covering jurisdiction, standing, debriefing, timeliness, filing, automatic stay, agency report, GAO timeline, alternative venues, and SBIR-specific risk flags. 20 document references total.
+v9 vs v10: V10 inventories 10 KB docs (V9 had 11). Quality maintained.
+Tools: v9=[knowledge_search, knowledge_fetch] | v10=[knowledge_search, knowledge_fetch]
+KB docs cited: V9=11 | V10=20 (+9 improvement, broader coverage)
+Verdict: Exceptional -- most thoroughly documented response in suite.</t>
+        </is>
+      </c>
+      <c r="BF13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excellent. I now have full content from all five core protest guidance documents. Here is the complete analysis:
+---
+## Knowledge Base Documents Found — Protest Guidance
+Before the analysis, here is every relevant document identified across all KB searches, with full file paths:
+---
+### 🗂️ Primary Protest Guidance Documents
+| # | Title | KB File Path |
+|---|-------|-------------|
+| 1 | **GAO Bid Protests – Essential Guide for Contracting Officers** (GAO-18-510SP, 10th Ed.) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt` |
+| 2 | **NIH Manual 6033-2: Stay Provisions for Protests** (2008, updated) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt` |
+| 3 | **NIH Policy Manual 6033-2: Stay Provisions for Protests** (2008 original version) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt` |
+| 4 | **NIH Manual 6033-1: CO's Statement of Facts and Circumstances in GAO Protests** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt` |
+| 5 | **FAR Companion Part 33: Protests, Disputes, and Appeals** (v2.0, Oct. 30, 2025) | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt` |
+| 6 | **ACQuipedia – Protests, Integrity, and Ethics** (DAU 2024/2025) | `eagle-knowledge-base/approved/legal-counselor/ethics-integrity/ACQuipedia_Protests_Integrity_Ethics.txt` |
+| 7 | **GAO Decision B-419831: Alpine Companies – Interested Party Status &amp; PIA** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419831_PIA_Allegations_Interested_Party.txt` |
+### 📋 Debriefing Requirements Documents
+| # | Title | KB File Path |
+|---|-------|-------------|
+| 8 | **FAR Part 15 – Contracting by Negotiation (RFO 2025/FAR 2.0)** *(§§ 15.206, 15.301 debriefing rules)* | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Source_Selection_RFO_2025.txt` |
+| 9 | **FAR Part 15 – Negotiation (RFO 2025)** *(debriefing + competitive range)* | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Negotiation_RFO_2025.txt` |
+| 10 | **FAR Companion Part 15: Negotiation and Source Selection Guidance** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_15_Negotiation_Source_Selection.txt` |
+| 11 | **ACQuipedia Source Selection and Evaluation Guide** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/ACQuipedia_Source_Selection_Evaluation.txt` |
+### 📌 Supporting SBIR/Small Business Documents
+| # | Title | KB File Path |
+|---|-------|-------------|
+| 12 | **ACQuipedia – Market Research and Small Business Programs** *(SBIR/STTR programs)* | `eagle-knowledge-base/approved/market-intelligence/market-research-guides/ACQuipedia_Market_Research_Small_Business.txt` |
+| 13 | **FAR Part 19 – Small Business Programs (RFO 2025)** | `eagle-knowledge-base/approved/market-intelligence/small-business/FAR_Part_19_Small_Business_RFO_2025.txt` |
+---
+## Analysis: SBIR Phase II Protest at GAO
+### ⚠️ CRITICAL THRESHOLD ISSUE: GAO Jurisdiction Over SBIR
+This is the most important issue to flag **before** anything else. The KB documents — particularly the GAO Essential Guide (4 C.F.R. § 21.5) and the ACQuipedia Protests guide — identify the boundaries of GAO jurisdiction. **SBIR Phase II awards involve a significant jurisdictional wrinkle:**
+- **SBIR Phase II competitions are negotiated procurements** (FAR Part 15 applies to competitive procedures). GAO **does** have jurisdiction to review whether the agency followed its stated evaluation criteria, complied with the SBIR solicitation, and acted consistent with applicable statutes and regulations.
+- However, **SBIR program decisions** — such as an agency's determination of technical merit under SBA's SBIR program policy directives — may be reviewable only to the extent they reflect compliance with the *solicitation's* evaluation criteria. GAO does not second-guess technical judgments where the agency has followed its stated methodology.
+- **SBA size standard challenges** (was the protester actually a small business?) go to **SBA, not GAO** (4 C.F.R. § 21.5(b)).
+- **Affirmative responsibility determinations** are generally not reviewed by GAO unless definitive responsibility criteria were not applied.
+**Bottom line:** The offeror can protest evaluation methodology, solicitation compliance, and procedural irregularities. It cannot protest purely technical merit judgments or SBA-jurisdictional matters.
+---
+### Step 1 — Interested Party Status (4 C.F.R. § 21.0(a))
+Per the GAO Essential Guide, the protester must be an **actual or prospective offeror with a direct economic interest** — i.e., a firm that would be in line for award if the protest were sustained. An offeror *eliminated* from Phase II competition qualifies **if** it can show it would have a reasonable prospect of award had the agency acted properly. This was reinforced in **GAO B-419831 (Alpine Companies)**: a firm whose own proposal was technically unacceptable lacked interested party status. The eliminated SBIR offeror must confirm its proposal was not itself fatally deficient independent of the challenged agency action.
+---
+### Step 2 — Timeliness (4 C.F.R. § 21.2) — Strictly Enforced
+This is the **most common reason for dismissal**. All deadlines are in **calendar days**.
+| Protest Basis | Deadline |
+|---------------|----------|
+| Solicitation impropriety apparent before proposals due | **Before** closing date for proposals |
+| All other grounds (e.g., evaluation errors) | **10 calendar days** after basis known or should have been known |
+| Basis arising from/before debriefing | **NOT before debriefing date offered**; then **10 days after debriefing held** |
+| Agency-level protest already filed → GAO | **10 days** after adverse agency action |
+**Strategic note from FC Part 33:** Agencies should offer debriefings promptly — doing so starts the 10-day clock and limits the protest window. For the offeror, *requesting a debriefing* is both a right and a strategic necessity — protest grounds discovered at debriefing must be filed within 10 days of the debriefing date.
+---
+### Step 3 — Debriefing Rights (FAR 15.206 / FAR 15.301 — RFO 2025)
+The eliminated SBIR offeror has the following debriefing rights:
+**Preaward Debriefing (FAR 15.206-2):**
+- Available if excluded from competitive range
+- Must **request within 3 days** of receiving exclusion notice
+- Minimum content: agency's evaluation of significant elements, summary of rationale for elimination, responses to questions about whether solicitation procedures were followed
+- **Cannot disclose:** number/identity of other offerors, content of other proposals, ranking of others
+**Postaward Debriefing (FAR 15.301-1):**
+- Available after award notice (within 3 days of award notice receipt)
+- Must be provided within **5 days** of written request to maximum extent practicable
+- Minimum content: significant weaknesses/deficiencies, overall evaluated cost/price and technical rating of awardee vs. protester, past performance info, overall ranking (if developed), rationale for award
+- **Key protest timing rule:** The protest deadline is **not extended** when the government accommodates an untimely request or delays a preaward debriefing
+**FC Part 33 best practice:** The agency should use the debriefing as an opportunity to provide transparency — furnishing technical evaluation documentation relevant to the requesting vendor may *reduce* protest likelihood by resolving information gaps before a formal protest is filed.
+---
+### Step 4 — Filing at GAO (4 C.F.R. § 21.1)
+**Where:** GAO's **Electronic Protest Docketing System (EPDS)** at `epds.gao.gov` — mandatory except for classified protests.
+**Required contents of the protest:**
+1. Protester's name, address, email, phone/fax
+2. Electronic signature of protester or representative
+3. Agency name and solicitation/contract number
+4. **Detailed statement of legal and factual grounds** (with supporting documents) — this is routinely the basis for dismissal if inadequate
+5. Information establishing interested party status
+6. Information establishing timeliness
+7. Specific request for a ruling by the Comptroller General
+8. Form of relief requested
+**Copy to agency:** Complete copy must reach the CO (or designated location) **no later than 1 day** after filing with GAO.
+**Optional but strategic:** Request for protective order (needed to access awardee's proprietary proposal data through counsel), request for specific documents, request for hearing.
+---
+### Step 5 — The Agency Report &amp; NIH Response Process
+Per **NIH Manual 6033-1**, once NIH receives notice of a GAO protest:
+| NIH Internal Deadline | Action |
+|----------------------|--------|
+| **5 calendar days** from receipt of protest | All documentation (except CO Statement) due to OGC-GLD (4 copies) and NIH PCO (1 copy) |
+| **14 calendar days** | CO's Statement of Facts and Circumstances due |
+| **30 calendar days** | OGC-GLD submits complete Agency Report to GAO |
+**Document routing:** CO → CO Supervisor → Director, IC Office of Acquisitions → NIH PCO (DAPE/OAMP, 301-496-6014) → OGC-GLD (Departmental PCO, 202-619-0150).
+**Litigation hold** is triggered immediately upon receipt of the protest — all relevant records (including email) must be preserved. This overrides normal retention schedules.
+The CO's statement must address: (1) Background, (2) Chronology of Events, (3) Individual responses to each allegation, (4) Summary of recommendations.
+---
+### Step 6 — GAO Decision Timeline
+| Milestone | Timeframe |
+|-----------|-----------|
+| Agency report due | 30 days after GAO notice |
+| Protester comments on report | 10 days after report filed (failure = **dismissal of protest ground**) |
+| GAO decision — standard | **100 calendar days** from filing |
+| GAO decision — express option | **65 calendar days** (request within 5 days of filing; agency report due in 20 days) |
+**Three possible outcomes:** Dismiss (procedural/substantive defect), Deny (no violation, or violation didn't prejudice protester), or **Sustain** (agency violated statute/regulation and protester was prejudiced).
+If **sustained**, GAO may recommend: terminate contract, recompete, reissue solicitation, make new award — plus reimbursement of protest costs (filing, attorneys' fees, consultants).
+---
+### Step 7 — NIH Stay Provisions (NIH Manual 6033-2 / FAR 33.104)
+If a GAO protest is filed, a **statutory stay** is automatically triggered when the protest is received by GAO within:
+- **10 calendar days** after contract award, **OR**
+- **5 calendar days** after the debriefing date offered
+- *Whichever is later*
+**To override the stay and proceed with award or performance**, NIH must:
+| Protest Stage | Standard | Approval Chain |
+|---------------|----------|----------------|
+| **Pre-award (GAO protest)** | Urgent &amp; compelling circumstances + award likely within 30 days | CO prepares D&amp;F → IC Director → NIH PCO → HCA → **DASAMP (HHS)** |
+| **Post-award (GAO protest)** | Performance in best interest of US *or* urgent &amp; compelling | Same chain — HCA executes, DASAMP approves |
+| **Pre-award (agency protest)** | Urgent &amp; compelling *or* best interest | CO with PCO + OGC-GLD concurrence |
+| **Post-award (agency protest)** | Urgent &amp; compelling *or* best interest | HCA approval |
+**Critical:** HCA authority for GAO protest stay overrides is **not delegable**. It must go to the HHS Deputy Assistant Secretary for Acquisition Management and Policy (DASAMP). This typically takes several days — urgency must be documented thoroughly in the acquisition record.
+---
+### Step 8 — Alternative Venues &amp; Strategic Considerations
+The KB identifies **three protest venues** (ACQuipedia):
+1. **GAO** — fastest, least expensive, 100-day decision, automatic stay
+2. **Agency-level protest** — cheapest, informal, but no automatic stay in same way; if filed first and timely, subsequent GAO protest must be filed within 10 days of adverse agency action
+3. **U.S. Court of Federal Claims (COFC)** — more expensive, pre-award only, requires complaint + motion for preliminary injunction
+**GAO ADR options (FC Part 33 / 4 C.F.R. § 21.10):** Negotiation assistance and outcome prediction are available. ADR may resolve the protest without a written decision — favorable when the agency wants to avoid a formal ruling while correcting a genuine error.
+---
+### Summary Checklist for the Eliminated SBIR Phase II Offeror
+- [ ] **Confirm interested party status** — would you be in line for award if protest sustained?
+- [ ] **Identify the precise basis** — evaluation error, solicitation noncompliance, procedural defect? (Not SBA size or purely technical merit)
+- [ ] **Request a debriefing immediately** — within 3 days of exclusion/award notice; grounds discovered at debriefing must be protested within 10 days of debriefing
+- [ ] **File within 10 days** — calendar days, strictly enforced; day of knowledge does not count
+- [ ] **File in EPDS** — `epds.gao.gov`; include detailed factual and legal statement
+- [ ] **Serve the agency** — complete copy to CO within 1 day of filing
+- [ ] **Request protective order** if you need access to awardee's proprietary proposal data (requires attorney)
+- [ ] **Comment on agency report** within 10 days — failure to comment = dismissal of that ground
+- [ ] **Be aware of the stay** — automatic if filed within the CICA window; NIH must obtain HCA + DASAMP approval to override
+---
+*Sources: All analysis drawn directly from full-text content of KB documents listed above. FAR citations reflect FAR 2.0/RFO 2025 version implemented via HHS class deviation.*
+</t>
+        </is>
+      </c>
+      <c r="BG13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BJ13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK13" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BL13" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &gt; RO (improved)
+RO comparison: V11 provides comprehensive protest analysis with KB document inventory (7+ primary docs with full S3 paths), debriefing analysis, protest timeline, automatic stay provisions, agency report requirements, and SBIR-specific risk flags. 13,860 chars -- second deepest response in suite.
+v10 vs v11: V11 longer (13,860 vs 12,789 chars). Both use knowledge_search + knowledge_fetch. V11 adds more document citations.
+Tools: v10=[knowledge_search, knowledge_fetch] | v11=[knowledge_search, knowledge_fetch]
+KB docs cited: V10=20 | V11=20+ (maintained)
+Verdict: Exceptional -- most thoroughly documented protest response maintained.</t>
+        </is>
+      </c>
+      <c r="BM13" s="20" t="inlineStr">
+        <is>
+          <t>ERROR: All connection attempts failed</t>
+        </is>
+      </c>
+      <c r="BN13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excellent — the KB returned a comprehensive set of documents. Here is the full inventory followed by a structured analysis.
+---
+## 📚 Knowledge Base Documents Found — Protest Guidance
+### Core Protest Procedure Documents
+| # | Title | S3 Path |
+|---|-------|---------|
+| 1 | **GAO Bid Protests - Essential Guide for Contracting Officers** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_Bid_Protests_Essential_Guide_for_COs.txt` |
+| 2 | **FAR Companion Part 33: Protests, Disputes, and Appeals** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/FC_33_Protests_Disputes_Appeals.txt` |
+| 3 | **NIH Manual 6033-2: Stay Provisions for Protests** *(Detailed)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_2_Stay_Provisions_Protests.txt` |
+| 4 | **NIH Policy Manual 6033-2: Stay Provisions for Protests** *(Policy version)* | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_Policy_6033_2_Protest_Stay_Provisions_2008.txt` |
+| 5 | **NIH Manual 6033-1: CO's Statement of Facts and Circumstances in GAO Protests** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/NIH_6033_1_GAO_Protest_CO_Statement.txt` |
+### GAO Case Law — Protest Precedents
+| # | Title | S3 Path |
+|---|-------|---------|
+| 6 | **GAO B-409917.11: Gella LLC - Failure to Rebut Agency Arguments** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-409917_Failure_to_Rebut_Agency_Arguments.txt` |
+| 7 | **GAO B-419956.258: EPDS Filing Timeliness and Protest Procedures** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419956.258_EPDS_Filing_Timeliness.txt` |
+| 8 | **GAO B-419831: Alpine Companies - PIA Allegations &amp; Interested Party Status** | `eagle-knowledge-base/approved/legal-counselor/protest-guidance/GAO_B-419831_PIA_Allegations_Interested_Party.txt` |
+| 9 | **GAO B-421835: Vertex Aerospace - Past Performance Evaluation Blending** | `eagle-knowledge-base/approved/legal-counselor/case-law/evaluation/GAO_B-421835_Past_Performance_Evaluation_Blending.txt` |
+| 10 | **GAO B-423546: SPRS Past Performance, Contract Admin vs. Protest Jurisdiction** | `eagle-knowledge-base/approved/legal-counselor/case-law/past-performance/GAO_B-423546_SPRS_Past_Performance_Contract_Admin.txt` |
+### Source Selection / Debriefing Documents
+| # | Title | S3 Path |
+|---|-------|---------|
+| 11 | **FAR Part 15 - Contracting by Negotiation (RFO 2025)** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FAR_Part_15_Negotiation_RFO_2025.txt` |
+| 12 | **FAR Companion Part 15: Negotiation and Source Selection Guidance** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/FC_15_Negotiation_Source_Selection.txt` |
+| 13 | **ACQuipedia: Source Selection and Evaluation Guide** | `eagle-knowledge-base/approved/compliance-strategist/FAR-guidance/ACQuipedia_Source_Selection_Evaluation.txt` |
+| 14 | **ACQuipedia: Protests, Integrity, and Ethics** | `eagle-knowledge-base/approved/legal-counselor/ethics-integrity/ACQuipedia_Protests_Integrity_Ethics.txt` |
+### NIH SBIR/R&amp;D-Specific Documents
+| # | Title | S3 Path |
+|---|-------|---------|
+| 15 | **NIH Policy 6035: Broad Agency Announcements** *(excludes SBIR by name)* | `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Policy_6035_Broad_Agency_Announcements_2016.txt` |
+| 16 | **NIH Manual 6315-1 (Part 1): R&amp;D Contracts - Core Policy &amp; Presolicitation** | `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_6315_1_RD_Contracts_Part1_Presolicitation.txt` |
+| 17 | **NIH Manual 6315-1 (Part 3): R&amp;D Contracts - Definitions, Controls, Process Flow** | `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_6315_1_RD_Contracts_Part3_Definitions_Controls.txt` |
+| 18 | **NIH CIO-SP3 Proposal Compliance Guide** *(Phase elimination/protest lessons)* | `eagle-knowledge-base/approved/supervisor-core/core-procedures/NIH_CIO-SP3_Proposal_Compliance_Guide.txt` |
+---
+## ⚠️ SBIR-Specific Protest Jurisdiction — Critical Threshold Issue
+Before analyzing the standard protest process, there is a **critical threshold question** for a SBIR Phase II competitor: **GAO's jurisdiction is limited for SBIR competitions.**
+### The SBIR Protest Jurisdiction Problem
+The Small Business Innovation Research (SBIR) program operates under a **statutory framework distinct from standard FAR Part 15 competitions**. Under **15 U.S.C. § 638** and SBA's SBIR Policy Directive, the competitive selection of SBIR awardees involves:
+1. **Peer review / technical scoring** (not traditional source selection)
+2. **Agency discretion** in final selection based on technical merit and program relevance
+3. Selections based on scientific/technical evaluation, not purely FAR-based procedures
+GAO generally **does not review the merits** of SBIR award decisions involving scientific/technical judgments — it treats those as matters committed to agency discretion. However, GAO **will** review protests alleging:
+- Violation of statute or regulation in conducting the competition
+- Arbitrary application of stated evaluation criteria
+- Procedural errors (improper evaluation of eligibility requirements, etc.)
+**Bottom line for the offeror:** The merits of the technical evaluation are likely unreviewable at GAO. The protest must be grounded in a **procedural, regulatory, or eligibility violation**.
+---
+## 📋 The GAO Protest Process — Step by Step
+Assuming a viable protest ground exists, here is the full process drawn from the KB documents:
+---
+### STEP 1 — Request a Debriefing First (Critical Timing Anchor)
+**Authority: FAR 15.206-2 (preaward) / FAR 15.301 (postaward)**
+| Scenario | Timing | Action |
+|----------|--------|--------|
+| Eliminated from competitive range | Request preaward debriefing **within 3 days** of exclusion notice | FAR 15.206-1 |
+| Award made to another firm | Request postaward debriefing **within 3 days** of award notice | FAR 15.301 |
+| Agency must hold debriefing | **Within 5 days** of request | FAR 15.301 |
+**Why this matters for timeliness:** Under **4 C.F.R. § 21.2**, the 10-day protest clock does **not begin** until the debriefing is held. The FC 33 guidance is explicit:
+&gt; *"The automatic stay of performance at GAO is 10 days after contract award OR within 5 days of debriefing date offered — whichever is later."*
+The debriefing is both a protest-prevention mechanism and a clock-management tool. **Request it immediately.**
+**Required content of the debriefing (FAR 15.301-1(c)):**
+- Government's evaluation of offeror's significant weaknesses/deficiencies
+- Overall evaluated cost/price and technical rating of awardee AND debriefed offeror
+- Summary of rationale for award
+- Responses to questions about whether procedures were followed
+**May NOT disclose:** Point-by-point comparisons, trade secrets, other offerors' cost breakdowns, names of past performance references.
+---
+### STEP 2 — File at GAO Within 10 Days
+**Authority: 4 C.F.R. § 21.2 | GAO-18-510SP**
+**Deadline:** Not later than **10 calendar days** after the basis of the protest is known or should have been known — or 10 days after the debriefing is held (whichever applies).
+⚠️ **GAO strictly enforces this.** GAO B-419956.258 confirms a **10-minute late filing is untimely with no exceptions** unless EPDS suffers a system-wide failure during business hours.
+**Filing method:** GAO's **Electronic Protest Docketing System (EPDS)** at `epds.gao.gov` — exceptions only for classified information. Email to `protests@gao.gov` is **not valid** when EPDS is functioning.
+**Required filing elements (4 C.F.R. § 21.1(c)):**
+1. Protester name, address, email, phone/fax
+2. Electronic signature
+3. Agency name and solicitation/contract number
+4. **Detailed statement of legal AND factual grounds** (with supporting documents)
+5. Information establishing interested party status
+6. Information establishing timeliness
+7. Request for ruling by Comptroller General
+8. Form of relief requested
+**Copy to agency:** Complete protest must be furnished to the CO (or designated protest recipient) **no later than 1 day after** filing with GAO.
+---
+### STEP 3 — Interested Party Status
+**Authority: 4 C.F.R. § 21.0(a)**
+The offeror must be an **actual or prospective bidder or offeror with a direct economic interest** — meaning they would be in line for award if the protest were sustained.
+⚠️ **GAO B-419831 (Alpine Companies)** is the controlling KB case: an offeror whose own proposal was technically unacceptable **lacked interested party status** even when alleging procurement integrity violations. For SBIR Phase II, the protester must establish they were a qualified offeror who would have received award but for the alleged impropriety.
+---
+### STEP 4 — The Automatic Stay (CICA)
+**Authority: 31 U.S.C. § 3553 | FAR 33.104(b)-(c) | NIH Manual 6033-2**
+This is where NIH-specific procedures become critical:
+**When the automatic stay applies:**
+- GAO receives notice of protest within **10 calendar days** after contract award, OR
+- Within **5 calendar days** after the debriefing date offered — whichever is **later**
+**Effect:**
+- **Pre-award protest:** Award must be suspended pending GAO decision
+- **Post-award protest:** Contract performance must be suspended pending GAO decision
+**Override — the "notwithstanding" determination:**
+NIH may proceed with award or continue performance notwithstanding the stay, but **only** through a formal Determination &amp; Findings (D&amp;F) process:
+| Scenario | Legal Standard | Approval Chain |
+|----------|---------------|----------------|
+| Pre-award (GAO protest) | Urgent &amp; compelling circumstances + award likely within 30 days | CO → IC Director → NIH PCO → **HCA** → **DASAMP, OS, DHHS** |
+| Post-award (GAO protest) | Best interests of U.S. OR urgent &amp; compelling | Same chain — **HCA authority is NOT redelegable** |
+| Agency protest (pre-award) | Urgent &amp; compelling OR best interest | CO + PCO concurrence + **OGC-GLD concurrence** |
+| Agency protest (post-award) | Urgent &amp; compelling OR best interest | CO → PCO → **HCA approval** |
+The D&amp;F routing goes: **CO → IC Director, Office of Acquisitions → NIH PCO → HCA → DASAMP (via OGC-GLD)**. OGC-GLD notifies GAO if approved.
+---
+### STEP 5 — Agency Report (30 Days)
+**Authority: 4 C.F.R. § 21.3 | NIH Manual 6033-1**
+NIH's internal deadlines under Manual 6033-1:
+| Deadline | Action |
+|----------|--------|
+| **5 calendar days** from receipt of protest | Protest file (all documents except CO Statement) due to OGC-GLD (4 copies) and NIH PCO (1 copy) |
+| **14 calendar days** from receipt of protest | CO's Statement of Facts and Circumstances due |
+| **30 calendar days** from receipt of protest | OGC-GLD submits complete Agency Report to GAO |
+**Litigation hold is immediate:** Upon receipt of protest, ALL relevant records must be retained — this overrides all normal retention schedules.
+**CO's Statement must contain (4 sections per Manual 6033-1 Appendix 2):**
+1. **Background** — acquisition purpose, history, estimated value
+2. **Chronology of Events** — AP date, posting, proposals received, award date, debriefing dates
+3. **Statement of Issues, Findings &amp; Circumstances** — respond individually to EACH allegation
+4. **Summary of Recommendations and Conclusions**
+---
+### STEP 6 — Protester's Comments (10 Days After Agency Report)
+**Authority: 4 C.F.R. § 21.3(i)**
+The protester has **10 days** after the agency report is filed to submit written comments.
+**From GAO B-409917.11 (Gella LLC):** Failure to **substantively rebut** agency arguments results in those grounds being **deemed abandoned**. Generic disagreement without engaging specific agency arguments provides no basis for GAO to question agency reasonableness. The protester must address each agency argument specifically.
+**Failure to file comments at all = dismissal of protest.**
+---
+### STEP 7 — GAO Decision
+**Authority: 4 C.F.R. § 21.9**
+| Track | Timeline |
+|-------|----------|
+| Standard | Decision within **100 days** of filing |
+| Express option | Decision within **65 days** (request within 5 days of filing; agency report due in 20 days; comments due in 5 days) |
+**Three outcomes:**
+1. **Dismiss** — procedural/substantive defect
+2. **Deny** — agency did not violate statute/regulation, or violation did not prejudice protester
+3. **Sustain** — agency violated statute/regulation and protester was prejudiced
+**If sustained, GAO may recommend:**
+- Recompete the procurement
+- Terminate the contract
+- Issue a new solicitation
+- Reimburse protest costs (filing fees, reasonable attorneys' fees, consultant fees)
+---
+## 🔍 SBIR Phase II — Most Likely Viable Protest Grounds
+Given the SBIR context, the offeror should focus on:
+| Ground | Basis | KB Support |
+|--------|-------|-----------|
+| **Improper peer review** | Conflict of interest on SRG, failure to follow 42 CFR 52h | NIH 6315-1, Parts 1 &amp; 3 |
+| **Evaluation inconsistency** | Applied unstated criteria, deviated from RFP Section M factors | FC 33, FAR Part 15 |
+| **Improper past performance evaluation** | Blending of ratings without qualitative relevancy analysis | GAO B-421835 (Vertex) |
+| **Failure to conduct required debriefing** | Agency failed to provide required content under FAR 15.301 | FAR Part 15 RFO 2025 |
+| **Competitive range error** | Improper exclusion without adequate notice | FAR 15.206-1 |
+| **Procurement integrity violation** | Must be reported to agency within **14 days** of discovering possible violation — failure bars GAO review | GAO B-419831, ACQuipedia |
+---
+## ⏱️ Critical Timeline Summary
+```
+Day 0:  Award notice received
+Day 1:  Request debriefing (within 3 days — do not wait)
+Day 3:  Debriefing held (agency must hold within 5 days of request)
+Day 13: LAST DAY to file at GAO (10 days after debriefing)
+         → Also last day for automatic CICA stay to apply
+Day 14: Agency notified of protest (within 1 day of GAO filing)
+Day 5*: Protest file due to OGC-GLD and NIH PCO (*NIH internal — from receipt)
+Day 14*: CO Statement due (*NIH internal — from receipt)
+Day 30*: Agency Report submitted to GAO (*from GAO notification)
+Day 40:  Protester comments due (10 days after agency report)
+Day 100: GAO decision deadline (standard track)
+```
+---
+**One critical advisory:** If the SBIR elimination was based purely on **scientific/technical merit scoring**, that ground is almost certainly unreviewable at GAO. The protest needs to be grounded in a specific **procedural or regulatory violation**. Recommend consulting OGC-GLD before filing to assess viability — a losing protest extends uncertainty and may not be in the government's or the offeror's interest.
+**Sources:**
+- `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_6307_3_Special_Clearance_Procedures.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/NIH-policies/NIH_Policy_6307_3_Special_Clearance_Procedures_2014.txt`
+- `eagle-knowledge-base/approved/compliance-strategist/regulatory-policies/EO_14275_Restoring_Common_Sense_Federal_Procurement.txt`
+- `eagle-knowledge-base/approved/financial-advisor/cost-analysis-guides/NIH_6015_1_Financial_Analysis_Proposals.txt`
+</t>
+        </is>
+      </c>
+      <c r="BO13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BP13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR13" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS13" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT13" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &gt; RO (improved)
+RO comparison: V12 provides comprehensive protest analysis (15,242 chars) with KB document inventory (18 docs with full S3 paths), SBIR jurisdiction analysis, 7-step procedural walkthrough, NIH approval chain table, SBIR-specific protest vulnerabilities table, and critical timeline. Uses research tool alone.
+v11 vs v12: V12 longer (15,242 vs 13,860 V11 chars). Uses research instead of knowledge_search + knowledge_fetch -- simpler tool surface, same depth.
+Tools: v11=[knowledge_search, knowledge_fetch] | v12=[research]
+KB docs cited: V11=20+ | V12=18 (direct listing with S3 paths)
+Verdict: Exceptional -- tool simplification delivers same depth with fewer calls.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="409.5" customHeight="1">
       <c r="A14" s="20" t="n">
@@ -9240,6 +13521,107 @@
 Verdict: Document generated correctly but chat response too terse. User must navigate to document card. create_document should echo key sections back.</t>
         </is>
       </c>
+      <c r="AY14" s="20" t="inlineStr">
+        <is>
+          <t>Generated a draft sow document. You can open it from the document card.
+**Template:** Using template: Statement of Work (SOW) Template - Eagle v2 (eagle-knowledge-base/approved/supervisor-core/essential-templates/statement-of-work-template-eagle-v2.docx)</t>
+        </is>
+      </c>
+      <c r="AZ14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BA14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BC14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD14" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="BE14" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V10 &lt; RO (regression)
+RO comparison: RO provides context about the generated SOW including key sections, HHSAR security checklist mapping, and template selection rationale. V10 returns only 255 chars saying 'Generated a draft sow document.' Same regression as V9.
+v9 vs v10: No change. Both produce terse chat response.
+Tools: v9=[create_document] | v10=[create_document]
+KB docs cited: V10=1 (template path only)
+Source gap: RO reads HHSAR_CD_2024_01_OAMS_Security_Checklist_Guide -- V10 does not.
+Verdict: Document generated but chat response too terse. Needs echo-back.</t>
+        </is>
+      </c>
+      <c r="BF14" s="20" t="inlineStr">
+        <is>
+          <t>Generated a draft sow document. You can open it from the document card.
+**Template:** Using template: Statement of Work (SOW) Template - Eagle v2 (eagle-knowledge-base/approved/supervisor-core/essential-templates/statement-of-work-template-eagle-v2.docx)</t>
+        </is>
+      </c>
+      <c r="BG14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BH14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK14" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="BL14" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V11 &lt; RO (regression)
+RO comparison: RO provides context about the generated SOW including key sections, HHSAR security checklist mapping, and template selection rationale. V11 returns only 255 chars saying 'Generated a draft sow document.' Same regression as V9 and V10.
+v10 vs v11: No change. Both produce terse chat response after create_document.
+Tools: v10=[create_document] | v11=[create_document]
+KB docs cited: V11=1 (template path only)
+Source gap: RO reads HHSAR_CD_2024_01_OAMS_Security_Checklist_Guide -- V11 does not.
+Verdict: Document generated but chat response too terse. Needs echo-back. Persistent regression across V9/V10/V11.</t>
+        </is>
+      </c>
+      <c r="BM14" s="20" t="inlineStr">
+        <is>
+          <t>ERROR: All connection attempts failed</t>
+        </is>
+      </c>
+      <c r="BN14" s="20" t="inlineStr">
+        <is>
+          <t>Generated a draft sow document. You can open it from the document card.
+**Template:** Using template: Statement of Work (SOW) Template - Eagle v2 (eagle-knowledge-base/approved/supervisor-core/essential-templates/statement-of-work-template-eagle-v2.docx)</t>
+        </is>
+      </c>
+      <c r="BO14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BP14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="BR14" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BS14" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="BT14" s="20" t="inlineStr">
+        <is>
+          <t>EAGLE V12 &lt; RO (regression)
+RO comparison: RO provides context about the generated SOW including key sections, HHSAR security checklist mapping, and template selection rationale. V12 returns only 255 chars saying 'Generated a draft sow document.' Same regression as V9/V10/V11.
+v11 vs v12: No change. Both produce terse chat response after create_document.
+Tools: v11=[create_document] | v12=[create_document]
+KB docs cited: V12=1 (template path only)
+Source gap: RO reads HHSAR_CD_2024_01_OAMS_Security_Checklist_Guide -- V12 does not.
+Verdict: Document generated but chat response too terse. Persistent regression.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>